<commit_message>
Actualizacion automatica dashboard lun 27/07/2026 20:47:29,81
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -652,19 +652,19 @@
         <v>62.16238270093839</v>
       </c>
       <c r="T2" t="n">
-        <v>11814</v>
+        <v>11833</v>
       </c>
       <c r="U2" t="n">
-        <v>13.56018283392585</v>
+        <v>13.54686047494296</v>
       </c>
       <c r="V2" t="n">
-        <v>65.38852209243271</v>
+        <v>65.36803853629681</v>
       </c>
       <c r="W2" t="n">
-        <v>-7.231330833964806</v>
+        <v>-7.244653192947702</v>
       </c>
       <c r="X2" t="n">
-        <v>-3.598531211750306</v>
+        <v>-3.443492452060384</v>
       </c>
     </row>
     <row r="3">
@@ -804,19 +804,19 @@
         <v>39.73451327433628</v>
       </c>
       <c r="T4" t="n">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="U4" t="n">
-        <v>0.1060445387062566</v>
+        <v>0.1053740779768177</v>
       </c>
       <c r="V4" t="n">
-        <v>33.19194061505832</v>
+        <v>33.2982086406744</v>
       </c>
       <c r="W4" t="n">
-        <v>-23.52227404536454</v>
+        <v>-23.52294450609398</v>
       </c>
       <c r="X4" t="n">
-        <v>-16.54867256637168</v>
+        <v>-16.01769911504425</v>
       </c>
     </row>
     <row r="5">
@@ -880,19 +880,19 @@
         <v>56.85258964143426</v>
       </c>
       <c r="T5" t="n">
-        <v>2085</v>
+        <v>2093</v>
       </c>
       <c r="U5" t="n">
-        <v>38.99280575539568</v>
+        <v>38.84376493072146</v>
       </c>
       <c r="V5" t="n">
-        <v>53.04556354916067</v>
+        <v>52.98614429049212</v>
       </c>
       <c r="W5" t="n">
-        <v>-6.8637679497836</v>
+        <v>-7.012808774457824</v>
       </c>
       <c r="X5" t="n">
-        <v>-16.93227091633466</v>
+        <v>-16.61354581673307</v>
       </c>
     </row>
     <row r="6">
@@ -956,19 +956,19 @@
         <v>60.76099053978854</v>
       </c>
       <c r="T6" t="n">
-        <v>24810</v>
+        <v>24828</v>
       </c>
       <c r="U6" t="n">
-        <v>58.62152357920194</v>
+        <v>58.65152247462543</v>
       </c>
       <c r="V6" t="n">
-        <v>63.25272067714631</v>
+        <v>63.27936201063316</v>
       </c>
       <c r="W6" t="n">
-        <v>0.7994590271707835</v>
+        <v>0.8294579225942726</v>
       </c>
       <c r="X6" t="n">
-        <v>-13.71035058430718</v>
+        <v>-13.64774624373957</v>
       </c>
     </row>
     <row r="7">
@@ -1032,19 +1032,19 @@
         <v>61.65678803274061</v>
       </c>
       <c r="T7" t="n">
-        <v>26958</v>
+        <v>27032</v>
       </c>
       <c r="U7" t="n">
-        <v>36.28607463461681</v>
+        <v>36.23113347144125</v>
       </c>
       <c r="V7" t="n">
-        <v>61.89628310705542</v>
+        <v>61.84522047943178</v>
       </c>
       <c r="W7" t="n">
-        <v>-10.03060614438404</v>
+        <v>-10.08554730755959</v>
       </c>
       <c r="X7" t="n">
-        <v>-4.889923793395427</v>
+        <v>-4.62884561106407</v>
       </c>
     </row>
     <row r="8">
@@ -1108,19 +1108,19 @@
         <v>45.21468784135787</v>
       </c>
       <c r="T8" t="n">
-        <v>11154</v>
+        <v>11183</v>
       </c>
       <c r="U8" t="n">
-        <v>36.50708266092882</v>
+        <v>36.41241169632478</v>
       </c>
       <c r="V8" t="n">
-        <v>53.25443786982249</v>
+        <v>53.11633729768398</v>
       </c>
       <c r="W8" t="n">
-        <v>0.8042005501818181</v>
+        <v>0.7095295855777835</v>
       </c>
       <c r="X8" t="n">
-        <v>-6.27678346357449</v>
+        <v>-6.033106461641879</v>
       </c>
     </row>
     <row r="9">
@@ -1260,19 +1260,19 @@
         <v>33.59223300970874</v>
       </c>
       <c r="T10" t="n">
-        <v>1798</v>
+        <v>1804</v>
       </c>
       <c r="U10" t="n">
-        <v>2.780867630700778</v>
+        <v>2.771618625277162</v>
       </c>
       <c r="V10" t="n">
-        <v>36.26251390433816</v>
+        <v>36.30820399113082</v>
       </c>
       <c r="W10" t="n">
-        <v>-8.481268291629316</v>
+        <v>-8.490517297052934</v>
       </c>
       <c r="X10" t="n">
-        <v>74.5631067961165</v>
+        <v>75.14563106796116</v>
       </c>
     </row>
     <row r="11">
@@ -1336,19 +1336,19 @@
         <v>74.40353659771201</v>
       </c>
       <c r="T11" t="n">
-        <v>81490</v>
+        <v>81630</v>
       </c>
       <c r="U11" t="n">
-        <v>67.52730396367652</v>
+        <v>67.49356854097758</v>
       </c>
       <c r="V11" t="n">
-        <v>73.65934470487177</v>
+        <v>73.63714320715424</v>
       </c>
       <c r="W11" t="n">
-        <v>-4.299150777096727</v>
+        <v>-4.332886199795666</v>
       </c>
       <c r="X11" t="n">
-        <v>-8.334176987367686</v>
+        <v>-8.176694900955015</v>
       </c>
     </row>
     <row r="12">
@@ -1412,19 +1412,19 @@
         <v>75.20695379142226</v>
       </c>
       <c r="T12" t="n">
-        <v>297851</v>
+        <v>298142</v>
       </c>
       <c r="U12" t="n">
-        <v>56.99527616157071</v>
+        <v>57.00941162264961</v>
       </c>
       <c r="V12" t="n">
-        <v>74.65108393122736</v>
+        <v>74.65704261727633</v>
       </c>
       <c r="W12" t="n">
-        <v>-5.033609150561325</v>
+        <v>-5.019473689482432</v>
       </c>
       <c r="X12" t="n">
-        <v>7.249053899805198</v>
+        <v>7.353836071712775</v>
       </c>
     </row>
     <row r="13">
@@ -1488,19 +1488,19 @@
         <v>60.68562662261034</v>
       </c>
       <c r="T13" t="n">
-        <v>51823</v>
+        <v>51873</v>
       </c>
       <c r="U13" t="n">
-        <v>27.55147328406306</v>
+        <v>27.56347232664392</v>
       </c>
       <c r="V13" t="n">
-        <v>60.28018447407521</v>
+        <v>60.28762554700904</v>
       </c>
       <c r="W13" t="n">
-        <v>0.3978268361045991</v>
+        <v>0.4098258786854565</v>
       </c>
       <c r="X13" t="n">
-        <v>1.925497600503501</v>
+        <v>2.023837620958225</v>
       </c>
     </row>
     <row r="14">
@@ -1564,19 +1564,19 @@
         <v>62.77658116310946</v>
       </c>
       <c r="T14" t="n">
-        <v>5578</v>
+        <v>5581</v>
       </c>
       <c r="U14" t="n">
-        <v>33.70383650053783</v>
+        <v>33.7394732126859</v>
       </c>
       <c r="V14" t="n">
-        <v>59.59125134456794</v>
+        <v>59.61297258555815</v>
       </c>
       <c r="W14" t="n">
-        <v>-3.421677499853793</v>
+        <v>-3.386040787705717</v>
       </c>
       <c r="X14" t="n">
-        <v>9.222635598198552</v>
+        <v>9.281378500097905</v>
       </c>
     </row>
     <row r="15">
@@ -1640,19 +1640,19 @@
         <v>81.03823437985702</v>
       </c>
       <c r="T15" t="n">
-        <v>14355</v>
+        <v>14367</v>
       </c>
       <c r="U15" t="n">
-        <v>59.7352838732149</v>
+        <v>59.76891487436487</v>
       </c>
       <c r="V15" t="n">
-        <v>74.24590734935562</v>
+        <v>74.26741838936451</v>
       </c>
       <c r="W15" t="n">
-        <v>-10.98277643141675</v>
+        <v>-10.94914543026678</v>
       </c>
       <c r="X15" t="n">
-        <v>-10.75536213863848</v>
+        <v>-10.68075847062481</v>
       </c>
     </row>
   </sheetData>
@@ -1742,19 +1742,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11814</v>
+        <v>11833</v>
       </c>
       <c r="C4" t="n">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="D4" t="n">
-        <v>13.56018283392585</v>
+        <v>13.54686047494296</v>
       </c>
       <c r="E4" t="n">
-        <v>7725</v>
+        <v>7735</v>
       </c>
       <c r="F4" t="n">
-        <v>65.38852209243271</v>
+        <v>65.36803853629681</v>
       </c>
     </row>
     <row r="5">
@@ -1786,19 +1786,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1060445387062566</v>
+        <v>0.1053740779768177</v>
       </c>
       <c r="E6" t="n">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F6" t="n">
-        <v>33.19194061505832</v>
+        <v>33.2982086406744</v>
       </c>
     </row>
     <row r="7">
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2085</v>
+        <v>2093</v>
       </c>
       <c r="C7" t="n">
         <v>813</v>
       </c>
       <c r="D7" t="n">
-        <v>38.99280575539568</v>
+        <v>38.84376493072146</v>
       </c>
       <c r="E7" t="n">
-        <v>1106</v>
+        <v>1109</v>
       </c>
       <c r="F7" t="n">
-        <v>53.04556354916067</v>
+        <v>52.98614429049212</v>
       </c>
     </row>
     <row r="8">
@@ -1830,19 +1830,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24810</v>
+        <v>24828</v>
       </c>
       <c r="C8" t="n">
-        <v>14544</v>
+        <v>14562</v>
       </c>
       <c r="D8" t="n">
-        <v>58.62152357920194</v>
+        <v>58.65152247462543</v>
       </c>
       <c r="E8" t="n">
-        <v>15693</v>
+        <v>15711</v>
       </c>
       <c r="F8" t="n">
-        <v>63.25272067714631</v>
+        <v>63.27936201063316</v>
       </c>
     </row>
     <row r="9">
@@ -1852,19 +1852,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>26958</v>
+        <v>27032</v>
       </c>
       <c r="C9" t="n">
-        <v>9782</v>
+        <v>9794</v>
       </c>
       <c r="D9" t="n">
-        <v>36.28607463461681</v>
+        <v>36.23113347144125</v>
       </c>
       <c r="E9" t="n">
-        <v>16686</v>
+        <v>16718</v>
       </c>
       <c r="F9" t="n">
-        <v>61.89628310705542</v>
+        <v>61.84522047943178</v>
       </c>
     </row>
     <row r="10">
@@ -1874,19 +1874,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11154</v>
+        <v>11183</v>
       </c>
       <c r="C10" t="n">
         <v>4072</v>
       </c>
       <c r="D10" t="n">
-        <v>36.50708266092882</v>
+        <v>36.41241169632478</v>
       </c>
       <c r="E10" t="n">
         <v>5940</v>
       </c>
       <c r="F10" t="n">
-        <v>53.25443786982249</v>
+        <v>53.11633729768398</v>
       </c>
     </row>
     <row r="11">
@@ -1918,19 +1918,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1798</v>
+        <v>1804</v>
       </c>
       <c r="C12" t="n">
         <v>50</v>
       </c>
       <c r="D12" t="n">
-        <v>2.780867630700778</v>
+        <v>2.771618625277162</v>
       </c>
       <c r="E12" t="n">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="F12" t="n">
-        <v>36.26251390433816</v>
+        <v>36.30820399113082</v>
       </c>
     </row>
     <row r="13">
@@ -1940,19 +1940,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>81490</v>
+        <v>81630</v>
       </c>
       <c r="C13" t="n">
-        <v>55028</v>
+        <v>55095</v>
       </c>
       <c r="D13" t="n">
-        <v>67.52730396367652</v>
+        <v>67.49356854097758</v>
       </c>
       <c r="E13" t="n">
-        <v>60025</v>
+        <v>60110</v>
       </c>
       <c r="F13" t="n">
-        <v>73.65934470487177</v>
+        <v>73.63714320715424</v>
       </c>
     </row>
     <row r="14">
@@ -1962,19 +1962,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>297851</v>
+        <v>298142</v>
       </c>
       <c r="C14" t="n">
-        <v>169761</v>
+        <v>169969</v>
       </c>
       <c r="D14" t="n">
-        <v>56.99527616157071</v>
+        <v>57.00941162264961</v>
       </c>
       <c r="E14" t="n">
-        <v>222349</v>
+        <v>222584</v>
       </c>
       <c r="F14" t="n">
-        <v>74.65108393122736</v>
+        <v>74.65704261727633</v>
       </c>
     </row>
     <row r="15">
@@ -1984,19 +1984,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>51823</v>
+        <v>51873</v>
       </c>
       <c r="C15" t="n">
-        <v>14278</v>
+        <v>14298</v>
       </c>
       <c r="D15" t="n">
-        <v>27.55147328406306</v>
+        <v>27.56347232664392</v>
       </c>
       <c r="E15" t="n">
-        <v>31239</v>
+        <v>31273</v>
       </c>
       <c r="F15" t="n">
-        <v>60.28018447407521</v>
+        <v>60.28762554700904</v>
       </c>
     </row>
     <row r="16">
@@ -2006,19 +2006,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5578</v>
+        <v>5581</v>
       </c>
       <c r="C16" t="n">
-        <v>1880</v>
+        <v>1883</v>
       </c>
       <c r="D16" t="n">
-        <v>33.70383650053783</v>
+        <v>33.7394732126859</v>
       </c>
       <c r="E16" t="n">
-        <v>3324</v>
+        <v>3327</v>
       </c>
       <c r="F16" t="n">
-        <v>59.59125134456794</v>
+        <v>59.61297258555815</v>
       </c>
     </row>
     <row r="17">
@@ -2028,19 +2028,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>14355</v>
+        <v>14367</v>
       </c>
       <c r="C17" t="n">
-        <v>8575</v>
+        <v>8587</v>
       </c>
       <c r="D17" t="n">
-        <v>59.7352838732149</v>
+        <v>59.76891487436487</v>
       </c>
       <c r="E17" t="n">
-        <v>10658</v>
+        <v>10670</v>
       </c>
       <c r="F17" t="n">
-        <v>74.24590734935562</v>
+        <v>74.26741838936451</v>
       </c>
     </row>
     <row r="18"/>
@@ -2141,19 +2141,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="D22" t="n">
-        <v>15.56577195172701</v>
+        <v>15.55606155125806</v>
       </c>
       <c r="E22" t="n">
-        <v>8.175000000000001</v>
+        <v>8.166666666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2594295325287835</v>
+        <v>0.2592676925209676</v>
       </c>
       <c r="G22" t="n">
-        <v>0.13625</v>
+        <v>0.1361111111111111</v>
       </c>
       <c r="H22" t="n">
         <v>267.2242802303263</v>
@@ -2192,40 +2192,40 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10212</v>
+        <v>10230</v>
       </c>
       <c r="D23" t="n">
-        <v>241.3881919963442</v>
+        <v>241.1290795047247</v>
       </c>
       <c r="E23" t="n">
-        <v>72.99166666666667</v>
+        <v>72.88333333333333</v>
       </c>
       <c r="F23" t="n">
-        <v>4.023136533272402</v>
+        <v>4.018817991745411</v>
       </c>
       <c r="G23" t="n">
-        <v>1.216527777777778</v>
+        <v>1.214722222222222</v>
       </c>
       <c r="H23" t="n">
-        <v>256.1652396176774</v>
+        <v>255.9123212979586</v>
       </c>
       <c r="I23" t="n">
-        <v>89.36666666666666</v>
+        <v>89.2</v>
       </c>
       <c r="J23" t="n">
-        <v>4.269420660294623</v>
+        <v>4.265205354965977</v>
       </c>
       <c r="K23" t="n">
-        <v>1.489444444444444</v>
+        <v>1.486666666666667</v>
       </c>
       <c r="L23" t="n">
-        <v>14.38749458820395</v>
+        <v>14.37771627102866</v>
       </c>
       <c r="M23" t="n">
         <v>6.2</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2397915764700659</v>
+        <v>0.2396286045171444</v>
       </c>
       <c r="O23" t="n">
         <v>0.1033333333333333</v>
@@ -2372,22 +2372,22 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="D27" t="n">
-        <v>647.171797593772</v>
+        <v>643.6988396624473</v>
       </c>
       <c r="E27" t="n">
-        <v>109.675</v>
+        <v>109.6</v>
       </c>
       <c r="F27" t="n">
-        <v>10.78619662656287</v>
+        <v>10.72831399437412</v>
       </c>
       <c r="G27" t="n">
-        <v>1.827916666666667</v>
+        <v>1.826666666666667</v>
       </c>
       <c r="H27" t="n">
-        <v>5140.077918781725</v>
+        <v>5140.077918781726</v>
       </c>
       <c r="I27" t="n">
         <v>4559.65</v>
@@ -2474,22 +2474,22 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1272</v>
+        <v>1280</v>
       </c>
       <c r="D29" t="n">
-        <v>247.2197196016772</v>
+        <v>246.0678776041667</v>
       </c>
       <c r="E29" t="n">
-        <v>72.18333333333334</v>
+        <v>71.95833333333334</v>
       </c>
       <c r="F29" t="n">
-        <v>4.120328660027952</v>
+        <v>4.101131293402778</v>
       </c>
       <c r="G29" t="n">
-        <v>1.203055555555556</v>
+        <v>1.199305555555556</v>
       </c>
       <c r="H29" t="n">
-        <v>996.4106321839082</v>
+        <v>996.410632183908</v>
       </c>
       <c r="I29" t="n">
         <v>928.5333333333333</v>
@@ -2525,43 +2525,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>14544</v>
+        <v>14562</v>
       </c>
       <c r="D30" t="n">
-        <v>25.0593016593326</v>
+        <v>25.0723126402051</v>
       </c>
       <c r="E30" t="n">
-        <v>29.96666666666667</v>
+        <v>30.35833333333333</v>
       </c>
       <c r="F30" t="n">
-        <v>0.4176550276555433</v>
+        <v>0.4178718773367516</v>
       </c>
       <c r="G30" t="n">
-        <v>0.4994444444444444</v>
+        <v>0.5059722222222223</v>
       </c>
       <c r="H30" t="n">
-        <v>407.3452705775352</v>
+        <v>406.4914607948443</v>
       </c>
       <c r="I30" t="n">
-        <v>236.4333333333333</v>
+        <v>234.6666666666667</v>
       </c>
       <c r="J30" t="n">
-        <v>6.789087842958921</v>
+        <v>6.774857679914071</v>
       </c>
       <c r="K30" t="n">
-        <v>3.940555555555556</v>
+        <v>3.911111111111111</v>
       </c>
       <c r="L30" t="n">
-        <v>382.0105035781814</v>
+        <v>381.1289676572383</v>
       </c>
       <c r="M30" t="n">
-        <v>209.0333333333333</v>
+        <v>206.85</v>
       </c>
       <c r="N30" t="n">
-        <v>6.366841726303024</v>
+        <v>6.352149460953973</v>
       </c>
       <c r="O30" t="n">
-        <v>3.483888888888889</v>
+        <v>3.4475</v>
       </c>
     </row>
     <row r="31">
@@ -2627,43 +2627,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9782</v>
+        <v>9794</v>
       </c>
       <c r="D32" t="n">
-        <v>335.9100678116268</v>
+        <v>335.534854672929</v>
       </c>
       <c r="E32" t="n">
         <v>35.16666666666666</v>
       </c>
       <c r="F32" t="n">
-        <v>5.598501130193781</v>
+        <v>5.59224757788215</v>
       </c>
       <c r="G32" t="n">
         <v>0.586111111111111</v>
       </c>
       <c r="H32" t="n">
-        <v>671.2512349656358</v>
+        <v>670.5325289575288</v>
       </c>
       <c r="I32" t="n">
-        <v>408.0166666666667</v>
+        <v>407.125</v>
       </c>
       <c r="J32" t="n">
-        <v>11.18752058276059</v>
+        <v>11.17554214929215</v>
       </c>
       <c r="K32" t="n">
-        <v>6.800277777777778</v>
+        <v>6.785416666666666</v>
       </c>
       <c r="L32" t="n">
-        <v>252.6233848797251</v>
+        <v>252.3976662376662</v>
       </c>
       <c r="M32" t="n">
-        <v>71.375</v>
+        <v>71.38333333333334</v>
       </c>
       <c r="N32" t="n">
-        <v>4.210389747995419</v>
+        <v>4.206627770627771</v>
       </c>
       <c r="O32" t="n">
-        <v>1.189583333333333</v>
+        <v>1.189722222222222</v>
       </c>
     </row>
     <row r="33">
@@ -2678,43 +2678,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>17176</v>
+        <v>17238</v>
       </c>
       <c r="D33" t="n">
-        <v>397.3392310976557</v>
+        <v>396.0638376455119</v>
       </c>
       <c r="E33" t="n">
-        <v>76.31666666666666</v>
+        <v>75.86666666666666</v>
       </c>
       <c r="F33" t="n">
-        <v>6.622320518294261</v>
+        <v>6.601063960758531</v>
       </c>
       <c r="G33" t="n">
-        <v>1.271944444444444</v>
+        <v>1.264444444444444</v>
       </c>
       <c r="H33" t="n">
-        <v>683.2241667190414</v>
+        <v>682.3947678795482</v>
       </c>
       <c r="I33" t="n">
-        <v>418.4333333333333</v>
+        <v>415.375</v>
       </c>
       <c r="J33" t="n">
-        <v>11.38706944531735</v>
+        <v>11.37324613132581</v>
       </c>
       <c r="K33" t="n">
-        <v>6.973888888888889</v>
+        <v>6.922916666666667</v>
       </c>
       <c r="L33" t="n">
-        <v>265.2057098862422</v>
+        <v>265.075495608532</v>
       </c>
       <c r="M33" t="n">
-        <v>61.45</v>
+        <v>61.54166666666666</v>
       </c>
       <c r="N33" t="n">
-        <v>4.420095164770703</v>
+        <v>4.417924926808866</v>
       </c>
       <c r="O33" t="n">
-        <v>1.024166666666667</v>
+        <v>1.025694444444444</v>
       </c>
     </row>
     <row r="34">
@@ -2780,19 +2780,19 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7082</v>
+        <v>7111</v>
       </c>
       <c r="D35" t="n">
-        <v>1355.628633625153</v>
+        <v>1350.259972812075</v>
       </c>
       <c r="E35" t="n">
-        <v>1098.558333333333</v>
+        <v>1096.266666666667</v>
       </c>
       <c r="F35" t="n">
-        <v>22.59381056041921</v>
+        <v>22.50433288020125</v>
       </c>
       <c r="G35" t="n">
-        <v>18.30930555555555</v>
+        <v>18.27111111111111</v>
       </c>
       <c r="H35" t="n">
         <v>2042.850454861669</v>
@@ -2807,7 +2807,7 @@
         <v>28.30166666666667</v>
       </c>
       <c r="L35" t="n">
-        <v>655.5163001016749</v>
+        <v>655.516300101675</v>
       </c>
       <c r="M35" t="n">
         <v>502.9</v>
@@ -2984,16 +2984,16 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1748</v>
+        <v>1754</v>
       </c>
       <c r="D39" t="n">
-        <v>175.2134630053394</v>
+        <v>174.8544469783352</v>
       </c>
       <c r="E39" t="n">
         <v>78.14166666666667</v>
       </c>
       <c r="F39" t="n">
-        <v>2.920224383422324</v>
+        <v>2.914240782972254</v>
       </c>
       <c r="G39" t="n">
         <v>1.302361111111111</v>
@@ -3011,7 +3011,7 @@
         <v>7.153333333333333</v>
       </c>
       <c r="L39" t="n">
-        <v>325.2852533650039</v>
+        <v>325.285253365004</v>
       </c>
       <c r="M39" t="n">
         <v>159.2583333333333</v>
@@ -3035,43 +3035,43 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>55028</v>
+        <v>55095</v>
       </c>
       <c r="D40" t="n">
-        <v>456.9012396719246</v>
+        <v>456.4585546177814</v>
       </c>
       <c r="E40" t="n">
-        <v>46.15833333333333</v>
+        <v>46.16666666666666</v>
       </c>
       <c r="F40" t="n">
-        <v>7.615020661198744</v>
+        <v>7.607642576963023</v>
       </c>
       <c r="G40" t="n">
-        <v>0.7693055555555555</v>
+        <v>0.7694444444444444</v>
       </c>
       <c r="H40" t="n">
-        <v>570.9486520624024</v>
+        <v>570.2220280258701</v>
       </c>
       <c r="I40" t="n">
-        <v>194.6666666666667</v>
+        <v>192.7583333333333</v>
       </c>
       <c r="J40" t="n">
-        <v>9.515810867706707</v>
+        <v>9.503700467097833</v>
       </c>
       <c r="K40" t="n">
-        <v>3.244444444444444</v>
+        <v>3.212638888888889</v>
       </c>
       <c r="L40" t="n">
-        <v>91.05161598241317</v>
+        <v>91.06445308489889</v>
       </c>
       <c r="M40" t="n">
-        <v>47.88333333333333</v>
+        <v>47.725</v>
       </c>
       <c r="N40" t="n">
-        <v>1.517526933040219</v>
+        <v>1.517740884748315</v>
       </c>
       <c r="O40" t="n">
-        <v>0.7980555555555555</v>
+        <v>0.7954166666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3086,43 +3086,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>26462</v>
+        <v>26535</v>
       </c>
       <c r="D41" t="n">
-        <v>765.5217135263144</v>
+        <v>763.8958614408642</v>
       </c>
       <c r="E41" t="n">
-        <v>703.2166666666667</v>
+        <v>701.2333333333333</v>
       </c>
       <c r="F41" t="n">
-        <v>12.75869522543858</v>
+        <v>12.73159769068107</v>
       </c>
       <c r="G41" t="n">
-        <v>11.72027777777778</v>
+        <v>11.68722222222222</v>
       </c>
       <c r="H41" t="n">
-        <v>883.1373427357962</v>
+        <v>880.1673776679158</v>
       </c>
       <c r="I41" t="n">
-        <v>830.9333333333334</v>
+        <v>824.2333333333333</v>
       </c>
       <c r="J41" t="n">
-        <v>14.71895571226327</v>
+        <v>14.66945629446526</v>
       </c>
       <c r="K41" t="n">
-        <v>13.84888888888889</v>
+        <v>13.73722222222222</v>
       </c>
       <c r="L41" t="n">
-        <v>110.6807944012608</v>
+        <v>110.5557258857614</v>
       </c>
       <c r="M41" t="n">
-        <v>88.33333333333333</v>
+        <v>88.08333333333333</v>
       </c>
       <c r="N41" t="n">
-        <v>1.84467990668768</v>
+        <v>1.842595431429356</v>
       </c>
       <c r="O41" t="n">
-        <v>1.472222222222222</v>
+        <v>1.468055555555555</v>
       </c>
     </row>
     <row r="42">
@@ -3137,43 +3137,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>169761</v>
+        <v>169969</v>
       </c>
       <c r="D42" t="n">
-        <v>9.439170657571529</v>
+        <v>9.46689827752904</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0.1573195109595255</v>
+        <v>0.1577816379588173</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>457.5126901732752</v>
+        <v>457.3888882150799</v>
       </c>
       <c r="I42" t="n">
-        <v>181.8</v>
+        <v>181.7166666666667</v>
       </c>
       <c r="J42" t="n">
-        <v>7.625211502887921</v>
+        <v>7.623148136917997</v>
       </c>
       <c r="K42" t="n">
-        <v>3.03</v>
+        <v>3.028611111111111</v>
       </c>
       <c r="L42" t="n">
-        <v>447.5398902920001</v>
+        <v>447.3871237338005</v>
       </c>
       <c r="M42" t="n">
-        <v>173.4833333333333</v>
+        <v>173.3666666666667</v>
       </c>
       <c r="N42" t="n">
-        <v>7.458998171533334</v>
+        <v>7.456452062230009</v>
       </c>
       <c r="O42" t="n">
-        <v>2.891388888888889</v>
+        <v>2.889444444444444</v>
       </c>
     </row>
     <row r="43">
@@ -3188,43 +3188,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>128090</v>
+        <v>128173</v>
       </c>
       <c r="D43" t="n">
-        <v>158.8924631118744</v>
+        <v>158.8526204166764</v>
       </c>
       <c r="E43" t="n">
-        <v>90.16666666666667</v>
+        <v>90.18333333333334</v>
       </c>
       <c r="F43" t="n">
-        <v>2.648207718531242</v>
+        <v>2.647543673611274</v>
       </c>
       <c r="G43" t="n">
-        <v>1.502777777777778</v>
+        <v>1.503055555555556</v>
       </c>
       <c r="H43" t="n">
-        <v>564.7490247153886</v>
+        <v>564.5380232836731</v>
       </c>
       <c r="I43" t="n">
-        <v>268.6166666666667</v>
+        <v>268.3166666666667</v>
       </c>
       <c r="J43" t="n">
-        <v>9.412483745256477</v>
+        <v>9.408967054727885</v>
       </c>
       <c r="K43" t="n">
-        <v>4.476944444444444</v>
+        <v>4.471944444444444</v>
       </c>
       <c r="L43" t="n">
-        <v>404.8180747295646</v>
+        <v>404.7194923168235</v>
       </c>
       <c r="M43" t="n">
-        <v>124.8166666666667</v>
+        <v>124.7666666666667</v>
       </c>
       <c r="N43" t="n">
-        <v>6.746967912159413</v>
+        <v>6.74532487194706</v>
       </c>
       <c r="O43" t="n">
-        <v>2.080277777777778</v>
+        <v>2.079444444444444</v>
       </c>
     </row>
     <row r="44">
@@ -3239,16 +3239,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>14278</v>
+        <v>14298</v>
       </c>
       <c r="D44" t="n">
-        <v>22.87138488116917</v>
+        <v>22.88172704807199</v>
       </c>
       <c r="E44" t="n">
         <v>15.76666666666667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.381189748019486</v>
+        <v>0.3813621174678665</v>
       </c>
       <c r="G44" t="n">
         <v>0.2627777777777778</v>
@@ -3290,43 +3290,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>37545</v>
+        <v>37575</v>
       </c>
       <c r="D45" t="n">
-        <v>276.0242531184801</v>
+        <v>275.8161281880683</v>
       </c>
       <c r="E45" t="n">
-        <v>30.13333333333333</v>
+        <v>30.08333333333333</v>
       </c>
       <c r="F45" t="n">
-        <v>4.600404218641335</v>
+        <v>4.596935469801139</v>
       </c>
       <c r="G45" t="n">
-        <v>0.5022222222222222</v>
+        <v>0.5013888888888889</v>
       </c>
       <c r="H45" t="n">
-        <v>1157.121097672075</v>
+        <v>1158.280942173817</v>
       </c>
       <c r="I45" t="n">
-        <v>964.2416666666667</v>
+        <v>966.9166666666666</v>
       </c>
       <c r="J45" t="n">
-        <v>19.28535162786791</v>
+        <v>19.30468236956361</v>
       </c>
       <c r="K45" t="n">
-        <v>16.07069444444444</v>
+        <v>16.11527777777778</v>
       </c>
       <c r="L45" t="n">
-        <v>883.1915799267313</v>
+        <v>882.1988717666482</v>
       </c>
       <c r="M45" t="n">
-        <v>626.4749999999999</v>
+        <v>623.2166666666667</v>
       </c>
       <c r="N45" t="n">
-        <v>14.71985966544552</v>
+        <v>14.70331452944414</v>
       </c>
       <c r="O45" t="n">
-        <v>10.44125</v>
+        <v>10.38694444444445</v>
       </c>
     </row>
     <row r="46">
@@ -3341,19 +3341,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1880</v>
+        <v>1883</v>
       </c>
       <c r="D46" t="n">
-        <v>21.82038120567376</v>
+        <v>21.84235262878385</v>
       </c>
       <c r="E46" t="n">
-        <v>15.625</v>
+        <v>15.63333333333333</v>
       </c>
       <c r="F46" t="n">
-        <v>0.3636730200945627</v>
+        <v>0.364039210479731</v>
       </c>
       <c r="G46" t="n">
-        <v>0.2604166666666666</v>
+        <v>0.2605555555555555</v>
       </c>
       <c r="H46" t="n">
         <v>2674.306204858831</v>
@@ -3407,28 +3407,28 @@
         <v>1.113333333333333</v>
       </c>
       <c r="H47" t="n">
-        <v>3018.061434297476</v>
+        <v>3017.137768031189</v>
       </c>
       <c r="I47" t="n">
         <v>2793.966666666667</v>
       </c>
       <c r="J47" t="n">
-        <v>50.30102390495794</v>
+        <v>50.28562946718649</v>
       </c>
       <c r="K47" t="n">
         <v>46.56611111111111</v>
       </c>
       <c r="L47" t="n">
-        <v>2783.231795038458</v>
+        <v>2782.372964045918</v>
       </c>
       <c r="M47" t="n">
-        <v>2721.3</v>
+        <v>2720.941666666667</v>
       </c>
       <c r="N47" t="n">
-        <v>46.38719658397429</v>
+        <v>46.37288273409862</v>
       </c>
       <c r="O47" t="n">
-        <v>45.355</v>
+        <v>45.34902777777778</v>
       </c>
     </row>
     <row r="48">
@@ -3443,19 +3443,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>8575</v>
+        <v>8587</v>
       </c>
       <c r="D48" t="n">
-        <v>24.45673663751215</v>
+        <v>24.47225262994449</v>
       </c>
       <c r="E48" t="n">
-        <v>15.93333333333333</v>
+        <v>15.95</v>
       </c>
       <c r="F48" t="n">
-        <v>0.4076122772918691</v>
+        <v>0.4078708771657415</v>
       </c>
       <c r="G48" t="n">
-        <v>0.2655555555555555</v>
+        <v>0.2658333333333333</v>
       </c>
       <c r="H48" t="n">
         <v>401.9148910217957</v>
@@ -3464,13 +3464,13 @@
         <v>333.3166666666667</v>
       </c>
       <c r="J48" t="n">
-        <v>6.698581517029927</v>
+        <v>6.698581517029926</v>
       </c>
       <c r="K48" t="n">
         <v>5.555277777777778</v>
       </c>
       <c r="L48" t="n">
-        <v>377.2225854829034</v>
+        <v>377.2225854829035</v>
       </c>
       <c r="M48" t="n">
         <v>307.7833333333334</v>
@@ -3509,28 +3509,28 @@
         <v>1.909166666666667</v>
       </c>
       <c r="H49" t="n">
-        <v>660.2463036303631</v>
+        <v>662.1981225710015</v>
       </c>
       <c r="I49" t="n">
-        <v>619.4166666666666</v>
+        <v>619.9833333333333</v>
       </c>
       <c r="J49" t="n">
-        <v>11.00410506050605</v>
+        <v>11.03663537618336</v>
       </c>
       <c r="K49" t="n">
-        <v>10.32361111111111</v>
+        <v>10.33305555555556</v>
       </c>
       <c r="L49" t="n">
-        <v>366.00599759976</v>
+        <v>365.7400627802691</v>
       </c>
       <c r="M49" t="n">
-        <v>231.5833333333333</v>
+        <v>231.0833333333333</v>
       </c>
       <c r="N49" t="n">
-        <v>6.100099959995999</v>
+        <v>6.095667713004484</v>
       </c>
       <c r="O49" t="n">
-        <v>3.859722222222222</v>
+        <v>3.851388888888889</v>
       </c>
     </row>
   </sheetData>
@@ -14685,19 +14685,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10404</v>
+        <v>10412</v>
       </c>
       <c r="C4" t="n">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D4" t="n">
-        <v>4.267589388696654</v>
+        <v>4.273914713791779</v>
       </c>
       <c r="E4" t="n">
-        <v>5280.212500000001</v>
+        <v>5268.391797752809</v>
       </c>
       <c r="F4" t="n">
-        <v>1419.698766967872</v>
+        <v>1420.712420888934</v>
       </c>
     </row>
     <row r="5">
@@ -14707,19 +14707,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>355370</v>
+        <v>355788</v>
       </c>
       <c r="C5" t="n">
-        <v>259399</v>
+        <v>259720</v>
       </c>
       <c r="D5" t="n">
-        <v>72.99406252638096</v>
+        <v>72.9985272128346</v>
       </c>
       <c r="E5" t="n">
-        <v>2804.386483324146</v>
+        <v>2805.224925719237</v>
       </c>
       <c r="F5" t="n">
-        <v>4811.868217326068</v>
+        <v>4810.073803087396</v>
       </c>
     </row>
     <row r="6">
@@ -14729,19 +14729,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>108560</v>
+        <v>108742</v>
       </c>
       <c r="C6" t="n">
-        <v>5039</v>
+        <v>5048</v>
       </c>
       <c r="D6" t="n">
-        <v>4.641672807663964</v>
+        <v>4.64218057420316</v>
       </c>
       <c r="E6" t="n">
-        <v>1589.1411291923</v>
+        <v>1586.872999207607</v>
       </c>
       <c r="F6" t="n">
-        <v>3585.539301851702</v>
+        <v>3589.012339739908</v>
       </c>
     </row>
     <row r="7">
@@ -14751,19 +14751,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60814</v>
+        <v>60862</v>
       </c>
       <c r="C7" t="n">
-        <v>17959</v>
+        <v>17969</v>
       </c>
       <c r="D7" t="n">
-        <v>29.53102903936594</v>
+        <v>29.52416943248661</v>
       </c>
       <c r="E7" t="n">
-        <v>542.9248473745755</v>
+        <v>542.6518634314654</v>
       </c>
       <c r="F7" t="n">
-        <v>4399.380149107456</v>
+        <v>4395.639700184179</v>
       </c>
     </row>
     <row r="8"/>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard jue 30/07/2026  9:32:07,04
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -652,19 +652,19 @@
         <v>62.16238270093839</v>
       </c>
       <c r="T2" t="n">
-        <v>11833</v>
+        <v>12469</v>
       </c>
       <c r="U2" t="n">
-        <v>13.54686047494296</v>
+        <v>13.36113561632849</v>
       </c>
       <c r="V2" t="n">
-        <v>65.36803853629681</v>
+        <v>65.22575988451359</v>
       </c>
       <c r="W2" t="n">
-        <v>-7.244653192947702</v>
+        <v>-7.430378051562164</v>
       </c>
       <c r="X2" t="n">
-        <v>-3.443492452060384</v>
+        <v>1.746226030191758</v>
       </c>
     </row>
     <row r="3">
@@ -728,19 +728,19 @@
         <v>77.97356828193833</v>
       </c>
       <c r="T3" t="n">
-        <v>684</v>
+        <v>731</v>
       </c>
       <c r="U3" t="n">
-        <v>27.63157894736842</v>
+        <v>26.67578659370725</v>
       </c>
       <c r="V3" t="n">
-        <v>76.75438596491229</v>
+        <v>77.4281805745554</v>
       </c>
       <c r="W3" t="n">
-        <v>-16.56812736687533</v>
+        <v>-17.5239197205365</v>
       </c>
       <c r="X3" t="n">
-        <v>0.4405286343612335</v>
+        <v>7.342143906020558</v>
       </c>
     </row>
     <row r="4">
@@ -804,19 +804,19 @@
         <v>39.73451327433628</v>
       </c>
       <c r="T4" t="n">
-        <v>949</v>
+        <v>997</v>
       </c>
       <c r="U4" t="n">
-        <v>0.1053740779768177</v>
+        <v>0.2006018054162488</v>
       </c>
       <c r="V4" t="n">
-        <v>33.2982086406744</v>
+        <v>34.40320962888666</v>
       </c>
       <c r="W4" t="n">
-        <v>-23.52294450609398</v>
+        <v>-23.42771677865455</v>
       </c>
       <c r="X4" t="n">
-        <v>-16.01769911504425</v>
+        <v>-11.76991150442478</v>
       </c>
     </row>
     <row r="5">
@@ -880,19 +880,19 @@
         <v>56.85258964143426</v>
       </c>
       <c r="T5" t="n">
-        <v>2093</v>
+        <v>2270</v>
       </c>
       <c r="U5" t="n">
-        <v>38.84376493072146</v>
+        <v>38.28193832599119</v>
       </c>
       <c r="V5" t="n">
-        <v>52.98614429049212</v>
+        <v>52.51101321585902</v>
       </c>
       <c r="W5" t="n">
-        <v>-7.012808774457824</v>
+        <v>-7.574635379188088</v>
       </c>
       <c r="X5" t="n">
-        <v>-16.61354581673307</v>
+        <v>-9.561752988047809</v>
       </c>
     </row>
     <row r="6">
@@ -956,19 +956,19 @@
         <v>60.76099053978854</v>
       </c>
       <c r="T6" t="n">
-        <v>24828</v>
+        <v>26727</v>
       </c>
       <c r="U6" t="n">
-        <v>58.65152247462543</v>
+        <v>59.67373816739626</v>
       </c>
       <c r="V6" t="n">
-        <v>63.27936201063316</v>
+        <v>64.24589366558162</v>
       </c>
       <c r="W6" t="n">
-        <v>0.8294579225942726</v>
+        <v>1.851673615365101</v>
       </c>
       <c r="X6" t="n">
-        <v>-13.64774624373957</v>
+        <v>-7.042988313856427</v>
       </c>
     </row>
     <row r="7">
@@ -1032,19 +1032,19 @@
         <v>61.65678803274061</v>
       </c>
       <c r="T7" t="n">
-        <v>27032</v>
+        <v>28890</v>
       </c>
       <c r="U7" t="n">
-        <v>36.23113347144125</v>
+        <v>35.93284873658705</v>
       </c>
       <c r="V7" t="n">
-        <v>61.84522047943178</v>
+        <v>61.83108341986847</v>
       </c>
       <c r="W7" t="n">
-        <v>-10.08554730755959</v>
+        <v>-10.38383204241379</v>
       </c>
       <c r="X7" t="n">
-        <v>-4.62884561106407</v>
+        <v>1.926333615580017</v>
       </c>
     </row>
     <row r="8">
@@ -1108,19 +1108,19 @@
         <v>45.21468784135787</v>
       </c>
       <c r="T8" t="n">
-        <v>11183</v>
+        <v>12043</v>
       </c>
       <c r="U8" t="n">
-        <v>36.41241169632478</v>
+        <v>36.61047911649921</v>
       </c>
       <c r="V8" t="n">
-        <v>53.11633729768398</v>
+        <v>53.88192310885992</v>
       </c>
       <c r="W8" t="n">
-        <v>0.7095295855777835</v>
+        <v>0.9075970057522156</v>
       </c>
       <c r="X8" t="n">
-        <v>-6.033106461641879</v>
+        <v>1.193177043945887</v>
       </c>
     </row>
     <row r="9">
@@ -1184,19 +1184,19 @@
         <v>69.81926219361227</v>
       </c>
       <c r="T9" t="n">
-        <v>3805</v>
+        <v>4053</v>
       </c>
       <c r="U9" t="n">
-        <v>59.55321944809461</v>
+        <v>60.00493461633359</v>
       </c>
       <c r="V9" t="n">
-        <v>67.72667542706965</v>
+        <v>68.04835924006909</v>
       </c>
       <c r="W9" t="n">
-        <v>1.296225142573441</v>
+        <v>1.747940310812417</v>
       </c>
       <c r="X9" t="n">
-        <v>-5.793513245852934</v>
+        <v>0.3466204506065858</v>
       </c>
     </row>
     <row r="10">
@@ -1260,19 +1260,19 @@
         <v>33.59223300970874</v>
       </c>
       <c r="T10" t="n">
-        <v>1804</v>
+        <v>1960</v>
       </c>
       <c r="U10" t="n">
-        <v>2.771618625277162</v>
+        <v>2.704081632653061</v>
       </c>
       <c r="V10" t="n">
-        <v>36.30820399113082</v>
+        <v>36.63265306122449</v>
       </c>
       <c r="W10" t="n">
-        <v>-8.490517297052934</v>
+        <v>-8.558054289677035</v>
       </c>
       <c r="X10" t="n">
-        <v>75.14563106796116</v>
+        <v>90.29126213592234</v>
       </c>
     </row>
     <row r="11">
@@ -1336,19 +1336,19 @@
         <v>74.40353659771201</v>
       </c>
       <c r="T11" t="n">
-        <v>81630</v>
+        <v>84764</v>
       </c>
       <c r="U11" t="n">
-        <v>67.49356854097758</v>
+        <v>68.68717851918267</v>
       </c>
       <c r="V11" t="n">
-        <v>73.63714320715424</v>
+        <v>74.60714454249445</v>
       </c>
       <c r="W11" t="n">
-        <v>-4.332886199795666</v>
+        <v>-3.139276221590578</v>
       </c>
       <c r="X11" t="n">
-        <v>-8.176694900955015</v>
+        <v>-4.651345909402806</v>
       </c>
     </row>
     <row r="12">
@@ -1412,19 +1412,19 @@
         <v>75.20695379142226</v>
       </c>
       <c r="T12" t="n">
-        <v>298142</v>
+        <v>313901</v>
       </c>
       <c r="U12" t="n">
-        <v>57.00941162264961</v>
+        <v>56.96827980796493</v>
       </c>
       <c r="V12" t="n">
-        <v>74.65704261727633</v>
+        <v>74.83569660498055</v>
       </c>
       <c r="W12" t="n">
-        <v>-5.019473689482432</v>
+        <v>-5.060605504167114</v>
       </c>
       <c r="X12" t="n">
-        <v>7.353836071712775</v>
+        <v>13.02827678336736</v>
       </c>
     </row>
     <row r="13">
@@ -1488,19 +1488,19 @@
         <v>60.68562662261034</v>
       </c>
       <c r="T13" t="n">
-        <v>51873</v>
+        <v>56356</v>
       </c>
       <c r="U13" t="n">
-        <v>27.56347232664392</v>
+        <v>27.64568102775214</v>
       </c>
       <c r="V13" t="n">
-        <v>60.28762554700904</v>
+        <v>60.61111505429768</v>
       </c>
       <c r="W13" t="n">
-        <v>0.4098258786854565</v>
+        <v>0.4920345797936818</v>
       </c>
       <c r="X13" t="n">
-        <v>2.023837620958225</v>
+        <v>10.8410038549288</v>
       </c>
     </row>
     <row r="14">
@@ -1564,19 +1564,19 @@
         <v>62.77658116310946</v>
       </c>
       <c r="T14" t="n">
-        <v>5581</v>
+        <v>5987</v>
       </c>
       <c r="U14" t="n">
-        <v>33.7394732126859</v>
+        <v>33.62284950726575</v>
       </c>
       <c r="V14" t="n">
-        <v>59.61297258555815</v>
+        <v>60.04676799732754</v>
       </c>
       <c r="W14" t="n">
-        <v>-3.386040787705717</v>
+        <v>-3.50266449312587</v>
       </c>
       <c r="X14" t="n">
-        <v>9.281378500097905</v>
+        <v>17.23125122381046</v>
       </c>
     </row>
     <row r="15">
@@ -1640,19 +1640,19 @@
         <v>81.03823437985702</v>
       </c>
       <c r="T15" t="n">
-        <v>14367</v>
+        <v>15521</v>
       </c>
       <c r="U15" t="n">
-        <v>59.76891487436487</v>
+        <v>59.28741704787063</v>
       </c>
       <c r="V15" t="n">
-        <v>74.26741838936451</v>
+        <v>74.15759293859932</v>
       </c>
       <c r="W15" t="n">
-        <v>-10.94914543026678</v>
+        <v>-11.43064325676102</v>
       </c>
       <c r="X15" t="n">
-        <v>-10.68075847062481</v>
+        <v>-3.506372396642835</v>
       </c>
     </row>
   </sheetData>
@@ -1742,19 +1742,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11833</v>
+        <v>12469</v>
       </c>
       <c r="C4" t="n">
-        <v>1603</v>
+        <v>1666</v>
       </c>
       <c r="D4" t="n">
-        <v>13.54686047494296</v>
+        <v>13.36113561632849</v>
       </c>
       <c r="E4" t="n">
-        <v>7735</v>
+        <v>8133</v>
       </c>
       <c r="F4" t="n">
-        <v>65.36803853629681</v>
+        <v>65.22575988451359</v>
       </c>
     </row>
     <row r="5">
@@ -1764,19 +1764,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>684</v>
+        <v>731</v>
       </c>
       <c r="C5" t="n">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D5" t="n">
-        <v>27.63157894736842</v>
+        <v>26.67578659370725</v>
       </c>
       <c r="E5" t="n">
-        <v>525</v>
+        <v>566</v>
       </c>
       <c r="F5" t="n">
-        <v>76.75438596491229</v>
+        <v>77.4281805745554</v>
       </c>
     </row>
     <row r="6">
@@ -1786,19 +1786,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>949</v>
+        <v>997</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1053740779768177</v>
+        <v>0.2006018054162488</v>
       </c>
       <c r="E6" t="n">
-        <v>316</v>
+        <v>343</v>
       </c>
       <c r="F6" t="n">
-        <v>33.2982086406744</v>
+        <v>34.40320962888666</v>
       </c>
     </row>
     <row r="7">
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2093</v>
+        <v>2270</v>
       </c>
       <c r="C7" t="n">
-        <v>813</v>
+        <v>869</v>
       </c>
       <c r="D7" t="n">
-        <v>38.84376493072146</v>
+        <v>38.28193832599119</v>
       </c>
       <c r="E7" t="n">
-        <v>1109</v>
+        <v>1192</v>
       </c>
       <c r="F7" t="n">
-        <v>52.98614429049212</v>
+        <v>52.51101321585902</v>
       </c>
     </row>
     <row r="8">
@@ -1830,19 +1830,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24828</v>
+        <v>26727</v>
       </c>
       <c r="C8" t="n">
-        <v>14562</v>
+        <v>15949</v>
       </c>
       <c r="D8" t="n">
-        <v>58.65152247462543</v>
+        <v>59.67373816739626</v>
       </c>
       <c r="E8" t="n">
-        <v>15711</v>
+        <v>17171</v>
       </c>
       <c r="F8" t="n">
-        <v>63.27936201063316</v>
+        <v>64.24589366558162</v>
       </c>
     </row>
     <row r="9">
@@ -1852,19 +1852,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>27032</v>
+        <v>28890</v>
       </c>
       <c r="C9" t="n">
-        <v>9794</v>
+        <v>10381</v>
       </c>
       <c r="D9" t="n">
-        <v>36.23113347144125</v>
+        <v>35.93284873658705</v>
       </c>
       <c r="E9" t="n">
-        <v>16718</v>
+        <v>17863</v>
       </c>
       <c r="F9" t="n">
-        <v>61.84522047943178</v>
+        <v>61.83108341986847</v>
       </c>
     </row>
     <row r="10">
@@ -1874,19 +1874,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11183</v>
+        <v>12043</v>
       </c>
       <c r="C10" t="n">
-        <v>4072</v>
+        <v>4409</v>
       </c>
       <c r="D10" t="n">
-        <v>36.41241169632478</v>
+        <v>36.61047911649921</v>
       </c>
       <c r="E10" t="n">
-        <v>5940</v>
+        <v>6489</v>
       </c>
       <c r="F10" t="n">
-        <v>53.11633729768398</v>
+        <v>53.88192310885992</v>
       </c>
     </row>
     <row r="11">
@@ -1896,19 +1896,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3805</v>
+        <v>4053</v>
       </c>
       <c r="C11" t="n">
-        <v>2266</v>
+        <v>2432</v>
       </c>
       <c r="D11" t="n">
-        <v>59.55321944809461</v>
+        <v>60.00493461633359</v>
       </c>
       <c r="E11" t="n">
-        <v>2577</v>
+        <v>2758</v>
       </c>
       <c r="F11" t="n">
-        <v>67.72667542706965</v>
+        <v>68.04835924006909</v>
       </c>
     </row>
     <row r="12">
@@ -1918,19 +1918,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1804</v>
+        <v>1960</v>
       </c>
       <c r="C12" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D12" t="n">
-        <v>2.771618625277162</v>
+        <v>2.704081632653061</v>
       </c>
       <c r="E12" t="n">
-        <v>655</v>
+        <v>718</v>
       </c>
       <c r="F12" t="n">
-        <v>36.30820399113082</v>
+        <v>36.63265306122449</v>
       </c>
     </row>
     <row r="13">
@@ -1940,19 +1940,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>81630</v>
+        <v>84764</v>
       </c>
       <c r="C13" t="n">
-        <v>55095</v>
+        <v>58222</v>
       </c>
       <c r="D13" t="n">
-        <v>67.49356854097758</v>
+        <v>68.68717851918267</v>
       </c>
       <c r="E13" t="n">
-        <v>60110</v>
+        <v>63240</v>
       </c>
       <c r="F13" t="n">
-        <v>73.63714320715424</v>
+        <v>74.60714454249445</v>
       </c>
     </row>
     <row r="14">
@@ -1962,19 +1962,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>298142</v>
+        <v>313901</v>
       </c>
       <c r="C14" t="n">
-        <v>169969</v>
+        <v>178824</v>
       </c>
       <c r="D14" t="n">
-        <v>57.00941162264961</v>
+        <v>56.96827980796493</v>
       </c>
       <c r="E14" t="n">
-        <v>222584</v>
+        <v>234910</v>
       </c>
       <c r="F14" t="n">
-        <v>74.65704261727633</v>
+        <v>74.83569660498055</v>
       </c>
     </row>
     <row r="15">
@@ -1984,19 +1984,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>51873</v>
+        <v>56356</v>
       </c>
       <c r="C15" t="n">
-        <v>14298</v>
+        <v>15580</v>
       </c>
       <c r="D15" t="n">
-        <v>27.56347232664392</v>
+        <v>27.64568102775214</v>
       </c>
       <c r="E15" t="n">
-        <v>31273</v>
+        <v>34158</v>
       </c>
       <c r="F15" t="n">
-        <v>60.28762554700904</v>
+        <v>60.61111505429768</v>
       </c>
     </row>
     <row r="16">
@@ -2006,19 +2006,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5581</v>
+        <v>5987</v>
       </c>
       <c r="C16" t="n">
-        <v>1883</v>
+        <v>2013</v>
       </c>
       <c r="D16" t="n">
-        <v>33.7394732126859</v>
+        <v>33.62284950726575</v>
       </c>
       <c r="E16" t="n">
-        <v>3327</v>
+        <v>3595</v>
       </c>
       <c r="F16" t="n">
-        <v>59.61297258555815</v>
+        <v>60.04676799732754</v>
       </c>
     </row>
     <row r="17">
@@ -2028,19 +2028,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>14367</v>
+        <v>15521</v>
       </c>
       <c r="C17" t="n">
-        <v>8587</v>
+        <v>9202</v>
       </c>
       <c r="D17" t="n">
-        <v>59.76891487436487</v>
+        <v>59.28741704787063</v>
       </c>
       <c r="E17" t="n">
-        <v>10670</v>
+        <v>11510</v>
       </c>
       <c r="F17" t="n">
-        <v>74.26741838936451</v>
+        <v>74.15759293859932</v>
       </c>
     </row>
     <row r="18"/>
@@ -2141,43 +2141,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1603</v>
+        <v>1666</v>
       </c>
       <c r="D22" t="n">
-        <v>15.55606155125806</v>
+        <v>15.84285714285714</v>
       </c>
       <c r="E22" t="n">
-        <v>8.166666666666666</v>
+        <v>8.316666666666666</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2592676925209676</v>
+        <v>0.264047619047619</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1361111111111111</v>
+        <v>0.1386111111111111</v>
       </c>
       <c r="H22" t="n">
-        <v>267.2242802303263</v>
+        <v>269.7315813953488</v>
       </c>
       <c r="I22" t="n">
-        <v>125.7666666666667</v>
+        <v>130.1666666666667</v>
       </c>
       <c r="J22" t="n">
-        <v>4.453738003838771</v>
+        <v>4.495526356589148</v>
       </c>
       <c r="K22" t="n">
-        <v>2.096111111111111</v>
+        <v>2.169444444444444</v>
       </c>
       <c r="L22" t="n">
-        <v>245.057949456174</v>
+        <v>247.1540000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>104.35</v>
+        <v>107.1</v>
       </c>
       <c r="N22" t="n">
-        <v>4.084299157602901</v>
+        <v>4.119233333333333</v>
       </c>
       <c r="O22" t="n">
-        <v>1.739166666666667</v>
+        <v>1.785</v>
       </c>
     </row>
     <row r="23">
@@ -2192,43 +2192,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10230</v>
+        <v>10803</v>
       </c>
       <c r="D23" t="n">
-        <v>241.1290795047247</v>
+        <v>237.3427057298898</v>
       </c>
       <c r="E23" t="n">
-        <v>72.88333333333333</v>
+        <v>70.33333333333333</v>
       </c>
       <c r="F23" t="n">
-        <v>4.018817991745411</v>
+        <v>3.955711762164831</v>
       </c>
       <c r="G23" t="n">
-        <v>1.214722222222222</v>
+        <v>1.172222222222222</v>
       </c>
       <c r="H23" t="n">
-        <v>255.9123212979586</v>
+        <v>251.6846655970807</v>
       </c>
       <c r="I23" t="n">
-        <v>89.2</v>
+        <v>86.35833333333332</v>
       </c>
       <c r="J23" t="n">
-        <v>4.265205354965977</v>
+        <v>4.194744426618011</v>
       </c>
       <c r="K23" t="n">
-        <v>1.486666666666667</v>
+        <v>1.439305555555555</v>
       </c>
       <c r="L23" t="n">
-        <v>14.37771627102866</v>
+        <v>13.96958600729835</v>
       </c>
       <c r="M23" t="n">
-        <v>6.2</v>
+        <v>6.091666666666667</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2396286045171444</v>
+        <v>0.2328264334549725</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1033333333333333</v>
+        <v>0.1015277777777778</v>
       </c>
     </row>
     <row r="24">
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -2264,7 +2264,7 @@
         <v>17.46666666666667</v>
       </c>
       <c r="J24" t="n">
-        <v>2.673711873638343</v>
+        <v>2.673711873638344</v>
       </c>
       <c r="K24" t="n">
         <v>0.2911111111111111</v>
@@ -2276,7 +2276,7 @@
         <v>17.46666666666667</v>
       </c>
       <c r="N24" t="n">
-        <v>2.673711873638343</v>
+        <v>2.673711873638344</v>
       </c>
       <c r="O24" t="n">
         <v>0.2911111111111111</v>
@@ -2294,40 +2294,40 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>495</v>
+        <v>536</v>
       </c>
       <c r="D25" t="n">
-        <v>294.9030976430976</v>
+        <v>287.6420087064677</v>
       </c>
       <c r="E25" t="n">
-        <v>15.78333333333333</v>
+        <v>15.56666666666667</v>
       </c>
       <c r="F25" t="n">
-        <v>4.91505162738496</v>
+        <v>4.794033478441128</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2630555555555555</v>
+        <v>0.2594444444444444</v>
       </c>
       <c r="H25" t="n">
-        <v>305.334756097561</v>
+        <v>298.4999374609131</v>
       </c>
       <c r="I25" t="n">
-        <v>22.35</v>
+        <v>21.75</v>
       </c>
       <c r="J25" t="n">
-        <v>5.088912601626016</v>
+        <v>4.974998957681885</v>
       </c>
       <c r="K25" t="n">
-        <v>0.3725</v>
+        <v>0.3625</v>
       </c>
       <c r="L25" t="n">
-        <v>11.84231029810298</v>
+        <v>12.20093808630394</v>
       </c>
       <c r="M25" t="n">
         <v>2.216666666666667</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1973718383017164</v>
+        <v>0.2033489681050657</v>
       </c>
       <c r="O25" t="n">
         <v>0.03694444444444445</v>
@@ -2345,7 +2345,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -2372,43 +2372,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>948</v>
+        <v>995</v>
       </c>
       <c r="D27" t="n">
-        <v>643.6988396624473</v>
+        <v>625.0669849246232</v>
       </c>
       <c r="E27" t="n">
-        <v>109.6</v>
+        <v>109.5833333333333</v>
       </c>
       <c r="F27" t="n">
-        <v>10.72831399437412</v>
+        <v>10.41778308207705</v>
       </c>
       <c r="G27" t="n">
-        <v>1.826666666666667</v>
+        <v>1.826388888888889</v>
       </c>
       <c r="H27" t="n">
-        <v>5140.077918781726</v>
+        <v>5234.074379178606</v>
       </c>
       <c r="I27" t="n">
-        <v>4559.65</v>
+        <v>4576.133333333333</v>
       </c>
       <c r="J27" t="n">
-        <v>85.66796531302877</v>
+        <v>87.2345729863101</v>
       </c>
       <c r="K27" t="n">
-        <v>75.99416666666666</v>
+        <v>76.2688888888889</v>
       </c>
       <c r="L27" t="n">
-        <v>4348.762887760858</v>
+        <v>4417.962774594078</v>
       </c>
       <c r="M27" t="n">
-        <v>4221.483333333334</v>
+        <v>4222.5</v>
       </c>
       <c r="N27" t="n">
-        <v>72.47938146268096</v>
+        <v>73.63271290990131</v>
       </c>
       <c r="O27" t="n">
-        <v>70.35805555555557</v>
+        <v>70.375</v>
       </c>
     </row>
     <row r="28">
@@ -2423,43 +2423,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>813</v>
+        <v>869</v>
       </c>
       <c r="D28" t="n">
-        <v>22.93337433374334</v>
+        <v>23.74468738013042</v>
       </c>
       <c r="E28" t="n">
-        <v>15.61666666666667</v>
+        <v>15.9</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3822229055623889</v>
+        <v>0.3957447896688403</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2602777777777778</v>
+        <v>0.265</v>
       </c>
       <c r="H28" t="n">
-        <v>750.9658333333333</v>
+        <v>743.2020961775586</v>
       </c>
       <c r="I28" t="n">
-        <v>740.8666666666667</v>
+        <v>736.0333333333333</v>
       </c>
       <c r="J28" t="n">
-        <v>12.51609722222222</v>
+        <v>12.38670160295931</v>
       </c>
       <c r="K28" t="n">
-        <v>12.34777777777778</v>
+        <v>12.26722222222222</v>
       </c>
       <c r="L28" t="n">
-        <v>727.8457692307692</v>
+        <v>719.6077887381834</v>
       </c>
       <c r="M28" t="n">
-        <v>717.9333333333334</v>
+        <v>708.9666666666667</v>
       </c>
       <c r="N28" t="n">
-        <v>12.13076282051282</v>
+        <v>11.99346314563639</v>
       </c>
       <c r="O28" t="n">
-        <v>11.96555555555556</v>
+        <v>11.81611111111111</v>
       </c>
     </row>
     <row r="29">
@@ -2474,43 +2474,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1280</v>
+        <v>1401</v>
       </c>
       <c r="D29" t="n">
-        <v>246.0678776041667</v>
+        <v>247.4369260052343</v>
       </c>
       <c r="E29" t="n">
-        <v>71.95833333333334</v>
+        <v>70.56666666666666</v>
       </c>
       <c r="F29" t="n">
-        <v>4.101131293402778</v>
+        <v>4.123948766753906</v>
       </c>
       <c r="G29" t="n">
-        <v>1.199305555555556</v>
+        <v>1.176111111111111</v>
       </c>
       <c r="H29" t="n">
-        <v>996.410632183908</v>
+        <v>986.9147304479878</v>
       </c>
       <c r="I29" t="n">
-        <v>928.5333333333333</v>
+        <v>923.55</v>
       </c>
       <c r="J29" t="n">
-        <v>16.6068438697318</v>
+        <v>16.4485788407998</v>
       </c>
       <c r="K29" t="n">
-        <v>15.47555555555556</v>
+        <v>15.3925</v>
       </c>
       <c r="L29" t="n">
-        <v>746.1134646962233</v>
+        <v>732.9659200202481</v>
       </c>
       <c r="M29" t="n">
-        <v>841.7</v>
+        <v>814.6833333333333</v>
       </c>
       <c r="N29" t="n">
-        <v>12.43522441160372</v>
+        <v>12.21609866700413</v>
       </c>
       <c r="O29" t="n">
-        <v>14.02833333333333</v>
+        <v>13.57805555555555</v>
       </c>
     </row>
     <row r="30">
@@ -2525,43 +2525,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>14562</v>
+        <v>15949</v>
       </c>
       <c r="D30" t="n">
-        <v>25.0723126402051</v>
+        <v>25.97564842100863</v>
       </c>
       <c r="E30" t="n">
-        <v>30.35833333333333</v>
+        <v>35.21666666666667</v>
       </c>
       <c r="F30" t="n">
-        <v>0.4178718773367516</v>
+        <v>0.4329274736834772</v>
       </c>
       <c r="G30" t="n">
-        <v>0.5059722222222223</v>
+        <v>0.5869444444444445</v>
       </c>
       <c r="H30" t="n">
-        <v>406.4914607948443</v>
+        <v>403.3587395256829</v>
       </c>
       <c r="I30" t="n">
-        <v>234.6666666666667</v>
+        <v>229.9833333333333</v>
       </c>
       <c r="J30" t="n">
-        <v>6.774857679914071</v>
+        <v>6.722645658761382</v>
       </c>
       <c r="K30" t="n">
-        <v>3.911111111111111</v>
+        <v>3.833055555555555</v>
       </c>
       <c r="L30" t="n">
-        <v>381.1289676572383</v>
+        <v>377.2942855237715</v>
       </c>
       <c r="M30" t="n">
-        <v>206.85</v>
+        <v>201.6833333333333</v>
       </c>
       <c r="N30" t="n">
-        <v>6.352149460953973</v>
+        <v>6.288238092062857</v>
       </c>
       <c r="O30" t="n">
-        <v>3.4475</v>
+        <v>3.361388888888889</v>
       </c>
     </row>
     <row r="31">
@@ -2576,43 +2576,43 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>10266</v>
+        <v>10778</v>
       </c>
       <c r="D31" t="n">
-        <v>1728.066228326515</v>
+        <v>1714.68124574751</v>
       </c>
       <c r="E31" t="n">
-        <v>1274.208333333333</v>
+        <v>1280.675</v>
       </c>
       <c r="F31" t="n">
-        <v>28.80110380544191</v>
+        <v>28.5780207624585</v>
       </c>
       <c r="G31" t="n">
-        <v>21.23680555555556</v>
+        <v>21.34458333333333</v>
       </c>
       <c r="H31" t="n">
-        <v>1987.976269129287</v>
+        <v>1969.435136085167</v>
       </c>
       <c r="I31" t="n">
-        <v>1509.266666666667</v>
+        <v>1509.6</v>
       </c>
       <c r="J31" t="n">
-        <v>33.13293781882146</v>
+        <v>32.82391893475278</v>
       </c>
       <c r="K31" t="n">
-        <v>25.15444444444444</v>
+        <v>25.16</v>
       </c>
       <c r="L31" t="n">
-        <v>261.2267739665787</v>
+        <v>255.9635248234073</v>
       </c>
       <c r="M31" t="n">
-        <v>247.6666666666667</v>
+        <v>247.65</v>
       </c>
       <c r="N31" t="n">
-        <v>4.353779566109646</v>
+        <v>4.266058747056789</v>
       </c>
       <c r="O31" t="n">
-        <v>4.127777777777777</v>
+        <v>4.1275</v>
       </c>
     </row>
     <row r="32">
@@ -2627,43 +2627,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>9794</v>
+        <v>10381</v>
       </c>
       <c r="D32" t="n">
-        <v>335.534854672929</v>
+        <v>325.7597935330571</v>
       </c>
       <c r="E32" t="n">
-        <v>35.16666666666666</v>
+        <v>35.3</v>
       </c>
       <c r="F32" t="n">
-        <v>5.59224757788215</v>
+        <v>5.42932989221762</v>
       </c>
       <c r="G32" t="n">
-        <v>0.586111111111111</v>
+        <v>0.5883333333333333</v>
       </c>
       <c r="H32" t="n">
-        <v>670.5325289575288</v>
+        <v>661.5398333538059</v>
       </c>
       <c r="I32" t="n">
-        <v>407.125</v>
+        <v>410.95</v>
       </c>
       <c r="J32" t="n">
-        <v>11.17554214929215</v>
+        <v>11.0256638892301</v>
       </c>
       <c r="K32" t="n">
-        <v>6.785416666666666</v>
+        <v>6.849166666666666</v>
       </c>
       <c r="L32" t="n">
-        <v>252.3976662376662</v>
+        <v>251.3512099250706</v>
       </c>
       <c r="M32" t="n">
-        <v>71.38333333333334</v>
+        <v>70.26666666666667</v>
       </c>
       <c r="N32" t="n">
-        <v>4.206627770627771</v>
+        <v>4.18918683208451</v>
       </c>
       <c r="O32" t="n">
-        <v>1.189722222222222</v>
+        <v>1.171111111111111</v>
       </c>
     </row>
     <row r="33">
@@ -2678,43 +2678,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>17238</v>
+        <v>18509</v>
       </c>
       <c r="D33" t="n">
-        <v>396.0638376455119</v>
+        <v>380.8550047724531</v>
       </c>
       <c r="E33" t="n">
-        <v>75.86666666666666</v>
+        <v>70.01666666666667</v>
       </c>
       <c r="F33" t="n">
-        <v>6.601063960758531</v>
+        <v>6.347583412874218</v>
       </c>
       <c r="G33" t="n">
-        <v>1.264444444444444</v>
+        <v>1.166944444444444</v>
       </c>
       <c r="H33" t="n">
-        <v>682.3947678795482</v>
+        <v>670.2795347519393</v>
       </c>
       <c r="I33" t="n">
-        <v>415.375</v>
+        <v>401.1666666666667</v>
       </c>
       <c r="J33" t="n">
-        <v>11.37324613132581</v>
+        <v>11.17132557919899</v>
       </c>
       <c r="K33" t="n">
-        <v>6.922916666666667</v>
+        <v>6.686111111111112</v>
       </c>
       <c r="L33" t="n">
-        <v>265.075495608532</v>
+        <v>268.6653858178478</v>
       </c>
       <c r="M33" t="n">
-        <v>61.54166666666666</v>
+        <v>62.65</v>
       </c>
       <c r="N33" t="n">
-        <v>4.417924926808866</v>
+        <v>4.477756430297465</v>
       </c>
       <c r="O33" t="n">
-        <v>1.025694444444444</v>
+        <v>1.044166666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2729,43 +2729,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4072</v>
+        <v>4409</v>
       </c>
       <c r="D34" t="n">
-        <v>1116.376088736084</v>
+        <v>1077.047629848038</v>
       </c>
       <c r="E34" t="n">
-        <v>938.2583333333333</v>
+        <v>911.7166666666667</v>
       </c>
       <c r="F34" t="n">
-        <v>18.6062681456014</v>
+        <v>17.95079383080063</v>
       </c>
       <c r="G34" t="n">
-        <v>15.63763888888889</v>
+        <v>15.19527777777778</v>
       </c>
       <c r="H34" t="n">
-        <v>1780.46858463792</v>
+        <v>1751.806763035622</v>
       </c>
       <c r="I34" t="n">
-        <v>1520.166666666667</v>
+        <v>1508.683333333333</v>
       </c>
       <c r="J34" t="n">
-        <v>29.674476410632</v>
+        <v>29.19677938392703</v>
       </c>
       <c r="K34" t="n">
-        <v>25.33611111111111</v>
+        <v>25.14472222222222</v>
       </c>
       <c r="L34" t="n">
-        <v>621.805937013641</v>
+        <v>613.2702331784546</v>
       </c>
       <c r="M34" t="n">
-        <v>515.6333333333333</v>
+        <v>502.9083333333333</v>
       </c>
       <c r="N34" t="n">
-        <v>10.36343228356068</v>
+        <v>10.22117055297424</v>
       </c>
       <c r="O34" t="n">
-        <v>8.593888888888889</v>
+        <v>8.381805555555555</v>
       </c>
     </row>
     <row r="35">
@@ -2780,43 +2780,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7111</v>
+        <v>7634</v>
       </c>
       <c r="D35" t="n">
-        <v>1350.259972812075</v>
+        <v>1327.760097371409</v>
       </c>
       <c r="E35" t="n">
-        <v>1096.266666666667</v>
+        <v>1086.491666666667</v>
       </c>
       <c r="F35" t="n">
-        <v>22.50433288020125</v>
+        <v>22.12933495619014</v>
       </c>
       <c r="G35" t="n">
-        <v>18.27111111111111</v>
+        <v>18.10819444444444</v>
       </c>
       <c r="H35" t="n">
-        <v>2042.850454861669</v>
+        <v>2014.113464042468</v>
       </c>
       <c r="I35" t="n">
-        <v>1698.1</v>
+        <v>1680.375</v>
       </c>
       <c r="J35" t="n">
-        <v>34.04750758102781</v>
+        <v>33.56855773404114</v>
       </c>
       <c r="K35" t="n">
-        <v>28.30166666666667</v>
+        <v>28.00625</v>
       </c>
       <c r="L35" t="n">
-        <v>655.516300101675</v>
+        <v>644.2678811097757</v>
       </c>
       <c r="M35" t="n">
-        <v>502.9</v>
+        <v>458.7</v>
       </c>
       <c r="N35" t="n">
-        <v>10.92527166836125</v>
+        <v>10.73779801849626</v>
       </c>
       <c r="O35" t="n">
-        <v>8.381666666666666</v>
+        <v>7.645</v>
       </c>
     </row>
     <row r="36">
@@ -2831,43 +2831,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2266</v>
+        <v>2432</v>
       </c>
       <c r="D36" t="n">
-        <v>24.59055604589585</v>
+        <v>25.26774259868421</v>
       </c>
       <c r="E36" t="n">
-        <v>16</v>
+        <v>33.99166666666666</v>
       </c>
       <c r="F36" t="n">
-        <v>0.4098426007649308</v>
+        <v>0.4211290433114034</v>
       </c>
       <c r="G36" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.5665277777777777</v>
       </c>
       <c r="H36" t="n">
-        <v>3095.120325802226</v>
+        <v>3001.039899680803</v>
       </c>
       <c r="I36" t="n">
-        <v>3008.95</v>
+        <v>2917.183333333333</v>
       </c>
       <c r="J36" t="n">
-        <v>51.58533876337044</v>
+        <v>50.01733166134672</v>
       </c>
       <c r="K36" t="n">
-        <v>50.14916666666667</v>
+        <v>48.61972222222222</v>
       </c>
       <c r="L36" t="n">
-        <v>3070.148526522593</v>
+        <v>2975.308732330141</v>
       </c>
       <c r="M36" t="n">
-        <v>2989.025</v>
+        <v>2886.166666666667</v>
       </c>
       <c r="N36" t="n">
-        <v>51.16914210870988</v>
+        <v>49.58847887216901</v>
       </c>
       <c r="O36" t="n">
-        <v>49.81708333333334</v>
+        <v>48.10277777777777</v>
       </c>
     </row>
     <row r="37">
@@ -2882,43 +2882,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1539</v>
+        <v>1621</v>
       </c>
       <c r="D37" t="n">
-        <v>2740.954732510289</v>
+        <v>2696.191610117212</v>
       </c>
       <c r="E37" t="n">
-        <v>2573.033333333333</v>
+        <v>2525.516666666667</v>
       </c>
       <c r="F37" t="n">
-        <v>45.68257887517147</v>
+        <v>44.93652683528686</v>
       </c>
       <c r="G37" t="n">
-        <v>42.88388888888889</v>
+        <v>42.09194444444445</v>
       </c>
       <c r="H37" t="n">
-        <v>3469.459366970334</v>
+        <v>3415.084254327564</v>
       </c>
       <c r="I37" t="n">
-        <v>3888.516666666667</v>
+        <v>3515.458333333333</v>
       </c>
       <c r="J37" t="n">
-        <v>57.8243227828389</v>
+        <v>56.91807090545939</v>
       </c>
       <c r="K37" t="n">
-        <v>64.80861111111112</v>
+        <v>58.59097222222222</v>
       </c>
       <c r="L37" t="n">
-        <v>599.3787316047653</v>
+        <v>587.6498557478916</v>
       </c>
       <c r="M37" t="n">
-        <v>335.3</v>
+        <v>341.7666666666667</v>
       </c>
       <c r="N37" t="n">
-        <v>9.989645526746088</v>
+        <v>9.794164262464861</v>
       </c>
       <c r="O37" t="n">
-        <v>5.588333333333334</v>
+        <v>5.696111111111112</v>
       </c>
     </row>
     <row r="38">
@@ -2933,7 +2933,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -2984,43 +2984,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1754</v>
+        <v>1907</v>
       </c>
       <c r="D39" t="n">
-        <v>174.8544469783352</v>
+        <v>177.0102954029016</v>
       </c>
       <c r="E39" t="n">
-        <v>78.14166666666667</v>
+        <v>78.18333333333334</v>
       </c>
       <c r="F39" t="n">
-        <v>2.914240782972254</v>
+        <v>2.95017159004836</v>
       </c>
       <c r="G39" t="n">
-        <v>1.302361111111111</v>
+        <v>1.303055555555556</v>
       </c>
       <c r="H39" t="n">
-        <v>502.2929829770388</v>
+        <v>494.6693649937039</v>
       </c>
       <c r="I39" t="n">
-        <v>429.2</v>
+        <v>426.15</v>
       </c>
       <c r="J39" t="n">
-        <v>8.37154971628398</v>
+        <v>8.244489416561731</v>
       </c>
       <c r="K39" t="n">
-        <v>7.153333333333333</v>
+        <v>7.1025</v>
       </c>
       <c r="L39" t="n">
-        <v>325.285253365004</v>
+        <v>315.7854380284224</v>
       </c>
       <c r="M39" t="n">
-        <v>159.2583333333333</v>
+        <v>160.9</v>
       </c>
       <c r="N39" t="n">
-        <v>5.421420889416733</v>
+        <v>5.26309063380704</v>
       </c>
       <c r="O39" t="n">
-        <v>2.654305555555555</v>
+        <v>2.681666666666667</v>
       </c>
     </row>
     <row r="40">
@@ -3035,43 +3035,43 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>55095</v>
+        <v>58222</v>
       </c>
       <c r="D40" t="n">
-        <v>456.4585546177814</v>
+        <v>433.8536446703995</v>
       </c>
       <c r="E40" t="n">
-        <v>46.16666666666666</v>
+        <v>44.41666666666666</v>
       </c>
       <c r="F40" t="n">
-        <v>7.607642576963023</v>
+        <v>7.230894077839991</v>
       </c>
       <c r="G40" t="n">
-        <v>0.7694444444444444</v>
+        <v>0.7402777777777777</v>
       </c>
       <c r="H40" t="n">
-        <v>570.2220280258701</v>
+        <v>559.491776377834</v>
       </c>
       <c r="I40" t="n">
-        <v>192.7583333333333</v>
+        <v>169.4666666666666</v>
       </c>
       <c r="J40" t="n">
-        <v>9.503700467097833</v>
+        <v>9.324862939630565</v>
       </c>
       <c r="K40" t="n">
-        <v>3.212638888888889</v>
+        <v>2.824444444444444</v>
       </c>
       <c r="L40" t="n">
-        <v>91.06445308489889</v>
+        <v>89.25040269342487</v>
       </c>
       <c r="M40" t="n">
-        <v>47.725</v>
+        <v>45.56666666666667</v>
       </c>
       <c r="N40" t="n">
-        <v>1.517740884748315</v>
+        <v>1.487506711557081</v>
       </c>
       <c r="O40" t="n">
-        <v>0.7954166666666667</v>
+        <v>0.7594444444444445</v>
       </c>
     </row>
     <row r="41">
@@ -3086,40 +3086,40 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>26535</v>
+        <v>26542</v>
       </c>
       <c r="D41" t="n">
-        <v>763.8958614408642</v>
+        <v>763.7284461105668</v>
       </c>
       <c r="E41" t="n">
-        <v>701.2333333333333</v>
+        <v>701.1666666666666</v>
       </c>
       <c r="F41" t="n">
-        <v>12.73159769068107</v>
+        <v>12.72880743517612</v>
       </c>
       <c r="G41" t="n">
-        <v>11.68722222222222</v>
+        <v>11.68611111111111</v>
       </c>
       <c r="H41" t="n">
-        <v>880.1673776679158</v>
+        <v>880.0281653180266</v>
       </c>
       <c r="I41" t="n">
-        <v>824.2333333333333</v>
+        <v>823.9666666666667</v>
       </c>
       <c r="J41" t="n">
-        <v>14.66945629446526</v>
+        <v>14.66713608863378</v>
       </c>
       <c r="K41" t="n">
-        <v>13.73722222222222</v>
+        <v>13.73277777777778</v>
       </c>
       <c r="L41" t="n">
-        <v>110.5557258857614</v>
+        <v>110.5443011652782</v>
       </c>
       <c r="M41" t="n">
         <v>88.08333333333333</v>
       </c>
       <c r="N41" t="n">
-        <v>1.842595431429356</v>
+        <v>1.842405019421302</v>
       </c>
       <c r="O41" t="n">
         <v>1.468055555555555</v>
@@ -3137,43 +3137,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>169969</v>
+        <v>178824</v>
       </c>
       <c r="D42" t="n">
-        <v>9.46689827752904</v>
+        <v>10.63374416558553</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0.1577816379588173</v>
+        <v>0.1772290694264255</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>457.3888882150799</v>
+        <v>454.7356620713077</v>
       </c>
       <c r="I42" t="n">
-        <v>181.7166666666667</v>
+        <v>182.45</v>
       </c>
       <c r="J42" t="n">
-        <v>7.623148136917997</v>
+        <v>7.57892770118846</v>
       </c>
       <c r="K42" t="n">
-        <v>3.028611111111111</v>
+        <v>3.040833333333333</v>
       </c>
       <c r="L42" t="n">
-        <v>447.3871237338005</v>
+        <v>443.6333169981</v>
       </c>
       <c r="M42" t="n">
-        <v>173.3666666666667</v>
+        <v>173.1</v>
       </c>
       <c r="N42" t="n">
-        <v>7.456452062230009</v>
+        <v>7.393888616635001</v>
       </c>
       <c r="O42" t="n">
-        <v>2.889444444444444</v>
+        <v>2.885</v>
       </c>
     </row>
     <row r="43">
@@ -3188,43 +3188,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>128173</v>
+        <v>135077</v>
       </c>
       <c r="D43" t="n">
-        <v>158.8526204166764</v>
+        <v>158.4470555066123</v>
       </c>
       <c r="E43" t="n">
-        <v>90.18333333333334</v>
+        <v>89.63333333333334</v>
       </c>
       <c r="F43" t="n">
-        <v>2.647543673611274</v>
+        <v>2.640784258443539</v>
       </c>
       <c r="G43" t="n">
-        <v>1.503055555555556</v>
+        <v>1.493888888888889</v>
       </c>
       <c r="H43" t="n">
-        <v>564.5380232836731</v>
+        <v>559.8444851731206</v>
       </c>
       <c r="I43" t="n">
-        <v>268.3166666666667</v>
+        <v>265.95</v>
       </c>
       <c r="J43" t="n">
-        <v>9.408967054727885</v>
+        <v>9.330741419552011</v>
       </c>
       <c r="K43" t="n">
-        <v>4.471944444444444</v>
+        <v>4.4325</v>
       </c>
       <c r="L43" t="n">
-        <v>404.7194923168235</v>
+        <v>401.2843708132173</v>
       </c>
       <c r="M43" t="n">
-        <v>124.7666666666667</v>
+        <v>124.6833333333333</v>
       </c>
       <c r="N43" t="n">
-        <v>6.74532487194706</v>
+        <v>6.688072846886955</v>
       </c>
       <c r="O43" t="n">
-        <v>2.079444444444444</v>
+        <v>2.078055555555556</v>
       </c>
     </row>
     <row r="44">
@@ -3239,43 +3239,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>14298</v>
+        <v>15580</v>
       </c>
       <c r="D44" t="n">
-        <v>22.88172704807199</v>
+        <v>23.78660248181429</v>
       </c>
       <c r="E44" t="n">
-        <v>15.76666666666667</v>
+        <v>35.11666666666667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.3813621174678665</v>
+        <v>0.3964433746969049</v>
       </c>
       <c r="G44" t="n">
-        <v>0.2627777777777778</v>
+        <v>0.5852777777777778</v>
       </c>
       <c r="H44" t="n">
-        <v>1072.777328145266</v>
+        <v>1045.016539155539</v>
       </c>
       <c r="I44" t="n">
-        <v>897.5916666666667</v>
+        <v>883.6833333333333</v>
       </c>
       <c r="J44" t="n">
-        <v>17.87962213575443</v>
+        <v>17.41694231925899</v>
       </c>
       <c r="K44" t="n">
-        <v>14.95986111111111</v>
+        <v>14.72805555555555</v>
       </c>
       <c r="L44" t="n">
-        <v>1048.810608300908</v>
+        <v>1020.208036809816</v>
       </c>
       <c r="M44" t="n">
-        <v>867.0666666666667</v>
+        <v>854.7333333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>17.48017680501513</v>
+        <v>17.0034672801636</v>
       </c>
       <c r="O44" t="n">
-        <v>14.45111111111111</v>
+        <v>14.24555555555556</v>
       </c>
     </row>
     <row r="45">
@@ -3290,43 +3290,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>37575</v>
+        <v>40776</v>
       </c>
       <c r="D45" t="n">
-        <v>275.8161281880683</v>
+        <v>269.3652540710222</v>
       </c>
       <c r="E45" t="n">
-        <v>30.08333333333333</v>
+        <v>29.26666666666667</v>
       </c>
       <c r="F45" t="n">
-        <v>4.596935469801139</v>
+        <v>4.489420901183703</v>
       </c>
       <c r="G45" t="n">
-        <v>0.5013888888888889</v>
+        <v>0.4877777777777778</v>
       </c>
       <c r="H45" t="n">
-        <v>1158.280942173817</v>
+        <v>1109.394442379511</v>
       </c>
       <c r="I45" t="n">
-        <v>966.9166666666666</v>
+        <v>940.25</v>
       </c>
       <c r="J45" t="n">
-        <v>19.30468236956361</v>
+        <v>18.48990737299185</v>
       </c>
       <c r="K45" t="n">
-        <v>16.11527777777778</v>
+        <v>15.67083333333333</v>
       </c>
       <c r="L45" t="n">
-        <v>882.1988717666482</v>
+        <v>838.5768925113717</v>
       </c>
       <c r="M45" t="n">
-        <v>623.2166666666667</v>
+        <v>560.1416666666667</v>
       </c>
       <c r="N45" t="n">
-        <v>14.70331452944414</v>
+        <v>13.9762815418562</v>
       </c>
       <c r="O45" t="n">
-        <v>10.38694444444445</v>
+        <v>9.335694444444444</v>
       </c>
     </row>
     <row r="46">
@@ -3341,43 +3341,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1883</v>
+        <v>2013</v>
       </c>
       <c r="D46" t="n">
-        <v>21.84235262878385</v>
+        <v>22.5016724623282</v>
       </c>
       <c r="E46" t="n">
-        <v>15.63333333333333</v>
+        <v>15.8</v>
       </c>
       <c r="F46" t="n">
-        <v>0.364039210479731</v>
+        <v>0.3750278743721366</v>
       </c>
       <c r="G46" t="n">
-        <v>0.2605555555555555</v>
+        <v>0.2633333333333334</v>
       </c>
       <c r="H46" t="n">
-        <v>2674.306204858831</v>
+        <v>2722.767684108527</v>
       </c>
       <c r="I46" t="n">
-        <v>2573.7</v>
+        <v>2597.383333333333</v>
       </c>
       <c r="J46" t="n">
-        <v>44.57177008098052</v>
+        <v>45.37946140180878</v>
       </c>
       <c r="K46" t="n">
-        <v>42.895</v>
+        <v>43.28972222222222</v>
       </c>
       <c r="L46" t="n">
-        <v>2651.866174217553</v>
+        <v>2698.824602713178</v>
       </c>
       <c r="M46" t="n">
-        <v>2543.116666666667</v>
+        <v>2565.6</v>
       </c>
       <c r="N46" t="n">
-        <v>44.19776957029255</v>
+        <v>44.98041004521964</v>
       </c>
       <c r="O46" t="n">
-        <v>42.38527777777778</v>
+        <v>42.76</v>
       </c>
     </row>
     <row r="47">
@@ -3392,43 +3392,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3698</v>
+        <v>3974</v>
       </c>
       <c r="D47" t="n">
-        <v>233.1295790517397</v>
+        <v>229.3043449085723</v>
       </c>
       <c r="E47" t="n">
-        <v>66.80000000000001</v>
+        <v>64.82499999999999</v>
       </c>
       <c r="F47" t="n">
-        <v>3.885492984195662</v>
+        <v>3.82173908180954</v>
       </c>
       <c r="G47" t="n">
-        <v>1.113333333333333</v>
+        <v>1.080416666666667</v>
       </c>
       <c r="H47" t="n">
-        <v>3017.137768031189</v>
+        <v>3067.137811504591</v>
       </c>
       <c r="I47" t="n">
-        <v>2793.966666666667</v>
+        <v>2839.375</v>
       </c>
       <c r="J47" t="n">
-        <v>50.28562946718649</v>
+        <v>51.1189635250765</v>
       </c>
       <c r="K47" t="n">
-        <v>46.56611111111111</v>
+        <v>47.32291666666666</v>
       </c>
       <c r="L47" t="n">
-        <v>2782.372964045918</v>
+        <v>2830.710652051715</v>
       </c>
       <c r="M47" t="n">
-        <v>2720.941666666667</v>
+        <v>2761.025</v>
       </c>
       <c r="N47" t="n">
-        <v>46.37288273409862</v>
+        <v>47.17851086752857</v>
       </c>
       <c r="O47" t="n">
-        <v>45.34902777777778</v>
+        <v>46.01708333333333</v>
       </c>
     </row>
     <row r="48">
@@ -3443,43 +3443,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>8587</v>
+        <v>9202</v>
       </c>
       <c r="D48" t="n">
-        <v>24.47225262994449</v>
+        <v>25.18171412011882</v>
       </c>
       <c r="E48" t="n">
-        <v>15.95</v>
+        <v>35.08333333333334</v>
       </c>
       <c r="F48" t="n">
-        <v>0.4078708771657415</v>
+        <v>0.4196952353353136</v>
       </c>
       <c r="G48" t="n">
-        <v>0.2658333333333333</v>
+        <v>0.5847222222222223</v>
       </c>
       <c r="H48" t="n">
-        <v>401.9148910217957</v>
+        <v>398.8258138929196</v>
       </c>
       <c r="I48" t="n">
-        <v>333.3166666666667</v>
+        <v>340.1833333333333</v>
       </c>
       <c r="J48" t="n">
-        <v>6.698581517029926</v>
+        <v>6.647096898215326</v>
       </c>
       <c r="K48" t="n">
-        <v>5.555277777777778</v>
+        <v>5.669722222222222</v>
       </c>
       <c r="L48" t="n">
-        <v>377.2225854829035</v>
+        <v>373.37683707259</v>
       </c>
       <c r="M48" t="n">
-        <v>307.7833333333334</v>
+        <v>313.8833333333333</v>
       </c>
       <c r="N48" t="n">
-        <v>6.287043091381723</v>
+        <v>6.222947284543166</v>
       </c>
       <c r="O48" t="n">
-        <v>5.129722222222223</v>
+        <v>5.231388888888889</v>
       </c>
     </row>
     <row r="49">
@@ -3494,43 +3494,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>5780</v>
+        <v>6319</v>
       </c>
       <c r="D49" t="n">
-        <v>292.8930940023068</v>
+        <v>283.5945244500712</v>
       </c>
       <c r="E49" t="n">
-        <v>114.55</v>
+        <v>106.2</v>
       </c>
       <c r="F49" t="n">
-        <v>4.881551566705113</v>
+        <v>4.726575407501187</v>
       </c>
       <c r="G49" t="n">
-        <v>1.909166666666667</v>
+        <v>1.77</v>
       </c>
       <c r="H49" t="n">
-        <v>662.1981225710015</v>
+        <v>640.4575871459695</v>
       </c>
       <c r="I49" t="n">
-        <v>619.9833333333333</v>
+        <v>598.5666666666666</v>
       </c>
       <c r="J49" t="n">
-        <v>11.03663537618336</v>
+        <v>10.67429311909949</v>
       </c>
       <c r="K49" t="n">
-        <v>10.33305555555556</v>
+        <v>9.976111111111113</v>
       </c>
       <c r="L49" t="n">
-        <v>365.7400627802691</v>
+        <v>356.0240196078431</v>
       </c>
       <c r="M49" t="n">
-        <v>231.0833333333333</v>
+        <v>220.2</v>
       </c>
       <c r="N49" t="n">
-        <v>6.095667713004484</v>
+        <v>5.933733660130718</v>
       </c>
       <c r="O49" t="n">
-        <v>3.851388888888889</v>
+        <v>3.67</v>
       </c>
     </row>
   </sheetData>
@@ -14685,19 +14685,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10412</v>
+        <v>10831</v>
       </c>
       <c r="C4" t="n">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="D4" t="n">
-        <v>4.273914713791779</v>
+        <v>4.219370325916351</v>
       </c>
       <c r="E4" t="n">
-        <v>5268.391797752809</v>
+        <v>5131.676914660832</v>
       </c>
       <c r="F4" t="n">
-        <v>1420.712420888934</v>
+        <v>1424.696596202044</v>
       </c>
     </row>
     <row r="5">
@@ -14707,19 +14707,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>355788</v>
+        <v>378363</v>
       </c>
       <c r="C5" t="n">
-        <v>259720</v>
+        <v>275514</v>
       </c>
       <c r="D5" t="n">
-        <v>72.9985272128346</v>
+        <v>72.81737379183483</v>
       </c>
       <c r="E5" t="n">
-        <v>2805.224925719237</v>
+        <v>2893.03943856864</v>
       </c>
       <c r="F5" t="n">
-        <v>4810.073803087396</v>
+        <v>4877.385439090317</v>
       </c>
     </row>
     <row r="6">
@@ -14729,19 +14729,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>108742</v>
+        <v>114879</v>
       </c>
       <c r="C6" t="n">
-        <v>5048</v>
+        <v>5330</v>
       </c>
       <c r="D6" t="n">
-        <v>4.64218057420316</v>
+        <v>4.63966434248209</v>
       </c>
       <c r="E6" t="n">
-        <v>1586.872999207607</v>
+        <v>1882.875110694184</v>
       </c>
       <c r="F6" t="n">
-        <v>3589.012339739908</v>
+        <v>3649.217590639714</v>
       </c>
     </row>
     <row r="7">
@@ -14751,19 +14751,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60862</v>
+        <v>62596</v>
       </c>
       <c r="C7" t="n">
-        <v>17969</v>
+        <v>18496</v>
       </c>
       <c r="D7" t="n">
-        <v>29.52416943248661</v>
+        <v>29.54821394338296</v>
       </c>
       <c r="E7" t="n">
-        <v>542.6518634314654</v>
+        <v>536.2528051470588</v>
       </c>
       <c r="F7" t="n">
-        <v>4395.639700184179</v>
+        <v>4368.450453514739</v>
       </c>
     </row>
     <row r="8"/>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard jue 30/07/2026 15:43:49,44
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -652,19 +652,19 @@
         <v>62.16238270093839</v>
       </c>
       <c r="T2" t="n">
-        <v>12469</v>
+        <v>12647</v>
       </c>
       <c r="U2" t="n">
-        <v>13.36113561632849</v>
+        <v>13.29959674231043</v>
       </c>
       <c r="V2" t="n">
-        <v>65.22575988451359</v>
+        <v>65.23286154819324</v>
       </c>
       <c r="W2" t="n">
-        <v>-7.430378051562164</v>
+        <v>-7.491916925580229</v>
       </c>
       <c r="X2" t="n">
-        <v>1.746226030191758</v>
+        <v>3.198694410444716</v>
       </c>
     </row>
     <row r="3">
@@ -728,19 +728,19 @@
         <v>77.97356828193833</v>
       </c>
       <c r="T3" t="n">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="U3" t="n">
-        <v>26.67578659370725</v>
+        <v>26.6304347826087</v>
       </c>
       <c r="V3" t="n">
-        <v>77.4281805745554</v>
+        <v>77.30978260869566</v>
       </c>
       <c r="W3" t="n">
-        <v>-17.5239197205365</v>
+        <v>-17.56927153163506</v>
       </c>
       <c r="X3" t="n">
-        <v>7.342143906020558</v>
+        <v>8.076358296622614</v>
       </c>
     </row>
     <row r="4">
@@ -804,19 +804,19 @@
         <v>39.73451327433628</v>
       </c>
       <c r="T4" t="n">
-        <v>997</v>
+        <v>1005</v>
       </c>
       <c r="U4" t="n">
-        <v>0.2006018054162488</v>
+        <v>0.1990049751243781</v>
       </c>
       <c r="V4" t="n">
-        <v>34.40320962888666</v>
+        <v>34.5273631840796</v>
       </c>
       <c r="W4" t="n">
-        <v>-23.42771677865455</v>
+        <v>-23.42931360894642</v>
       </c>
       <c r="X4" t="n">
-        <v>-11.76991150442478</v>
+        <v>-11.06194690265487</v>
       </c>
     </row>
     <row r="5">
@@ -880,19 +880,19 @@
         <v>56.85258964143426</v>
       </c>
       <c r="T5" t="n">
-        <v>2270</v>
+        <v>2298</v>
       </c>
       <c r="U5" t="n">
-        <v>38.28193832599119</v>
+        <v>38.16362053959965</v>
       </c>
       <c r="V5" t="n">
-        <v>52.51101321585902</v>
+        <v>52.26283724978242</v>
       </c>
       <c r="W5" t="n">
-        <v>-7.574635379188088</v>
+        <v>-7.692953165579631</v>
       </c>
       <c r="X5" t="n">
-        <v>-9.561752988047809</v>
+        <v>-8.446215139442231</v>
       </c>
     </row>
     <row r="6">
@@ -956,19 +956,19 @@
         <v>60.76099053978854</v>
       </c>
       <c r="T6" t="n">
-        <v>26727</v>
+        <v>27095</v>
       </c>
       <c r="U6" t="n">
-        <v>59.67373816739626</v>
+        <v>59.25078427754198</v>
       </c>
       <c r="V6" t="n">
-        <v>64.24589366558162</v>
+        <v>63.90477947960878</v>
       </c>
       <c r="W6" t="n">
-        <v>1.851673615365101</v>
+        <v>1.428719725510824</v>
       </c>
       <c r="X6" t="n">
-        <v>-7.042988313856427</v>
+        <v>-5.76307735114079</v>
       </c>
     </row>
     <row r="7">
@@ -1032,19 +1032,19 @@
         <v>61.65678803274061</v>
       </c>
       <c r="T7" t="n">
-        <v>28890</v>
+        <v>29151</v>
       </c>
       <c r="U7" t="n">
-        <v>35.93284873658705</v>
+        <v>35.88213097320846</v>
       </c>
       <c r="V7" t="n">
-        <v>61.83108341986847</v>
+        <v>61.81606119858667</v>
       </c>
       <c r="W7" t="n">
-        <v>-10.38383204241379</v>
+        <v>-10.43454980579239</v>
       </c>
       <c r="X7" t="n">
-        <v>1.926333615580017</v>
+        <v>2.847163420829805</v>
       </c>
     </row>
     <row r="8">
@@ -1108,19 +1108,19 @@
         <v>45.21468784135787</v>
       </c>
       <c r="T8" t="n">
-        <v>12043</v>
+        <v>12123</v>
       </c>
       <c r="U8" t="n">
-        <v>36.61047911649921</v>
+        <v>36.6493442217273</v>
       </c>
       <c r="V8" t="n">
-        <v>53.88192310885992</v>
+        <v>53.93054524457642</v>
       </c>
       <c r="W8" t="n">
-        <v>0.9075970057522156</v>
+        <v>0.9464621109802991</v>
       </c>
       <c r="X8" t="n">
-        <v>1.193177043945887</v>
+        <v>1.86538946307033</v>
       </c>
     </row>
     <row r="9">
@@ -1184,19 +1184,19 @@
         <v>69.81926219361227</v>
       </c>
       <c r="T9" t="n">
-        <v>4053</v>
+        <v>4126</v>
       </c>
       <c r="U9" t="n">
-        <v>60.00493461633359</v>
+        <v>59.57343674260785</v>
       </c>
       <c r="V9" t="n">
-        <v>68.04835924006909</v>
+        <v>67.69268056228793</v>
       </c>
       <c r="W9" t="n">
-        <v>1.747940310812417</v>
+        <v>1.316442437086685</v>
       </c>
       <c r="X9" t="n">
-        <v>0.3466204506065858</v>
+        <v>2.153998514483783</v>
       </c>
     </row>
     <row r="10">
@@ -1260,19 +1260,19 @@
         <v>33.59223300970874</v>
       </c>
       <c r="T10" t="n">
-        <v>1960</v>
+        <v>1986</v>
       </c>
       <c r="U10" t="n">
-        <v>2.704081632653061</v>
+        <v>2.668680765357502</v>
       </c>
       <c r="V10" t="n">
-        <v>36.63265306122449</v>
+        <v>36.90835850956697</v>
       </c>
       <c r="W10" t="n">
-        <v>-8.558054289677035</v>
+        <v>-8.593455156972594</v>
       </c>
       <c r="X10" t="n">
-        <v>90.29126213592234</v>
+        <v>92.81553398058252</v>
       </c>
     </row>
     <row r="11">
@@ -1336,19 +1336,19 @@
         <v>74.40353659771201</v>
       </c>
       <c r="T11" t="n">
-        <v>84764</v>
+        <v>87015</v>
       </c>
       <c r="U11" t="n">
-        <v>68.68717851918267</v>
+        <v>67.47572257656725</v>
       </c>
       <c r="V11" t="n">
-        <v>74.60714454249445</v>
+        <v>73.46319600068954</v>
       </c>
       <c r="W11" t="n">
-        <v>-3.139276221590578</v>
+        <v>-4.350732164205994</v>
       </c>
       <c r="X11" t="n">
-        <v>-4.651345909402806</v>
+        <v>-2.119258934296224</v>
       </c>
     </row>
     <row r="12">
@@ -1412,19 +1412,19 @@
         <v>75.20695379142226</v>
       </c>
       <c r="T12" t="n">
-        <v>313901</v>
+        <v>316256</v>
       </c>
       <c r="U12" t="n">
-        <v>56.96827980796493</v>
+        <v>56.92287260953152</v>
       </c>
       <c r="V12" t="n">
-        <v>74.83569660498055</v>
+        <v>74.83715723970454</v>
       </c>
       <c r="W12" t="n">
-        <v>-5.060605504167114</v>
+        <v>-5.106012702600523</v>
       </c>
       <c r="X12" t="n">
-        <v>13.02827678336736</v>
+        <v>13.87625621581527</v>
       </c>
     </row>
     <row r="13">
@@ -1488,19 +1488,19 @@
         <v>60.68562662261034</v>
       </c>
       <c r="T13" t="n">
-        <v>56356</v>
+        <v>56960</v>
       </c>
       <c r="U13" t="n">
-        <v>27.64568102775214</v>
+        <v>27.49824438202247</v>
       </c>
       <c r="V13" t="n">
-        <v>60.61111505429768</v>
+        <v>60.59339887640449</v>
       </c>
       <c r="W13" t="n">
-        <v>0.4920345797936818</v>
+        <v>0.3445979340640122</v>
       </c>
       <c r="X13" t="n">
-        <v>10.8410038549288</v>
+        <v>12.02895130202187</v>
       </c>
     </row>
     <row r="14">
@@ -1564,19 +1564,19 @@
         <v>62.77658116310946</v>
       </c>
       <c r="T14" t="n">
-        <v>5987</v>
+        <v>6051</v>
       </c>
       <c r="U14" t="n">
-        <v>33.62284950726575</v>
+        <v>33.56470004957858</v>
       </c>
       <c r="V14" t="n">
-        <v>60.04676799732754</v>
+        <v>60.02313667162452</v>
       </c>
       <c r="W14" t="n">
-        <v>-3.50266449312587</v>
+        <v>-3.560813950813035</v>
       </c>
       <c r="X14" t="n">
-        <v>17.23125122381046</v>
+        <v>18.48443313099667</v>
       </c>
     </row>
     <row r="15">
@@ -1640,19 +1640,19 @@
         <v>81.03823437985702</v>
       </c>
       <c r="T15" t="n">
-        <v>15521</v>
+        <v>15597</v>
       </c>
       <c r="U15" t="n">
-        <v>59.28741704787063</v>
+        <v>59.40244918894659</v>
       </c>
       <c r="V15" t="n">
-        <v>74.15759293859932</v>
+        <v>74.25787010322497</v>
       </c>
       <c r="W15" t="n">
-        <v>-11.43064325676102</v>
+        <v>-11.31561111568506</v>
       </c>
       <c r="X15" t="n">
-        <v>-3.506372396642835</v>
+        <v>-3.033882499222878</v>
       </c>
     </row>
   </sheetData>
@@ -1742,19 +1742,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12469</v>
+        <v>12647</v>
       </c>
       <c r="C4" t="n">
-        <v>1666</v>
+        <v>1682</v>
       </c>
       <c r="D4" t="n">
-        <v>13.36113561632849</v>
+        <v>13.29959674231043</v>
       </c>
       <c r="E4" t="n">
-        <v>8133</v>
+        <v>8250</v>
       </c>
       <c r="F4" t="n">
-        <v>65.22575988451359</v>
+        <v>65.23286154819324</v>
       </c>
     </row>
     <row r="5">
@@ -1764,19 +1764,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="C5" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D5" t="n">
-        <v>26.67578659370725</v>
+        <v>26.6304347826087</v>
       </c>
       <c r="E5" t="n">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="F5" t="n">
-        <v>77.4281805745554</v>
+        <v>77.30978260869566</v>
       </c>
     </row>
     <row r="6">
@@ -1786,19 +1786,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>997</v>
+        <v>1005</v>
       </c>
       <c r="C6" t="n">
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2006018054162488</v>
+        <v>0.1990049751243781</v>
       </c>
       <c r="E6" t="n">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="F6" t="n">
-        <v>34.40320962888666</v>
+        <v>34.5273631840796</v>
       </c>
     </row>
     <row r="7">
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2270</v>
+        <v>2298</v>
       </c>
       <c r="C7" t="n">
-        <v>869</v>
+        <v>877</v>
       </c>
       <c r="D7" t="n">
-        <v>38.28193832599119</v>
+        <v>38.16362053959965</v>
       </c>
       <c r="E7" t="n">
-        <v>1192</v>
+        <v>1201</v>
       </c>
       <c r="F7" t="n">
-        <v>52.51101321585902</v>
+        <v>52.26283724978242</v>
       </c>
     </row>
     <row r="8">
@@ -1830,19 +1830,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26727</v>
+        <v>27095</v>
       </c>
       <c r="C8" t="n">
-        <v>15949</v>
+        <v>16054</v>
       </c>
       <c r="D8" t="n">
-        <v>59.67373816739626</v>
+        <v>59.25078427754198</v>
       </c>
       <c r="E8" t="n">
-        <v>17171</v>
+        <v>17315</v>
       </c>
       <c r="F8" t="n">
-        <v>64.24589366558162</v>
+        <v>63.90477947960878</v>
       </c>
     </row>
     <row r="9">
@@ -1852,19 +1852,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>28890</v>
+        <v>29151</v>
       </c>
       <c r="C9" t="n">
-        <v>10381</v>
+        <v>10460</v>
       </c>
       <c r="D9" t="n">
-        <v>35.93284873658705</v>
+        <v>35.88213097320846</v>
       </c>
       <c r="E9" t="n">
-        <v>17863</v>
+        <v>18020</v>
       </c>
       <c r="F9" t="n">
-        <v>61.83108341986847</v>
+        <v>61.81606119858667</v>
       </c>
     </row>
     <row r="10">
@@ -1874,19 +1874,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>12043</v>
+        <v>12123</v>
       </c>
       <c r="C10" t="n">
-        <v>4409</v>
+        <v>4443</v>
       </c>
       <c r="D10" t="n">
-        <v>36.61047911649921</v>
+        <v>36.6493442217273</v>
       </c>
       <c r="E10" t="n">
-        <v>6489</v>
+        <v>6538</v>
       </c>
       <c r="F10" t="n">
-        <v>53.88192310885992</v>
+        <v>53.93054524457642</v>
       </c>
     </row>
     <row r="11">
@@ -1896,19 +1896,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4053</v>
+        <v>4126</v>
       </c>
       <c r="C11" t="n">
-        <v>2432</v>
+        <v>2458</v>
       </c>
       <c r="D11" t="n">
-        <v>60.00493461633359</v>
+        <v>59.57343674260785</v>
       </c>
       <c r="E11" t="n">
-        <v>2758</v>
+        <v>2793</v>
       </c>
       <c r="F11" t="n">
-        <v>68.04835924006909</v>
+        <v>67.69268056228793</v>
       </c>
     </row>
     <row r="12">
@@ -1918,19 +1918,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1960</v>
+        <v>1986</v>
       </c>
       <c r="C12" t="n">
         <v>53</v>
       </c>
       <c r="D12" t="n">
-        <v>2.704081632653061</v>
+        <v>2.668680765357502</v>
       </c>
       <c r="E12" t="n">
-        <v>718</v>
+        <v>733</v>
       </c>
       <c r="F12" t="n">
-        <v>36.63265306122449</v>
+        <v>36.90835850956697</v>
       </c>
     </row>
     <row r="13">
@@ -1940,19 +1940,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>84764</v>
+        <v>87015</v>
       </c>
       <c r="C13" t="n">
-        <v>58222</v>
+        <v>58714</v>
       </c>
       <c r="D13" t="n">
-        <v>68.68717851918267</v>
+        <v>67.47572257656725</v>
       </c>
       <c r="E13" t="n">
-        <v>63240</v>
+        <v>63924</v>
       </c>
       <c r="F13" t="n">
-        <v>74.60714454249445</v>
+        <v>73.46319600068954</v>
       </c>
     </row>
     <row r="14">
@@ -1962,19 +1962,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>313901</v>
+        <v>316256</v>
       </c>
       <c r="C14" t="n">
-        <v>178824</v>
+        <v>180022</v>
       </c>
       <c r="D14" t="n">
-        <v>56.96827980796493</v>
+        <v>56.92287260953152</v>
       </c>
       <c r="E14" t="n">
-        <v>234910</v>
+        <v>236677</v>
       </c>
       <c r="F14" t="n">
-        <v>74.83569660498055</v>
+        <v>74.83715723970454</v>
       </c>
     </row>
     <row r="15">
@@ -1984,19 +1984,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>56356</v>
+        <v>56960</v>
       </c>
       <c r="C15" t="n">
-        <v>15580</v>
+        <v>15663</v>
       </c>
       <c r="D15" t="n">
-        <v>27.64568102775214</v>
+        <v>27.49824438202247</v>
       </c>
       <c r="E15" t="n">
-        <v>34158</v>
+        <v>34514</v>
       </c>
       <c r="F15" t="n">
-        <v>60.61111505429768</v>
+        <v>60.59339887640449</v>
       </c>
     </row>
     <row r="16">
@@ -2006,19 +2006,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5987</v>
+        <v>6051</v>
       </c>
       <c r="C16" t="n">
-        <v>2013</v>
+        <v>2031</v>
       </c>
       <c r="D16" t="n">
-        <v>33.62284950726575</v>
+        <v>33.56470004957858</v>
       </c>
       <c r="E16" t="n">
-        <v>3595</v>
+        <v>3632</v>
       </c>
       <c r="F16" t="n">
-        <v>60.04676799732754</v>
+        <v>60.02313667162452</v>
       </c>
     </row>
     <row r="17">
@@ -2028,19 +2028,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15521</v>
+        <v>15597</v>
       </c>
       <c r="C17" t="n">
-        <v>9202</v>
+        <v>9265</v>
       </c>
       <c r="D17" t="n">
-        <v>59.28741704787063</v>
+        <v>59.40244918894659</v>
       </c>
       <c r="E17" t="n">
-        <v>11510</v>
+        <v>11582</v>
       </c>
       <c r="F17" t="n">
-        <v>74.15759293859932</v>
+        <v>74.25787010322497</v>
       </c>
     </row>
     <row r="18"/>
@@ -2141,40 +2141,40 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1666</v>
+        <v>1682</v>
       </c>
       <c r="D22" t="n">
-        <v>15.84285714285714</v>
+        <v>15.75559849385652</v>
       </c>
       <c r="E22" t="n">
-        <v>8.316666666666666</v>
+        <v>8.258333333333333</v>
       </c>
       <c r="F22" t="n">
-        <v>0.264047619047619</v>
+        <v>0.262593308230942</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1386111111111111</v>
+        <v>0.1376388888888889</v>
       </c>
       <c r="H22" t="n">
-        <v>269.7315813953488</v>
+        <v>269.6064669738863</v>
       </c>
       <c r="I22" t="n">
-        <v>130.1666666666667</v>
+        <v>130.2333333333333</v>
       </c>
       <c r="J22" t="n">
-        <v>4.495526356589148</v>
+        <v>4.493441116231438</v>
       </c>
       <c r="K22" t="n">
-        <v>2.169444444444444</v>
+        <v>2.170555555555555</v>
       </c>
       <c r="L22" t="n">
-        <v>247.1540000000001</v>
+        <v>246.9095698924731</v>
       </c>
       <c r="M22" t="n">
         <v>107.1</v>
       </c>
       <c r="N22" t="n">
-        <v>4.119233333333333</v>
+        <v>4.115159498207885</v>
       </c>
       <c r="O22" t="n">
         <v>1.785</v>
@@ -2192,43 +2192,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10803</v>
+        <v>10965</v>
       </c>
       <c r="D23" t="n">
-        <v>237.3427057298898</v>
+        <v>239.0794148046816</v>
       </c>
       <c r="E23" t="n">
-        <v>70.33333333333333</v>
+        <v>71.75</v>
       </c>
       <c r="F23" t="n">
-        <v>3.955711762164831</v>
+        <v>3.984656913411359</v>
       </c>
       <c r="G23" t="n">
-        <v>1.172222222222222</v>
+        <v>1.195833333333333</v>
       </c>
       <c r="H23" t="n">
-        <v>251.6846655970807</v>
+        <v>253.3141631034269</v>
       </c>
       <c r="I23" t="n">
-        <v>86.35833333333332</v>
+        <v>87.77500000000001</v>
       </c>
       <c r="J23" t="n">
-        <v>4.194744426618011</v>
+        <v>4.221902718390449</v>
       </c>
       <c r="K23" t="n">
-        <v>1.439305555555555</v>
+        <v>1.462916666666667</v>
       </c>
       <c r="L23" t="n">
-        <v>13.96958600729835</v>
+        <v>13.8345649749024</v>
       </c>
       <c r="M23" t="n">
-        <v>6.091666666666667</v>
+        <v>6.033333333333333</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2328264334549725</v>
+        <v>0.23057608291504</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1015277777777778</v>
+        <v>0.1005555555555556</v>
       </c>
     </row>
     <row r="24">
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -2294,40 +2294,40 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="D25" t="n">
-        <v>287.6420087064677</v>
+        <v>286.0467901234568</v>
       </c>
       <c r="E25" t="n">
         <v>15.56666666666667</v>
       </c>
       <c r="F25" t="n">
-        <v>4.794033478441128</v>
+        <v>4.767446502057613</v>
       </c>
       <c r="G25" t="n">
         <v>0.2594444444444444</v>
       </c>
       <c r="H25" t="n">
-        <v>298.4999374609131</v>
+        <v>296.8302296710118</v>
       </c>
       <c r="I25" t="n">
         <v>21.75</v>
       </c>
       <c r="J25" t="n">
-        <v>4.974998957681885</v>
+        <v>4.947170494516863</v>
       </c>
       <c r="K25" t="n">
         <v>0.3625</v>
       </c>
       <c r="L25" t="n">
-        <v>12.20093808630394</v>
+        <v>12.12535692116698</v>
       </c>
       <c r="M25" t="n">
         <v>2.216666666666667</v>
       </c>
       <c r="N25" t="n">
-        <v>0.2033489681050657</v>
+        <v>0.2020892820194496</v>
       </c>
       <c r="O25" t="n">
         <v>0.03694444444444445</v>
@@ -2372,19 +2372,19 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>995</v>
+        <v>1003</v>
       </c>
       <c r="D27" t="n">
-        <v>625.0669849246232</v>
+        <v>736.7651877700233</v>
       </c>
       <c r="E27" t="n">
-        <v>109.5833333333333</v>
+        <v>110.6333333333333</v>
       </c>
       <c r="F27" t="n">
-        <v>10.41778308207705</v>
+        <v>12.27941979616705</v>
       </c>
       <c r="G27" t="n">
-        <v>1.826388888888889</v>
+        <v>1.843888888888889</v>
       </c>
       <c r="H27" t="n">
         <v>5234.074379178606</v>
@@ -2423,19 +2423,19 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>869</v>
+        <v>877</v>
       </c>
       <c r="D28" t="n">
-        <v>23.74468738013042</v>
+        <v>23.85226149752946</v>
       </c>
       <c r="E28" t="n">
-        <v>15.9</v>
+        <v>15.91666666666667</v>
       </c>
       <c r="F28" t="n">
-        <v>0.3957447896688403</v>
+        <v>0.397537691625491</v>
       </c>
       <c r="G28" t="n">
-        <v>0.265</v>
+        <v>0.2652777777777778</v>
       </c>
       <c r="H28" t="n">
         <v>743.2020961775586</v>
@@ -2450,7 +2450,7 @@
         <v>12.26722222222222</v>
       </c>
       <c r="L28" t="n">
-        <v>719.6077887381834</v>
+        <v>719.6077887381832</v>
       </c>
       <c r="M28" t="n">
         <v>708.9666666666667</v>
@@ -2474,19 +2474,19 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1401</v>
+        <v>1421</v>
       </c>
       <c r="D29" t="n">
-        <v>247.4369260052343</v>
+        <v>256.8724724372507</v>
       </c>
       <c r="E29" t="n">
-        <v>70.56666666666666</v>
+        <v>72.21666666666667</v>
       </c>
       <c r="F29" t="n">
-        <v>4.123948766753906</v>
+        <v>4.281207873954179</v>
       </c>
       <c r="G29" t="n">
-        <v>1.176111111111111</v>
+        <v>1.203611111111111</v>
       </c>
       <c r="H29" t="n">
         <v>986.9147304479878</v>
@@ -2507,7 +2507,7 @@
         <v>814.6833333333333</v>
       </c>
       <c r="N29" t="n">
-        <v>12.21609866700413</v>
+        <v>12.21609866700414</v>
       </c>
       <c r="O29" t="n">
         <v>13.57805555555555</v>
@@ -2525,43 +2525,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>15949</v>
+        <v>16054</v>
       </c>
       <c r="D30" t="n">
-        <v>25.97564842100863</v>
+        <v>26.03604086209044</v>
       </c>
       <c r="E30" t="n">
         <v>35.21666666666667</v>
       </c>
       <c r="F30" t="n">
-        <v>0.4329274736834772</v>
+        <v>0.4339340143681741</v>
       </c>
       <c r="G30" t="n">
         <v>0.5869444444444445</v>
       </c>
       <c r="H30" t="n">
-        <v>403.3587395256829</v>
+        <v>408.7599069566159</v>
       </c>
       <c r="I30" t="n">
-        <v>229.9833333333333</v>
+        <v>243.5333333333333</v>
       </c>
       <c r="J30" t="n">
-        <v>6.722645658761382</v>
+        <v>6.812665115943598</v>
       </c>
       <c r="K30" t="n">
-        <v>3.833055555555555</v>
+        <v>4.058888888888889</v>
       </c>
       <c r="L30" t="n">
-        <v>377.2942855237715</v>
+        <v>382.4440776804068</v>
       </c>
       <c r="M30" t="n">
-        <v>201.6833333333333</v>
+        <v>213.55</v>
       </c>
       <c r="N30" t="n">
-        <v>6.288238092062857</v>
+        <v>6.374067961340113</v>
       </c>
       <c r="O30" t="n">
-        <v>3.361388888888889</v>
+        <v>3.559166666666667</v>
       </c>
     </row>
     <row r="31">
@@ -2576,22 +2576,22 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>10778</v>
+        <v>11041</v>
       </c>
       <c r="D31" t="n">
-        <v>1714.68124574751</v>
+        <v>1705.794076623494</v>
       </c>
       <c r="E31" t="n">
-        <v>1280.675</v>
+        <v>1279.883333333333</v>
       </c>
       <c r="F31" t="n">
-        <v>28.5780207624585</v>
+        <v>28.42990127705824</v>
       </c>
       <c r="G31" t="n">
-        <v>21.34458333333333</v>
+        <v>21.33138888888889</v>
       </c>
       <c r="H31" t="n">
-        <v>1969.435136085167</v>
+        <v>1969.435136085166</v>
       </c>
       <c r="I31" t="n">
         <v>1509.6</v>
@@ -2627,43 +2627,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>10381</v>
+        <v>10460</v>
       </c>
       <c r="D32" t="n">
-        <v>325.7597935330571</v>
+        <v>327.0361217335882</v>
       </c>
       <c r="E32" t="n">
         <v>35.3</v>
       </c>
       <c r="F32" t="n">
-        <v>5.42932989221762</v>
+        <v>5.450602028893138</v>
       </c>
       <c r="G32" t="n">
         <v>0.5883333333333333</v>
       </c>
       <c r="H32" t="n">
-        <v>661.5398333538059</v>
+        <v>659.9170174589733</v>
       </c>
       <c r="I32" t="n">
-        <v>410.95</v>
+        <v>414.7833333333334</v>
       </c>
       <c r="J32" t="n">
-        <v>11.0256638892301</v>
+        <v>10.99861695764956</v>
       </c>
       <c r="K32" t="n">
-        <v>6.849166666666666</v>
+        <v>6.913055555555556</v>
       </c>
       <c r="L32" t="n">
-        <v>251.3512099250706</v>
+        <v>250.9853151082617</v>
       </c>
       <c r="M32" t="n">
-        <v>70.26666666666667</v>
+        <v>69.93333333333334</v>
       </c>
       <c r="N32" t="n">
-        <v>4.18918683208451</v>
+        <v>4.183088585137695</v>
       </c>
       <c r="O32" t="n">
-        <v>1.171111111111111</v>
+        <v>1.165555555555556</v>
       </c>
     </row>
     <row r="33">
@@ -2678,43 +2678,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>18509</v>
+        <v>18691</v>
       </c>
       <c r="D33" t="n">
-        <v>380.8550047724531</v>
+        <v>383.9539903340289</v>
       </c>
       <c r="E33" t="n">
-        <v>70.01666666666667</v>
+        <v>72.33333333333333</v>
       </c>
       <c r="F33" t="n">
-        <v>6.347583412874218</v>
+        <v>6.399233172233814</v>
       </c>
       <c r="G33" t="n">
-        <v>1.166944444444444</v>
+        <v>1.205555555555555</v>
       </c>
       <c r="H33" t="n">
-        <v>670.2795347519393</v>
+        <v>673.1323341419275</v>
       </c>
       <c r="I33" t="n">
-        <v>401.1666666666667</v>
+        <v>409.3916666666667</v>
       </c>
       <c r="J33" t="n">
-        <v>11.17132557919899</v>
+        <v>11.21887223569879</v>
       </c>
       <c r="K33" t="n">
-        <v>6.686111111111112</v>
+        <v>6.823194444444444</v>
       </c>
       <c r="L33" t="n">
-        <v>268.6653858178478</v>
+        <v>270.3307891494359</v>
       </c>
       <c r="M33" t="n">
-        <v>62.65</v>
+        <v>62.48333333333333</v>
       </c>
       <c r="N33" t="n">
-        <v>4.477756430297465</v>
+        <v>4.505513152490598</v>
       </c>
       <c r="O33" t="n">
-        <v>1.044166666666667</v>
+        <v>1.041388888888889</v>
       </c>
     </row>
     <row r="34">
@@ -2729,43 +2729,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4409</v>
+        <v>4443</v>
       </c>
       <c r="D34" t="n">
-        <v>1077.047629848038</v>
+        <v>1091.020624202866</v>
       </c>
       <c r="E34" t="n">
-        <v>911.7166666666667</v>
+        <v>924.0666666666667</v>
       </c>
       <c r="F34" t="n">
-        <v>17.95079383080063</v>
+        <v>18.18367707004777</v>
       </c>
       <c r="G34" t="n">
-        <v>15.19527777777778</v>
+        <v>15.40111111111111</v>
       </c>
       <c r="H34" t="n">
-        <v>1751.806763035622</v>
+        <v>1751.367634408602</v>
       </c>
       <c r="I34" t="n">
-        <v>1508.683333333333</v>
+        <v>1508.583333333333</v>
       </c>
       <c r="J34" t="n">
-        <v>29.19677938392703</v>
+        <v>29.1894605734767</v>
       </c>
       <c r="K34" t="n">
-        <v>25.14472222222222</v>
+        <v>25.14305555555556</v>
       </c>
       <c r="L34" t="n">
-        <v>613.2702331784546</v>
+        <v>613.1157032258064</v>
       </c>
       <c r="M34" t="n">
-        <v>502.9083333333333</v>
+        <v>502.9</v>
       </c>
       <c r="N34" t="n">
-        <v>10.22117055297424</v>
+        <v>10.21859505376344</v>
       </c>
       <c r="O34" t="n">
-        <v>8.381805555555555</v>
+        <v>8.381666666666666</v>
       </c>
     </row>
     <row r="35">
@@ -2780,40 +2780,40 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7634</v>
+        <v>7680</v>
       </c>
       <c r="D35" t="n">
-        <v>1327.760097371409</v>
+        <v>1355.200323350695</v>
       </c>
       <c r="E35" t="n">
-        <v>1086.491666666667</v>
+        <v>1100.466666666667</v>
       </c>
       <c r="F35" t="n">
-        <v>22.12933495619014</v>
+        <v>22.58667205584491</v>
       </c>
       <c r="G35" t="n">
-        <v>18.10819444444444</v>
+        <v>18.34111111111111</v>
       </c>
       <c r="H35" t="n">
-        <v>2014.113464042468</v>
+        <v>2013.66546760789</v>
       </c>
       <c r="I35" t="n">
-        <v>1680.375</v>
+        <v>1680.291666666667</v>
       </c>
       <c r="J35" t="n">
-        <v>33.56855773404114</v>
+        <v>33.56109112679817</v>
       </c>
       <c r="K35" t="n">
-        <v>28.00625</v>
+        <v>28.00486111111111</v>
       </c>
       <c r="L35" t="n">
-        <v>644.2678811097757</v>
+        <v>644.1454841293681</v>
       </c>
       <c r="M35" t="n">
         <v>458.7</v>
       </c>
       <c r="N35" t="n">
-        <v>10.73779801849626</v>
+        <v>10.7357580688228</v>
       </c>
       <c r="O35" t="n">
         <v>7.645</v>
@@ -2831,43 +2831,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2432</v>
+        <v>2458</v>
       </c>
       <c r="D36" t="n">
-        <v>25.26774259868421</v>
+        <v>25.37641036072688</v>
       </c>
       <c r="E36" t="n">
-        <v>33.99166666666666</v>
+        <v>35.1</v>
       </c>
       <c r="F36" t="n">
-        <v>0.4211290433114034</v>
+        <v>0.4229401726787813</v>
       </c>
       <c r="G36" t="n">
-        <v>0.5665277777777777</v>
+        <v>0.5850000000000001</v>
       </c>
       <c r="H36" t="n">
-        <v>3001.039899680803</v>
+        <v>2953.639493876346</v>
       </c>
       <c r="I36" t="n">
-        <v>2917.183333333333</v>
+        <v>2883.45</v>
       </c>
       <c r="J36" t="n">
-        <v>50.01733166134672</v>
+        <v>49.22732489793911</v>
       </c>
       <c r="K36" t="n">
-        <v>48.61972222222222</v>
+        <v>48.0575</v>
       </c>
       <c r="L36" t="n">
-        <v>2975.308732330141</v>
+        <v>2927.620835177807</v>
       </c>
       <c r="M36" t="n">
-        <v>2886.166666666667</v>
+        <v>2850.25</v>
       </c>
       <c r="N36" t="n">
-        <v>49.58847887216901</v>
+        <v>48.79368058629678</v>
       </c>
       <c r="O36" t="n">
-        <v>48.10277777777777</v>
+        <v>47.50416666666667</v>
       </c>
     </row>
     <row r="37">
@@ -2882,43 +2882,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1621</v>
+        <v>1668</v>
       </c>
       <c r="D37" t="n">
-        <v>2696.191610117212</v>
+        <v>2677.354226618705</v>
       </c>
       <c r="E37" t="n">
-        <v>2525.516666666667</v>
+        <v>2493.416666666667</v>
       </c>
       <c r="F37" t="n">
-        <v>44.93652683528686</v>
+        <v>44.62257044364509</v>
       </c>
       <c r="G37" t="n">
-        <v>42.09194444444445</v>
+        <v>41.55694444444444</v>
       </c>
       <c r="H37" t="n">
-        <v>3415.084254327564</v>
+        <v>3384.641198017669</v>
       </c>
       <c r="I37" t="n">
-        <v>3515.458333333333</v>
+        <v>3296.966666666667</v>
       </c>
       <c r="J37" t="n">
-        <v>56.91807090545939</v>
+        <v>56.41068663362781</v>
       </c>
       <c r="K37" t="n">
-        <v>58.59097222222222</v>
+        <v>54.94944444444445</v>
       </c>
       <c r="L37" t="n">
-        <v>587.6498557478916</v>
+        <v>577.6309523809524</v>
       </c>
       <c r="M37" t="n">
-        <v>341.7666666666667</v>
+        <v>336.0333333333334</v>
       </c>
       <c r="N37" t="n">
-        <v>9.794164262464861</v>
+        <v>9.62718253968254</v>
       </c>
       <c r="O37" t="n">
-        <v>5.696111111111112</v>
+        <v>5.600555555555556</v>
       </c>
     </row>
     <row r="38">
@@ -2948,28 +2948,28 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>91.14285714285715</v>
+        <v>101.7916666666667</v>
       </c>
       <c r="I38" t="n">
-        <v>2.216666666666667</v>
+        <v>2.291666666666667</v>
       </c>
       <c r="J38" t="n">
-        <v>1.519047619047619</v>
+        <v>1.696527777777778</v>
       </c>
       <c r="K38" t="n">
-        <v>0.03694444444444445</v>
+        <v>0.03819444444444445</v>
       </c>
       <c r="L38" t="n">
-        <v>91.14285714285715</v>
+        <v>101.7916666666667</v>
       </c>
       <c r="M38" t="n">
-        <v>2.216666666666667</v>
+        <v>2.291666666666667</v>
       </c>
       <c r="N38" t="n">
-        <v>1.519047619047619</v>
+        <v>1.696527777777778</v>
       </c>
       <c r="O38" t="n">
-        <v>0.03694444444444445</v>
+        <v>0.03819444444444445</v>
       </c>
     </row>
     <row r="39">
@@ -2984,43 +2984,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1907</v>
+        <v>1933</v>
       </c>
       <c r="D39" t="n">
-        <v>177.0102954029016</v>
+        <v>180.3992757371961</v>
       </c>
       <c r="E39" t="n">
-        <v>78.18333333333334</v>
+        <v>79.18333333333334</v>
       </c>
       <c r="F39" t="n">
-        <v>2.95017159004836</v>
+        <v>3.006654595619934</v>
       </c>
       <c r="G39" t="n">
-        <v>1.303055555555556</v>
+        <v>1.319722222222222</v>
       </c>
       <c r="H39" t="n">
-        <v>494.6693649937039</v>
+        <v>494.9470420017873</v>
       </c>
       <c r="I39" t="n">
-        <v>426.15</v>
+        <v>428.9166666666667</v>
       </c>
       <c r="J39" t="n">
-        <v>8.244489416561731</v>
+        <v>8.249117366696455</v>
       </c>
       <c r="K39" t="n">
-        <v>7.1025</v>
+        <v>7.148611111111111</v>
       </c>
       <c r="L39" t="n">
-        <v>315.7854380284224</v>
+        <v>314.2220643431635</v>
       </c>
       <c r="M39" t="n">
-        <v>160.9</v>
+        <v>156.5333333333333</v>
       </c>
       <c r="N39" t="n">
-        <v>5.26309063380704</v>
+        <v>5.237034405719392</v>
       </c>
       <c r="O39" t="n">
-        <v>2.681666666666667</v>
+        <v>2.608888888888889</v>
       </c>
     </row>
     <row r="40">
@@ -3035,43 +3035,43 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>58222</v>
+        <v>58714</v>
       </c>
       <c r="D40" t="n">
-        <v>433.8536446703995</v>
+        <v>499.8174211715548</v>
       </c>
       <c r="E40" t="n">
-        <v>44.41666666666666</v>
+        <v>50.08333333333334</v>
       </c>
       <c r="F40" t="n">
-        <v>7.230894077839991</v>
+        <v>8.330290352859247</v>
       </c>
       <c r="G40" t="n">
-        <v>0.7402777777777777</v>
+        <v>0.8347222222222224</v>
       </c>
       <c r="H40" t="n">
-        <v>559.491776377834</v>
+        <v>615.368107337996</v>
       </c>
       <c r="I40" t="n">
-        <v>169.4666666666666</v>
+        <v>212.1166666666667</v>
       </c>
       <c r="J40" t="n">
-        <v>9.324862939630565</v>
+        <v>10.25613512229993</v>
       </c>
       <c r="K40" t="n">
-        <v>2.824444444444444</v>
+        <v>3.535277777777778</v>
       </c>
       <c r="L40" t="n">
-        <v>89.25040269342487</v>
+        <v>90.70259971445611</v>
       </c>
       <c r="M40" t="n">
-        <v>45.56666666666667</v>
+        <v>49.45</v>
       </c>
       <c r="N40" t="n">
-        <v>1.487506711557081</v>
+        <v>1.511709995240935</v>
       </c>
       <c r="O40" t="n">
-        <v>0.7594444444444445</v>
+        <v>0.8241666666666667</v>
       </c>
     </row>
     <row r="41">
@@ -3086,43 +3086,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>26542</v>
+        <v>28301</v>
       </c>
       <c r="D41" t="n">
-        <v>763.7284461105668</v>
+        <v>837.8153557589249</v>
       </c>
       <c r="E41" t="n">
-        <v>701.1666666666666</v>
+        <v>737.6</v>
       </c>
       <c r="F41" t="n">
-        <v>12.72880743517612</v>
+        <v>13.96358926264875</v>
       </c>
       <c r="G41" t="n">
-        <v>11.68611111111111</v>
+        <v>12.29333333333333</v>
       </c>
       <c r="H41" t="n">
-        <v>880.0281653180266</v>
+        <v>926.8915458195862</v>
       </c>
       <c r="I41" t="n">
-        <v>823.9666666666667</v>
+        <v>851.425</v>
       </c>
       <c r="J41" t="n">
-        <v>14.66713608863378</v>
+        <v>15.44819243032644</v>
       </c>
       <c r="K41" t="n">
-        <v>13.73277777777778</v>
+        <v>14.19041666666667</v>
       </c>
       <c r="L41" t="n">
-        <v>110.5443011652782</v>
+        <v>109.5894082968874</v>
       </c>
       <c r="M41" t="n">
-        <v>88.08333333333333</v>
+        <v>87.84999999999999</v>
       </c>
       <c r="N41" t="n">
-        <v>1.842405019421302</v>
+        <v>1.826490138281456</v>
       </c>
       <c r="O41" t="n">
-        <v>1.468055555555555</v>
+        <v>1.464166666666667</v>
       </c>
     </row>
     <row r="42">
@@ -3137,43 +3137,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>178824</v>
+        <v>180022</v>
       </c>
       <c r="D42" t="n">
-        <v>10.63374416558553</v>
+        <v>10.78492823099399</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0.1772290694264255</v>
+        <v>0.1797488038498998</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>454.7356620713077</v>
+        <v>455.2786757257804</v>
       </c>
       <c r="I42" t="n">
-        <v>182.45</v>
+        <v>183.5666666666667</v>
       </c>
       <c r="J42" t="n">
-        <v>7.57892770118846</v>
+        <v>7.587977928763004</v>
       </c>
       <c r="K42" t="n">
-        <v>3.040833333333333</v>
+        <v>3.059444444444444</v>
       </c>
       <c r="L42" t="n">
-        <v>443.6333169981</v>
+        <v>443.8825595075036</v>
       </c>
       <c r="M42" t="n">
-        <v>173.1</v>
+        <v>174.0333333333333</v>
       </c>
       <c r="N42" t="n">
-        <v>7.393888616635001</v>
+        <v>7.398042658458395</v>
       </c>
       <c r="O42" t="n">
-        <v>2.885</v>
+        <v>2.900555555555556</v>
       </c>
     </row>
     <row r="43">
@@ -3188,43 +3188,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>135077</v>
+        <v>136234</v>
       </c>
       <c r="D43" t="n">
-        <v>158.4470555066123</v>
+        <v>158.0131446628594</v>
       </c>
       <c r="E43" t="n">
-        <v>89.63333333333334</v>
+        <v>89.43333333333334</v>
       </c>
       <c r="F43" t="n">
-        <v>2.640784258443539</v>
+        <v>2.633552411047659</v>
       </c>
       <c r="G43" t="n">
-        <v>1.493888888888889</v>
+        <v>1.490555555555556</v>
       </c>
       <c r="H43" t="n">
-        <v>559.8444851731206</v>
+        <v>559.4842872999272</v>
       </c>
       <c r="I43" t="n">
-        <v>265.95</v>
+        <v>266.8333333333333</v>
       </c>
       <c r="J43" t="n">
-        <v>9.330741419552011</v>
+        <v>9.324738121665453</v>
       </c>
       <c r="K43" t="n">
-        <v>4.4325</v>
+        <v>4.447222222222222</v>
       </c>
       <c r="L43" t="n">
-        <v>401.2843708132173</v>
+        <v>400.5331938847704</v>
       </c>
       <c r="M43" t="n">
-        <v>124.6833333333333</v>
+        <v>124.775</v>
       </c>
       <c r="N43" t="n">
-        <v>6.688072846886955</v>
+        <v>6.675553231412841</v>
       </c>
       <c r="O43" t="n">
-        <v>2.078055555555556</v>
+        <v>2.079583333333333</v>
       </c>
     </row>
     <row r="44">
@@ -3239,43 +3239,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>15580</v>
+        <v>15663</v>
       </c>
       <c r="D44" t="n">
-        <v>23.78660248181429</v>
+        <v>23.82856732426738</v>
       </c>
       <c r="E44" t="n">
         <v>35.11666666666667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.3964433746969049</v>
+        <v>0.3971427887377897</v>
       </c>
       <c r="G44" t="n">
         <v>0.5852777777777778</v>
       </c>
       <c r="H44" t="n">
-        <v>1045.016539155539</v>
+        <v>1035.069069343066</v>
       </c>
       <c r="I44" t="n">
-        <v>883.6833333333333</v>
+        <v>871.3666666666667</v>
       </c>
       <c r="J44" t="n">
-        <v>17.41694231925899</v>
+        <v>17.25115115571776</v>
       </c>
       <c r="K44" t="n">
-        <v>14.72805555555555</v>
+        <v>14.52277777777778</v>
       </c>
       <c r="L44" t="n">
-        <v>1020.208036809816</v>
+        <v>1009.963363279057</v>
       </c>
       <c r="M44" t="n">
-        <v>854.7333333333333</v>
+        <v>843.9833333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>17.0034672801636</v>
+        <v>16.83272272131761</v>
       </c>
       <c r="O44" t="n">
-        <v>14.24555555555556</v>
+        <v>14.06638888888889</v>
       </c>
     </row>
     <row r="45">
@@ -3290,43 +3290,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>40776</v>
+        <v>41297</v>
       </c>
       <c r="D45" t="n">
-        <v>269.3652540710222</v>
+        <v>268.0716286897353</v>
       </c>
       <c r="E45" t="n">
-        <v>29.26666666666667</v>
+        <v>29.2</v>
       </c>
       <c r="F45" t="n">
-        <v>4.489420901183703</v>
+        <v>4.467860478162256</v>
       </c>
       <c r="G45" t="n">
-        <v>0.4877777777777778</v>
+        <v>0.4866666666666666</v>
       </c>
       <c r="H45" t="n">
-        <v>1109.394442379511</v>
+        <v>1102.388018471002</v>
       </c>
       <c r="I45" t="n">
-        <v>940.25</v>
+        <v>937.9666666666667</v>
       </c>
       <c r="J45" t="n">
-        <v>18.48990737299185</v>
+        <v>18.37313364118337</v>
       </c>
       <c r="K45" t="n">
-        <v>15.67083333333333</v>
+        <v>15.63277777777778</v>
       </c>
       <c r="L45" t="n">
-        <v>838.5768925113717</v>
+        <v>834.0250546441005</v>
       </c>
       <c r="M45" t="n">
-        <v>560.1416666666667</v>
+        <v>562.1833333333333</v>
       </c>
       <c r="N45" t="n">
-        <v>13.9762815418562</v>
+        <v>13.90041757740168</v>
       </c>
       <c r="O45" t="n">
-        <v>9.335694444444444</v>
+        <v>9.369722222222221</v>
       </c>
     </row>
     <row r="46">
@@ -3341,19 +3341,19 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2013</v>
+        <v>2031</v>
       </c>
       <c r="D46" t="n">
-        <v>22.5016724623282</v>
+        <v>22.61802888560643</v>
       </c>
       <c r="E46" t="n">
-        <v>15.8</v>
+        <v>15.81666666666667</v>
       </c>
       <c r="F46" t="n">
-        <v>0.3750278743721366</v>
+        <v>0.3769671480934406</v>
       </c>
       <c r="G46" t="n">
-        <v>0.2633333333333334</v>
+        <v>0.2636111111111111</v>
       </c>
       <c r="H46" t="n">
         <v>2722.767684108527</v>
@@ -3392,43 +3392,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3974</v>
+        <v>4020</v>
       </c>
       <c r="D47" t="n">
-        <v>229.3043449085723</v>
+        <v>229.5184618573798</v>
       </c>
       <c r="E47" t="n">
-        <v>64.82499999999999</v>
+        <v>65.125</v>
       </c>
       <c r="F47" t="n">
-        <v>3.82173908180954</v>
+        <v>3.825307697622996</v>
       </c>
       <c r="G47" t="n">
-        <v>1.080416666666667</v>
+        <v>1.085416666666667</v>
       </c>
       <c r="H47" t="n">
-        <v>3067.137811504591</v>
+        <v>3065.697476591761</v>
       </c>
       <c r="I47" t="n">
-        <v>2839.375</v>
+        <v>2839.333333333333</v>
       </c>
       <c r="J47" t="n">
-        <v>51.1189635250765</v>
+        <v>51.094957943196</v>
       </c>
       <c r="K47" t="n">
-        <v>47.32291666666666</v>
+        <v>47.32222222222222</v>
       </c>
       <c r="L47" t="n">
-        <v>2830.710652051715</v>
+        <v>2829.254887640449</v>
       </c>
       <c r="M47" t="n">
-        <v>2761.025</v>
+        <v>2760.65</v>
       </c>
       <c r="N47" t="n">
-        <v>47.17851086752857</v>
+        <v>47.15424812734083</v>
       </c>
       <c r="O47" t="n">
-        <v>46.01708333333333</v>
+        <v>46.01083333333333</v>
       </c>
     </row>
     <row r="48">
@@ -3443,43 +3443,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9202</v>
+        <v>9265</v>
       </c>
       <c r="D48" t="n">
-        <v>25.18171412011882</v>
+        <v>25.25211009174312</v>
       </c>
       <c r="E48" t="n">
-        <v>35.08333333333334</v>
+        <v>35.1</v>
       </c>
       <c r="F48" t="n">
-        <v>0.4196952353353136</v>
+        <v>0.420868501529052</v>
       </c>
       <c r="G48" t="n">
-        <v>0.5847222222222223</v>
+        <v>0.5850000000000001</v>
       </c>
       <c r="H48" t="n">
-        <v>398.8258138929196</v>
+        <v>397.865464930826</v>
       </c>
       <c r="I48" t="n">
-        <v>340.1833333333333</v>
+        <v>337.9333333333333</v>
       </c>
       <c r="J48" t="n">
-        <v>6.647096898215326</v>
+        <v>6.631091082180433</v>
       </c>
       <c r="K48" t="n">
-        <v>5.669722222222222</v>
+        <v>5.632222222222222</v>
       </c>
       <c r="L48" t="n">
-        <v>373.37683707259</v>
+        <v>372.3851192463188</v>
       </c>
       <c r="M48" t="n">
-        <v>313.8833333333333</v>
+        <v>310.9833333333333</v>
       </c>
       <c r="N48" t="n">
-        <v>6.222947284543166</v>
+        <v>6.206418654105313</v>
       </c>
       <c r="O48" t="n">
-        <v>5.231388888888889</v>
+        <v>5.183055555555556</v>
       </c>
     </row>
     <row r="49">
@@ -3494,43 +3494,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6319</v>
+        <v>6332</v>
       </c>
       <c r="D49" t="n">
-        <v>283.5945244500712</v>
+        <v>284.0647425773847</v>
       </c>
       <c r="E49" t="n">
-        <v>106.2</v>
+        <v>106.6</v>
       </c>
       <c r="F49" t="n">
-        <v>4.726575407501187</v>
+        <v>4.734412376289746</v>
       </c>
       <c r="G49" t="n">
-        <v>1.77</v>
+        <v>1.776666666666667</v>
       </c>
       <c r="H49" t="n">
-        <v>640.4575871459695</v>
+        <v>640.2324615718863</v>
       </c>
       <c r="I49" t="n">
-        <v>598.5666666666666</v>
+        <v>598.3833333333333</v>
       </c>
       <c r="J49" t="n">
-        <v>10.67429311909949</v>
+        <v>10.67054102619811</v>
       </c>
       <c r="K49" t="n">
-        <v>9.976111111111113</v>
+        <v>9.973055555555556</v>
       </c>
       <c r="L49" t="n">
-        <v>356.0240196078431</v>
+        <v>355.8073108467764</v>
       </c>
       <c r="M49" t="n">
-        <v>220.2</v>
+        <v>219.3</v>
       </c>
       <c r="N49" t="n">
-        <v>5.933733660130718</v>
+        <v>5.930121847446273</v>
       </c>
       <c r="O49" t="n">
-        <v>3.67</v>
+        <v>3.655</v>
       </c>
     </row>
   </sheetData>
@@ -14685,19 +14685,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10831</v>
+        <v>11251</v>
       </c>
       <c r="C4" t="n">
-        <v>457</v>
+        <v>478</v>
       </c>
       <c r="D4" t="n">
-        <v>4.219370325916351</v>
+        <v>4.248511243445027</v>
       </c>
       <c r="E4" t="n">
-        <v>5131.676914660832</v>
+        <v>4918.933786610879</v>
       </c>
       <c r="F4" t="n">
-        <v>1424.696596202044</v>
+        <v>1395.479407685881</v>
       </c>
     </row>
     <row r="5">
@@ -14707,19 +14707,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>378363</v>
+        <v>381565</v>
       </c>
       <c r="C5" t="n">
-        <v>275514</v>
+        <v>277390</v>
       </c>
       <c r="D5" t="n">
-        <v>72.81737379183483</v>
+        <v>72.697967580884</v>
       </c>
       <c r="E5" t="n">
-        <v>2893.03943856864</v>
+        <v>2895.874611657955</v>
       </c>
       <c r="F5" t="n">
-        <v>4877.385439090317</v>
+        <v>4963.101685769139</v>
       </c>
     </row>
     <row r="6">
@@ -14729,19 +14729,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>114879</v>
+        <v>117083</v>
       </c>
       <c r="C6" t="n">
-        <v>5330</v>
+        <v>5428</v>
       </c>
       <c r="D6" t="n">
-        <v>4.63966434248209</v>
+        <v>4.63602743353006</v>
       </c>
       <c r="E6" t="n">
-        <v>1882.875110694184</v>
+        <v>1881.129489683124</v>
       </c>
       <c r="F6" t="n">
-        <v>3649.217590639714</v>
+        <v>3714.470015288075</v>
       </c>
     </row>
     <row r="7">
@@ -14751,19 +14751,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62596</v>
+        <v>63147</v>
       </c>
       <c r="C7" t="n">
-        <v>18496</v>
+        <v>18624</v>
       </c>
       <c r="D7" t="n">
-        <v>29.54821394338296</v>
+        <v>29.49308755760369</v>
       </c>
       <c r="E7" t="n">
-        <v>536.2528051470588</v>
+        <v>535.1113479381443</v>
       </c>
       <c r="F7" t="n">
-        <v>4368.450453514739</v>
+        <v>4363.276148732116</v>
       </c>
     </row>
     <row r="8"/>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard vie 31/07/2026  8:44:10,71
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -652,19 +652,19 @@
         <v>62.16238270093839</v>
       </c>
       <c r="T2" t="n">
-        <v>12647</v>
+        <v>12813</v>
       </c>
       <c r="U2" t="n">
-        <v>13.29959674231043</v>
+        <v>13.38484351830173</v>
       </c>
       <c r="V2" t="n">
-        <v>65.23286154819324</v>
+        <v>65.29306173417623</v>
       </c>
       <c r="W2" t="n">
-        <v>-7.491916925580229</v>
+        <v>-7.406670149588933</v>
       </c>
       <c r="X2" t="n">
-        <v>3.198694410444716</v>
+        <v>4.553243574051407</v>
       </c>
     </row>
     <row r="3">
@@ -728,19 +728,19 @@
         <v>77.97356828193833</v>
       </c>
       <c r="T3" t="n">
-        <v>736</v>
+        <v>745</v>
       </c>
       <c r="U3" t="n">
-        <v>26.6304347826087</v>
+        <v>26.71140939597316</v>
       </c>
       <c r="V3" t="n">
-        <v>77.30978260869566</v>
+        <v>77.58389261744966</v>
       </c>
       <c r="W3" t="n">
-        <v>-17.56927153163506</v>
+        <v>-17.4882969182706</v>
       </c>
       <c r="X3" t="n">
-        <v>8.076358296622614</v>
+        <v>9.397944199706314</v>
       </c>
     </row>
     <row r="4">
@@ -804,19 +804,19 @@
         <v>39.73451327433628</v>
       </c>
       <c r="T4" t="n">
-        <v>1005</v>
+        <v>1027</v>
       </c>
       <c r="U4" t="n">
-        <v>0.1990049751243781</v>
+        <v>0.1947419668938656</v>
       </c>
       <c r="V4" t="n">
-        <v>34.5273631840796</v>
+        <v>34.85881207400195</v>
       </c>
       <c r="W4" t="n">
-        <v>-23.42931360894642</v>
+        <v>-23.43357661717693</v>
       </c>
       <c r="X4" t="n">
-        <v>-11.06194690265487</v>
+        <v>-9.115044247787612</v>
       </c>
     </row>
     <row r="5">
@@ -880,19 +880,19 @@
         <v>56.85258964143426</v>
       </c>
       <c r="T5" t="n">
-        <v>2298</v>
+        <v>2357</v>
       </c>
       <c r="U5" t="n">
-        <v>38.16362053959965</v>
+        <v>38.56597369537548</v>
       </c>
       <c r="V5" t="n">
-        <v>52.26283724978242</v>
+        <v>52.69410267288927</v>
       </c>
       <c r="W5" t="n">
-        <v>-7.692953165579631</v>
+        <v>-7.290600009803804</v>
       </c>
       <c r="X5" t="n">
-        <v>-8.446215139442231</v>
+        <v>-6.095617529880478</v>
       </c>
     </row>
     <row r="6">
@@ -956,19 +956,19 @@
         <v>60.76099053978854</v>
       </c>
       <c r="T6" t="n">
-        <v>27095</v>
+        <v>27487</v>
       </c>
       <c r="U6" t="n">
-        <v>59.25078427754198</v>
+        <v>59.83192054425729</v>
       </c>
       <c r="V6" t="n">
-        <v>63.90477947960878</v>
+        <v>64.41954378433441</v>
       </c>
       <c r="W6" t="n">
-        <v>1.428719725510824</v>
+        <v>2.009855992226129</v>
       </c>
       <c r="X6" t="n">
-        <v>-5.76307735114079</v>
+        <v>-4.399693934335003</v>
       </c>
     </row>
     <row r="7">
@@ -1032,19 +1032,19 @@
         <v>61.65678803274061</v>
       </c>
       <c r="T7" t="n">
-        <v>29151</v>
+        <v>29682</v>
       </c>
       <c r="U7" t="n">
-        <v>35.88213097320846</v>
+        <v>35.82305774543494</v>
       </c>
       <c r="V7" t="n">
-        <v>61.81606119858667</v>
+        <v>61.85567010309278</v>
       </c>
       <c r="W7" t="n">
-        <v>-10.43454980579239</v>
+        <v>-10.4936230335659</v>
       </c>
       <c r="X7" t="n">
-        <v>2.847163420829805</v>
+        <v>4.720575783234547</v>
       </c>
     </row>
     <row r="8">
@@ -1108,19 +1108,19 @@
         <v>45.21468784135787</v>
       </c>
       <c r="T8" t="n">
-        <v>12123</v>
+        <v>12432</v>
       </c>
       <c r="U8" t="n">
-        <v>36.6493442217273</v>
+        <v>36.58301158301158</v>
       </c>
       <c r="V8" t="n">
-        <v>53.93054524457642</v>
+        <v>53.9494851994852</v>
       </c>
       <c r="W8" t="n">
-        <v>0.9464621109802991</v>
+        <v>0.8801294722645849</v>
       </c>
       <c r="X8" t="n">
-        <v>1.86538946307033</v>
+        <v>4.461809931938492</v>
       </c>
     </row>
     <row r="9">
@@ -1184,19 +1184,19 @@
         <v>69.81926219361227</v>
       </c>
       <c r="T9" t="n">
-        <v>4126</v>
+        <v>4204</v>
       </c>
       <c r="U9" t="n">
-        <v>59.57343674260785</v>
+        <v>60.08563273073264</v>
       </c>
       <c r="V9" t="n">
-        <v>67.69268056228793</v>
+        <v>68.22074215033301</v>
       </c>
       <c r="W9" t="n">
-        <v>1.316442437086685</v>
+        <v>1.828638425211473</v>
       </c>
       <c r="X9" t="n">
-        <v>2.153998514483783</v>
+        <v>4.085169596434761</v>
       </c>
     </row>
     <row r="10">
@@ -1260,19 +1260,19 @@
         <v>33.59223300970874</v>
       </c>
       <c r="T10" t="n">
-        <v>1986</v>
+        <v>2028</v>
       </c>
       <c r="U10" t="n">
-        <v>2.668680765357502</v>
+        <v>2.761341222879684</v>
       </c>
       <c r="V10" t="n">
-        <v>36.90835850956697</v>
+        <v>36.93293885601578</v>
       </c>
       <c r="W10" t="n">
-        <v>-8.593455156972594</v>
+        <v>-8.500794699450411</v>
       </c>
       <c r="X10" t="n">
-        <v>92.81553398058252</v>
+        <v>96.89320388349515</v>
       </c>
     </row>
     <row r="11">
@@ -1336,19 +1336,19 @@
         <v>74.40353659771201</v>
       </c>
       <c r="T11" t="n">
-        <v>87015</v>
+        <v>88544</v>
       </c>
       <c r="U11" t="n">
-        <v>67.47572257656725</v>
+        <v>67.6736989519335</v>
       </c>
       <c r="V11" t="n">
-        <v>73.46319600068954</v>
+        <v>73.6447415973979</v>
       </c>
       <c r="W11" t="n">
-        <v>-4.350732164205994</v>
+        <v>-4.152755788839741</v>
       </c>
       <c r="X11" t="n">
-        <v>-2.119258934296224</v>
+        <v>-0.3993295762607004</v>
       </c>
     </row>
     <row r="12">
@@ -1412,19 +1412,19 @@
         <v>75.20695379142226</v>
       </c>
       <c r="T12" t="n">
-        <v>316256</v>
+        <v>320396</v>
       </c>
       <c r="U12" t="n">
-        <v>56.92287260953152</v>
+        <v>56.989475524039</v>
       </c>
       <c r="V12" t="n">
-        <v>74.83715723970454</v>
+        <v>74.93570456560008</v>
       </c>
       <c r="W12" t="n">
-        <v>-5.106012702600523</v>
+        <v>-5.039409788093039</v>
       </c>
       <c r="X12" t="n">
-        <v>13.87625621581527</v>
+        <v>15.36697165120139</v>
       </c>
     </row>
     <row r="13">
@@ -1488,19 +1488,19 @@
         <v>60.68562662261034</v>
       </c>
       <c r="T13" t="n">
-        <v>56960</v>
+        <v>57892</v>
       </c>
       <c r="U13" t="n">
-        <v>27.49824438202247</v>
+        <v>27.6152145374145</v>
       </c>
       <c r="V13" t="n">
-        <v>60.59339887640449</v>
+        <v>60.82532992468735</v>
       </c>
       <c r="W13" t="n">
-        <v>0.3445979340640122</v>
+        <v>0.4615680894560334</v>
       </c>
       <c r="X13" t="n">
-        <v>12.02895130202187</v>
+        <v>13.86200928329793</v>
       </c>
     </row>
     <row r="14">
@@ -1564,19 +1564,19 @@
         <v>62.77658116310946</v>
       </c>
       <c r="T14" t="n">
-        <v>6051</v>
+        <v>6156</v>
       </c>
       <c r="U14" t="n">
-        <v>33.56470004957858</v>
+        <v>33.67446393762184</v>
       </c>
       <c r="V14" t="n">
-        <v>60.02313667162452</v>
+        <v>60.31513970110461</v>
       </c>
       <c r="W14" t="n">
-        <v>-3.560813950813035</v>
+        <v>-3.451050062769781</v>
       </c>
       <c r="X14" t="n">
-        <v>18.48443313099667</v>
+        <v>20.54043469747405</v>
       </c>
     </row>
     <row r="15">
@@ -1640,19 +1640,19 @@
         <v>81.03823437985702</v>
       </c>
       <c r="T15" t="n">
-        <v>15597</v>
+        <v>16006</v>
       </c>
       <c r="U15" t="n">
-        <v>59.40244918894659</v>
+        <v>59.19655129326502</v>
       </c>
       <c r="V15" t="n">
-        <v>74.25787010322497</v>
+        <v>74.15969011620642</v>
       </c>
       <c r="W15" t="n">
-        <v>-11.31561111568506</v>
+        <v>-11.52150901136663</v>
       </c>
       <c r="X15" t="n">
-        <v>-3.033882499222878</v>
+        <v>-0.4911408144233759</v>
       </c>
     </row>
   </sheetData>
@@ -1742,19 +1742,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12647</v>
+        <v>12813</v>
       </c>
       <c r="C4" t="n">
-        <v>1682</v>
+        <v>1715</v>
       </c>
       <c r="D4" t="n">
-        <v>13.29959674231043</v>
+        <v>13.38484351830173</v>
       </c>
       <c r="E4" t="n">
-        <v>8250</v>
+        <v>8366</v>
       </c>
       <c r="F4" t="n">
-        <v>65.23286154819324</v>
+        <v>65.29306173417623</v>
       </c>
     </row>
     <row r="5">
@@ -1764,19 +1764,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>736</v>
+        <v>745</v>
       </c>
       <c r="C5" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D5" t="n">
-        <v>26.6304347826087</v>
+        <v>26.71140939597316</v>
       </c>
       <c r="E5" t="n">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="F5" t="n">
-        <v>77.30978260869566</v>
+        <v>77.58389261744966</v>
       </c>
     </row>
     <row r="6">
@@ -1786,19 +1786,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1005</v>
+        <v>1027</v>
       </c>
       <c r="C6" t="n">
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1990049751243781</v>
+        <v>0.1947419668938656</v>
       </c>
       <c r="E6" t="n">
-        <v>347</v>
+        <v>358</v>
       </c>
       <c r="F6" t="n">
-        <v>34.5273631840796</v>
+        <v>34.85881207400195</v>
       </c>
     </row>
     <row r="7">
@@ -1808,19 +1808,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2298</v>
+        <v>2357</v>
       </c>
       <c r="C7" t="n">
-        <v>877</v>
+        <v>909</v>
       </c>
       <c r="D7" t="n">
-        <v>38.16362053959965</v>
+        <v>38.56597369537548</v>
       </c>
       <c r="E7" t="n">
-        <v>1201</v>
+        <v>1242</v>
       </c>
       <c r="F7" t="n">
-        <v>52.26283724978242</v>
+        <v>52.69410267288927</v>
       </c>
     </row>
     <row r="8">
@@ -1830,19 +1830,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27095</v>
+        <v>27487</v>
       </c>
       <c r="C8" t="n">
-        <v>16054</v>
+        <v>16446</v>
       </c>
       <c r="D8" t="n">
-        <v>59.25078427754198</v>
+        <v>59.83192054425729</v>
       </c>
       <c r="E8" t="n">
-        <v>17315</v>
+        <v>17707</v>
       </c>
       <c r="F8" t="n">
-        <v>63.90477947960878</v>
+        <v>64.41954378433441</v>
       </c>
     </row>
     <row r="9">
@@ -1852,19 +1852,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>29151</v>
+        <v>29682</v>
       </c>
       <c r="C9" t="n">
-        <v>10460</v>
+        <v>10633</v>
       </c>
       <c r="D9" t="n">
-        <v>35.88213097320846</v>
+        <v>35.82305774543494</v>
       </c>
       <c r="E9" t="n">
-        <v>18020</v>
+        <v>18360</v>
       </c>
       <c r="F9" t="n">
-        <v>61.81606119858667</v>
+        <v>61.85567010309278</v>
       </c>
     </row>
     <row r="10">
@@ -1874,19 +1874,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>12123</v>
+        <v>12432</v>
       </c>
       <c r="C10" t="n">
-        <v>4443</v>
+        <v>4548</v>
       </c>
       <c r="D10" t="n">
-        <v>36.6493442217273</v>
+        <v>36.58301158301158</v>
       </c>
       <c r="E10" t="n">
-        <v>6538</v>
+        <v>6707</v>
       </c>
       <c r="F10" t="n">
-        <v>53.93054524457642</v>
+        <v>53.9494851994852</v>
       </c>
     </row>
     <row r="11">
@@ -1896,19 +1896,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4126</v>
+        <v>4204</v>
       </c>
       <c r="C11" t="n">
-        <v>2458</v>
+        <v>2526</v>
       </c>
       <c r="D11" t="n">
-        <v>59.57343674260785</v>
+        <v>60.08563273073264</v>
       </c>
       <c r="E11" t="n">
-        <v>2793</v>
+        <v>2868</v>
       </c>
       <c r="F11" t="n">
-        <v>67.69268056228793</v>
+        <v>68.22074215033301</v>
       </c>
     </row>
     <row r="12">
@@ -1918,19 +1918,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1986</v>
+        <v>2028</v>
       </c>
       <c r="C12" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D12" t="n">
-        <v>2.668680765357502</v>
+        <v>2.761341222879684</v>
       </c>
       <c r="E12" t="n">
-        <v>733</v>
+        <v>749</v>
       </c>
       <c r="F12" t="n">
-        <v>36.90835850956697</v>
+        <v>36.93293885601578</v>
       </c>
     </row>
     <row r="13">
@@ -1940,19 +1940,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>87015</v>
+        <v>88544</v>
       </c>
       <c r="C13" t="n">
-        <v>58714</v>
+        <v>59921</v>
       </c>
       <c r="D13" t="n">
-        <v>67.47572257656725</v>
+        <v>67.6736989519335</v>
       </c>
       <c r="E13" t="n">
-        <v>63924</v>
+        <v>65208</v>
       </c>
       <c r="F13" t="n">
-        <v>73.46319600068954</v>
+        <v>73.6447415973979</v>
       </c>
     </row>
     <row r="14">
@@ -1962,19 +1962,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>316256</v>
+        <v>320396</v>
       </c>
       <c r="C14" t="n">
-        <v>180022</v>
+        <v>182592</v>
       </c>
       <c r="D14" t="n">
-        <v>56.92287260953152</v>
+        <v>56.989475524039</v>
       </c>
       <c r="E14" t="n">
-        <v>236677</v>
+        <v>240091</v>
       </c>
       <c r="F14" t="n">
-        <v>74.83715723970454</v>
+        <v>74.93570456560008</v>
       </c>
     </row>
     <row r="15">
@@ -1984,19 +1984,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>56960</v>
+        <v>57892</v>
       </c>
       <c r="C15" t="n">
-        <v>15663</v>
+        <v>15987</v>
       </c>
       <c r="D15" t="n">
-        <v>27.49824438202247</v>
+        <v>27.6152145374145</v>
       </c>
       <c r="E15" t="n">
-        <v>34514</v>
+        <v>35213</v>
       </c>
       <c r="F15" t="n">
-        <v>60.59339887640449</v>
+        <v>60.82532992468735</v>
       </c>
     </row>
     <row r="16">
@@ -2006,19 +2006,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6051</v>
+        <v>6156</v>
       </c>
       <c r="C16" t="n">
-        <v>2031</v>
+        <v>2073</v>
       </c>
       <c r="D16" t="n">
-        <v>33.56470004957858</v>
+        <v>33.67446393762184</v>
       </c>
       <c r="E16" t="n">
-        <v>3632</v>
+        <v>3713</v>
       </c>
       <c r="F16" t="n">
-        <v>60.02313667162452</v>
+        <v>60.31513970110461</v>
       </c>
     </row>
     <row r="17">
@@ -2028,19 +2028,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15597</v>
+        <v>16006</v>
       </c>
       <c r="C17" t="n">
-        <v>9265</v>
+        <v>9475</v>
       </c>
       <c r="D17" t="n">
-        <v>59.40244918894659</v>
+        <v>59.19655129326502</v>
       </c>
       <c r="E17" t="n">
-        <v>11582</v>
+        <v>11870</v>
       </c>
       <c r="F17" t="n">
-        <v>74.25787010322497</v>
+        <v>74.15969011620642</v>
       </c>
     </row>
     <row r="18"/>
@@ -2141,43 +2141,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1682</v>
+        <v>1715</v>
       </c>
       <c r="D22" t="n">
-        <v>15.75559849385652</v>
+        <v>16.03368318756074</v>
       </c>
       <c r="E22" t="n">
-        <v>8.258333333333333</v>
+        <v>8.433333333333334</v>
       </c>
       <c r="F22" t="n">
-        <v>0.262593308230942</v>
+        <v>0.2672280531260123</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1376388888888889</v>
+        <v>0.1405555555555556</v>
       </c>
       <c r="H22" t="n">
-        <v>269.6064669738863</v>
+        <v>268.2327380952381</v>
       </c>
       <c r="I22" t="n">
-        <v>130.2333333333333</v>
+        <v>126.9166666666667</v>
       </c>
       <c r="J22" t="n">
-        <v>4.493441116231438</v>
+        <v>4.470545634920635</v>
       </c>
       <c r="K22" t="n">
-        <v>2.170555555555555</v>
+        <v>2.115277777777778</v>
       </c>
       <c r="L22" t="n">
-        <v>246.9095698924731</v>
+        <v>245.4521214896215</v>
       </c>
       <c r="M22" t="n">
-        <v>107.1</v>
+        <v>105.0666666666667</v>
       </c>
       <c r="N22" t="n">
-        <v>4.115159498207885</v>
+        <v>4.090868691493692</v>
       </c>
       <c r="O22" t="n">
-        <v>1.785</v>
+        <v>1.751111111111111</v>
       </c>
     </row>
     <row r="23">
@@ -2192,43 +2192,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>10965</v>
+        <v>11098</v>
       </c>
       <c r="D23" t="n">
-        <v>239.0794148046816</v>
+        <v>236.6539271340181</v>
       </c>
       <c r="E23" t="n">
-        <v>71.75</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>3.984656913411359</v>
+        <v>3.944232118900302</v>
       </c>
       <c r="G23" t="n">
-        <v>1.195833333333333</v>
+        <v>1.165</v>
       </c>
       <c r="H23" t="n">
-        <v>253.3141631034269</v>
+        <v>250.8468099436689</v>
       </c>
       <c r="I23" t="n">
-        <v>87.77500000000001</v>
+        <v>85.81666666666666</v>
       </c>
       <c r="J23" t="n">
-        <v>4.221902718390449</v>
+        <v>4.180780165727814</v>
       </c>
       <c r="K23" t="n">
-        <v>1.462916666666667</v>
+        <v>1.430277777777778</v>
       </c>
       <c r="L23" t="n">
-        <v>13.8345649749024</v>
+        <v>13.79189780798433</v>
       </c>
       <c r="M23" t="n">
-        <v>6.033333333333333</v>
+        <v>6.066666666666666</v>
       </c>
       <c r="N23" t="n">
-        <v>0.23057608291504</v>
+        <v>0.2298649634664054</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1005555555555556</v>
+        <v>0.1011111111111111</v>
       </c>
     </row>
     <row r="24">
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -2294,40 +2294,40 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="D25" t="n">
-        <v>286.0467901234568</v>
+        <v>283.0639499389499</v>
       </c>
       <c r="E25" t="n">
-        <v>15.56666666666667</v>
+        <v>15.30833333333333</v>
       </c>
       <c r="F25" t="n">
-        <v>4.767446502057613</v>
+        <v>4.717732498982499</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2594444444444444</v>
+        <v>0.2551388888888889</v>
       </c>
       <c r="H25" t="n">
-        <v>296.8302296710118</v>
+        <v>293.805095150399</v>
       </c>
       <c r="I25" t="n">
-        <v>21.75</v>
+        <v>21.68333333333333</v>
       </c>
       <c r="J25" t="n">
-        <v>4.947170494516863</v>
+        <v>4.896751585839984</v>
       </c>
       <c r="K25" t="n">
-        <v>0.3625</v>
+        <v>0.3613888888888889</v>
       </c>
       <c r="L25" t="n">
-        <v>12.12535692116698</v>
+        <v>12.08471454880295</v>
       </c>
       <c r="M25" t="n">
         <v>2.216666666666667</v>
       </c>
       <c r="N25" t="n">
-        <v>0.2020892820194496</v>
+        <v>0.2014119091467158</v>
       </c>
       <c r="O25" t="n">
         <v>0.03694444444444445</v>
@@ -2372,43 +2372,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1003</v>
+        <v>1025</v>
       </c>
       <c r="D27" t="n">
-        <v>736.7651877700233</v>
+        <v>723.6870569105691</v>
       </c>
       <c r="E27" t="n">
-        <v>110.6333333333333</v>
+        <v>108.9833333333333</v>
       </c>
       <c r="F27" t="n">
-        <v>12.27941979616705</v>
+        <v>12.06145094850948</v>
       </c>
       <c r="G27" t="n">
-        <v>1.843888888888889</v>
+        <v>1.816388888888889</v>
       </c>
       <c r="H27" t="n">
-        <v>5234.074379178606</v>
+        <v>5170.702463167587</v>
       </c>
       <c r="I27" t="n">
-        <v>4576.133333333333</v>
+        <v>4525.016666666666</v>
       </c>
       <c r="J27" t="n">
-        <v>87.2345729863101</v>
+        <v>86.17837438612646</v>
       </c>
       <c r="K27" t="n">
-        <v>76.2688888888889</v>
+        <v>75.41694444444445</v>
       </c>
       <c r="L27" t="n">
-        <v>4417.962774594078</v>
+        <v>4377.41197053407</v>
       </c>
       <c r="M27" t="n">
-        <v>4222.5</v>
+        <v>4206.866666666667</v>
       </c>
       <c r="N27" t="n">
-        <v>73.63271290990131</v>
+        <v>72.95686617556784</v>
       </c>
       <c r="O27" t="n">
-        <v>70.375</v>
+        <v>70.11444444444444</v>
       </c>
     </row>
     <row r="28">
@@ -2423,43 +2423,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>877</v>
+        <v>909</v>
       </c>
       <c r="D28" t="n">
-        <v>23.85226149752946</v>
+        <v>33.56343967730106</v>
       </c>
       <c r="E28" t="n">
-        <v>15.91666666666667</v>
+        <v>21.53333333333333</v>
       </c>
       <c r="F28" t="n">
-        <v>0.397537691625491</v>
+        <v>0.559390661288351</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2652777777777778</v>
+        <v>0.3588888888888889</v>
       </c>
       <c r="H28" t="n">
-        <v>743.2020961775586</v>
+        <v>743.1556015779092</v>
       </c>
       <c r="I28" t="n">
         <v>736.0333333333333</v>
       </c>
       <c r="J28" t="n">
-        <v>12.38670160295931</v>
+        <v>12.38592669296515</v>
       </c>
       <c r="K28" t="n">
         <v>12.26722222222222</v>
       </c>
       <c r="L28" t="n">
-        <v>719.6077887381832</v>
+        <v>709.0769625246547</v>
       </c>
       <c r="M28" t="n">
-        <v>708.9666666666667</v>
+        <v>701.9833333333333</v>
       </c>
       <c r="N28" t="n">
-        <v>11.99346314563639</v>
+        <v>11.81794937541091</v>
       </c>
       <c r="O28" t="n">
-        <v>11.81611111111111</v>
+        <v>11.69972222222222</v>
       </c>
     </row>
     <row r="29">
@@ -2474,43 +2474,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1421</v>
+        <v>1448</v>
       </c>
       <c r="D29" t="n">
-        <v>256.8724724372507</v>
+        <v>261.1618899631676</v>
       </c>
       <c r="E29" t="n">
-        <v>72.21666666666667</v>
+        <v>72.38333333333333</v>
       </c>
       <c r="F29" t="n">
-        <v>4.281207873954179</v>
+        <v>4.352698166052793</v>
       </c>
       <c r="G29" t="n">
-        <v>1.203611111111111</v>
+        <v>1.206388888888889</v>
       </c>
       <c r="H29" t="n">
-        <v>986.9147304479878</v>
+        <v>990.9516739980447</v>
       </c>
       <c r="I29" t="n">
-        <v>923.55</v>
+        <v>928.2833333333333</v>
       </c>
       <c r="J29" t="n">
-        <v>16.4485788407998</v>
+        <v>16.51586123330075</v>
       </c>
       <c r="K29" t="n">
-        <v>15.3925</v>
+        <v>15.47138888888889</v>
       </c>
       <c r="L29" t="n">
-        <v>732.9659200202481</v>
+        <v>725.6427663734116</v>
       </c>
       <c r="M29" t="n">
-        <v>814.6833333333333</v>
+        <v>813.45</v>
       </c>
       <c r="N29" t="n">
-        <v>12.21609866700414</v>
+        <v>12.09404610622353</v>
       </c>
       <c r="O29" t="n">
-        <v>13.57805555555555</v>
+        <v>13.5575</v>
       </c>
     </row>
     <row r="30">
@@ -2525,43 +2525,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>16054</v>
+        <v>16446</v>
       </c>
       <c r="D30" t="n">
-        <v>26.03604086209044</v>
+        <v>26.26299100085127</v>
       </c>
       <c r="E30" t="n">
-        <v>35.21666666666667</v>
+        <v>35.25</v>
       </c>
       <c r="F30" t="n">
-        <v>0.4339340143681741</v>
+        <v>0.4377165166808545</v>
       </c>
       <c r="G30" t="n">
-        <v>0.5869444444444445</v>
+        <v>0.5875</v>
       </c>
       <c r="H30" t="n">
-        <v>408.7599069566159</v>
+        <v>405.1169703580136</v>
       </c>
       <c r="I30" t="n">
-        <v>243.5333333333333</v>
+        <v>234.925</v>
       </c>
       <c r="J30" t="n">
-        <v>6.812665115943598</v>
+        <v>6.751949505966894</v>
       </c>
       <c r="K30" t="n">
-        <v>4.058888888888889</v>
+        <v>3.915416666666666</v>
       </c>
       <c r="L30" t="n">
-        <v>382.4440776804068</v>
+        <v>378.6940673253775</v>
       </c>
       <c r="M30" t="n">
-        <v>213.55</v>
+        <v>206.7</v>
       </c>
       <c r="N30" t="n">
-        <v>6.374067961340113</v>
+        <v>6.311567788756292</v>
       </c>
       <c r="O30" t="n">
-        <v>3.559166666666667</v>
+        <v>3.445</v>
       </c>
     </row>
     <row r="31">
@@ -2591,28 +2591,28 @@
         <v>21.33138888888889</v>
       </c>
       <c r="H31" t="n">
-        <v>1969.435136085166</v>
+        <v>1957.352044979763</v>
       </c>
       <c r="I31" t="n">
-        <v>1509.6</v>
+        <v>1507.958333333333</v>
       </c>
       <c r="J31" t="n">
-        <v>32.82391893475278</v>
+        <v>32.62253408299604</v>
       </c>
       <c r="K31" t="n">
-        <v>25.16</v>
+        <v>25.13263888888889</v>
       </c>
       <c r="L31" t="n">
-        <v>255.9635248234073</v>
+        <v>253.0812377594986</v>
       </c>
       <c r="M31" t="n">
-        <v>247.65</v>
+        <v>247.6333333333333</v>
       </c>
       <c r="N31" t="n">
-        <v>4.266058747056789</v>
+        <v>4.218020629324977</v>
       </c>
       <c r="O31" t="n">
-        <v>4.1275</v>
+        <v>4.127222222222222</v>
       </c>
     </row>
     <row r="32">
@@ -2627,43 +2627,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>10460</v>
+        <v>10633</v>
       </c>
       <c r="D32" t="n">
-        <v>327.0361217335882</v>
+        <v>322.2131242358694</v>
       </c>
       <c r="E32" t="n">
-        <v>35.3</v>
+        <v>35.31666666666667</v>
       </c>
       <c r="F32" t="n">
-        <v>5.450602028893138</v>
+        <v>5.370218737264492</v>
       </c>
       <c r="G32" t="n">
-        <v>0.5883333333333333</v>
+        <v>0.5886111111111112</v>
       </c>
       <c r="H32" t="n">
-        <v>659.9170174589733</v>
+        <v>656.6801168186909</v>
       </c>
       <c r="I32" t="n">
-        <v>414.7833333333334</v>
+        <v>408.3583333333333</v>
       </c>
       <c r="J32" t="n">
-        <v>10.99861695764956</v>
+        <v>10.94466861364485</v>
       </c>
       <c r="K32" t="n">
-        <v>6.913055555555556</v>
+        <v>6.805972222222222</v>
       </c>
       <c r="L32" t="n">
-        <v>250.9853151082617</v>
+        <v>250.6613818210914</v>
       </c>
       <c r="M32" t="n">
-        <v>69.93333333333334</v>
+        <v>69.95</v>
       </c>
       <c r="N32" t="n">
-        <v>4.183088585137695</v>
+        <v>4.17768969701819</v>
       </c>
       <c r="O32" t="n">
-        <v>1.165555555555556</v>
+        <v>1.165833333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2678,43 +2678,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>18691</v>
+        <v>19049</v>
       </c>
       <c r="D33" t="n">
-        <v>383.9539903340289</v>
+        <v>377.6164680560659</v>
       </c>
       <c r="E33" t="n">
-        <v>72.33333333333333</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="F33" t="n">
-        <v>6.399233172233814</v>
+        <v>6.293607800934433</v>
       </c>
       <c r="G33" t="n">
-        <v>1.205555555555555</v>
+        <v>1.164166666666667</v>
       </c>
       <c r="H33" t="n">
-        <v>673.1323341419275</v>
+        <v>668.9687925073141</v>
       </c>
       <c r="I33" t="n">
-        <v>409.3916666666667</v>
+        <v>397.4583333333334</v>
       </c>
       <c r="J33" t="n">
-        <v>11.21887223569879</v>
+        <v>11.1494798751219</v>
       </c>
       <c r="K33" t="n">
-        <v>6.823194444444444</v>
+        <v>6.624305555555555</v>
       </c>
       <c r="L33" t="n">
-        <v>270.3307891494359</v>
+        <v>270.55061647479</v>
       </c>
       <c r="M33" t="n">
-        <v>62.48333333333333</v>
+        <v>62.79166666666666</v>
       </c>
       <c r="N33" t="n">
-        <v>4.505513152490598</v>
+        <v>4.509176941246501</v>
       </c>
       <c r="O33" t="n">
-        <v>1.041388888888889</v>
+        <v>1.046527777777778</v>
       </c>
     </row>
     <row r="34">
@@ -2729,43 +2729,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>4443</v>
+        <v>4548</v>
       </c>
       <c r="D34" t="n">
-        <v>1091.020624202866</v>
+        <v>1066.653228525359</v>
       </c>
       <c r="E34" t="n">
-        <v>924.0666666666667</v>
+        <v>904.0083333333333</v>
       </c>
       <c r="F34" t="n">
-        <v>18.18367707004777</v>
+        <v>17.77755380875599</v>
       </c>
       <c r="G34" t="n">
-        <v>15.40111111111111</v>
+        <v>15.06680555555556</v>
       </c>
       <c r="H34" t="n">
-        <v>1751.367634408602</v>
+        <v>1738.814140906425</v>
       </c>
       <c r="I34" t="n">
-        <v>1508.583333333333</v>
+        <v>1500.233333333333</v>
       </c>
       <c r="J34" t="n">
-        <v>29.1894605734767</v>
+        <v>28.98023568177376</v>
       </c>
       <c r="K34" t="n">
-        <v>25.14305555555556</v>
+        <v>25.00388888888889</v>
       </c>
       <c r="L34" t="n">
-        <v>613.1157032258064</v>
+        <v>606.1989402697495</v>
       </c>
       <c r="M34" t="n">
-        <v>502.9</v>
+        <v>501.9666666666666</v>
       </c>
       <c r="N34" t="n">
-        <v>10.21859505376344</v>
+        <v>10.10331567116249</v>
       </c>
       <c r="O34" t="n">
-        <v>8.381666666666666</v>
+        <v>8.366111111111111</v>
       </c>
     </row>
     <row r="35">
@@ -2780,43 +2780,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7680</v>
+        <v>7884</v>
       </c>
       <c r="D35" t="n">
-        <v>1355.200323350695</v>
+        <v>1323.480991036699</v>
       </c>
       <c r="E35" t="n">
-        <v>1100.466666666667</v>
+        <v>1083.775</v>
       </c>
       <c r="F35" t="n">
-        <v>22.58667205584491</v>
+        <v>22.05801651727831</v>
       </c>
       <c r="G35" t="n">
-        <v>18.34111111111111</v>
+        <v>18.06291666666667</v>
       </c>
       <c r="H35" t="n">
-        <v>2013.66546760789</v>
+        <v>1999.430839513354</v>
       </c>
       <c r="I35" t="n">
-        <v>1680.291666666667</v>
+        <v>1672.433333333333</v>
       </c>
       <c r="J35" t="n">
-        <v>33.56109112679817</v>
+        <v>33.32384732522256</v>
       </c>
       <c r="K35" t="n">
-        <v>28.00486111111111</v>
+        <v>27.87388888888889</v>
       </c>
       <c r="L35" t="n">
-        <v>644.1454841293681</v>
+        <v>634.6497091755125</v>
       </c>
       <c r="M35" t="n">
-        <v>458.7</v>
+        <v>457.1</v>
       </c>
       <c r="N35" t="n">
-        <v>10.7357580688228</v>
+        <v>10.57749515292521</v>
       </c>
       <c r="O35" t="n">
-        <v>7.645</v>
+        <v>7.618333333333334</v>
       </c>
     </row>
     <row r="36">
@@ -2831,43 +2831,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2458</v>
+        <v>2526</v>
       </c>
       <c r="D36" t="n">
-        <v>25.37641036072688</v>
+        <v>25.63712721034574</v>
       </c>
       <c r="E36" t="n">
-        <v>35.1</v>
+        <v>35.16666666666666</v>
       </c>
       <c r="F36" t="n">
-        <v>0.4229401726787813</v>
+        <v>0.4272854535057623</v>
       </c>
       <c r="G36" t="n">
-        <v>0.5850000000000001</v>
+        <v>0.586111111111111</v>
       </c>
       <c r="H36" t="n">
-        <v>2953.639493876346</v>
+        <v>2950.183716475096</v>
       </c>
       <c r="I36" t="n">
-        <v>2883.45</v>
+        <v>2882.225</v>
       </c>
       <c r="J36" t="n">
-        <v>49.22732489793911</v>
+        <v>49.16972860791827</v>
       </c>
       <c r="K36" t="n">
-        <v>48.0575</v>
+        <v>48.03708333333333</v>
       </c>
       <c r="L36" t="n">
-        <v>2927.620835177807</v>
+        <v>2924.152247273799</v>
       </c>
       <c r="M36" t="n">
-        <v>2850.25</v>
+        <v>2848.575</v>
       </c>
       <c r="N36" t="n">
-        <v>48.79368058629678</v>
+        <v>48.73587078789665</v>
       </c>
       <c r="O36" t="n">
-        <v>47.50416666666667</v>
+        <v>47.47625</v>
       </c>
     </row>
     <row r="37">
@@ -2882,43 +2882,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1668</v>
+        <v>1678</v>
       </c>
       <c r="D37" t="n">
-        <v>2677.354226618705</v>
+        <v>2661.582886372666</v>
       </c>
       <c r="E37" t="n">
-        <v>2493.416666666667</v>
+        <v>2478.275</v>
       </c>
       <c r="F37" t="n">
-        <v>44.62257044364509</v>
+        <v>44.35971477287777</v>
       </c>
       <c r="G37" t="n">
-        <v>41.55694444444444</v>
+        <v>41.30458333333333</v>
       </c>
       <c r="H37" t="n">
-        <v>3384.641198017669</v>
+        <v>3366.662692802057</v>
       </c>
       <c r="I37" t="n">
-        <v>3296.966666666667</v>
+        <v>3265.941666666667</v>
       </c>
       <c r="J37" t="n">
-        <v>56.41068663362781</v>
+        <v>56.11104488003427</v>
       </c>
       <c r="K37" t="n">
-        <v>54.94944444444445</v>
+        <v>54.43236111111111</v>
       </c>
       <c r="L37" t="n">
-        <v>577.6309523809524</v>
+        <v>575.670029991431</v>
       </c>
       <c r="M37" t="n">
-        <v>336.0333333333334</v>
+        <v>335.525</v>
       </c>
       <c r="N37" t="n">
-        <v>9.62718253968254</v>
+        <v>9.594500499857183</v>
       </c>
       <c r="O37" t="n">
-        <v>5.600555555555556</v>
+        <v>5.592083333333333</v>
       </c>
     </row>
     <row r="38">
@@ -2933,7 +2933,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -2984,43 +2984,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1933</v>
+        <v>1972</v>
       </c>
       <c r="D39" t="n">
-        <v>180.3992757371961</v>
+        <v>178.508392494929</v>
       </c>
       <c r="E39" t="n">
         <v>79.18333333333334</v>
       </c>
       <c r="F39" t="n">
-        <v>3.006654595619934</v>
+        <v>2.975139874915484</v>
       </c>
       <c r="G39" t="n">
         <v>1.319722222222222</v>
       </c>
       <c r="H39" t="n">
-        <v>494.9470420017873</v>
+        <v>491.5866684082201</v>
       </c>
       <c r="I39" t="n">
-        <v>428.9166666666667</v>
+        <v>416.4416666666667</v>
       </c>
       <c r="J39" t="n">
-        <v>8.249117366696455</v>
+        <v>8.193111140137002</v>
       </c>
       <c r="K39" t="n">
-        <v>7.148611111111111</v>
+        <v>6.940694444444444</v>
       </c>
       <c r="L39" t="n">
-        <v>314.2220643431635</v>
+        <v>311.5510884709161</v>
       </c>
       <c r="M39" t="n">
-        <v>156.5333333333333</v>
+        <v>154.9916666666667</v>
       </c>
       <c r="N39" t="n">
-        <v>5.237034405719392</v>
+        <v>5.192518141181934</v>
       </c>
       <c r="O39" t="n">
-        <v>2.608888888888889</v>
+        <v>2.583194444444445</v>
       </c>
     </row>
     <row r="40">
@@ -3035,43 +3035,43 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>58714</v>
+        <v>59921</v>
       </c>
       <c r="D40" t="n">
-        <v>499.8174211715548</v>
+        <v>490.567163153708</v>
       </c>
       <c r="E40" t="n">
-        <v>50.08333333333334</v>
+        <v>45</v>
       </c>
       <c r="F40" t="n">
-        <v>8.330290352859247</v>
+        <v>8.176119385895133</v>
       </c>
       <c r="G40" t="n">
-        <v>0.8347222222222224</v>
+        <v>0.75</v>
       </c>
       <c r="H40" t="n">
-        <v>615.368107337996</v>
+        <v>611.0832309299897</v>
       </c>
       <c r="I40" t="n">
-        <v>212.1166666666667</v>
+        <v>200.3333333333333</v>
       </c>
       <c r="J40" t="n">
-        <v>10.25613512229993</v>
+        <v>10.18472051549983</v>
       </c>
       <c r="K40" t="n">
-        <v>3.535277777777778</v>
+        <v>3.338888888888889</v>
       </c>
       <c r="L40" t="n">
-        <v>90.70259971445611</v>
+        <v>90.37999164054335</v>
       </c>
       <c r="M40" t="n">
-        <v>49.45</v>
+        <v>48.58333333333334</v>
       </c>
       <c r="N40" t="n">
-        <v>1.511709995240935</v>
+        <v>1.506333194009056</v>
       </c>
       <c r="O40" t="n">
-        <v>0.8241666666666667</v>
+        <v>0.8097222222222222</v>
       </c>
     </row>
     <row r="41">
@@ -3086,43 +3086,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>28301</v>
+        <v>28623</v>
       </c>
       <c r="D41" t="n">
-        <v>837.8153557589249</v>
+        <v>830.8317151707832</v>
       </c>
       <c r="E41" t="n">
-        <v>737.6</v>
+        <v>725.4666666666667</v>
       </c>
       <c r="F41" t="n">
-        <v>13.96358926264875</v>
+        <v>13.84719525284639</v>
       </c>
       <c r="G41" t="n">
-        <v>12.29333333333333</v>
+        <v>12.09111111111111</v>
       </c>
       <c r="H41" t="n">
-        <v>926.8915458195862</v>
+        <v>946.3680715032921</v>
       </c>
       <c r="I41" t="n">
-        <v>851.425</v>
+        <v>848.5166666666667</v>
       </c>
       <c r="J41" t="n">
-        <v>15.44819243032644</v>
+        <v>15.77280119172153</v>
       </c>
       <c r="K41" t="n">
-        <v>14.19041666666667</v>
+        <v>14.14194444444444</v>
       </c>
       <c r="L41" t="n">
-        <v>109.5894082968874</v>
+        <v>108.6917365085226</v>
       </c>
       <c r="M41" t="n">
-        <v>87.84999999999999</v>
+        <v>86.96666666666667</v>
       </c>
       <c r="N41" t="n">
-        <v>1.826490138281456</v>
+        <v>1.811528941808709</v>
       </c>
       <c r="O41" t="n">
-        <v>1.464166666666667</v>
+        <v>1.449444444444445</v>
       </c>
     </row>
     <row r="42">
@@ -3137,43 +3137,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>180022</v>
+        <v>182592</v>
       </c>
       <c r="D42" t="n">
-        <v>10.78492823099399</v>
+        <v>11.09793136245473</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0.1797488038498998</v>
+        <v>0.1849655227075788</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>455.2786757257804</v>
+        <v>453.349332416155</v>
       </c>
       <c r="I42" t="n">
-        <v>183.5666666666667</v>
+        <v>182.7333333333333</v>
       </c>
       <c r="J42" t="n">
-        <v>7.587977928763004</v>
+        <v>7.555822206935916</v>
       </c>
       <c r="K42" t="n">
-        <v>3.059444444444444</v>
+        <v>3.045555555555555</v>
       </c>
       <c r="L42" t="n">
-        <v>443.8825595075036</v>
+        <v>441.726237822669</v>
       </c>
       <c r="M42" t="n">
-        <v>174.0333333333333</v>
+        <v>172.8833333333333</v>
       </c>
       <c r="N42" t="n">
-        <v>7.398042658458395</v>
+        <v>7.362103963711153</v>
       </c>
       <c r="O42" t="n">
-        <v>2.900555555555556</v>
+        <v>2.881388888888889</v>
       </c>
     </row>
     <row r="43">
@@ -3188,43 +3188,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>136234</v>
+        <v>137804</v>
       </c>
       <c r="D43" t="n">
-        <v>158.0131446628594</v>
+        <v>156.9309387487542</v>
       </c>
       <c r="E43" t="n">
-        <v>89.43333333333334</v>
+        <v>88.96666666666667</v>
       </c>
       <c r="F43" t="n">
-        <v>2.633552411047659</v>
+        <v>2.615515645812572</v>
       </c>
       <c r="G43" t="n">
-        <v>1.490555555555556</v>
+        <v>1.482777777777778</v>
       </c>
       <c r="H43" t="n">
-        <v>559.4842872999272</v>
+        <v>556.2643231660055</v>
       </c>
       <c r="I43" t="n">
-        <v>266.8333333333333</v>
+        <v>263.475</v>
       </c>
       <c r="J43" t="n">
-        <v>9.324738121665453</v>
+        <v>9.271072052766758</v>
       </c>
       <c r="K43" t="n">
-        <v>4.447222222222222</v>
+        <v>4.391249999999999</v>
       </c>
       <c r="L43" t="n">
-        <v>400.5331938847704</v>
+        <v>398.2182079768183</v>
       </c>
       <c r="M43" t="n">
-        <v>124.775</v>
+        <v>124.15</v>
       </c>
       <c r="N43" t="n">
-        <v>6.675553231412841</v>
+        <v>6.636970132946971</v>
       </c>
       <c r="O43" t="n">
-        <v>2.079583333333333</v>
+        <v>2.069166666666667</v>
       </c>
     </row>
     <row r="44">
@@ -3239,40 +3239,40 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>15663</v>
+        <v>15987</v>
       </c>
       <c r="D44" t="n">
-        <v>23.82856732426738</v>
+        <v>24.03482204290987</v>
       </c>
       <c r="E44" t="n">
-        <v>35.11666666666667</v>
+        <v>35.15</v>
       </c>
       <c r="F44" t="n">
-        <v>0.3971427887377897</v>
+        <v>0.4005803673818311</v>
       </c>
       <c r="G44" t="n">
-        <v>0.5852777777777778</v>
+        <v>0.5858333333333333</v>
       </c>
       <c r="H44" t="n">
-        <v>1035.069069343066</v>
+        <v>1035.003140571268</v>
       </c>
       <c r="I44" t="n">
-        <v>871.3666666666667</v>
+        <v>871.2666666666667</v>
       </c>
       <c r="J44" t="n">
-        <v>17.25115115571776</v>
+        <v>17.25005234285447</v>
       </c>
       <c r="K44" t="n">
-        <v>14.52277777777778</v>
+        <v>14.52111111111111</v>
       </c>
       <c r="L44" t="n">
-        <v>1009.963363279057</v>
+        <v>1009.896698013896</v>
       </c>
       <c r="M44" t="n">
         <v>843.9833333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>16.83272272131761</v>
+        <v>16.83161163356493</v>
       </c>
       <c r="O44" t="n">
         <v>14.06638888888889</v>
@@ -3290,43 +3290,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>41297</v>
+        <v>41905</v>
       </c>
       <c r="D45" t="n">
-        <v>268.0716286897353</v>
+        <v>264.3851219027164</v>
       </c>
       <c r="E45" t="n">
-        <v>29.2</v>
+        <v>28.26666666666667</v>
       </c>
       <c r="F45" t="n">
-        <v>4.467860478162256</v>
+        <v>4.406418698378608</v>
       </c>
       <c r="G45" t="n">
-        <v>0.4866666666666666</v>
+        <v>0.4711111111111111</v>
       </c>
       <c r="H45" t="n">
-        <v>1102.388018471002</v>
+        <v>1102.18878353756</v>
       </c>
       <c r="I45" t="n">
-        <v>937.9666666666667</v>
+        <v>937.7666666666667</v>
       </c>
       <c r="J45" t="n">
-        <v>18.37313364118337</v>
+        <v>18.36981305895932</v>
       </c>
       <c r="K45" t="n">
-        <v>15.63277777777778</v>
+        <v>15.62944444444444</v>
       </c>
       <c r="L45" t="n">
-        <v>834.0250546441005</v>
+        <v>833.926264000069</v>
       </c>
       <c r="M45" t="n">
-        <v>562.1833333333333</v>
+        <v>562.0333333333333</v>
       </c>
       <c r="N45" t="n">
-        <v>13.90041757740168</v>
+        <v>13.89877106666782</v>
       </c>
       <c r="O45" t="n">
-        <v>9.369722222222221</v>
+        <v>9.367222222222221</v>
       </c>
     </row>
     <row r="46">
@@ -3341,43 +3341,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2031</v>
+        <v>2073</v>
       </c>
       <c r="D46" t="n">
-        <v>22.61802888560643</v>
+        <v>22.86252612960283</v>
       </c>
       <c r="E46" t="n">
-        <v>15.81666666666667</v>
+        <v>15.9</v>
       </c>
       <c r="F46" t="n">
-        <v>0.3769671480934406</v>
+        <v>0.3810421021600472</v>
       </c>
       <c r="G46" t="n">
-        <v>0.2636111111111111</v>
+        <v>0.265</v>
       </c>
       <c r="H46" t="n">
-        <v>2722.767684108527</v>
+        <v>2708.867042677195</v>
       </c>
       <c r="I46" t="n">
-        <v>2597.383333333333</v>
+        <v>2578.316666666667</v>
       </c>
       <c r="J46" t="n">
-        <v>45.37946140180878</v>
+        <v>45.14778404461991</v>
       </c>
       <c r="K46" t="n">
-        <v>43.28972222222222</v>
+        <v>42.97194444444445</v>
       </c>
       <c r="L46" t="n">
-        <v>2698.824602713178</v>
+        <v>2684.575502914082</v>
       </c>
       <c r="M46" t="n">
-        <v>2565.6</v>
+        <v>2549.25</v>
       </c>
       <c r="N46" t="n">
-        <v>44.98041004521964</v>
+        <v>44.74292504856803</v>
       </c>
       <c r="O46" t="n">
-        <v>42.76</v>
+        <v>42.4875</v>
       </c>
     </row>
     <row r="47">
@@ -3392,43 +3392,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>4020</v>
+        <v>4083</v>
       </c>
       <c r="D47" t="n">
-        <v>229.5184618573798</v>
+        <v>226.3140256347457</v>
       </c>
       <c r="E47" t="n">
-        <v>65.125</v>
+        <v>62.91666666666666</v>
       </c>
       <c r="F47" t="n">
-        <v>3.825307697622996</v>
+        <v>3.771900427245761</v>
       </c>
       <c r="G47" t="n">
-        <v>1.085416666666667</v>
+        <v>1.048611111111111</v>
       </c>
       <c r="H47" t="n">
-        <v>3065.697476591761</v>
+        <v>3040.647868217054</v>
       </c>
       <c r="I47" t="n">
-        <v>2839.333333333333</v>
+        <v>2826.325</v>
       </c>
       <c r="J47" t="n">
-        <v>51.094957943196</v>
+        <v>50.67746447028424</v>
       </c>
       <c r="K47" t="n">
-        <v>47.32222222222222</v>
+        <v>47.10541666666667</v>
       </c>
       <c r="L47" t="n">
-        <v>2829.254887640449</v>
+        <v>2808.780124391563</v>
       </c>
       <c r="M47" t="n">
-        <v>2760.65</v>
+        <v>2753.566666666667</v>
       </c>
       <c r="N47" t="n">
-        <v>47.15424812734083</v>
+        <v>46.81300207319271</v>
       </c>
       <c r="O47" t="n">
-        <v>46.01083333333333</v>
+        <v>45.89277777777778</v>
       </c>
     </row>
     <row r="48">
@@ -3443,43 +3443,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9265</v>
+        <v>9475</v>
       </c>
       <c r="D48" t="n">
-        <v>25.25211009174312</v>
+        <v>25.47298153034301</v>
       </c>
       <c r="E48" t="n">
-        <v>35.1</v>
+        <v>35.15</v>
       </c>
       <c r="F48" t="n">
-        <v>0.420868501529052</v>
+        <v>0.4245496921723835</v>
       </c>
       <c r="G48" t="n">
-        <v>0.5850000000000001</v>
+        <v>0.5858333333333333</v>
       </c>
       <c r="H48" t="n">
-        <v>397.865464930826</v>
+        <v>396.7051839404452</v>
       </c>
       <c r="I48" t="n">
-        <v>337.9333333333333</v>
+        <v>340.05</v>
       </c>
       <c r="J48" t="n">
-        <v>6.631091082180433</v>
+        <v>6.611753065674087</v>
       </c>
       <c r="K48" t="n">
-        <v>5.632222222222222</v>
+        <v>5.6675</v>
       </c>
       <c r="L48" t="n">
-        <v>372.3851192463188</v>
+        <v>370.9658373084707</v>
       </c>
       <c r="M48" t="n">
-        <v>310.9833333333333</v>
+        <v>311.75</v>
       </c>
       <c r="N48" t="n">
-        <v>6.206418654105313</v>
+        <v>6.182763955141177</v>
       </c>
       <c r="O48" t="n">
-        <v>5.183055555555556</v>
+        <v>5.195833333333334</v>
       </c>
     </row>
     <row r="49">
@@ -3494,43 +3494,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6332</v>
+        <v>6531</v>
       </c>
       <c r="D49" t="n">
-        <v>284.0647425773847</v>
+        <v>283.6982621344358</v>
       </c>
       <c r="E49" t="n">
-        <v>106.6</v>
+        <v>105.8</v>
       </c>
       <c r="F49" t="n">
-        <v>4.734412376289746</v>
+        <v>4.728304368907263</v>
       </c>
       <c r="G49" t="n">
-        <v>1.776666666666667</v>
+        <v>1.763333333333333</v>
       </c>
       <c r="H49" t="n">
-        <v>640.2324615718863</v>
+        <v>638.6656776094277</v>
       </c>
       <c r="I49" t="n">
-        <v>598.3833333333333</v>
+        <v>593.575</v>
       </c>
       <c r="J49" t="n">
-        <v>10.67054102619811</v>
+        <v>10.64442796015713</v>
       </c>
       <c r="K49" t="n">
-        <v>9.973055555555556</v>
+        <v>9.892916666666666</v>
       </c>
       <c r="L49" t="n">
-        <v>355.8073108467764</v>
+        <v>353.0083017676768</v>
       </c>
       <c r="M49" t="n">
-        <v>219.3</v>
+        <v>208.3166666666667</v>
       </c>
       <c r="N49" t="n">
-        <v>5.930121847446273</v>
+        <v>5.883471696127946</v>
       </c>
       <c r="O49" t="n">
-        <v>3.655</v>
+        <v>3.471944444444444</v>
       </c>
     </row>
   </sheetData>
@@ -14685,19 +14685,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11251</v>
+        <v>11362</v>
       </c>
       <c r="C4" t="n">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="D4" t="n">
-        <v>4.248511243445027</v>
+        <v>4.224608343601479</v>
       </c>
       <c r="E4" t="n">
-        <v>4918.933786610879</v>
+        <v>4898.479895833332</v>
       </c>
       <c r="F4" t="n">
-        <v>1395.479407685881</v>
+        <v>1388.356319518471</v>
       </c>
     </row>
     <row r="5">
@@ -14707,19 +14707,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>381565</v>
+        <v>388288</v>
       </c>
       <c r="C5" t="n">
-        <v>277390</v>
+        <v>282340</v>
       </c>
       <c r="D5" t="n">
-        <v>72.697967580884</v>
+        <v>72.71406790835668</v>
       </c>
       <c r="E5" t="n">
-        <v>2895.874611657955</v>
+        <v>2922.888139929873</v>
       </c>
       <c r="F5" t="n">
-        <v>4963.101685769139</v>
+        <v>4919.06169889946</v>
       </c>
     </row>
     <row r="6">
@@ -14729,19 +14729,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>117083</v>
+        <v>118561</v>
       </c>
       <c r="C6" t="n">
-        <v>5428</v>
+        <v>5505</v>
       </c>
       <c r="D6" t="n">
-        <v>4.63602743353006</v>
+        <v>4.643179460362176</v>
       </c>
       <c r="E6" t="n">
-        <v>1881.129489683124</v>
+        <v>1864.616138056312</v>
       </c>
       <c r="F6" t="n">
-        <v>3714.470015288075</v>
+        <v>3683.792526862705</v>
       </c>
     </row>
     <row r="7">
@@ -14751,19 +14751,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>63147</v>
+        <v>63558</v>
       </c>
       <c r="C7" t="n">
-        <v>18624</v>
+        <v>18757</v>
       </c>
       <c r="D7" t="n">
-        <v>29.49308755760369</v>
+        <v>29.51162717517858</v>
       </c>
       <c r="E7" t="n">
-        <v>535.1113479381443</v>
+        <v>537.9021183558139</v>
       </c>
       <c r="F7" t="n">
-        <v>4363.276148732116</v>
+        <v>4341.114168656949</v>
       </c>
     </row>
     <row r="8"/>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard jue 13/08/2026 11:25:35,42
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -680,19 +680,19 @@
         <v>65.29306173417623</v>
       </c>
       <c r="W2" t="n">
-        <v>2947</v>
+        <v>4214</v>
       </c>
       <c r="X2" t="n">
-        <v>12.35154394299287</v>
+        <v>16.49264356905553</v>
       </c>
       <c r="Y2" t="n">
-        <v>69.22293858160842</v>
+        <v>70.45562411010916</v>
       </c>
       <c r="Z2" t="n">
-        <v>-1.033299575308851</v>
+        <v>3.107800050753802</v>
       </c>
       <c r="AA2" t="n">
-        <v>-76.9999219542652</v>
+        <v>-67.11152735503005</v>
       </c>
     </row>
     <row r="3">
@@ -765,19 +765,19 @@
         <v>77.58389261744966</v>
       </c>
       <c r="W3" t="n">
-        <v>159</v>
+        <v>196</v>
       </c>
       <c r="X3" t="n">
-        <v>8.176100628930817</v>
+        <v>8.673469387755102</v>
       </c>
       <c r="Y3" t="n">
-        <v>79.87421383647799</v>
+        <v>80.61224489795919</v>
       </c>
       <c r="Z3" t="n">
-        <v>-18.53530876704234</v>
+        <v>-18.03794000821805</v>
       </c>
       <c r="AA3" t="n">
-        <v>-78.65771812080537</v>
+        <v>-73.69127516778524</v>
       </c>
     </row>
     <row r="4">
@@ -850,19 +850,19 @@
         <v>34.85881207400195</v>
       </c>
       <c r="W4" t="n">
-        <v>120</v>
+        <v>194</v>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>23.71134020618556</v>
       </c>
       <c r="Y4" t="n">
-        <v>53.33333333333334</v>
+        <v>64.43298969072166</v>
       </c>
       <c r="Z4" t="n">
-        <v>-0.1947419668938656</v>
+        <v>23.5165982392917</v>
       </c>
       <c r="AA4" t="n">
-        <v>-88.31548198636806</v>
+        <v>-81.11002921129503</v>
       </c>
     </row>
     <row r="5">
@@ -935,19 +935,19 @@
         <v>52.69410267288927</v>
       </c>
       <c r="W5" t="n">
-        <v>603</v>
+        <v>883</v>
       </c>
       <c r="X5" t="n">
-        <v>42.45439469320066</v>
+        <v>50.16987542468856</v>
       </c>
       <c r="Y5" t="n">
-        <v>55.38971807628524</v>
+        <v>61.26840317100793</v>
       </c>
       <c r="Z5" t="n">
-        <v>3.888420997825186</v>
+        <v>11.60390172931308</v>
       </c>
       <c r="AA5" t="n">
-        <v>-74.41663131098855</v>
+        <v>-62.537123462028</v>
       </c>
     </row>
     <row r="6">
@@ -1020,19 +1020,19 @@
         <v>64.41954378433441</v>
       </c>
       <c r="W6" t="n">
-        <v>5257</v>
+        <v>8112</v>
       </c>
       <c r="X6" t="n">
-        <v>72.70306258322236</v>
+        <v>73.96449704142012</v>
       </c>
       <c r="Y6" t="n">
-        <v>77.28742628875784</v>
+        <v>78.31607495069034</v>
       </c>
       <c r="Z6" t="n">
-        <v>12.87114203896508</v>
+        <v>14.13257649716283</v>
       </c>
       <c r="AA6" t="n">
-        <v>-80.87459526321534</v>
+        <v>-70.4878669916688</v>
       </c>
     </row>
     <row r="7">
@@ -1105,19 +1105,19 @@
         <v>61.85549639414975</v>
       </c>
       <c r="W7" t="n">
-        <v>7307</v>
+        <v>10548</v>
       </c>
       <c r="X7" t="n">
-        <v>32.88627343643082</v>
+        <v>34.27189988623436</v>
       </c>
       <c r="Y7" t="n">
-        <v>64.80087587245107</v>
+        <v>63.65187713310581</v>
       </c>
       <c r="Z7" t="n">
-        <v>-2.946442072095159</v>
+        <v>-1.560815622291621</v>
       </c>
       <c r="AA7" t="n">
-        <v>-75.37574981465256</v>
+        <v>-64.45373053851857</v>
       </c>
     </row>
     <row r="8">
@@ -1190,19 +1190,19 @@
         <v>53.9494851994852</v>
       </c>
       <c r="W8" t="n">
-        <v>2336</v>
+        <v>3262</v>
       </c>
       <c r="X8" t="n">
-        <v>40.88184931506849</v>
+        <v>43.28632740649908</v>
       </c>
       <c r="Y8" t="n">
-        <v>61.90068493150685</v>
+        <v>63.18209687308399</v>
       </c>
       <c r="Z8" t="n">
-        <v>4.29883773205691</v>
+        <v>6.7033158234875</v>
       </c>
       <c r="AA8" t="n">
-        <v>-81.20978120978121</v>
+        <v>-73.76126126126125</v>
       </c>
     </row>
     <row r="9">
@@ -1275,19 +1275,19 @@
         <v>68.22074215033301</v>
       </c>
       <c r="W9" t="n">
-        <v>764</v>
+        <v>1142</v>
       </c>
       <c r="X9" t="n">
-        <v>64.92146596858639</v>
+        <v>66.28721541155866</v>
       </c>
       <c r="Y9" t="n">
-        <v>74.60732984293193</v>
+        <v>74.25569176882661</v>
       </c>
       <c r="Z9" t="n">
-        <v>4.835833237853748</v>
+        <v>6.201582680826021</v>
       </c>
       <c r="AA9" t="n">
-        <v>-81.82683158896289</v>
+        <v>-72.83539486203615</v>
       </c>
     </row>
     <row r="10">
@@ -1360,19 +1360,19 @@
         <v>36.93293885601578</v>
       </c>
       <c r="W10" t="n">
-        <v>573</v>
+        <v>954</v>
       </c>
       <c r="X10" t="n">
-        <v>3.141361256544502</v>
+        <v>20.33542976939203</v>
       </c>
       <c r="Y10" t="n">
-        <v>44.50261780104712</v>
+        <v>53.77358490566038</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.3800200336648181</v>
+        <v>17.57408854651235</v>
       </c>
       <c r="AA10" t="n">
-        <v>-71.7455621301775</v>
+        <v>-52.95857988165681</v>
       </c>
     </row>
     <row r="11">
@@ -1445,19 +1445,19 @@
         <v>73.6447415973979</v>
       </c>
       <c r="W11" t="n">
-        <v>17102</v>
+        <v>28014</v>
       </c>
       <c r="X11" t="n">
-        <v>70.94491872295639</v>
+        <v>76.84015135289498</v>
       </c>
       <c r="Y11" t="n">
-        <v>77.02607882119051</v>
+        <v>81.50210608981223</v>
       </c>
       <c r="Z11" t="n">
-        <v>3.271219771022885</v>
+        <v>9.166452400961475</v>
       </c>
       <c r="AA11" t="n">
-        <v>-80.6853089989158</v>
+        <v>-68.36149259125406</v>
       </c>
     </row>
     <row r="12">
@@ -1530,19 +1530,19 @@
         <v>74.93570456560008</v>
       </c>
       <c r="W12" t="n">
-        <v>56382</v>
+        <v>78006</v>
       </c>
       <c r="X12" t="n">
-        <v>56.93838459082686</v>
+        <v>58.08527549162885</v>
       </c>
       <c r="Y12" t="n">
-        <v>79.28594232201766</v>
+        <v>78.56575135246007</v>
       </c>
       <c r="Z12" t="n">
-        <v>-0.0510909332121372</v>
+        <v>1.095799967589848</v>
       </c>
       <c r="AA12" t="n">
-        <v>-82.40240202749098</v>
+        <v>-75.65325409805365</v>
       </c>
     </row>
     <row r="13">
@@ -1615,19 +1615,19 @@
         <v>60.82532992468735</v>
       </c>
       <c r="W13" t="n">
-        <v>10924</v>
+        <v>14665</v>
       </c>
       <c r="X13" t="n">
-        <v>27.6913218601245</v>
+        <v>30.35117627003068</v>
       </c>
       <c r="Y13" t="n">
-        <v>62.71512266569022</v>
+        <v>64.99147630412547</v>
       </c>
       <c r="Z13" t="n">
-        <v>0.07610732271000131</v>
+        <v>2.73596173261619</v>
       </c>
       <c r="AA13" t="n">
-        <v>-81.13038070890623</v>
+        <v>-74.66834795826712</v>
       </c>
     </row>
     <row r="14">
@@ -1700,19 +1700,19 @@
         <v>60.31513970110461</v>
       </c>
       <c r="W14" t="n">
-        <v>1297</v>
+        <v>1666</v>
       </c>
       <c r="X14" t="n">
-        <v>37.62528912875867</v>
+        <v>41.05642256902761</v>
       </c>
       <c r="Y14" t="n">
-        <v>66.07555898226677</v>
+        <v>68.36734693877551</v>
       </c>
       <c r="Z14" t="n">
-        <v>3.950825191136836</v>
+        <v>7.381958631405773</v>
       </c>
       <c r="AA14" t="n">
-        <v>-78.93112410656271</v>
+        <v>-72.93697205977908</v>
       </c>
     </row>
     <row r="15">
@@ -1785,19 +1785,19 @@
         <v>74.15969011620642</v>
       </c>
       <c r="W15" t="n">
-        <v>3663</v>
+        <v>5428</v>
       </c>
       <c r="X15" t="n">
-        <v>65.92956592956592</v>
+        <v>67.74134119380987</v>
       </c>
       <c r="Y15" t="n">
-        <v>78.56947856947856</v>
+        <v>79.93736182756079</v>
       </c>
       <c r="Z15" t="n">
-        <v>6.733014636300908</v>
+        <v>8.544789900544856</v>
       </c>
       <c r="AA15" t="n">
-        <v>-77.11483193802324</v>
+        <v>-66.08771710608522</v>
       </c>
     </row>
   </sheetData>
@@ -1876,19 +1876,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1692</v>
+        <v>2870</v>
       </c>
       <c r="C4" t="n">
-        <v>62</v>
+        <v>441</v>
       </c>
       <c r="D4" t="n">
-        <v>3.664302600472813</v>
+        <v>15.36585365853658</v>
       </c>
       <c r="E4" t="n">
-        <v>450.2996774193548</v>
+        <v>669.0308163265305</v>
       </c>
       <c r="F4" t="n">
-        <v>1200.708503067485</v>
+        <v>1297.273589954714</v>
       </c>
     </row>
     <row r="5">
@@ -1898,19 +1898,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79526</v>
+        <v>111451</v>
       </c>
       <c r="C5" t="n">
-        <v>55921</v>
+        <v>80869</v>
       </c>
       <c r="D5" t="n">
-        <v>70.31788345949752</v>
+        <v>72.56013853621771</v>
       </c>
       <c r="E5" t="n">
-        <v>3361.120403211673</v>
+        <v>4036.01766286216</v>
       </c>
       <c r="F5" t="n">
-        <v>5659.866565134505</v>
+        <v>5854.246933326794</v>
       </c>
     </row>
     <row r="6">
@@ -1920,19 +1920,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22938</v>
+        <v>34695</v>
       </c>
       <c r="C6" t="n">
-        <v>907</v>
+        <v>4317</v>
       </c>
       <c r="D6" t="n">
-        <v>3.954137239515215</v>
+        <v>12.44271508862949</v>
       </c>
       <c r="E6" t="n">
-        <v>1462.600496141125</v>
+        <v>9107.960889506601</v>
       </c>
       <c r="F6" t="n">
-        <v>4536.925464568109</v>
+        <v>4469.714320228455</v>
       </c>
     </row>
     <row r="7">
@@ -1942,19 +1942,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5278</v>
+        <v>8268</v>
       </c>
       <c r="C7" t="n">
-        <v>1601</v>
+        <v>3200</v>
       </c>
       <c r="D7" t="n">
-        <v>30.33345964380447</v>
+        <v>38.70343492985002</v>
       </c>
       <c r="E7" t="n">
-        <v>390.8595502810743</v>
+        <v>842.7509875000001</v>
       </c>
       <c r="F7" t="n">
-        <v>2761.018683709546</v>
+        <v>3799.223310970797</v>
       </c>
     </row>
     <row r="8"/>
@@ -2996,19 +2996,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2947</v>
+        <v>4214</v>
       </c>
       <c r="C4" t="n">
-        <v>364</v>
+        <v>695</v>
       </c>
       <c r="D4" t="n">
-        <v>12.35154394299287</v>
+        <v>16.49264356905553</v>
       </c>
       <c r="E4" t="n">
-        <v>2040</v>
+        <v>2969</v>
       </c>
       <c r="F4" t="n">
-        <v>69.22293858160842</v>
+        <v>70.45562411010916</v>
       </c>
     </row>
     <row r="5">
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>159</v>
+        <v>196</v>
       </c>
       <c r="C5" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D5" t="n">
-        <v>8.176100628930817</v>
+        <v>8.673469387755102</v>
       </c>
       <c r="E5" t="n">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="F5" t="n">
-        <v>79.87421383647799</v>
+        <v>80.61224489795919</v>
       </c>
     </row>
     <row r="6">
@@ -3040,19 +3040,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>120</v>
+        <v>194</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>23.71134020618556</v>
       </c>
       <c r="E6" t="n">
-        <v>64</v>
+        <v>125</v>
       </c>
       <c r="F6" t="n">
-        <v>53.33333333333334</v>
+        <v>64.43298969072166</v>
       </c>
     </row>
     <row r="7">
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>603</v>
+        <v>883</v>
       </c>
       <c r="C7" t="n">
-        <v>256</v>
+        <v>443</v>
       </c>
       <c r="D7" t="n">
-        <v>42.45439469320066</v>
+        <v>50.16987542468856</v>
       </c>
       <c r="E7" t="n">
-        <v>334</v>
+        <v>541</v>
       </c>
       <c r="F7" t="n">
-        <v>55.38971807628524</v>
+        <v>61.26840317100793</v>
       </c>
     </row>
     <row r="8">
@@ -3084,19 +3084,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5257</v>
+        <v>8112</v>
       </c>
       <c r="C8" t="n">
-        <v>3822</v>
+        <v>6000</v>
       </c>
       <c r="D8" t="n">
-        <v>72.70306258322236</v>
+        <v>73.96449704142012</v>
       </c>
       <c r="E8" t="n">
-        <v>4063</v>
+        <v>6353</v>
       </c>
       <c r="F8" t="n">
-        <v>77.28742628875784</v>
+        <v>78.31607495069034</v>
       </c>
     </row>
     <row r="9">
@@ -3106,19 +3106,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7307</v>
+        <v>10548</v>
       </c>
       <c r="C9" t="n">
-        <v>2403</v>
+        <v>3615</v>
       </c>
       <c r="D9" t="n">
-        <v>32.88627343643082</v>
+        <v>34.27189988623436</v>
       </c>
       <c r="E9" t="n">
-        <v>4735</v>
+        <v>6714</v>
       </c>
       <c r="F9" t="n">
-        <v>64.80087587245107</v>
+        <v>63.65187713310581</v>
       </c>
     </row>
     <row r="10">
@@ -3128,19 +3128,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2336</v>
+        <v>3262</v>
       </c>
       <c r="C10" t="n">
-        <v>955</v>
+        <v>1412</v>
       </c>
       <c r="D10" t="n">
-        <v>40.88184931506849</v>
+        <v>43.28632740649908</v>
       </c>
       <c r="E10" t="n">
-        <v>1446</v>
+        <v>2061</v>
       </c>
       <c r="F10" t="n">
-        <v>61.90068493150685</v>
+        <v>63.18209687308399</v>
       </c>
     </row>
     <row r="11">
@@ -3150,19 +3150,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>764</v>
+        <v>1142</v>
       </c>
       <c r="C11" t="n">
-        <v>496</v>
+        <v>757</v>
       </c>
       <c r="D11" t="n">
-        <v>64.92146596858639</v>
+        <v>66.28721541155866</v>
       </c>
       <c r="E11" t="n">
-        <v>570</v>
+        <v>848</v>
       </c>
       <c r="F11" t="n">
-        <v>74.60732984293193</v>
+        <v>74.25569176882661</v>
       </c>
     </row>
     <row r="12">
@@ -3172,19 +3172,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>573</v>
+        <v>954</v>
       </c>
       <c r="C12" t="n">
-        <v>18</v>
+        <v>194</v>
       </c>
       <c r="D12" t="n">
-        <v>3.141361256544502</v>
+        <v>20.33542976939203</v>
       </c>
       <c r="E12" t="n">
-        <v>255</v>
+        <v>513</v>
       </c>
       <c r="F12" t="n">
-        <v>44.50261780104712</v>
+        <v>53.77358490566038</v>
       </c>
     </row>
     <row r="13">
@@ -3194,19 +3194,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>17102</v>
+        <v>28014</v>
       </c>
       <c r="C13" t="n">
-        <v>12133</v>
+        <v>21526</v>
       </c>
       <c r="D13" t="n">
-        <v>70.94491872295639</v>
+        <v>76.84015135289498</v>
       </c>
       <c r="E13" t="n">
-        <v>13173</v>
+        <v>22832</v>
       </c>
       <c r="F13" t="n">
-        <v>77.02607882119051</v>
+        <v>81.50210608981223</v>
       </c>
     </row>
     <row r="14">
@@ -3216,19 +3216,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>56382</v>
+        <v>78006</v>
       </c>
       <c r="C14" t="n">
-        <v>32103</v>
+        <v>45310</v>
       </c>
       <c r="D14" t="n">
-        <v>56.93838459082686</v>
+        <v>58.08527549162885</v>
       </c>
       <c r="E14" t="n">
-        <v>44703</v>
+        <v>61286</v>
       </c>
       <c r="F14" t="n">
-        <v>79.28594232201766</v>
+        <v>78.56575135246007</v>
       </c>
     </row>
     <row r="15">
@@ -3238,19 +3238,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10924</v>
+        <v>14665</v>
       </c>
       <c r="C15" t="n">
-        <v>3025</v>
+        <v>4451</v>
       </c>
       <c r="D15" t="n">
-        <v>27.6913218601245</v>
+        <v>30.35117627003068</v>
       </c>
       <c r="E15" t="n">
-        <v>6851</v>
+        <v>9531</v>
       </c>
       <c r="F15" t="n">
-        <v>62.71512266569022</v>
+        <v>64.99147630412547</v>
       </c>
     </row>
     <row r="16">
@@ -3260,19 +3260,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1297</v>
+        <v>1666</v>
       </c>
       <c r="C16" t="n">
-        <v>488</v>
+        <v>684</v>
       </c>
       <c r="D16" t="n">
-        <v>37.62528912875867</v>
+        <v>41.05642256902761</v>
       </c>
       <c r="E16" t="n">
-        <v>857</v>
+        <v>1139</v>
       </c>
       <c r="F16" t="n">
-        <v>66.07555898226677</v>
+        <v>68.36734693877551</v>
       </c>
     </row>
     <row r="17">
@@ -3282,19 +3282,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3663</v>
+        <v>5428</v>
       </c>
       <c r="C17" t="n">
-        <v>2415</v>
+        <v>3677</v>
       </c>
       <c r="D17" t="n">
-        <v>65.92956592956592</v>
+        <v>67.74134119380987</v>
       </c>
       <c r="E17" t="n">
-        <v>2878</v>
+        <v>4339</v>
       </c>
       <c r="F17" t="n">
-        <v>78.56947856947856</v>
+        <v>79.93736182756079</v>
       </c>
     </row>
     <row r="18"/>
@@ -3395,43 +3395,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>364</v>
+        <v>695</v>
       </c>
       <c r="D22" t="n">
-        <v>18.68630952380953</v>
+        <v>12.42040767386091</v>
       </c>
       <c r="E22" t="n">
-        <v>20.39166666666667</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3114384920634921</v>
+        <v>0.2070067945643485</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3398611111111111</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>294.0441558441559</v>
+        <v>288.4700733752621</v>
       </c>
       <c r="I22" t="n">
-        <v>144.3666666666667</v>
+        <v>136.1333333333333</v>
       </c>
       <c r="J22" t="n">
-        <v>4.90073593073593</v>
+        <v>4.807834556254367</v>
       </c>
       <c r="K22" t="n">
-        <v>2.406111111111111</v>
+        <v>2.268888888888889</v>
       </c>
       <c r="L22" t="n">
-        <v>266.8016594516595</v>
+        <v>263.1197589098533</v>
       </c>
       <c r="M22" t="n">
-        <v>114.1666666666667</v>
+        <v>104.6833333333333</v>
       </c>
       <c r="N22" t="n">
-        <v>4.446694324194324</v>
+        <v>4.385329315164221</v>
       </c>
       <c r="O22" t="n">
-        <v>1.902777777777778</v>
+        <v>1.744722222222222</v>
       </c>
     </row>
     <row r="23">
@@ -3446,43 +3446,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2583</v>
+        <v>3519</v>
       </c>
       <c r="D23" t="n">
-        <v>221.0288875983998</v>
+        <v>214.5087288055319</v>
       </c>
       <c r="E23" t="n">
-        <v>68.06666666666666</v>
+        <v>65.75</v>
       </c>
       <c r="F23" t="n">
-        <v>3.683814793306663</v>
+        <v>3.575145480092198</v>
       </c>
       <c r="G23" t="n">
-        <v>1.134444444444444</v>
+        <v>1.095833333333333</v>
       </c>
       <c r="H23" t="n">
-        <v>232.8639325990034</v>
+        <v>226.3614373440798</v>
       </c>
       <c r="I23" t="n">
-        <v>84.79166666666667</v>
+        <v>80.95833333333334</v>
       </c>
       <c r="J23" t="n">
-        <v>3.881065543316724</v>
+        <v>3.77269062240133</v>
       </c>
       <c r="K23" t="n">
-        <v>1.413194444444445</v>
+        <v>1.349305555555556</v>
       </c>
       <c r="L23" t="n">
-        <v>11.23388408077629</v>
+        <v>11.28678276722318</v>
       </c>
       <c r="M23" t="n">
-        <v>5.316666666666666</v>
+        <v>5.416666666666667</v>
       </c>
       <c r="N23" t="n">
-        <v>0.1872314013462715</v>
+        <v>0.1881130461203863</v>
       </c>
       <c r="O23" t="n">
-        <v>0.08861111111111111</v>
+        <v>0.09027777777777778</v>
       </c>
     </row>
     <row r="24">
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -3524,43 +3524,43 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>146</v>
+        <v>179</v>
       </c>
       <c r="D25" t="n">
-        <v>378.9694063926941</v>
+        <v>330.0571694599628</v>
       </c>
       <c r="E25" t="n">
-        <v>20.59166666666667</v>
+        <v>17.75</v>
       </c>
       <c r="F25" t="n">
-        <v>6.316156773211568</v>
+        <v>5.500952824332713</v>
       </c>
       <c r="G25" t="n">
-        <v>0.3431944444444445</v>
+        <v>0.2958333333333333</v>
       </c>
       <c r="H25" t="n">
-        <v>390.0368055555555</v>
+        <v>338.8777153558053</v>
       </c>
       <c r="I25" t="n">
-        <v>33.08333333333334</v>
+        <v>26.225</v>
       </c>
       <c r="J25" t="n">
-        <v>6.500613425925927</v>
+        <v>5.647961922596754</v>
       </c>
       <c r="K25" t="n">
-        <v>0.5513888888888889</v>
+        <v>0.4370833333333333</v>
       </c>
       <c r="L25" t="n">
-        <v>34.19363425925926</v>
+        <v>29.82237827715356</v>
       </c>
       <c r="M25" t="n">
-        <v>2.383333333333333</v>
+        <v>2.416666666666667</v>
       </c>
       <c r="N25" t="n">
-        <v>0.5698939043209876</v>
+        <v>0.4970396379525593</v>
       </c>
       <c r="O25" t="n">
-        <v>0.03972222222222222</v>
+        <v>0.04027777777777778</v>
       </c>
     </row>
     <row r="26">
@@ -3575,6 +3575,18 @@
         </is>
       </c>
       <c r="C26" t="n">
+        <v>46</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3590,43 +3602,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>120</v>
+        <v>148</v>
       </c>
       <c r="D27" t="n">
-        <v>684.9763888888888</v>
+        <v>617.0925675675675</v>
       </c>
       <c r="E27" t="n">
-        <v>134.875</v>
+        <v>146.225</v>
       </c>
       <c r="F27" t="n">
-        <v>11.41627314814815</v>
+        <v>10.28487612612613</v>
       </c>
       <c r="G27" t="n">
-        <v>2.247916666666667</v>
+        <v>2.437083333333333</v>
       </c>
       <c r="H27" t="n">
-        <v>3371.798015873016</v>
+        <v>4337.126763990268</v>
       </c>
       <c r="I27" t="n">
-        <v>2578.8</v>
+        <v>3253.15</v>
       </c>
       <c r="J27" t="n">
-        <v>56.1966335978836</v>
+        <v>72.28544606650446</v>
       </c>
       <c r="K27" t="n">
-        <v>42.98</v>
+        <v>54.21916666666667</v>
       </c>
       <c r="L27" t="n">
-        <v>2235.24126984127</v>
+        <v>3683.415936739659</v>
       </c>
       <c r="M27" t="n">
-        <v>2341.016666666667</v>
+        <v>3048.033333333333</v>
       </c>
       <c r="N27" t="n">
-        <v>37.25402116402116</v>
+        <v>61.39026561232765</v>
       </c>
       <c r="O27" t="n">
-        <v>39.01694444444445</v>
+        <v>50.80055555555555</v>
       </c>
     </row>
     <row r="28">
@@ -3641,43 +3653,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>256</v>
+        <v>443</v>
       </c>
       <c r="D28" t="n">
-        <v>237.0017578125</v>
+        <v>187.3192249811889</v>
       </c>
       <c r="E28" t="n">
-        <v>35.575</v>
+        <v>20.8</v>
       </c>
       <c r="F28" t="n">
-        <v>3.950029296875</v>
+        <v>3.121987083019814</v>
       </c>
       <c r="G28" t="n">
-        <v>0.5929166666666668</v>
+        <v>0.3466666666666667</v>
       </c>
       <c r="H28" t="n">
-        <v>898.0271144278607</v>
+        <v>943.2666666666668</v>
       </c>
       <c r="I28" t="n">
-        <v>877.7333333333333</v>
+        <v>933.9166666666666</v>
       </c>
       <c r="J28" t="n">
-        <v>14.96711857379768</v>
+        <v>15.72111111111111</v>
       </c>
       <c r="K28" t="n">
-        <v>14.62888888888889</v>
+        <v>15.56527777777778</v>
       </c>
       <c r="L28" t="n">
-        <v>628.157048092869</v>
+        <v>704.8952840300107</v>
       </c>
       <c r="M28" t="n">
-        <v>679.9166666666666</v>
+        <v>780.0166666666667</v>
       </c>
       <c r="N28" t="n">
-        <v>10.46928413488115</v>
+        <v>11.74825473383351</v>
       </c>
       <c r="O28" t="n">
-        <v>11.33194444444444</v>
+        <v>13.00027777777778</v>
       </c>
     </row>
     <row r="29">
@@ -3692,43 +3704,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>347</v>
+        <v>440</v>
       </c>
       <c r="D29" t="n">
-        <v>804.7110470701249</v>
+        <v>721.0587878787878</v>
       </c>
       <c r="E29" t="n">
-        <v>223.3333333333333</v>
+        <v>209.675</v>
       </c>
       <c r="F29" t="n">
-        <v>13.41185078450208</v>
+        <v>12.01764646464646</v>
       </c>
       <c r="G29" t="n">
-        <v>3.722222222222222</v>
+        <v>3.494583333333334</v>
       </c>
       <c r="H29" t="n">
-        <v>1508.786793540946</v>
+        <v>1588.609744779583</v>
       </c>
       <c r="I29" t="n">
-        <v>1142.75</v>
+        <v>1201.183333333333</v>
       </c>
       <c r="J29" t="n">
-        <v>25.14644655901577</v>
+        <v>26.47682907965971</v>
       </c>
       <c r="K29" t="n">
-        <v>19.04583333333333</v>
+        <v>20.01972222222222</v>
       </c>
       <c r="L29" t="n">
-        <v>671.4643598615918</v>
+        <v>862.5654292343387</v>
       </c>
       <c r="M29" t="n">
-        <v>754.7666666666667</v>
+        <v>946.4666666666667</v>
       </c>
       <c r="N29" t="n">
-        <v>11.19107266435986</v>
+        <v>14.37609048723898</v>
       </c>
       <c r="O29" t="n">
-        <v>12.57944444444444</v>
+        <v>15.77444444444444</v>
       </c>
     </row>
     <row r="30">
@@ -3743,43 +3755,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3822</v>
+        <v>6000</v>
       </c>
       <c r="D30" t="n">
-        <v>29.39793738008024</v>
+        <v>23.09763333333333</v>
       </c>
       <c r="E30" t="n">
-        <v>35.06666666666667</v>
+        <v>20.71666666666667</v>
       </c>
       <c r="F30" t="n">
-        <v>0.4899656230013373</v>
+        <v>0.3849605555555555</v>
       </c>
       <c r="G30" t="n">
-        <v>0.5844444444444445</v>
+        <v>0.3452777777777777</v>
       </c>
       <c r="H30" t="n">
-        <v>437.4889844169801</v>
+        <v>407.2903135911899</v>
       </c>
       <c r="I30" t="n">
-        <v>433.1666666666666</v>
+        <v>272.025</v>
       </c>
       <c r="J30" t="n">
-        <v>7.291483073616336</v>
+        <v>6.788171893186498</v>
       </c>
       <c r="K30" t="n">
-        <v>7.219444444444445</v>
+        <v>4.53375</v>
       </c>
       <c r="L30" t="n">
-        <v>407.9347617768224</v>
+        <v>379.9723576416868</v>
       </c>
       <c r="M30" t="n">
-        <v>405.3166666666667</v>
+        <v>240.8833333333333</v>
       </c>
       <c r="N30" t="n">
-        <v>6.798912696280375</v>
+        <v>6.332872627361447</v>
       </c>
       <c r="O30" t="n">
-        <v>6.755277777777778</v>
+        <v>4.014722222222223</v>
       </c>
     </row>
     <row r="31">
@@ -3794,43 +3806,43 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1435</v>
+        <v>2112</v>
       </c>
       <c r="D31" t="n">
-        <v>2049.078919860627</v>
+        <v>1885.034098800505</v>
       </c>
       <c r="E31" t="n">
-        <v>1522.066666666667</v>
+        <v>1421.458333333333</v>
       </c>
       <c r="F31" t="n">
-        <v>34.15131533101045</v>
+        <v>31.41723498000841</v>
       </c>
       <c r="G31" t="n">
-        <v>25.36777777777778</v>
+        <v>23.69097222222222</v>
       </c>
       <c r="H31" t="n">
-        <v>1971.404618141715</v>
+        <v>2093.89307069706</v>
       </c>
       <c r="I31" t="n">
-        <v>1569.4</v>
+        <v>1598.15</v>
       </c>
       <c r="J31" t="n">
-        <v>32.85674363569525</v>
+        <v>34.898217844951</v>
       </c>
       <c r="K31" t="n">
-        <v>26.15666666666667</v>
+        <v>26.63583333333334</v>
       </c>
       <c r="L31" t="n">
-        <v>190.3124345188861</v>
+        <v>205.5923026098447</v>
       </c>
       <c r="M31" t="n">
-        <v>225.75</v>
+        <v>226.2916666666667</v>
       </c>
       <c r="N31" t="n">
-        <v>3.171873908648102</v>
+        <v>3.426538376830746</v>
       </c>
       <c r="O31" t="n">
-        <v>3.7625</v>
+        <v>3.771527777777778</v>
       </c>
     </row>
     <row r="32">
@@ -3845,43 +3857,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2403</v>
+        <v>3615</v>
       </c>
       <c r="D32" t="n">
-        <v>350.2745665140797</v>
+        <v>417.9553019824804</v>
       </c>
       <c r="E32" t="n">
-        <v>35.15</v>
+        <v>20.88333333333333</v>
       </c>
       <c r="F32" t="n">
-        <v>5.837909441901327</v>
+        <v>6.965921699708007</v>
       </c>
       <c r="G32" t="n">
-        <v>0.5858333333333333</v>
+        <v>0.3480555555555556</v>
       </c>
       <c r="H32" t="n">
-        <v>716.5163727219283</v>
+        <v>804.7200405604719</v>
       </c>
       <c r="I32" t="n">
-        <v>522.3833333333333</v>
+        <v>525.5666666666666</v>
       </c>
       <c r="J32" t="n">
-        <v>11.94193954536547</v>
+        <v>13.41200067600787</v>
       </c>
       <c r="K32" t="n">
-        <v>8.706388888888888</v>
+        <v>8.759444444444444</v>
       </c>
       <c r="L32" t="n">
-        <v>231.0370958259847</v>
+        <v>253.8350294985251</v>
       </c>
       <c r="M32" t="n">
-        <v>46.9</v>
+        <v>54.15833333333333</v>
       </c>
       <c r="N32" t="n">
-        <v>3.850618263766412</v>
+        <v>4.230583824975418</v>
       </c>
       <c r="O32" t="n">
-        <v>0.7816666666666666</v>
+        <v>0.902638888888889</v>
       </c>
     </row>
     <row r="33">
@@ -3896,43 +3908,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4904</v>
+        <v>6933</v>
       </c>
       <c r="D33" t="n">
-        <v>326.1417482327352</v>
+        <v>412.6410620702919</v>
       </c>
       <c r="E33" t="n">
-        <v>45.45</v>
+        <v>54.56666666666667</v>
       </c>
       <c r="F33" t="n">
-        <v>5.43569580387892</v>
+        <v>6.877351034504864</v>
       </c>
       <c r="G33" t="n">
-        <v>0.7575000000000001</v>
+        <v>0.9094444444444445</v>
       </c>
       <c r="H33" t="n">
-        <v>592.7979711486538</v>
+        <v>686.5703359375001</v>
       </c>
       <c r="I33" t="n">
-        <v>289.8833333333333</v>
+        <v>326.9</v>
       </c>
       <c r="J33" t="n">
-        <v>9.879966185810897</v>
+        <v>11.44283893229167</v>
       </c>
       <c r="K33" t="n">
-        <v>4.831388888888889</v>
+        <v>5.448333333333332</v>
       </c>
       <c r="L33" t="n">
-        <v>241.0157216693667</v>
+        <v>248.14771875</v>
       </c>
       <c r="M33" t="n">
-        <v>65.28333333333333</v>
+        <v>63.94166666666666</v>
       </c>
       <c r="N33" t="n">
-        <v>4.016928694489445</v>
+        <v>4.135795312499999</v>
       </c>
       <c r="O33" t="n">
-        <v>1.088055555555556</v>
+        <v>1.065694444444444</v>
       </c>
     </row>
     <row r="34">
@@ -3947,43 +3959,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>955</v>
+        <v>1412</v>
       </c>
       <c r="D34" t="n">
-        <v>1803.980802792321</v>
+        <v>1775.183781869688</v>
       </c>
       <c r="E34" t="n">
-        <v>1456.133333333333</v>
+        <v>1776.116666666667</v>
       </c>
       <c r="F34" t="n">
-        <v>30.06634671320535</v>
+        <v>29.58639636449481</v>
       </c>
       <c r="G34" t="n">
-        <v>24.26888888888889</v>
+        <v>29.60194444444445</v>
       </c>
       <c r="H34" t="n">
-        <v>2490.034151785715</v>
+        <v>2664.186404416839</v>
       </c>
       <c r="I34" t="n">
-        <v>2178.1</v>
+        <v>2635.85</v>
       </c>
       <c r="J34" t="n">
-        <v>41.50056919642857</v>
+        <v>44.40310674028066</v>
       </c>
       <c r="K34" t="n">
-        <v>36.30166666666666</v>
+        <v>43.93083333333334</v>
       </c>
       <c r="L34" t="n">
-        <v>486.3879960317461</v>
+        <v>586.1867322291235</v>
       </c>
       <c r="M34" t="n">
-        <v>525.45</v>
+        <v>525.4166666666666</v>
       </c>
       <c r="N34" t="n">
-        <v>8.1064666005291</v>
+        <v>9.769778870485393</v>
       </c>
       <c r="O34" t="n">
-        <v>8.7575</v>
+        <v>8.756944444444445</v>
       </c>
     </row>
     <row r="35">
@@ -3998,43 +4010,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1381</v>
+        <v>1850</v>
       </c>
       <c r="D35" t="n">
-        <v>2040.944219164857</v>
+        <v>2125.079423423424</v>
       </c>
       <c r="E35" t="n">
-        <v>2009.483333333333</v>
+        <v>2124.641666666666</v>
       </c>
       <c r="F35" t="n">
-        <v>34.01573698608095</v>
+        <v>35.41799039039039</v>
       </c>
       <c r="G35" t="n">
-        <v>33.49138888888889</v>
+        <v>35.41069444444445</v>
       </c>
       <c r="H35" t="n">
-        <v>2686.576202239789</v>
+        <v>2787.761152968037</v>
       </c>
       <c r="I35" t="n">
-        <v>2400.666666666667</v>
+        <v>2703.5</v>
       </c>
       <c r="J35" t="n">
-        <v>44.77627003732982</v>
+        <v>46.46268588280061</v>
       </c>
       <c r="K35" t="n">
-        <v>40.01111111111111</v>
+        <v>45.05833333333334</v>
       </c>
       <c r="L35" t="n">
-        <v>468.0734683794466</v>
+        <v>556.6087785388128</v>
       </c>
       <c r="M35" t="n">
-        <v>524.9583333333334</v>
+        <v>524.4333333333333</v>
       </c>
       <c r="N35" t="n">
-        <v>7.801224472990778</v>
+        <v>9.27681297564688</v>
       </c>
       <c r="O35" t="n">
-        <v>8.749305555555555</v>
+        <v>8.740555555555554</v>
       </c>
     </row>
     <row r="36">
@@ -4049,43 +4061,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>496</v>
+        <v>757</v>
       </c>
       <c r="D36" t="n">
-        <v>29.20517473118279</v>
+        <v>22.18126376045795</v>
       </c>
       <c r="E36" t="n">
-        <v>23.95</v>
+        <v>20.65</v>
       </c>
       <c r="F36" t="n">
-        <v>0.48675291218638</v>
+        <v>0.3696877293409658</v>
       </c>
       <c r="G36" t="n">
-        <v>0.3991666666666667</v>
+        <v>0.3441666666666666</v>
       </c>
       <c r="H36" t="n">
-        <v>1335.057786357786</v>
+        <v>2096.005545722714</v>
       </c>
       <c r="I36" t="n">
-        <v>1389.016666666667</v>
+        <v>1685.566666666667</v>
       </c>
       <c r="J36" t="n">
-        <v>22.2509631059631</v>
+        <v>34.93342576204523</v>
       </c>
       <c r="K36" t="n">
-        <v>23.15027777777778</v>
+        <v>28.09277777777778</v>
       </c>
       <c r="L36" t="n">
-        <v>1301.38314028314</v>
+        <v>2067.918348082596</v>
       </c>
       <c r="M36" t="n">
-        <v>1346.666666666667</v>
+        <v>1638.2</v>
       </c>
       <c r="N36" t="n">
-        <v>21.689719004719</v>
+        <v>34.46530580137659</v>
       </c>
       <c r="O36" t="n">
-        <v>22.44444444444445</v>
+        <v>27.30333333333333</v>
       </c>
     </row>
     <row r="37">
@@ -4100,43 +4112,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>268</v>
+        <v>385</v>
       </c>
       <c r="D37" t="n">
-        <v>2182.42947761194</v>
+        <v>2319.501558441559</v>
       </c>
       <c r="E37" t="n">
-        <v>1671.025</v>
+        <v>2302.85</v>
       </c>
       <c r="F37" t="n">
-        <v>36.37382462686568</v>
+        <v>38.65835930735931</v>
       </c>
       <c r="G37" t="n">
-        <v>27.85041666666667</v>
+        <v>38.38083333333334</v>
       </c>
       <c r="H37" t="n">
-        <v>2559.436622807018</v>
+        <v>2713.626754385965</v>
       </c>
       <c r="I37" t="n">
-        <v>2293.066666666667</v>
+        <v>2717.991666666667</v>
       </c>
       <c r="J37" t="n">
-        <v>42.65727704678363</v>
+        <v>45.22711257309941</v>
       </c>
       <c r="K37" t="n">
-        <v>38.21777777777778</v>
+        <v>45.29986111111111</v>
       </c>
       <c r="L37" t="n">
-        <v>215.0663742690058</v>
+        <v>284.026461988304</v>
       </c>
       <c r="M37" t="n">
-        <v>158.0916666666667</v>
+        <v>232.3416666666667</v>
       </c>
       <c r="N37" t="n">
-        <v>3.584439571150097</v>
+        <v>4.733774366471735</v>
       </c>
       <c r="O37" t="n">
-        <v>2.634861111111111</v>
+        <v>3.872361111111111</v>
       </c>
     </row>
     <row r="38">
@@ -4151,7 +4163,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>18</v>
+        <v>194</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -4166,28 +4178,28 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>305.015</v>
+        <v>232.8547619047619</v>
       </c>
       <c r="I38" t="n">
-        <v>130.7833333333333</v>
+        <v>66.925</v>
       </c>
       <c r="J38" t="n">
-        <v>5.083583333333333</v>
+        <v>3.880912698412698</v>
       </c>
       <c r="K38" t="n">
-        <v>2.179722222222222</v>
+        <v>1.115416666666667</v>
       </c>
       <c r="L38" t="n">
-        <v>305.015</v>
+        <v>232.8547619047619</v>
       </c>
       <c r="M38" t="n">
-        <v>130.7833333333333</v>
+        <v>66.925</v>
       </c>
       <c r="N38" t="n">
-        <v>5.083583333333333</v>
+        <v>3.880912698412698</v>
       </c>
       <c r="O38" t="n">
-        <v>2.179722222222222</v>
+        <v>1.115416666666667</v>
       </c>
     </row>
     <row r="39">
@@ -4202,43 +4214,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>555</v>
+        <v>760</v>
       </c>
       <c r="D39" t="n">
-        <v>235.5743543543543</v>
+        <v>236.2387938596491</v>
       </c>
       <c r="E39" t="n">
-        <v>91.8</v>
+        <v>93.05000000000001</v>
       </c>
       <c r="F39" t="n">
-        <v>3.926239239239239</v>
+        <v>3.937313230994152</v>
       </c>
       <c r="G39" t="n">
-        <v>1.53</v>
+        <v>1.550833333333333</v>
       </c>
       <c r="H39" t="n">
-        <v>562.3424186617557</v>
+        <v>535.3983533600357</v>
       </c>
       <c r="I39" t="n">
-        <v>500.6166666666667</v>
+        <v>445.8666666666667</v>
       </c>
       <c r="J39" t="n">
-        <v>9.372373644362595</v>
+        <v>8.923305889333927</v>
       </c>
       <c r="K39" t="n">
-        <v>8.343611111111111</v>
+        <v>7.431111111111111</v>
       </c>
       <c r="L39" t="n">
-        <v>323.6876918354819</v>
+        <v>297.3450378282154</v>
       </c>
       <c r="M39" t="n">
-        <v>249.6666666666667</v>
+        <v>194.8166666666667</v>
       </c>
       <c r="N39" t="n">
-        <v>5.394794863924698</v>
+        <v>4.955750630470257</v>
       </c>
       <c r="O39" t="n">
-        <v>4.161111111111111</v>
+        <v>3.246944444444444</v>
       </c>
     </row>
     <row r="40">
@@ -4253,40 +4265,40 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>12133</v>
+        <v>21526</v>
       </c>
       <c r="D40" t="n">
-        <v>286.3783386906234</v>
+        <v>169.9221158908607</v>
       </c>
       <c r="E40" t="n">
-        <v>35.51666666666667</v>
+        <v>20.68333333333333</v>
       </c>
       <c r="F40" t="n">
-        <v>4.772972311510389</v>
+        <v>2.832035264847678</v>
       </c>
       <c r="G40" t="n">
-        <v>0.5919444444444444</v>
+        <v>0.3447222222222222</v>
       </c>
       <c r="H40" t="n">
-        <v>347.9983139677856</v>
+        <v>260.7236201449545</v>
       </c>
       <c r="I40" t="n">
-        <v>35.93333333333333</v>
+        <v>21.18333333333333</v>
       </c>
       <c r="J40" t="n">
-        <v>5.799971899463093</v>
+        <v>4.345393669082575</v>
       </c>
       <c r="K40" t="n">
-        <v>0.5988888888888888</v>
+        <v>0.3530555555555556</v>
       </c>
       <c r="L40" t="n">
-        <v>32.36273669002828</v>
+        <v>36.88921204237131</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.5393789448338047</v>
+        <v>0.6148202007061884</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -4304,43 +4316,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>4969</v>
+        <v>6488</v>
       </c>
       <c r="D41" t="n">
-        <v>925.4605118400751</v>
+        <v>798.2948520345253</v>
       </c>
       <c r="E41" t="n">
-        <v>752.8166666666667</v>
+        <v>643.3583333333333</v>
       </c>
       <c r="F41" t="n">
-        <v>15.42434186400125</v>
+        <v>13.30491420057542</v>
       </c>
       <c r="G41" t="n">
-        <v>12.54694444444445</v>
+        <v>10.72263888888889</v>
       </c>
       <c r="H41" t="n">
-        <v>909.4797028855211</v>
+        <v>885.273290113452</v>
       </c>
       <c r="I41" t="n">
-        <v>777.8833333333333</v>
+        <v>741.6166666666667</v>
       </c>
       <c r="J41" t="n">
-        <v>15.15799504809202</v>
+        <v>14.7545548352242</v>
       </c>
       <c r="K41" t="n">
-        <v>12.96472222222222</v>
+        <v>12.36027777777778</v>
       </c>
       <c r="L41" t="n">
-        <v>76.6857179553044</v>
+        <v>80.94260129659644</v>
       </c>
       <c r="M41" t="n">
-        <v>74.55</v>
+        <v>73.72499999999999</v>
       </c>
       <c r="N41" t="n">
-        <v>1.278095299255073</v>
+        <v>1.349043354943274</v>
       </c>
       <c r="O41" t="n">
-        <v>1.2425</v>
+        <v>1.22875</v>
       </c>
     </row>
     <row r="42">
@@ -4355,43 +4367,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>32103</v>
+        <v>45310</v>
       </c>
       <c r="D42" t="n">
-        <v>27.52259238492768</v>
+        <v>25.02397594350033</v>
       </c>
       <c r="E42" t="n">
-        <v>20.93333333333333</v>
+        <v>20.76666666666667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.458709873082128</v>
+        <v>0.4170662657250055</v>
       </c>
       <c r="G42" t="n">
-        <v>0.3488888888888889</v>
+        <v>0.3461111111111111</v>
       </c>
       <c r="H42" t="n">
-        <v>358.2117837626854</v>
+        <v>513.9659371931564</v>
       </c>
       <c r="I42" t="n">
-        <v>181.1833333333333</v>
+        <v>201.8</v>
       </c>
       <c r="J42" t="n">
-        <v>5.970196396044757</v>
+        <v>8.566098953219273</v>
       </c>
       <c r="K42" t="n">
-        <v>3.019722222222222</v>
+        <v>3.363333333333334</v>
       </c>
       <c r="L42" t="n">
-        <v>328.0706915170439</v>
+        <v>486.9684679752874</v>
       </c>
       <c r="M42" t="n">
-        <v>149.2666666666667</v>
+        <v>172.45</v>
       </c>
       <c r="N42" t="n">
-        <v>5.467844858617399</v>
+        <v>8.116141132921456</v>
       </c>
       <c r="O42" t="n">
-        <v>2.487777777777778</v>
+        <v>2.874166666666667</v>
       </c>
     </row>
     <row r="43">
@@ -4406,43 +4418,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>24279</v>
+        <v>32696</v>
       </c>
       <c r="D43" t="n">
-        <v>152.3982481431141</v>
+        <v>152.1490860247941</v>
       </c>
       <c r="E43" t="n">
-        <v>73.76666666666667</v>
+        <v>76.63333333333334</v>
       </c>
       <c r="F43" t="n">
-        <v>2.539970802385235</v>
+        <v>2.535818100413234</v>
       </c>
       <c r="G43" t="n">
-        <v>1.229444444444444</v>
+        <v>1.277222222222222</v>
       </c>
       <c r="H43" t="n">
-        <v>400.0978985373079</v>
+        <v>538.6446022542185</v>
       </c>
       <c r="I43" t="n">
-        <v>209.5</v>
+        <v>232.3666666666667</v>
       </c>
       <c r="J43" t="n">
-        <v>6.668298308955132</v>
+        <v>8.977410037570309</v>
       </c>
       <c r="K43" t="n">
-        <v>3.491666666666667</v>
+        <v>3.872777777777777</v>
       </c>
       <c r="L43" t="n">
-        <v>249.3663773683886</v>
+        <v>386.5592867070602</v>
       </c>
       <c r="M43" t="n">
-        <v>102.825</v>
+        <v>113.325</v>
       </c>
       <c r="N43" t="n">
-        <v>4.156106289473143</v>
+        <v>6.442654778451003</v>
       </c>
       <c r="O43" t="n">
-        <v>1.71375</v>
+        <v>1.88875</v>
       </c>
     </row>
     <row r="44">
@@ -4457,43 +4469,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3025</v>
+        <v>4451</v>
       </c>
       <c r="D44" t="n">
-        <v>25.20775757575758</v>
+        <v>20.47282633116154</v>
       </c>
       <c r="E44" t="n">
-        <v>20.85</v>
+        <v>20.61666666666667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.4201292929292929</v>
+        <v>0.3412137721860256</v>
       </c>
       <c r="G44" t="n">
-        <v>0.3475</v>
+        <v>0.3436111111111111</v>
       </c>
       <c r="H44" t="n">
-        <v>975.1987601842011</v>
+        <v>925.2382991669007</v>
       </c>
       <c r="I44" t="n">
-        <v>851.1333333333333</v>
+        <v>831.4</v>
       </c>
       <c r="J44" t="n">
-        <v>16.25331266973669</v>
+        <v>15.42063831944835</v>
       </c>
       <c r="K44" t="n">
-        <v>14.18555555555556</v>
+        <v>13.85666666666667</v>
       </c>
       <c r="L44" t="n">
-        <v>949.1032471366158</v>
+        <v>900.288912290555</v>
       </c>
       <c r="M44" t="n">
-        <v>828.5833333333334</v>
+        <v>809.9666666666667</v>
       </c>
       <c r="N44" t="n">
-        <v>15.81838745227693</v>
+        <v>15.00481520484258</v>
       </c>
       <c r="O44" t="n">
-        <v>13.80972222222222</v>
+        <v>13.49944444444444</v>
       </c>
     </row>
     <row r="45">
@@ -4508,43 +4520,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>7899</v>
+        <v>10214</v>
       </c>
       <c r="D45" t="n">
-        <v>210.7227497151538</v>
+        <v>191.2924450101168</v>
       </c>
       <c r="E45" t="n">
-        <v>23.45</v>
+        <v>19.95</v>
       </c>
       <c r="F45" t="n">
-        <v>3.512045828585897</v>
+        <v>3.18820741683528</v>
       </c>
       <c r="G45" t="n">
-        <v>0.3908333333333333</v>
+        <v>0.3325</v>
       </c>
       <c r="H45" t="n">
-        <v>811.1560036454772</v>
+        <v>837.4699847483478</v>
       </c>
       <c r="I45" t="n">
-        <v>792.8833333333333</v>
+        <v>853.2</v>
       </c>
       <c r="J45" t="n">
-        <v>13.51926672742462</v>
+        <v>13.95783307913913</v>
       </c>
       <c r="K45" t="n">
-        <v>13.21472222222222</v>
+        <v>14.22</v>
       </c>
       <c r="L45" t="n">
-        <v>598.9181453634085</v>
+        <v>645.3405660057617</v>
       </c>
       <c r="M45" t="n">
-        <v>423.95</v>
+        <v>485.65</v>
       </c>
       <c r="N45" t="n">
-        <v>9.981969089390141</v>
+        <v>10.75567610009603</v>
       </c>
       <c r="O45" t="n">
-        <v>7.065833333333333</v>
+        <v>8.094166666666666</v>
       </c>
     </row>
     <row r="46">
@@ -4559,43 +4571,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>488</v>
+        <v>684</v>
       </c>
       <c r="D46" t="n">
-        <v>24.9521174863388</v>
+        <v>19.69739278752436</v>
       </c>
       <c r="E46" t="n">
-        <v>20.85</v>
+        <v>20.63333333333333</v>
       </c>
       <c r="F46" t="n">
-        <v>0.4158686247723133</v>
+        <v>0.3282898797920728</v>
       </c>
       <c r="G46" t="n">
-        <v>0.3475</v>
+        <v>0.3438888888888889</v>
       </c>
       <c r="H46" t="n">
-        <v>2848.708794326241</v>
+        <v>3262.247438456421</v>
       </c>
       <c r="I46" t="n">
-        <v>2643.066666666667</v>
+        <v>2852.433333333333</v>
       </c>
       <c r="J46" t="n">
-        <v>47.47847990543735</v>
+        <v>54.37079064094033</v>
       </c>
       <c r="K46" t="n">
-        <v>44.05111111111111</v>
+        <v>47.54055555555556</v>
       </c>
       <c r="L46" t="n">
-        <v>2816.744397163121</v>
+        <v>3236.295908183633</v>
       </c>
       <c r="M46" t="n">
-        <v>2597.433333333333</v>
+        <v>2816.433333333333</v>
       </c>
       <c r="N46" t="n">
-        <v>46.94573995271867</v>
+        <v>53.93826513639387</v>
       </c>
       <c r="O46" t="n">
-        <v>43.29055555555556</v>
+        <v>46.94055555555556</v>
       </c>
     </row>
     <row r="47">
@@ -4610,43 +4622,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>809</v>
+        <v>982</v>
       </c>
       <c r="D47" t="n">
-        <v>215.8476926246394</v>
+        <v>203.6907162253904</v>
       </c>
       <c r="E47" t="n">
-        <v>38</v>
+        <v>38.29166666666667</v>
       </c>
       <c r="F47" t="n">
-        <v>3.597461543743992</v>
+        <v>3.394845270423173</v>
       </c>
       <c r="G47" t="n">
-        <v>0.6333333333333333</v>
+        <v>0.6381944444444445</v>
       </c>
       <c r="H47" t="n">
-        <v>3039.955669144981</v>
+        <v>3136.334719260839</v>
       </c>
       <c r="I47" t="n">
-        <v>2831.283333333333</v>
+        <v>2892.125</v>
       </c>
       <c r="J47" t="n">
-        <v>50.66592781908302</v>
+        <v>52.27224532101398</v>
       </c>
       <c r="K47" t="n">
-        <v>47.18805555555555</v>
+        <v>48.20208333333333</v>
       </c>
       <c r="L47" t="n">
-        <v>2844.073884758364</v>
+        <v>2927.867537313433</v>
       </c>
       <c r="M47" t="n">
-        <v>2806.391666666666</v>
+        <v>2816.091666666667</v>
       </c>
       <c r="N47" t="n">
-        <v>47.4012314126394</v>
+        <v>48.79779228855722</v>
       </c>
       <c r="O47" t="n">
-        <v>46.77319444444444</v>
+        <v>46.93486111111111</v>
       </c>
     </row>
     <row r="48">
@@ -4661,43 +4673,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2415</v>
+        <v>3677</v>
       </c>
       <c r="D48" t="n">
-        <v>29.62420289855073</v>
+        <v>23.22049224911613</v>
       </c>
       <c r="E48" t="n">
-        <v>35.1</v>
+        <v>20.7</v>
       </c>
       <c r="F48" t="n">
-        <v>0.4937367149758454</v>
+        <v>0.3870082041519355</v>
       </c>
       <c r="G48" t="n">
-        <v>0.5850000000000001</v>
+        <v>0.345</v>
       </c>
       <c r="H48" t="n">
-        <v>439.3307703904719</v>
+        <v>459.0204166666667</v>
       </c>
       <c r="I48" t="n">
-        <v>373.95</v>
+        <v>397.7333333333333</v>
       </c>
       <c r="J48" t="n">
-        <v>7.322179506507865</v>
+        <v>7.650340277777778</v>
       </c>
       <c r="K48" t="n">
-        <v>6.2325</v>
+        <v>6.628888888888889</v>
       </c>
       <c r="L48" t="n">
-        <v>408.8652344338912</v>
+        <v>431.2479550438596</v>
       </c>
       <c r="M48" t="n">
-        <v>342.9</v>
+        <v>359.6583333333333</v>
       </c>
       <c r="N48" t="n">
-        <v>6.814420573898186</v>
+        <v>7.187465917397661</v>
       </c>
       <c r="O48" t="n">
-        <v>5.715</v>
+        <v>5.994305555555556</v>
       </c>
     </row>
     <row r="49">
@@ -4712,43 +4724,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1248</v>
+        <v>1751</v>
       </c>
       <c r="D49" t="n">
-        <v>357.3351896367521</v>
+        <v>325.5730630116124</v>
       </c>
       <c r="E49" t="n">
-        <v>153.0833333333333</v>
+        <v>120.7666666666667</v>
       </c>
       <c r="F49" t="n">
-        <v>5.955586493945868</v>
+        <v>5.426217716860207</v>
       </c>
       <c r="G49" t="n">
-        <v>2.551388888888889</v>
+        <v>2.012777777777778</v>
       </c>
       <c r="H49" t="n">
-        <v>697.2663052905465</v>
+        <v>709.9369640787949</v>
       </c>
       <c r="I49" t="n">
-        <v>570.6</v>
+        <v>574.8916666666667</v>
       </c>
       <c r="J49" t="n">
-        <v>11.62110508817577</v>
+        <v>11.83228273464658</v>
       </c>
       <c r="K49" t="n">
-        <v>9.51</v>
+        <v>9.581527777777779</v>
       </c>
       <c r="L49" t="n">
-        <v>334.1105377276669</v>
+        <v>383.0971996910004</v>
       </c>
       <c r="M49" t="n">
-        <v>193.85</v>
+        <v>223.8083333333333</v>
       </c>
       <c r="N49" t="n">
-        <v>5.568508962127782</v>
+        <v>6.384953328183339</v>
       </c>
       <c r="O49" t="n">
-        <v>3.230833333333333</v>
+        <v>3.730138888888889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard mar 18/08/2026  8:13:02,05
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -680,19 +680,19 @@
         <v>65.29306173417623</v>
       </c>
       <c r="W2" t="n">
-        <v>4214</v>
+        <v>6029</v>
       </c>
       <c r="X2" t="n">
-        <v>16.49264356905553</v>
+        <v>17.93000497594958</v>
       </c>
       <c r="Y2" t="n">
-        <v>70.45562411010916</v>
+        <v>71.52098192071654</v>
       </c>
       <c r="Z2" t="n">
-        <v>3.107800050753802</v>
+        <v>4.545161457647851</v>
       </c>
       <c r="AA2" t="n">
-        <v>-67.11152735503005</v>
+        <v>-52.9462264887224</v>
       </c>
     </row>
     <row r="3">
@@ -765,19 +765,19 @@
         <v>77.58389261744966</v>
       </c>
       <c r="W3" t="n">
-        <v>196</v>
+        <v>284</v>
       </c>
       <c r="X3" t="n">
-        <v>8.673469387755102</v>
+        <v>9.859154929577464</v>
       </c>
       <c r="Y3" t="n">
-        <v>80.61224489795919</v>
+        <v>80.63380281690141</v>
       </c>
       <c r="Z3" t="n">
-        <v>-18.03794000821805</v>
+        <v>-16.85225446639569</v>
       </c>
       <c r="AA3" t="n">
-        <v>-73.69127516778524</v>
+        <v>-61.87919463087248</v>
       </c>
     </row>
     <row r="4">
@@ -850,19 +850,19 @@
         <v>34.85881207400195</v>
       </c>
       <c r="W4" t="n">
-        <v>194</v>
+        <v>226</v>
       </c>
       <c r="X4" t="n">
-        <v>23.71134020618556</v>
+        <v>21.23893805309735</v>
       </c>
       <c r="Y4" t="n">
-        <v>64.43298969072166</v>
+        <v>62.83185840707964</v>
       </c>
       <c r="Z4" t="n">
-        <v>23.5165982392917</v>
+        <v>21.04419608620348</v>
       </c>
       <c r="AA4" t="n">
-        <v>-81.11002921129503</v>
+        <v>-77.99415774099319</v>
       </c>
     </row>
     <row r="5">
@@ -935,19 +935,19 @@
         <v>52.69410267288927</v>
       </c>
       <c r="W5" t="n">
-        <v>883</v>
+        <v>1264</v>
       </c>
       <c r="X5" t="n">
-        <v>50.16987542468856</v>
+        <v>52.29430379746836</v>
       </c>
       <c r="Y5" t="n">
-        <v>61.26840317100793</v>
+        <v>60.68037974683544</v>
       </c>
       <c r="Z5" t="n">
-        <v>11.60390172931308</v>
+        <v>13.72833010209288</v>
       </c>
       <c r="AA5" t="n">
-        <v>-62.537123462028</v>
+        <v>-46.37250742469241</v>
       </c>
     </row>
     <row r="6">
@@ -1020,19 +1020,19 @@
         <v>64.41954378433441</v>
       </c>
       <c r="W6" t="n">
-        <v>8112</v>
+        <v>12405</v>
       </c>
       <c r="X6" t="n">
-        <v>73.96449704142012</v>
+        <v>75.67916162837565</v>
       </c>
       <c r="Y6" t="n">
-        <v>78.31607495069034</v>
+        <v>79.77428456267634</v>
       </c>
       <c r="Z6" t="n">
-        <v>14.13257649716283</v>
+        <v>15.84724108411837</v>
       </c>
       <c r="AA6" t="n">
-        <v>-70.4878669916688</v>
+        <v>-54.8695747080438</v>
       </c>
     </row>
     <row r="7">
@@ -1105,19 +1105,19 @@
         <v>61.85549639414975</v>
       </c>
       <c r="W7" t="n">
-        <v>10548</v>
+        <v>15471</v>
       </c>
       <c r="X7" t="n">
-        <v>34.27189988623436</v>
+        <v>40.26889018163015</v>
       </c>
       <c r="Y7" t="n">
-        <v>63.65187713310581</v>
+        <v>64.4431517031866</v>
       </c>
       <c r="Z7" t="n">
-        <v>-1.560815622291621</v>
+        <v>4.436174673104169</v>
       </c>
       <c r="AA7" t="n">
-        <v>-64.45373053851857</v>
+        <v>-47.86344948439712</v>
       </c>
     </row>
     <row r="8">
@@ -1190,19 +1190,19 @@
         <v>53.9494851994852</v>
       </c>
       <c r="W8" t="n">
-        <v>3262</v>
+        <v>4279</v>
       </c>
       <c r="X8" t="n">
-        <v>43.28632740649908</v>
+        <v>46.0855340032718</v>
       </c>
       <c r="Y8" t="n">
-        <v>63.18209687308399</v>
+        <v>63.16896471138116</v>
       </c>
       <c r="Z8" t="n">
-        <v>6.7033158234875</v>
+        <v>9.502522420260213</v>
       </c>
       <c r="AA8" t="n">
-        <v>-73.76126126126125</v>
+        <v>-65.58075933075934</v>
       </c>
     </row>
     <row r="9">
@@ -1275,19 +1275,19 @@
         <v>68.22074215033301</v>
       </c>
       <c r="W9" t="n">
-        <v>1142</v>
+        <v>1627</v>
       </c>
       <c r="X9" t="n">
-        <v>66.28721541155866</v>
+        <v>69.94468346650277</v>
       </c>
       <c r="Y9" t="n">
-        <v>74.25569176882661</v>
+        <v>76.64413030116779</v>
       </c>
       <c r="Z9" t="n">
-        <v>6.201582680826021</v>
+        <v>9.859050735770126</v>
       </c>
       <c r="AA9" t="n">
-        <v>-72.83539486203615</v>
+        <v>-61.29876308277831</v>
       </c>
     </row>
     <row r="10">
@@ -1360,19 +1360,19 @@
         <v>36.93293885601578</v>
       </c>
       <c r="W10" t="n">
-        <v>954</v>
+        <v>1413</v>
       </c>
       <c r="X10" t="n">
-        <v>20.33542976939203</v>
+        <v>21.37296532200991</v>
       </c>
       <c r="Y10" t="n">
-        <v>53.77358490566038</v>
+        <v>54.98938428874735</v>
       </c>
       <c r="Z10" t="n">
-        <v>17.57408854651235</v>
+        <v>18.61162409913022</v>
       </c>
       <c r="AA10" t="n">
-        <v>-52.95857988165681</v>
+        <v>-30.32544378698225</v>
       </c>
     </row>
     <row r="11">
@@ -1445,19 +1445,19 @@
         <v>73.6447415973979</v>
       </c>
       <c r="W11" t="n">
-        <v>28014</v>
+        <v>41977</v>
       </c>
       <c r="X11" t="n">
-        <v>76.84015135289498</v>
+        <v>77.93791838387688</v>
       </c>
       <c r="Y11" t="n">
-        <v>81.50210608981223</v>
+        <v>81.99013745622604</v>
       </c>
       <c r="Z11" t="n">
-        <v>9.166452400961475</v>
+        <v>10.26421943194337</v>
       </c>
       <c r="AA11" t="n">
-        <v>-68.36149259125406</v>
+        <v>-52.59193169497651</v>
       </c>
     </row>
     <row r="12">
@@ -1530,19 +1530,19 @@
         <v>74.93570456560008</v>
       </c>
       <c r="W12" t="n">
-        <v>78006</v>
+        <v>114113</v>
       </c>
       <c r="X12" t="n">
-        <v>58.08527549162885</v>
+        <v>59.29473416700989</v>
       </c>
       <c r="Y12" t="n">
-        <v>78.56575135246007</v>
+        <v>78.01389850411434</v>
       </c>
       <c r="Z12" t="n">
-        <v>1.095799967589848</v>
+        <v>2.305258642970884</v>
       </c>
       <c r="AA12" t="n">
-        <v>-75.65325409805365</v>
+        <v>-64.38376259379018</v>
       </c>
     </row>
     <row r="13">
@@ -1615,19 +1615,19 @@
         <v>60.82532992468735</v>
       </c>
       <c r="W13" t="n">
-        <v>14665</v>
+        <v>21432</v>
       </c>
       <c r="X13" t="n">
-        <v>30.35117627003068</v>
+        <v>35.70828667413214</v>
       </c>
       <c r="Y13" t="n">
-        <v>64.99147630412547</v>
+        <v>65.02892870474058</v>
       </c>
       <c r="Z13" t="n">
-        <v>2.73596173261619</v>
+        <v>8.093072136717645</v>
       </c>
       <c r="AA13" t="n">
-        <v>-74.66834795826712</v>
+        <v>-62.97934084156706</v>
       </c>
     </row>
     <row r="14">
@@ -1700,19 +1700,19 @@
         <v>60.31513970110461</v>
       </c>
       <c r="W14" t="n">
-        <v>1666</v>
+        <v>2278</v>
       </c>
       <c r="X14" t="n">
-        <v>41.05642256902761</v>
+        <v>43.06409130816506</v>
       </c>
       <c r="Y14" t="n">
-        <v>68.36734693877551</v>
+        <v>69.75417032484636</v>
       </c>
       <c r="Z14" t="n">
-        <v>7.381958631405773</v>
+        <v>9.389627370543224</v>
       </c>
       <c r="AA14" t="n">
-        <v>-72.93697205977908</v>
+        <v>-62.99545159194282</v>
       </c>
     </row>
     <row r="15">
@@ -1785,19 +1785,19 @@
         <v>74.15969011620642</v>
       </c>
       <c r="W15" t="n">
-        <v>5428</v>
+        <v>7846</v>
       </c>
       <c r="X15" t="n">
-        <v>67.74134119380987</v>
+        <v>68.69742543971449</v>
       </c>
       <c r="Y15" t="n">
-        <v>79.93736182756079</v>
+        <v>79.17410145296967</v>
       </c>
       <c r="Z15" t="n">
-        <v>8.544789900544856</v>
+        <v>9.500874146449476</v>
       </c>
       <c r="AA15" t="n">
-        <v>-66.08771710608522</v>
+        <v>-50.98088216918656</v>
       </c>
     </row>
   </sheetData>
@@ -1876,19 +1876,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2870</v>
+        <v>4637</v>
       </c>
       <c r="C4" t="n">
-        <v>441</v>
+        <v>717</v>
       </c>
       <c r="D4" t="n">
-        <v>15.36585365853658</v>
+        <v>15.4625835669614</v>
       </c>
       <c r="E4" t="n">
-        <v>669.0308163265305</v>
+        <v>640.6675034867503</v>
       </c>
       <c r="F4" t="n">
-        <v>1297.273589954714</v>
+        <v>1210.727375</v>
       </c>
     </row>
     <row r="5">
@@ -1898,19 +1898,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>111451</v>
+        <v>163034</v>
       </c>
       <c r="C5" t="n">
-        <v>80869</v>
+        <v>123063</v>
       </c>
       <c r="D5" t="n">
-        <v>72.56013853621771</v>
+        <v>75.48302808003238</v>
       </c>
       <c r="E5" t="n">
-        <v>4036.01766286216</v>
+        <v>4370.045520959995</v>
       </c>
       <c r="F5" t="n">
-        <v>5854.246933326794</v>
+        <v>6531.543080608441</v>
       </c>
     </row>
     <row r="6">
@@ -1920,19 +1920,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34695</v>
+        <v>50827</v>
       </c>
       <c r="C6" t="n">
-        <v>4317</v>
+        <v>6600</v>
       </c>
       <c r="D6" t="n">
-        <v>12.44271508862949</v>
+        <v>12.98522438861235</v>
       </c>
       <c r="E6" t="n">
-        <v>9107.960889506601</v>
+        <v>9818.861668181818</v>
       </c>
       <c r="F6" t="n">
-        <v>4469.714320228455</v>
+        <v>4235.714070361995</v>
       </c>
     </row>
     <row r="7">
@@ -1942,19 +1942,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8268</v>
+        <v>12146</v>
       </c>
       <c r="C7" t="n">
-        <v>3200</v>
+        <v>4871</v>
       </c>
       <c r="D7" t="n">
-        <v>38.70343492985002</v>
+        <v>40.10373785608431</v>
       </c>
       <c r="E7" t="n">
-        <v>842.7509875000001</v>
+        <v>886.6248624512421</v>
       </c>
       <c r="F7" t="n">
-        <v>3799.223310970797</v>
+        <v>3569.86883024055</v>
       </c>
     </row>
     <row r="8"/>
@@ -2996,19 +2996,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4214</v>
+        <v>6029</v>
       </c>
       <c r="C4" t="n">
-        <v>695</v>
+        <v>1081</v>
       </c>
       <c r="D4" t="n">
-        <v>16.49264356905553</v>
+        <v>17.93000497594958</v>
       </c>
       <c r="E4" t="n">
-        <v>2969</v>
+        <v>4312</v>
       </c>
       <c r="F4" t="n">
-        <v>70.45562411010916</v>
+        <v>71.52098192071654</v>
       </c>
     </row>
     <row r="5">
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>196</v>
+        <v>284</v>
       </c>
       <c r="C5" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="D5" t="n">
-        <v>8.673469387755102</v>
+        <v>9.859154929577464</v>
       </c>
       <c r="E5" t="n">
-        <v>158</v>
+        <v>229</v>
       </c>
       <c r="F5" t="n">
-        <v>80.61224489795919</v>
+        <v>80.63380281690141</v>
       </c>
     </row>
     <row r="6">
@@ -3040,19 +3040,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>194</v>
+        <v>226</v>
       </c>
       <c r="C6" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D6" t="n">
-        <v>23.71134020618556</v>
+        <v>21.23893805309735</v>
       </c>
       <c r="E6" t="n">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="F6" t="n">
-        <v>64.43298969072166</v>
+        <v>62.83185840707964</v>
       </c>
     </row>
     <row r="7">
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>883</v>
+        <v>1264</v>
       </c>
       <c r="C7" t="n">
-        <v>443</v>
+        <v>661</v>
       </c>
       <c r="D7" t="n">
-        <v>50.16987542468856</v>
+        <v>52.29430379746836</v>
       </c>
       <c r="E7" t="n">
-        <v>541</v>
+        <v>767</v>
       </c>
       <c r="F7" t="n">
-        <v>61.26840317100793</v>
+        <v>60.68037974683544</v>
       </c>
     </row>
     <row r="8">
@@ -3084,19 +3084,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8112</v>
+        <v>12405</v>
       </c>
       <c r="C8" t="n">
-        <v>6000</v>
+        <v>9388</v>
       </c>
       <c r="D8" t="n">
-        <v>73.96449704142012</v>
+        <v>75.67916162837565</v>
       </c>
       <c r="E8" t="n">
-        <v>6353</v>
+        <v>9896</v>
       </c>
       <c r="F8" t="n">
-        <v>78.31607495069034</v>
+        <v>79.77428456267634</v>
       </c>
     </row>
     <row r="9">
@@ -3106,19 +3106,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10548</v>
+        <v>15471</v>
       </c>
       <c r="C9" t="n">
-        <v>3615</v>
+        <v>6230</v>
       </c>
       <c r="D9" t="n">
-        <v>34.27189988623436</v>
+        <v>40.26889018163015</v>
       </c>
       <c r="E9" t="n">
-        <v>6714</v>
+        <v>9970</v>
       </c>
       <c r="F9" t="n">
-        <v>63.65187713310581</v>
+        <v>64.4431517031866</v>
       </c>
     </row>
     <row r="10">
@@ -3128,19 +3128,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3262</v>
+        <v>4279</v>
       </c>
       <c r="C10" t="n">
-        <v>1412</v>
+        <v>1972</v>
       </c>
       <c r="D10" t="n">
-        <v>43.28632740649908</v>
+        <v>46.0855340032718</v>
       </c>
       <c r="E10" t="n">
-        <v>2061</v>
+        <v>2703</v>
       </c>
       <c r="F10" t="n">
-        <v>63.18209687308399</v>
+        <v>63.16896471138116</v>
       </c>
     </row>
     <row r="11">
@@ -3150,19 +3150,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1142</v>
+        <v>1627</v>
       </c>
       <c r="C11" t="n">
-        <v>757</v>
+        <v>1138</v>
       </c>
       <c r="D11" t="n">
-        <v>66.28721541155866</v>
+        <v>69.94468346650277</v>
       </c>
       <c r="E11" t="n">
-        <v>848</v>
+        <v>1247</v>
       </c>
       <c r="F11" t="n">
-        <v>74.25569176882661</v>
+        <v>76.64413030116779</v>
       </c>
     </row>
     <row r="12">
@@ -3172,19 +3172,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>954</v>
+        <v>1413</v>
       </c>
       <c r="C12" t="n">
-        <v>194</v>
+        <v>302</v>
       </c>
       <c r="D12" t="n">
-        <v>20.33542976939203</v>
+        <v>21.37296532200991</v>
       </c>
       <c r="E12" t="n">
-        <v>513</v>
+        <v>777</v>
       </c>
       <c r="F12" t="n">
-        <v>53.77358490566038</v>
+        <v>54.98938428874735</v>
       </c>
     </row>
     <row r="13">
@@ -3194,19 +3194,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>28014</v>
+        <v>41977</v>
       </c>
       <c r="C13" t="n">
-        <v>21526</v>
+        <v>32716</v>
       </c>
       <c r="D13" t="n">
-        <v>76.84015135289498</v>
+        <v>77.93791838387688</v>
       </c>
       <c r="E13" t="n">
-        <v>22832</v>
+        <v>34417</v>
       </c>
       <c r="F13" t="n">
-        <v>81.50210608981223</v>
+        <v>81.99013745622604</v>
       </c>
     </row>
     <row r="14">
@@ -3216,19 +3216,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>78006</v>
+        <v>114113</v>
       </c>
       <c r="C14" t="n">
-        <v>45310</v>
+        <v>67663</v>
       </c>
       <c r="D14" t="n">
-        <v>58.08527549162885</v>
+        <v>59.29473416700989</v>
       </c>
       <c r="E14" t="n">
-        <v>61286</v>
+        <v>89024</v>
       </c>
       <c r="F14" t="n">
-        <v>78.56575135246007</v>
+        <v>78.01389850411434</v>
       </c>
     </row>
     <row r="15">
@@ -3238,19 +3238,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>14665</v>
+        <v>21432</v>
       </c>
       <c r="C15" t="n">
-        <v>4451</v>
+        <v>7653</v>
       </c>
       <c r="D15" t="n">
-        <v>30.35117627003068</v>
+        <v>35.70828667413214</v>
       </c>
       <c r="E15" t="n">
-        <v>9531</v>
+        <v>13937</v>
       </c>
       <c r="F15" t="n">
-        <v>64.99147630412547</v>
+        <v>65.02892870474058</v>
       </c>
     </row>
     <row r="16">
@@ -3260,19 +3260,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1666</v>
+        <v>2278</v>
       </c>
       <c r="C16" t="n">
-        <v>684</v>
+        <v>981</v>
       </c>
       <c r="D16" t="n">
-        <v>41.05642256902761</v>
+        <v>43.06409130816506</v>
       </c>
       <c r="E16" t="n">
-        <v>1139</v>
+        <v>1589</v>
       </c>
       <c r="F16" t="n">
-        <v>68.36734693877551</v>
+        <v>69.75417032484636</v>
       </c>
     </row>
     <row r="17">
@@ -3282,19 +3282,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5428</v>
+        <v>7846</v>
       </c>
       <c r="C17" t="n">
-        <v>3677</v>
+        <v>5390</v>
       </c>
       <c r="D17" t="n">
-        <v>67.74134119380987</v>
+        <v>68.69742543971449</v>
       </c>
       <c r="E17" t="n">
-        <v>4339</v>
+        <v>6212</v>
       </c>
       <c r="F17" t="n">
-        <v>79.93736182756079</v>
+        <v>79.17410145296967</v>
       </c>
     </row>
     <row r="18"/>
@@ -3395,43 +3395,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>695</v>
+        <v>1081</v>
       </c>
       <c r="D22" t="n">
-        <v>12.42040767386091</v>
+        <v>8.439855072463768</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>1.133333333333333</v>
       </c>
       <c r="F22" t="n">
-        <v>0.2070067945643485</v>
+        <v>0.1406642512077295</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>0.01888888888888889</v>
       </c>
       <c r="H22" t="n">
-        <v>288.4700733752621</v>
+        <v>247.1298784388996</v>
       </c>
       <c r="I22" t="n">
-        <v>136.1333333333333</v>
+        <v>95.2</v>
       </c>
       <c r="J22" t="n">
-        <v>4.807834556254367</v>
+        <v>4.118831307314992</v>
       </c>
       <c r="K22" t="n">
-        <v>2.268888888888889</v>
+        <v>1.586666666666667</v>
       </c>
       <c r="L22" t="n">
-        <v>263.1197589098533</v>
+        <v>230.7414267434421</v>
       </c>
       <c r="M22" t="n">
-        <v>104.6833333333333</v>
+        <v>74.31666666666666</v>
       </c>
       <c r="N22" t="n">
-        <v>4.385329315164221</v>
+        <v>3.845690445724035</v>
       </c>
       <c r="O22" t="n">
-        <v>1.744722222222222</v>
+        <v>1.238611111111111</v>
       </c>
     </row>
     <row r="23">
@@ -3446,43 +3446,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3519</v>
+        <v>4948</v>
       </c>
       <c r="D23" t="n">
-        <v>214.5087288055319</v>
+        <v>207.096948261924</v>
       </c>
       <c r="E23" t="n">
-        <v>65.75</v>
+        <v>62.76666666666667</v>
       </c>
       <c r="F23" t="n">
-        <v>3.575145480092198</v>
+        <v>3.4516158043654</v>
       </c>
       <c r="G23" t="n">
-        <v>1.095833333333333</v>
+        <v>1.046111111111111</v>
       </c>
       <c r="H23" t="n">
-        <v>226.3614373440798</v>
+        <v>220.2246247782781</v>
       </c>
       <c r="I23" t="n">
-        <v>80.95833333333334</v>
+        <v>78.84166666666667</v>
       </c>
       <c r="J23" t="n">
-        <v>3.77269062240133</v>
+        <v>3.670410412971301</v>
       </c>
       <c r="K23" t="n">
-        <v>1.349305555555556</v>
+        <v>1.314027777777778</v>
       </c>
       <c r="L23" t="n">
-        <v>11.28678276722318</v>
+        <v>12.35825487788239</v>
       </c>
       <c r="M23" t="n">
-        <v>5.416666666666667</v>
+        <v>5.916666666666667</v>
       </c>
       <c r="N23" t="n">
-        <v>0.1881130461203863</v>
+        <v>0.2059709146313731</v>
       </c>
       <c r="O23" t="n">
-        <v>0.09027777777777778</v>
+        <v>0.09861111111111112</v>
       </c>
     </row>
     <row r="24">
@@ -3497,7 +3497,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -3524,40 +3524,40 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>179</v>
+        <v>256</v>
       </c>
       <c r="D25" t="n">
-        <v>330.0571694599628</v>
+        <v>298.5602864583333</v>
       </c>
       <c r="E25" t="n">
-        <v>17.75</v>
+        <v>17.18333333333333</v>
       </c>
       <c r="F25" t="n">
-        <v>5.500952824332713</v>
+        <v>4.976004774305555</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2958333333333333</v>
+        <v>0.2863888888888889</v>
       </c>
       <c r="H25" t="n">
-        <v>338.8777153558053</v>
+        <v>307.1418635170604</v>
       </c>
       <c r="I25" t="n">
-        <v>26.225</v>
+        <v>22.56666666666667</v>
       </c>
       <c r="J25" t="n">
-        <v>5.647961922596754</v>
+        <v>5.119031058617673</v>
       </c>
       <c r="K25" t="n">
-        <v>0.4370833333333333</v>
+        <v>0.3761111111111111</v>
       </c>
       <c r="L25" t="n">
-        <v>29.82237827715356</v>
+        <v>22.45334645669292</v>
       </c>
       <c r="M25" t="n">
         <v>2.416666666666667</v>
       </c>
       <c r="N25" t="n">
-        <v>0.4970396379525593</v>
+        <v>0.3742224409448819</v>
       </c>
       <c r="O25" t="n">
         <v>0.04027777777777778</v>
@@ -3575,7 +3575,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -3602,43 +3602,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="D27" t="n">
-        <v>617.0925675675675</v>
+        <v>560.1910112359551</v>
       </c>
       <c r="E27" t="n">
-        <v>146.225</v>
+        <v>142.8333333333333</v>
       </c>
       <c r="F27" t="n">
-        <v>10.28487612612613</v>
+        <v>9.336516853932585</v>
       </c>
       <c r="G27" t="n">
-        <v>2.437083333333333</v>
+        <v>2.380555555555556</v>
       </c>
       <c r="H27" t="n">
-        <v>4337.126763990268</v>
+        <v>4010.026706827309</v>
       </c>
       <c r="I27" t="n">
-        <v>3253.15</v>
+        <v>2835.441666666667</v>
       </c>
       <c r="J27" t="n">
-        <v>72.28544606650446</v>
+        <v>66.83377844712183</v>
       </c>
       <c r="K27" t="n">
-        <v>54.21916666666667</v>
+        <v>47.25736111111111</v>
       </c>
       <c r="L27" t="n">
-        <v>3683.415936739659</v>
+        <v>3420.706526104418</v>
       </c>
       <c r="M27" t="n">
-        <v>3048.033333333333</v>
+        <v>2614.008333333333</v>
       </c>
       <c r="N27" t="n">
-        <v>61.39026561232765</v>
+        <v>57.01177543507362</v>
       </c>
       <c r="O27" t="n">
-        <v>50.80055555555555</v>
+        <v>43.56680555555556</v>
       </c>
     </row>
     <row r="28">
@@ -3653,43 +3653,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>443</v>
+        <v>661</v>
       </c>
       <c r="D28" t="n">
-        <v>187.3192249811889</v>
+        <v>169.2865607665154</v>
       </c>
       <c r="E28" t="n">
-        <v>20.8</v>
+        <v>20.45</v>
       </c>
       <c r="F28" t="n">
-        <v>3.121987083019814</v>
+        <v>2.821442679441923</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3466666666666667</v>
+        <v>0.3408333333333333</v>
       </c>
       <c r="H28" t="n">
-        <v>943.2666666666668</v>
+        <v>881.4934753211629</v>
       </c>
       <c r="I28" t="n">
-        <v>933.9166666666666</v>
+        <v>882.05</v>
       </c>
       <c r="J28" t="n">
-        <v>15.72111111111111</v>
+        <v>14.69155792201938</v>
       </c>
       <c r="K28" t="n">
-        <v>15.56527777777778</v>
+        <v>14.70083333333333</v>
       </c>
       <c r="L28" t="n">
-        <v>704.8952840300107</v>
+        <v>672.5099729546992</v>
       </c>
       <c r="M28" t="n">
-        <v>780.0166666666667</v>
+        <v>754.9666666666667</v>
       </c>
       <c r="N28" t="n">
-        <v>11.74825473383351</v>
+        <v>11.20849954924499</v>
       </c>
       <c r="O28" t="n">
-        <v>13.00027777777778</v>
+        <v>12.58277777777778</v>
       </c>
     </row>
     <row r="29">
@@ -3704,43 +3704,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>440</v>
+        <v>603</v>
       </c>
       <c r="D29" t="n">
-        <v>721.0587878787878</v>
+        <v>712.1982310668877</v>
       </c>
       <c r="E29" t="n">
-        <v>209.675</v>
+        <v>223.3333333333333</v>
       </c>
       <c r="F29" t="n">
-        <v>12.01764646464646</v>
+        <v>11.86997051778146</v>
       </c>
       <c r="G29" t="n">
-        <v>3.494583333333334</v>
+        <v>3.722222222222222</v>
       </c>
       <c r="H29" t="n">
-        <v>1588.609744779583</v>
+        <v>1511.047916666667</v>
       </c>
       <c r="I29" t="n">
-        <v>1201.183333333333</v>
+        <v>1134.358333333333</v>
       </c>
       <c r="J29" t="n">
-        <v>26.47682907965971</v>
+        <v>25.18413194444444</v>
       </c>
       <c r="K29" t="n">
-        <v>20.01972222222222</v>
+        <v>18.90597222222222</v>
       </c>
       <c r="L29" t="n">
-        <v>862.5654292343387</v>
+        <v>795.2763513513514</v>
       </c>
       <c r="M29" t="n">
-        <v>946.4666666666667</v>
+        <v>825.475</v>
       </c>
       <c r="N29" t="n">
-        <v>14.37609048723898</v>
+        <v>13.25460585585586</v>
       </c>
       <c r="O29" t="n">
-        <v>15.77444444444444</v>
+        <v>13.75791666666667</v>
       </c>
     </row>
     <row r="30">
@@ -3755,43 +3755,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6000</v>
+        <v>9388</v>
       </c>
       <c r="D30" t="n">
-        <v>23.09763333333333</v>
+        <v>15.85036216446528</v>
       </c>
       <c r="E30" t="n">
-        <v>20.71666666666667</v>
+        <v>20.25</v>
       </c>
       <c r="F30" t="n">
-        <v>0.3849605555555555</v>
+        <v>0.2641727027410879</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3452777777777777</v>
+        <v>0.3375</v>
       </c>
       <c r="H30" t="n">
-        <v>407.2903135911899</v>
+        <v>443.0361457129404</v>
       </c>
       <c r="I30" t="n">
-        <v>272.025</v>
+        <v>379.5</v>
       </c>
       <c r="J30" t="n">
-        <v>6.788171893186498</v>
+        <v>7.38393576188234</v>
       </c>
       <c r="K30" t="n">
-        <v>4.53375</v>
+        <v>6.325</v>
       </c>
       <c r="L30" t="n">
-        <v>379.9723576416868</v>
+        <v>424.3640404948418</v>
       </c>
       <c r="M30" t="n">
-        <v>240.8833333333333</v>
+        <v>366.5666666666667</v>
       </c>
       <c r="N30" t="n">
-        <v>6.332872627361447</v>
+        <v>7.072734008247363</v>
       </c>
       <c r="O30" t="n">
-        <v>4.014722222222223</v>
+        <v>6.109444444444445</v>
       </c>
     </row>
     <row r="31">
@@ -3806,43 +3806,43 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2112</v>
+        <v>3017</v>
       </c>
       <c r="D31" t="n">
-        <v>1885.034098800505</v>
+        <v>1912.681626339631</v>
       </c>
       <c r="E31" t="n">
-        <v>1421.458333333333</v>
+        <v>1480.5</v>
       </c>
       <c r="F31" t="n">
-        <v>31.41723498000841</v>
+        <v>31.87802710566051</v>
       </c>
       <c r="G31" t="n">
-        <v>23.69097222222222</v>
+        <v>24.675</v>
       </c>
       <c r="H31" t="n">
-        <v>2093.89307069706</v>
+        <v>2121.648593335639</v>
       </c>
       <c r="I31" t="n">
-        <v>1598.15</v>
+        <v>1660.916666666667</v>
       </c>
       <c r="J31" t="n">
-        <v>34.898217844951</v>
+        <v>35.36080988892732</v>
       </c>
       <c r="K31" t="n">
-        <v>26.63583333333334</v>
+        <v>27.68194444444445</v>
       </c>
       <c r="L31" t="n">
-        <v>205.5923026098447</v>
+        <v>207.3172258734002</v>
       </c>
       <c r="M31" t="n">
-        <v>226.2916666666667</v>
+        <v>234.8166666666667</v>
       </c>
       <c r="N31" t="n">
-        <v>3.426538376830746</v>
+        <v>3.455287097890004</v>
       </c>
       <c r="O31" t="n">
-        <v>3.771527777777778</v>
+        <v>3.913611111111111</v>
       </c>
     </row>
     <row r="32">
@@ -3857,43 +3857,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3615</v>
+        <v>6230</v>
       </c>
       <c r="D32" t="n">
-        <v>417.9553019824804</v>
+        <v>340.4267067950776</v>
       </c>
       <c r="E32" t="n">
-        <v>20.88333333333333</v>
+        <v>20.425</v>
       </c>
       <c r="F32" t="n">
-        <v>6.965921699708007</v>
+        <v>5.673778446584625</v>
       </c>
       <c r="G32" t="n">
-        <v>0.3480555555555556</v>
+        <v>0.3404166666666667</v>
       </c>
       <c r="H32" t="n">
-        <v>804.7200405604719</v>
+        <v>694.0605051985207</v>
       </c>
       <c r="I32" t="n">
-        <v>525.5666666666666</v>
+        <v>435.2166666666666</v>
       </c>
       <c r="J32" t="n">
-        <v>13.41200067600787</v>
+        <v>11.56767508664201</v>
       </c>
       <c r="K32" t="n">
-        <v>8.759444444444444</v>
+        <v>7.253611111111111</v>
       </c>
       <c r="L32" t="n">
-        <v>253.8350294985251</v>
+        <v>253.6920696392436</v>
       </c>
       <c r="M32" t="n">
-        <v>54.15833333333333</v>
+        <v>70.81666666666666</v>
       </c>
       <c r="N32" t="n">
-        <v>4.230583824975418</v>
+        <v>4.228201160654059</v>
       </c>
       <c r="O32" t="n">
-        <v>0.902638888888889</v>
+        <v>1.180277777777778</v>
       </c>
     </row>
     <row r="33">
@@ -3908,43 +3908,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6933</v>
+        <v>9241</v>
       </c>
       <c r="D33" t="n">
-        <v>412.6410620702919</v>
+        <v>401.3472585939472</v>
       </c>
       <c r="E33" t="n">
-        <v>54.56666666666667</v>
+        <v>62.76666666666667</v>
       </c>
       <c r="F33" t="n">
-        <v>6.877351034504864</v>
+        <v>6.689120976565787</v>
       </c>
       <c r="G33" t="n">
-        <v>0.9094444444444445</v>
+        <v>1.046111111111111</v>
       </c>
       <c r="H33" t="n">
-        <v>686.5703359375001</v>
+        <v>678.7645575771712</v>
       </c>
       <c r="I33" t="n">
-        <v>326.9</v>
+        <v>330.9</v>
       </c>
       <c r="J33" t="n">
-        <v>11.44283893229167</v>
+        <v>11.31274262628619</v>
       </c>
       <c r="K33" t="n">
-        <v>5.448333333333332</v>
+        <v>5.515000000000001</v>
       </c>
       <c r="L33" t="n">
-        <v>248.14771875</v>
+        <v>254.4889996889822</v>
       </c>
       <c r="M33" t="n">
-        <v>63.94166666666666</v>
+        <v>67.68333333333334</v>
       </c>
       <c r="N33" t="n">
-        <v>4.135795312499999</v>
+        <v>4.241483328149704</v>
       </c>
       <c r="O33" t="n">
-        <v>1.065694444444444</v>
+        <v>1.128055555555556</v>
       </c>
     </row>
     <row r="34">
@@ -3959,43 +3959,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1412</v>
+        <v>1972</v>
       </c>
       <c r="D34" t="n">
-        <v>1775.183781869688</v>
+        <v>1457.845884043272</v>
       </c>
       <c r="E34" t="n">
-        <v>1776.116666666667</v>
+        <v>1044.225</v>
       </c>
       <c r="F34" t="n">
-        <v>29.58639636449481</v>
+        <v>24.29743140072121</v>
       </c>
       <c r="G34" t="n">
-        <v>29.60194444444445</v>
+        <v>17.40375</v>
       </c>
       <c r="H34" t="n">
-        <v>2664.186404416839</v>
+        <v>2149.565047114252</v>
       </c>
       <c r="I34" t="n">
-        <v>2635.85</v>
+        <v>1648.433333333333</v>
       </c>
       <c r="J34" t="n">
-        <v>44.40310674028066</v>
+        <v>35.82608411857087</v>
       </c>
       <c r="K34" t="n">
-        <v>43.93083333333334</v>
+        <v>27.47388888888889</v>
       </c>
       <c r="L34" t="n">
-        <v>586.1867322291235</v>
+        <v>539.3833333333333</v>
       </c>
       <c r="M34" t="n">
-        <v>525.4166666666666</v>
+        <v>442.525</v>
       </c>
       <c r="N34" t="n">
-        <v>9.769778870485393</v>
+        <v>8.989722222222223</v>
       </c>
       <c r="O34" t="n">
-        <v>8.756944444444445</v>
+        <v>7.375416666666666</v>
       </c>
     </row>
     <row r="35">
@@ -4010,43 +4010,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1850</v>
+        <v>2307</v>
       </c>
       <c r="D35" t="n">
-        <v>2125.079423423424</v>
+        <v>1909.514658286375</v>
       </c>
       <c r="E35" t="n">
-        <v>2124.641666666666</v>
+        <v>1900.133333333333</v>
       </c>
       <c r="F35" t="n">
-        <v>35.41799039039039</v>
+        <v>31.82524430477292</v>
       </c>
       <c r="G35" t="n">
-        <v>35.41069444444445</v>
+        <v>31.66888888888889</v>
       </c>
       <c r="H35" t="n">
-        <v>2787.761152968037</v>
+        <v>2459.743304254668</v>
       </c>
       <c r="I35" t="n">
-        <v>2703.5</v>
+        <v>2366.15</v>
       </c>
       <c r="J35" t="n">
-        <v>46.46268588280061</v>
+        <v>40.9957217375778</v>
       </c>
       <c r="K35" t="n">
-        <v>45.05833333333334</v>
+        <v>39.43583333333333</v>
       </c>
       <c r="L35" t="n">
-        <v>556.6087785388128</v>
+        <v>536.72842822161</v>
       </c>
       <c r="M35" t="n">
-        <v>524.4333333333333</v>
+        <v>443.8916666666667</v>
       </c>
       <c r="N35" t="n">
-        <v>9.27681297564688</v>
+        <v>8.945473803693501</v>
       </c>
       <c r="O35" t="n">
-        <v>8.740555555555554</v>
+        <v>7.398194444444444</v>
       </c>
     </row>
     <row r="36">
@@ -4061,43 +4061,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>757</v>
+        <v>1138</v>
       </c>
       <c r="D36" t="n">
-        <v>22.18126376045795</v>
+        <v>17.06802870533099</v>
       </c>
       <c r="E36" t="n">
-        <v>20.65</v>
+        <v>20.35</v>
       </c>
       <c r="F36" t="n">
-        <v>0.3696877293409658</v>
+        <v>0.2844671450888498</v>
       </c>
       <c r="G36" t="n">
-        <v>0.3441666666666666</v>
+        <v>0.3391666666666667</v>
       </c>
       <c r="H36" t="n">
-        <v>2096.005545722714</v>
+        <v>2460.456875</v>
       </c>
       <c r="I36" t="n">
-        <v>1685.566666666667</v>
+        <v>1819.216666666667</v>
       </c>
       <c r="J36" t="n">
-        <v>34.93342576204523</v>
+        <v>41.00761458333332</v>
       </c>
       <c r="K36" t="n">
-        <v>28.09277777777778</v>
+        <v>30.32027777777778</v>
       </c>
       <c r="L36" t="n">
-        <v>2067.918348082596</v>
+        <v>2437.4168125</v>
       </c>
       <c r="M36" t="n">
-        <v>1638.2</v>
+        <v>1786.433333333333</v>
       </c>
       <c r="N36" t="n">
-        <v>34.46530580137659</v>
+        <v>40.62361354166666</v>
       </c>
       <c r="O36" t="n">
-        <v>27.30333333333333</v>
+        <v>29.77388888888889</v>
       </c>
     </row>
     <row r="37">
@@ -4112,43 +4112,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>385</v>
+        <v>489</v>
       </c>
       <c r="D37" t="n">
-        <v>2319.501558441559</v>
+        <v>2751.817246080436</v>
       </c>
       <c r="E37" t="n">
-        <v>2302.85</v>
+        <v>2518.9</v>
       </c>
       <c r="F37" t="n">
-        <v>38.65835930735931</v>
+        <v>45.86362076800727</v>
       </c>
       <c r="G37" t="n">
-        <v>38.38083333333334</v>
+        <v>41.98166666666667</v>
       </c>
       <c r="H37" t="n">
-        <v>2713.626754385965</v>
+        <v>3183.666215199398</v>
       </c>
       <c r="I37" t="n">
-        <v>2717.991666666667</v>
+        <v>2858.5</v>
       </c>
       <c r="J37" t="n">
-        <v>45.22711257309941</v>
+        <v>53.06110358665664</v>
       </c>
       <c r="K37" t="n">
-        <v>45.29986111111111</v>
+        <v>47.64166666666667</v>
       </c>
       <c r="L37" t="n">
-        <v>284.026461988304</v>
+        <v>286.4480060195636</v>
       </c>
       <c r="M37" t="n">
-        <v>232.3416666666667</v>
+        <v>289.4</v>
       </c>
       <c r="N37" t="n">
-        <v>4.733774366471735</v>
+        <v>4.774133433659394</v>
       </c>
       <c r="O37" t="n">
-        <v>3.872361111111111</v>
+        <v>4.823333333333333</v>
       </c>
     </row>
     <row r="38">
@@ -4163,7 +4163,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>194</v>
+        <v>302</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -4178,28 +4178,28 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>232.8547619047619</v>
+        <v>380.6364583333333</v>
       </c>
       <c r="I38" t="n">
-        <v>66.925</v>
+        <v>130.7833333333333</v>
       </c>
       <c r="J38" t="n">
-        <v>3.880912698412698</v>
+        <v>6.343940972222223</v>
       </c>
       <c r="K38" t="n">
-        <v>1.115416666666667</v>
+        <v>2.179722222222222</v>
       </c>
       <c r="L38" t="n">
-        <v>232.8547619047619</v>
+        <v>380.6364583333333</v>
       </c>
       <c r="M38" t="n">
-        <v>66.925</v>
+        <v>130.7833333333333</v>
       </c>
       <c r="N38" t="n">
-        <v>3.880912698412698</v>
+        <v>6.343940972222223</v>
       </c>
       <c r="O38" t="n">
-        <v>1.115416666666667</v>
+        <v>2.179722222222222</v>
       </c>
     </row>
     <row r="39">
@@ -4214,43 +4214,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>760</v>
+        <v>1111</v>
       </c>
       <c r="D39" t="n">
-        <v>236.2387938596491</v>
+        <v>218.8424542454246</v>
       </c>
       <c r="E39" t="n">
-        <v>93.05000000000001</v>
+        <v>89.98333333333333</v>
       </c>
       <c r="F39" t="n">
-        <v>3.937313230994152</v>
+        <v>3.647374237423743</v>
       </c>
       <c r="G39" t="n">
-        <v>1.550833333333333</v>
+        <v>1.499722222222222</v>
       </c>
       <c r="H39" t="n">
-        <v>535.3983533600357</v>
+        <v>544.346152676399</v>
       </c>
       <c r="I39" t="n">
-        <v>445.8666666666667</v>
+        <v>469.2416666666667</v>
       </c>
       <c r="J39" t="n">
-        <v>8.923305889333927</v>
+        <v>9.072435877939983</v>
       </c>
       <c r="K39" t="n">
-        <v>7.431111111111111</v>
+        <v>7.820694444444444</v>
       </c>
       <c r="L39" t="n">
-        <v>297.3450378282154</v>
+        <v>324.2905717761557</v>
       </c>
       <c r="M39" t="n">
-        <v>194.8166666666667</v>
+        <v>205.95</v>
       </c>
       <c r="N39" t="n">
-        <v>4.955750630470257</v>
+        <v>5.404842862935928</v>
       </c>
       <c r="O39" t="n">
-        <v>3.246944444444444</v>
+        <v>3.4325</v>
       </c>
     </row>
     <row r="40">
@@ -4265,40 +4265,40 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>21526</v>
+        <v>32716</v>
       </c>
       <c r="D40" t="n">
-        <v>169.9221158908607</v>
+        <v>125.122158882504</v>
       </c>
       <c r="E40" t="n">
-        <v>20.68333333333333</v>
+        <v>2.016666666666667</v>
       </c>
       <c r="F40" t="n">
-        <v>2.832035264847678</v>
+        <v>2.0853693147084</v>
       </c>
       <c r="G40" t="n">
-        <v>0.3447222222222222</v>
+        <v>0.03361111111111111</v>
       </c>
       <c r="H40" t="n">
-        <v>260.7236201449545</v>
+        <v>196.1111803203785</v>
       </c>
       <c r="I40" t="n">
-        <v>21.18333333333333</v>
+        <v>20.81666666666667</v>
       </c>
       <c r="J40" t="n">
-        <v>4.345393669082575</v>
+        <v>3.268519672006307</v>
       </c>
       <c r="K40" t="n">
-        <v>0.3530555555555556</v>
+        <v>0.3469444444444444</v>
       </c>
       <c r="L40" t="n">
-        <v>36.88921204237131</v>
+        <v>32.9230863301618</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.6148202007061884</v>
+        <v>0.5487181055026966</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -4316,43 +4316,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>6488</v>
+        <v>9261</v>
       </c>
       <c r="D41" t="n">
-        <v>798.2948520345253</v>
+        <v>798.685127596012</v>
       </c>
       <c r="E41" t="n">
-        <v>643.3583333333333</v>
+        <v>664.8166666666667</v>
       </c>
       <c r="F41" t="n">
-        <v>13.30491420057542</v>
+        <v>13.31141879326687</v>
       </c>
       <c r="G41" t="n">
-        <v>10.72263888888889</v>
+        <v>11.08027777777778</v>
       </c>
       <c r="H41" t="n">
-        <v>885.273290113452</v>
+        <v>895.375662270319</v>
       </c>
       <c r="I41" t="n">
-        <v>741.6166666666667</v>
+        <v>765.25</v>
       </c>
       <c r="J41" t="n">
-        <v>14.7545548352242</v>
+        <v>14.92292770450532</v>
       </c>
       <c r="K41" t="n">
-        <v>12.36027777777778</v>
+        <v>12.75416666666667</v>
       </c>
       <c r="L41" t="n">
-        <v>80.94260129659644</v>
+        <v>91.06264043888325</v>
       </c>
       <c r="M41" t="n">
-        <v>73.72499999999999</v>
+        <v>73.86666666666666</v>
       </c>
       <c r="N41" t="n">
-        <v>1.349043354943274</v>
+        <v>1.517710673981387</v>
       </c>
       <c r="O41" t="n">
-        <v>1.22875</v>
+        <v>1.231111111111111</v>
       </c>
     </row>
     <row r="42">
@@ -4367,43 +4367,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>45310</v>
+        <v>67663</v>
       </c>
       <c r="D42" t="n">
-        <v>25.02397594350033</v>
+        <v>17.49177196793915</v>
       </c>
       <c r="E42" t="n">
-        <v>20.76666666666667</v>
+        <v>20.41666666666667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.4170662657250055</v>
+        <v>0.2915295327989857</v>
       </c>
       <c r="G42" t="n">
-        <v>0.3461111111111111</v>
+        <v>0.3402777777777778</v>
       </c>
       <c r="H42" t="n">
-        <v>513.9659371931564</v>
+        <v>496.4281213396886</v>
       </c>
       <c r="I42" t="n">
-        <v>201.8</v>
+        <v>184.7833333333333</v>
       </c>
       <c r="J42" t="n">
-        <v>8.566098953219273</v>
+        <v>8.273802022328141</v>
       </c>
       <c r="K42" t="n">
-        <v>3.363333333333334</v>
+        <v>3.079722222222222</v>
       </c>
       <c r="L42" t="n">
-        <v>486.9684679752874</v>
+        <v>477.3967122429809</v>
       </c>
       <c r="M42" t="n">
-        <v>172.45</v>
+        <v>165.6833333333333</v>
       </c>
       <c r="N42" t="n">
-        <v>8.116141132921456</v>
+        <v>7.956611870716349</v>
       </c>
       <c r="O42" t="n">
-        <v>2.874166666666667</v>
+        <v>2.761388888888889</v>
       </c>
     </row>
     <row r="43">
@@ -4418,43 +4418,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>32696</v>
+        <v>46450</v>
       </c>
       <c r="D43" t="n">
-        <v>152.1490860247941</v>
+        <v>150.1527922497309</v>
       </c>
       <c r="E43" t="n">
-        <v>76.63333333333334</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="F43" t="n">
-        <v>2.535818100413234</v>
+        <v>2.502546537495515</v>
       </c>
       <c r="G43" t="n">
-        <v>1.277222222222222</v>
+        <v>1.3225</v>
       </c>
       <c r="H43" t="n">
-        <v>538.6446022542185</v>
+        <v>546.2368451085314</v>
       </c>
       <c r="I43" t="n">
-        <v>232.3666666666667</v>
+        <v>232.4833333333333</v>
       </c>
       <c r="J43" t="n">
-        <v>8.977410037570309</v>
+        <v>9.103947418475522</v>
       </c>
       <c r="K43" t="n">
-        <v>3.872777777777777</v>
+        <v>3.874722222222222</v>
       </c>
       <c r="L43" t="n">
-        <v>386.5592867070602</v>
+        <v>394.9053736622528</v>
       </c>
       <c r="M43" t="n">
-        <v>113.325</v>
+        <v>114.5333333333333</v>
       </c>
       <c r="N43" t="n">
-        <v>6.442654778451003</v>
+        <v>6.581756227704214</v>
       </c>
       <c r="O43" t="n">
-        <v>1.88875</v>
+        <v>1.908888888888889</v>
       </c>
     </row>
     <row r="44">
@@ -4469,43 +4469,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>4451</v>
+        <v>7653</v>
       </c>
       <c r="D44" t="n">
-        <v>20.47282633116154</v>
+        <v>13.17853565050743</v>
       </c>
       <c r="E44" t="n">
-        <v>20.61666666666667</v>
+        <v>1.95</v>
       </c>
       <c r="F44" t="n">
-        <v>0.3412137721860256</v>
+        <v>0.2196422608417904</v>
       </c>
       <c r="G44" t="n">
-        <v>0.3436111111111111</v>
+        <v>0.0325</v>
       </c>
       <c r="H44" t="n">
-        <v>925.2382991669007</v>
+        <v>820.3296343402226</v>
       </c>
       <c r="I44" t="n">
-        <v>831.4</v>
+        <v>799.7583333333333</v>
       </c>
       <c r="J44" t="n">
-        <v>15.42063831944835</v>
+        <v>13.67216057233704</v>
       </c>
       <c r="K44" t="n">
-        <v>13.85666666666667</v>
+        <v>13.32930555555556</v>
       </c>
       <c r="L44" t="n">
-        <v>900.288912290555</v>
+        <v>804.6955219925809</v>
       </c>
       <c r="M44" t="n">
-        <v>809.9666666666667</v>
+        <v>783.9333333333334</v>
       </c>
       <c r="N44" t="n">
-        <v>15.00481520484258</v>
+        <v>13.41159203320968</v>
       </c>
       <c r="O44" t="n">
-        <v>13.49944444444444</v>
+        <v>13.06555555555556</v>
       </c>
     </row>
     <row r="45">
@@ -4520,43 +4520,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>10214</v>
+        <v>13779</v>
       </c>
       <c r="D45" t="n">
-        <v>191.2924450101168</v>
+        <v>221.0427534654184</v>
       </c>
       <c r="E45" t="n">
-        <v>19.95</v>
+        <v>27.71666666666667</v>
       </c>
       <c r="F45" t="n">
-        <v>3.18820741683528</v>
+        <v>3.684045891090307</v>
       </c>
       <c r="G45" t="n">
-        <v>0.3325</v>
+        <v>0.4619444444444444</v>
       </c>
       <c r="H45" t="n">
-        <v>837.4699847483478</v>
+        <v>822.5919505577328</v>
       </c>
       <c r="I45" t="n">
-        <v>853.2</v>
+        <v>856.5083333333333</v>
       </c>
       <c r="J45" t="n">
-        <v>13.95783307913913</v>
+        <v>13.70986584262888</v>
       </c>
       <c r="K45" t="n">
-        <v>14.22</v>
+        <v>14.27513888888889</v>
       </c>
       <c r="L45" t="n">
-        <v>645.3405660057617</v>
+        <v>601.0616759622148</v>
       </c>
       <c r="M45" t="n">
-        <v>485.65</v>
+        <v>437.0083333333333</v>
       </c>
       <c r="N45" t="n">
-        <v>10.75567610009603</v>
+        <v>10.01769459937025</v>
       </c>
       <c r="O45" t="n">
-        <v>8.094166666666666</v>
+        <v>7.283472222222223</v>
       </c>
     </row>
     <row r="46">
@@ -4571,43 +4571,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>684</v>
+        <v>981</v>
       </c>
       <c r="D46" t="n">
-        <v>19.69739278752436</v>
+        <v>16.45504587155963</v>
       </c>
       <c r="E46" t="n">
-        <v>20.63333333333333</v>
+        <v>20.4</v>
       </c>
       <c r="F46" t="n">
-        <v>0.3282898797920728</v>
+        <v>0.2742507645259939</v>
       </c>
       <c r="G46" t="n">
-        <v>0.3438888888888889</v>
+        <v>0.34</v>
       </c>
       <c r="H46" t="n">
-        <v>3262.247438456421</v>
+        <v>3269.677423822715</v>
       </c>
       <c r="I46" t="n">
-        <v>2852.433333333333</v>
+        <v>2943.358333333334</v>
       </c>
       <c r="J46" t="n">
-        <v>54.37079064094033</v>
+        <v>54.49462373037858</v>
       </c>
       <c r="K46" t="n">
-        <v>47.54055555555556</v>
+        <v>49.05597222222222</v>
       </c>
       <c r="L46" t="n">
-        <v>3236.295908183633</v>
+        <v>3247.938481071099</v>
       </c>
       <c r="M46" t="n">
-        <v>2816.433333333333</v>
+        <v>2922.858333333333</v>
       </c>
       <c r="N46" t="n">
-        <v>53.93826513639387</v>
+        <v>54.13230801785164</v>
       </c>
       <c r="O46" t="n">
-        <v>46.94055555555556</v>
+        <v>48.71430555555555</v>
       </c>
     </row>
     <row r="47">
@@ -4622,43 +4622,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>982</v>
+        <v>1297</v>
       </c>
       <c r="D47" t="n">
-        <v>203.6907162253904</v>
+        <v>215.2599460292984</v>
       </c>
       <c r="E47" t="n">
-        <v>38.29166666666667</v>
+        <v>42.2</v>
       </c>
       <c r="F47" t="n">
-        <v>3.394845270423173</v>
+        <v>3.587665767154973</v>
       </c>
       <c r="G47" t="n">
-        <v>0.6381944444444445</v>
+        <v>0.7033333333333334</v>
       </c>
       <c r="H47" t="n">
-        <v>3136.334719260839</v>
+        <v>3262.960426796326</v>
       </c>
       <c r="I47" t="n">
-        <v>2892.125</v>
+        <v>2963.741666666667</v>
       </c>
       <c r="J47" t="n">
-        <v>52.27224532101398</v>
+        <v>54.38267377993878</v>
       </c>
       <c r="K47" t="n">
-        <v>48.20208333333333</v>
+        <v>49.39569444444444</v>
       </c>
       <c r="L47" t="n">
-        <v>2927.867537313433</v>
+        <v>3048.287722852512</v>
       </c>
       <c r="M47" t="n">
-        <v>2816.091666666667</v>
+        <v>2876.583333333333</v>
       </c>
       <c r="N47" t="n">
-        <v>48.79779228855722</v>
+        <v>50.80479538087521</v>
       </c>
       <c r="O47" t="n">
-        <v>46.93486111111111</v>
+        <v>47.94305555555555</v>
       </c>
     </row>
     <row r="48">
@@ -4673,43 +4673,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3677</v>
+        <v>5390</v>
       </c>
       <c r="D48" t="n">
-        <v>23.22049224911613</v>
+        <v>16.43401669758812</v>
       </c>
       <c r="E48" t="n">
-        <v>20.7</v>
+        <v>20.275</v>
       </c>
       <c r="F48" t="n">
-        <v>0.3870082041519355</v>
+        <v>0.2739002782931355</v>
       </c>
       <c r="G48" t="n">
-        <v>0.345</v>
+        <v>0.3379166666666667</v>
       </c>
       <c r="H48" t="n">
-        <v>459.0204166666667</v>
+        <v>418.4459716496709</v>
       </c>
       <c r="I48" t="n">
-        <v>397.7333333333333</v>
+        <v>353.15</v>
       </c>
       <c r="J48" t="n">
-        <v>7.650340277777778</v>
+        <v>6.974099527494515</v>
       </c>
       <c r="K48" t="n">
-        <v>6.628888888888889</v>
+        <v>5.885833333333333</v>
       </c>
       <c r="L48" t="n">
-        <v>431.2479550438596</v>
+        <v>399.4396940768062</v>
       </c>
       <c r="M48" t="n">
-        <v>359.6583333333333</v>
+        <v>327.8666666666667</v>
       </c>
       <c r="N48" t="n">
-        <v>7.187465917397661</v>
+        <v>6.657328234613438</v>
       </c>
       <c r="O48" t="n">
-        <v>5.994305555555556</v>
+        <v>5.464444444444444</v>
       </c>
     </row>
     <row r="49">
@@ -4724,43 +4724,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1751</v>
+        <v>2456</v>
       </c>
       <c r="D49" t="n">
-        <v>325.5730630116124</v>
+        <v>295.0677049402823</v>
       </c>
       <c r="E49" t="n">
-        <v>120.7666666666667</v>
+        <v>112.0916666666667</v>
       </c>
       <c r="F49" t="n">
-        <v>5.426217716860207</v>
+        <v>4.917795082338039</v>
       </c>
       <c r="G49" t="n">
-        <v>2.012777777777778</v>
+        <v>1.868194444444444</v>
       </c>
       <c r="H49" t="n">
-        <v>709.9369640787949</v>
+        <v>663.9142130584193</v>
       </c>
       <c r="I49" t="n">
-        <v>574.8916666666667</v>
+        <v>558.9833333333333</v>
       </c>
       <c r="J49" t="n">
-        <v>11.83228273464658</v>
+        <v>11.06523688430699</v>
       </c>
       <c r="K49" t="n">
-        <v>9.581527777777779</v>
+        <v>9.316388888888889</v>
       </c>
       <c r="L49" t="n">
-        <v>383.0971996910004</v>
+        <v>368.1101580756014</v>
       </c>
       <c r="M49" t="n">
-        <v>223.8083333333333</v>
+        <v>194.1333333333333</v>
       </c>
       <c r="N49" t="n">
-        <v>6.384953328183339</v>
+        <v>6.135169301260023</v>
       </c>
       <c r="O49" t="n">
-        <v>3.730138888888889</v>
+        <v>3.235555555555556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard mié 19/08/2026  9:45:39,77
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -680,19 +680,19 @@
         <v>65.29306173417623</v>
       </c>
       <c r="W2" t="n">
-        <v>6029</v>
+        <v>6604</v>
       </c>
       <c r="X2" t="n">
-        <v>17.93000497594958</v>
+        <v>19.41247728649304</v>
       </c>
       <c r="Y2" t="n">
-        <v>71.52098192071654</v>
+        <v>71.78982434887948</v>
       </c>
       <c r="Z2" t="n">
-        <v>4.545161457647851</v>
+        <v>6.027633768191311</v>
       </c>
       <c r="AA2" t="n">
-        <v>-52.9462264887224</v>
+        <v>-48.45859673768829</v>
       </c>
     </row>
     <row r="3">
@@ -765,19 +765,19 @@
         <v>77.58389261744966</v>
       </c>
       <c r="W3" t="n">
-        <v>284</v>
+        <v>307</v>
       </c>
       <c r="X3" t="n">
-        <v>9.859154929577464</v>
+        <v>11.07491856677524</v>
       </c>
       <c r="Y3" t="n">
-        <v>80.63380281690141</v>
+        <v>80.13029315960912</v>
       </c>
       <c r="Z3" t="n">
-        <v>-16.85225446639569</v>
+        <v>-15.63649082919791</v>
       </c>
       <c r="AA3" t="n">
-        <v>-61.87919463087248</v>
+        <v>-58.79194630872483</v>
       </c>
     </row>
     <row r="4">
@@ -850,19 +850,19 @@
         <v>34.85881207400195</v>
       </c>
       <c r="W4" t="n">
-        <v>226</v>
+        <v>249</v>
       </c>
       <c r="X4" t="n">
-        <v>21.23893805309735</v>
+        <v>19.67871485943775</v>
       </c>
       <c r="Y4" t="n">
-        <v>62.83185840707964</v>
+        <v>63.85542168674698</v>
       </c>
       <c r="Z4" t="n">
-        <v>21.04419608620348</v>
+        <v>19.48397289254389</v>
       </c>
       <c r="AA4" t="n">
-        <v>-77.99415774099319</v>
+        <v>-75.75462512171373</v>
       </c>
     </row>
     <row r="5">
@@ -935,19 +935,19 @@
         <v>52.69410267288927</v>
       </c>
       <c r="W5" t="n">
-        <v>1264</v>
+        <v>1346</v>
       </c>
       <c r="X5" t="n">
-        <v>52.29430379746836</v>
+        <v>53.04606240713225</v>
       </c>
       <c r="Y5" t="n">
-        <v>60.68037974683544</v>
+        <v>61.2184249628529</v>
       </c>
       <c r="Z5" t="n">
-        <v>13.72833010209288</v>
+        <v>14.48008871175677</v>
       </c>
       <c r="AA5" t="n">
-        <v>-46.37250742469241</v>
+        <v>-42.89350869749682</v>
       </c>
     </row>
     <row r="6">
@@ -1020,19 +1020,19 @@
         <v>64.41954378433441</v>
       </c>
       <c r="W6" t="n">
-        <v>12405</v>
+        <v>13198</v>
       </c>
       <c r="X6" t="n">
-        <v>75.67916162837565</v>
+        <v>75.80694044552206</v>
       </c>
       <c r="Y6" t="n">
-        <v>79.77428456267634</v>
+        <v>79.83785422033641</v>
       </c>
       <c r="Z6" t="n">
-        <v>15.84724108411837</v>
+        <v>15.97501990126477</v>
       </c>
       <c r="AA6" t="n">
-        <v>-54.8695747080438</v>
+        <v>-51.98457452613962</v>
       </c>
     </row>
     <row r="7">
@@ -1105,19 +1105,19 @@
         <v>61.85549639414975</v>
       </c>
       <c r="W7" t="n">
-        <v>15471</v>
+        <v>16611</v>
       </c>
       <c r="X7" t="n">
-        <v>40.26889018163015</v>
+        <v>41.13539220998133</v>
       </c>
       <c r="Y7" t="n">
-        <v>64.4431517031866</v>
+        <v>64.46330744687255</v>
       </c>
       <c r="Z7" t="n">
-        <v>4.436174673104169</v>
+        <v>5.302676701455354</v>
       </c>
       <c r="AA7" t="n">
-        <v>-47.86344948439712</v>
+        <v>-44.02170250050549</v>
       </c>
     </row>
     <row r="8">
@@ -1190,19 +1190,19 @@
         <v>53.9494851994852</v>
       </c>
       <c r="W8" t="n">
-        <v>4279</v>
+        <v>4601</v>
       </c>
       <c r="X8" t="n">
-        <v>46.0855340032718</v>
+        <v>46.27254944577266</v>
       </c>
       <c r="Y8" t="n">
-        <v>63.16896471138116</v>
+        <v>62.96457291893067</v>
       </c>
       <c r="Z8" t="n">
-        <v>9.502522420260213</v>
+        <v>9.689537862761078</v>
       </c>
       <c r="AA8" t="n">
-        <v>-65.58075933075934</v>
+        <v>-62.99066924066924</v>
       </c>
     </row>
     <row r="9">
@@ -1275,19 +1275,19 @@
         <v>68.22074215033301</v>
       </c>
       <c r="W9" t="n">
-        <v>1627</v>
+        <v>1812</v>
       </c>
       <c r="X9" t="n">
-        <v>69.94468346650277</v>
+        <v>69.81236203090508</v>
       </c>
       <c r="Y9" t="n">
-        <v>76.64413030116779</v>
+        <v>76.32450331125827</v>
       </c>
       <c r="Z9" t="n">
-        <v>9.859050735770126</v>
+        <v>9.726729300172437</v>
       </c>
       <c r="AA9" t="n">
-        <v>-61.29876308277831</v>
+        <v>-56.89819219790676</v>
       </c>
     </row>
     <row r="10">
@@ -1360,19 +1360,19 @@
         <v>36.93293885601578</v>
       </c>
       <c r="W10" t="n">
-        <v>1413</v>
+        <v>1529</v>
       </c>
       <c r="X10" t="n">
-        <v>21.37296532200991</v>
+        <v>22.04054937867888</v>
       </c>
       <c r="Y10" t="n">
-        <v>54.98938428874735</v>
+        <v>55.2648790058862</v>
       </c>
       <c r="Z10" t="n">
-        <v>18.61162409913022</v>
+        <v>19.27920815579919</v>
       </c>
       <c r="AA10" t="n">
-        <v>-30.32544378698225</v>
+        <v>-24.60552268244576</v>
       </c>
     </row>
     <row r="11">
@@ -1445,19 +1445,19 @@
         <v>73.6447415973979</v>
       </c>
       <c r="W11" t="n">
-        <v>41977</v>
+        <v>44703</v>
       </c>
       <c r="X11" t="n">
-        <v>77.93791838387688</v>
+        <v>78.02608326063127</v>
       </c>
       <c r="Y11" t="n">
-        <v>81.99013745622604</v>
+        <v>82.01239290427935</v>
       </c>
       <c r="Z11" t="n">
-        <v>10.26421943194337</v>
+        <v>10.35238430869776</v>
       </c>
       <c r="AA11" t="n">
-        <v>-52.59193169497651</v>
+        <v>-49.51323635706542</v>
       </c>
     </row>
     <row r="12">
@@ -1530,19 +1530,19 @@
         <v>74.93570456560008</v>
       </c>
       <c r="W12" t="n">
-        <v>114113</v>
+        <v>122745</v>
       </c>
       <c r="X12" t="n">
-        <v>59.29473416700989</v>
+        <v>59.44437655301642</v>
       </c>
       <c r="Y12" t="n">
-        <v>78.01389850411434</v>
+        <v>78.07568536396595</v>
       </c>
       <c r="Z12" t="n">
-        <v>2.305258642970884</v>
+        <v>2.454901028977417</v>
       </c>
       <c r="AA12" t="n">
-        <v>-64.38376259379018</v>
+        <v>-61.68959662417758</v>
       </c>
     </row>
     <row r="13">
@@ -1615,19 +1615,19 @@
         <v>60.82532992468735</v>
       </c>
       <c r="W13" t="n">
-        <v>21432</v>
+        <v>22527</v>
       </c>
       <c r="X13" t="n">
-        <v>35.70828667413214</v>
+        <v>37.32853908642962</v>
       </c>
       <c r="Y13" t="n">
-        <v>65.02892870474058</v>
+        <v>65.71225640342699</v>
       </c>
       <c r="Z13" t="n">
-        <v>8.093072136717645</v>
+        <v>9.713324549015127</v>
       </c>
       <c r="AA13" t="n">
-        <v>-62.97934084156706</v>
+        <v>-61.08788779105922</v>
       </c>
     </row>
     <row r="14">
@@ -1700,19 +1700,19 @@
         <v>60.31513970110461</v>
       </c>
       <c r="W14" t="n">
-        <v>2278</v>
+        <v>2750</v>
       </c>
       <c r="X14" t="n">
-        <v>43.06409130816506</v>
+        <v>45.12727272727273</v>
       </c>
       <c r="Y14" t="n">
-        <v>69.75417032484636</v>
+        <v>69.78181818181818</v>
       </c>
       <c r="Z14" t="n">
-        <v>9.389627370543224</v>
+        <v>11.45280878965089</v>
       </c>
       <c r="AA14" t="n">
-        <v>-62.99545159194282</v>
+        <v>-55.32813515269655</v>
       </c>
     </row>
     <row r="15">
@@ -1785,19 +1785,19 @@
         <v>74.15969011620642</v>
       </c>
       <c r="W15" t="n">
-        <v>7846</v>
+        <v>8322</v>
       </c>
       <c r="X15" t="n">
-        <v>68.69742543971449</v>
+        <v>69.13001682287911</v>
       </c>
       <c r="Y15" t="n">
-        <v>79.17410145296967</v>
+        <v>79.36794039894257</v>
       </c>
       <c r="Z15" t="n">
-        <v>9.500874146449476</v>
+        <v>9.933465529614097</v>
       </c>
       <c r="AA15" t="n">
-        <v>-50.98088216918656</v>
+        <v>-48.00699737598401</v>
       </c>
     </row>
   </sheetData>
@@ -1876,19 +1876,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4637</v>
+        <v>4990</v>
       </c>
       <c r="C4" t="n">
-        <v>717</v>
+        <v>776</v>
       </c>
       <c r="D4" t="n">
-        <v>15.4625835669614</v>
+        <v>15.55110220440882</v>
       </c>
       <c r="E4" t="n">
-        <v>640.6675034867503</v>
+        <v>619.7540463917526</v>
       </c>
       <c r="F4" t="n">
-        <v>1210.727375</v>
+        <v>1200.715939724727</v>
       </c>
     </row>
     <row r="5">
@@ -1898,19 +1898,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>163034</v>
+        <v>175083</v>
       </c>
       <c r="C5" t="n">
-        <v>123063</v>
+        <v>132816</v>
       </c>
       <c r="D5" t="n">
-        <v>75.48302808003238</v>
+        <v>75.858878360549</v>
       </c>
       <c r="E5" t="n">
-        <v>4370.045520959995</v>
+        <v>4358.244660281141</v>
       </c>
       <c r="F5" t="n">
-        <v>6531.543080608441</v>
+        <v>6468.804301819387</v>
       </c>
     </row>
     <row r="6">
@@ -1920,19 +1920,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50827</v>
+        <v>54268</v>
       </c>
       <c r="C6" t="n">
-        <v>6600</v>
+        <v>7093</v>
       </c>
       <c r="D6" t="n">
-        <v>12.98522438861235</v>
+        <v>13.07031768261222</v>
       </c>
       <c r="E6" t="n">
-        <v>9818.861668181818</v>
+        <v>9728.788553503453</v>
       </c>
       <c r="F6" t="n">
-        <v>4235.714070361995</v>
+        <v>4242.262514656069</v>
       </c>
     </row>
     <row r="7">
@@ -1942,19 +1942,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12146</v>
+        <v>12963</v>
       </c>
       <c r="C7" t="n">
-        <v>4871</v>
+        <v>5211</v>
       </c>
       <c r="D7" t="n">
-        <v>40.10373785608431</v>
+        <v>40.19902800277714</v>
       </c>
       <c r="E7" t="n">
-        <v>886.6248624512421</v>
+        <v>920.8495384763002</v>
       </c>
       <c r="F7" t="n">
-        <v>3569.86883024055</v>
+        <v>3515.792954076368</v>
       </c>
     </row>
     <row r="8"/>
@@ -2996,19 +2996,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6029</v>
+        <v>6604</v>
       </c>
       <c r="C4" t="n">
-        <v>1081</v>
+        <v>1282</v>
       </c>
       <c r="D4" t="n">
-        <v>17.93000497594958</v>
+        <v>19.41247728649304</v>
       </c>
       <c r="E4" t="n">
-        <v>4312</v>
+        <v>4741</v>
       </c>
       <c r="F4" t="n">
-        <v>71.52098192071654</v>
+        <v>71.78982434887948</v>
       </c>
     </row>
     <row r="5">
@@ -3018,19 +3018,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>284</v>
+        <v>307</v>
       </c>
       <c r="C5" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D5" t="n">
-        <v>9.859154929577464</v>
+        <v>11.07491856677524</v>
       </c>
       <c r="E5" t="n">
-        <v>229</v>
+        <v>246</v>
       </c>
       <c r="F5" t="n">
-        <v>80.63380281690141</v>
+        <v>80.13029315960912</v>
       </c>
     </row>
     <row r="6">
@@ -3040,19 +3040,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>226</v>
+        <v>249</v>
       </c>
       <c r="C6" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6" t="n">
-        <v>21.23893805309735</v>
+        <v>19.67871485943775</v>
       </c>
       <c r="E6" t="n">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="F6" t="n">
-        <v>62.83185840707964</v>
+        <v>63.85542168674698</v>
       </c>
     </row>
     <row r="7">
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1264</v>
+        <v>1346</v>
       </c>
       <c r="C7" t="n">
-        <v>661</v>
+        <v>714</v>
       </c>
       <c r="D7" t="n">
-        <v>52.29430379746836</v>
+        <v>53.04606240713225</v>
       </c>
       <c r="E7" t="n">
-        <v>767</v>
+        <v>824</v>
       </c>
       <c r="F7" t="n">
-        <v>60.68037974683544</v>
+        <v>61.2184249628529</v>
       </c>
     </row>
     <row r="8">
@@ -3084,19 +3084,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12405</v>
+        <v>13198</v>
       </c>
       <c r="C8" t="n">
-        <v>9388</v>
+        <v>10005</v>
       </c>
       <c r="D8" t="n">
-        <v>75.67916162837565</v>
+        <v>75.80694044552206</v>
       </c>
       <c r="E8" t="n">
-        <v>9896</v>
+        <v>10537</v>
       </c>
       <c r="F8" t="n">
-        <v>79.77428456267634</v>
+        <v>79.83785422033641</v>
       </c>
     </row>
     <row r="9">
@@ -3106,19 +3106,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15471</v>
+        <v>16611</v>
       </c>
       <c r="C9" t="n">
-        <v>6230</v>
+        <v>6833</v>
       </c>
       <c r="D9" t="n">
-        <v>40.26889018163015</v>
+        <v>41.13539220998133</v>
       </c>
       <c r="E9" t="n">
-        <v>9970</v>
+        <v>10708</v>
       </c>
       <c r="F9" t="n">
-        <v>64.4431517031866</v>
+        <v>64.46330744687255</v>
       </c>
     </row>
     <row r="10">
@@ -3128,19 +3128,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4279</v>
+        <v>4601</v>
       </c>
       <c r="C10" t="n">
-        <v>1972</v>
+        <v>2129</v>
       </c>
       <c r="D10" t="n">
-        <v>46.0855340032718</v>
+        <v>46.27254944577266</v>
       </c>
       <c r="E10" t="n">
-        <v>2703</v>
+        <v>2897</v>
       </c>
       <c r="F10" t="n">
-        <v>63.16896471138116</v>
+        <v>62.96457291893067</v>
       </c>
     </row>
     <row r="11">
@@ -3150,19 +3150,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1627</v>
+        <v>1812</v>
       </c>
       <c r="C11" t="n">
-        <v>1138</v>
+        <v>1265</v>
       </c>
       <c r="D11" t="n">
-        <v>69.94468346650277</v>
+        <v>69.81236203090508</v>
       </c>
       <c r="E11" t="n">
-        <v>1247</v>
+        <v>1383</v>
       </c>
       <c r="F11" t="n">
-        <v>76.64413030116779</v>
+        <v>76.32450331125827</v>
       </c>
     </row>
     <row r="12">
@@ -3172,19 +3172,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1413</v>
+        <v>1529</v>
       </c>
       <c r="C12" t="n">
-        <v>302</v>
+        <v>337</v>
       </c>
       <c r="D12" t="n">
-        <v>21.37296532200991</v>
+        <v>22.04054937867888</v>
       </c>
       <c r="E12" t="n">
-        <v>777</v>
+        <v>845</v>
       </c>
       <c r="F12" t="n">
-        <v>54.98938428874735</v>
+        <v>55.2648790058862</v>
       </c>
     </row>
     <row r="13">
@@ -3194,19 +3194,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>41977</v>
+        <v>44703</v>
       </c>
       <c r="C13" t="n">
-        <v>32716</v>
+        <v>34880</v>
       </c>
       <c r="D13" t="n">
-        <v>77.93791838387688</v>
+        <v>78.02608326063127</v>
       </c>
       <c r="E13" t="n">
-        <v>34417</v>
+        <v>36662</v>
       </c>
       <c r="F13" t="n">
-        <v>81.99013745622604</v>
+        <v>82.01239290427935</v>
       </c>
     </row>
     <row r="14">
@@ -3216,19 +3216,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>114113</v>
+        <v>122745</v>
       </c>
       <c r="C14" t="n">
-        <v>67663</v>
+        <v>72965</v>
       </c>
       <c r="D14" t="n">
-        <v>59.29473416700989</v>
+        <v>59.44437655301642</v>
       </c>
       <c r="E14" t="n">
-        <v>89024</v>
+        <v>95834</v>
       </c>
       <c r="F14" t="n">
-        <v>78.01389850411434</v>
+        <v>78.07568536396595</v>
       </c>
     </row>
     <row r="15">
@@ -3238,19 +3238,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>21432</v>
+        <v>22527</v>
       </c>
       <c r="C15" t="n">
-        <v>7653</v>
+        <v>8409</v>
       </c>
       <c r="D15" t="n">
-        <v>35.70828667413214</v>
+        <v>37.32853908642962</v>
       </c>
       <c r="E15" t="n">
-        <v>13937</v>
+        <v>14803</v>
       </c>
       <c r="F15" t="n">
-        <v>65.02892870474058</v>
+        <v>65.71225640342699</v>
       </c>
     </row>
     <row r="16">
@@ -3260,19 +3260,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2278</v>
+        <v>2750</v>
       </c>
       <c r="C16" t="n">
-        <v>981</v>
+        <v>1241</v>
       </c>
       <c r="D16" t="n">
-        <v>43.06409130816506</v>
+        <v>45.12727272727273</v>
       </c>
       <c r="E16" t="n">
-        <v>1589</v>
+        <v>1919</v>
       </c>
       <c r="F16" t="n">
-        <v>69.75417032484636</v>
+        <v>69.78181818181818</v>
       </c>
     </row>
     <row r="17">
@@ -3282,19 +3282,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7846</v>
+        <v>8322</v>
       </c>
       <c r="C17" t="n">
-        <v>5390</v>
+        <v>5753</v>
       </c>
       <c r="D17" t="n">
-        <v>68.69742543971449</v>
+        <v>69.13001682287911</v>
       </c>
       <c r="E17" t="n">
-        <v>6212</v>
+        <v>6605</v>
       </c>
       <c r="F17" t="n">
-        <v>79.17410145296967</v>
+        <v>79.36794039894257</v>
       </c>
     </row>
     <row r="18"/>
@@ -3395,43 +3395,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1081</v>
+        <v>1282</v>
       </c>
       <c r="D22" t="n">
-        <v>8.439855072463768</v>
+        <v>7.261245449817992</v>
       </c>
       <c r="E22" t="n">
-        <v>1.133333333333333</v>
+        <v>1.166666666666667</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1406642512077295</v>
+        <v>0.1210207574969665</v>
       </c>
       <c r="G22" t="n">
-        <v>0.01888888888888889</v>
+        <v>0.01944444444444444</v>
       </c>
       <c r="H22" t="n">
-        <v>247.1298784388996</v>
+        <v>229.8576046634871</v>
       </c>
       <c r="I22" t="n">
-        <v>95.2</v>
+        <v>85.51666666666667</v>
       </c>
       <c r="J22" t="n">
-        <v>4.118831307314992</v>
+        <v>3.830960077724784</v>
       </c>
       <c r="K22" t="n">
-        <v>1.586666666666667</v>
+        <v>1.425277777777778</v>
       </c>
       <c r="L22" t="n">
-        <v>230.7414267434421</v>
+        <v>216.0112082670906</v>
       </c>
       <c r="M22" t="n">
-        <v>74.31666666666666</v>
+        <v>65.16666666666667</v>
       </c>
       <c r="N22" t="n">
-        <v>3.845690445724035</v>
+        <v>3.60018680445151</v>
       </c>
       <c r="O22" t="n">
-        <v>1.238611111111111</v>
+        <v>1.086111111111111</v>
       </c>
     </row>
     <row r="23">
@@ -3446,43 +3446,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>4948</v>
+        <v>5322</v>
       </c>
       <c r="D23" t="n">
-        <v>207.096948261924</v>
+        <v>212.851769384943</v>
       </c>
       <c r="E23" t="n">
-        <v>62.76666666666667</v>
+        <v>64.47499999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>3.4516158043654</v>
+        <v>3.54752948974905</v>
       </c>
       <c r="G23" t="n">
-        <v>1.046111111111111</v>
+        <v>1.074583333333333</v>
       </c>
       <c r="H23" t="n">
-        <v>220.2246247782781</v>
+        <v>226.9829493526276</v>
       </c>
       <c r="I23" t="n">
-        <v>78.84166666666667</v>
+        <v>81.13333333333333</v>
       </c>
       <c r="J23" t="n">
-        <v>3.670410412971301</v>
+        <v>3.783049155877126</v>
       </c>
       <c r="K23" t="n">
-        <v>1.314027777777778</v>
+        <v>1.352222222222222</v>
       </c>
       <c r="L23" t="n">
-        <v>12.35825487788239</v>
+        <v>13.4155972328002</v>
       </c>
       <c r="M23" t="n">
-        <v>5.916666666666667</v>
+        <v>6.333333333333333</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2059709146313731</v>
+        <v>0.2235932872133367</v>
       </c>
       <c r="O23" t="n">
-        <v>0.09861111111111112</v>
+        <v>0.1055555555555556</v>
       </c>
     </row>
     <row r="24">
@@ -3497,16 +3497,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>0.05784313725490196</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>0.0009640522875816992</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -3524,43 +3524,43 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>256</v>
+        <v>273</v>
       </c>
       <c r="D25" t="n">
-        <v>298.5602864583333</v>
+        <v>288.3046398046398</v>
       </c>
       <c r="E25" t="n">
-        <v>17.18333333333333</v>
+        <v>17.65</v>
       </c>
       <c r="F25" t="n">
-        <v>4.976004774305555</v>
+        <v>4.80507733007733</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2863888888888889</v>
+        <v>0.2941666666666666</v>
       </c>
       <c r="H25" t="n">
-        <v>307.1418635170604</v>
+        <v>296.4760493827161</v>
       </c>
       <c r="I25" t="n">
-        <v>22.56666666666667</v>
+        <v>23.40833333333333</v>
       </c>
       <c r="J25" t="n">
-        <v>5.119031058617673</v>
+        <v>4.941267489711935</v>
       </c>
       <c r="K25" t="n">
-        <v>0.3761111111111111</v>
+        <v>0.3901388888888889</v>
       </c>
       <c r="L25" t="n">
-        <v>22.45334645669292</v>
+        <v>21.64302469135802</v>
       </c>
       <c r="M25" t="n">
-        <v>2.416666666666667</v>
+        <v>2.383333333333333</v>
       </c>
       <c r="N25" t="n">
-        <v>0.3742224409448819</v>
+        <v>0.3607170781893004</v>
       </c>
       <c r="O25" t="n">
-        <v>0.04027777777777778</v>
+        <v>0.03972222222222222</v>
       </c>
     </row>
     <row r="26">
@@ -3575,7 +3575,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -3602,43 +3602,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>178</v>
+        <v>200</v>
       </c>
       <c r="D27" t="n">
-        <v>560.1910112359551</v>
+        <v>1009.216333333333</v>
       </c>
       <c r="E27" t="n">
-        <v>142.8333333333333</v>
+        <v>134.1416666666667</v>
       </c>
       <c r="F27" t="n">
-        <v>9.336516853932585</v>
+        <v>16.82027222222222</v>
       </c>
       <c r="G27" t="n">
-        <v>2.380555555555556</v>
+        <v>2.235694444444444</v>
       </c>
       <c r="H27" t="n">
-        <v>4010.026706827309</v>
+        <v>4845.113992869875</v>
       </c>
       <c r="I27" t="n">
-        <v>2835.441666666667</v>
+        <v>3120.266666666667</v>
       </c>
       <c r="J27" t="n">
-        <v>66.83377844712183</v>
+        <v>80.75189988116459</v>
       </c>
       <c r="K27" t="n">
-        <v>47.25736111111111</v>
+        <v>52.00444444444445</v>
       </c>
       <c r="L27" t="n">
-        <v>3420.706526104418</v>
+        <v>3775.846613190731</v>
       </c>
       <c r="M27" t="n">
-        <v>2614.008333333333</v>
+        <v>2715.933333333333</v>
       </c>
       <c r="N27" t="n">
-        <v>57.01177543507362</v>
+        <v>62.93077688651218</v>
       </c>
       <c r="O27" t="n">
-        <v>43.56680555555556</v>
+        <v>45.26555555555556</v>
       </c>
     </row>
     <row r="28">
@@ -3653,43 +3653,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>661</v>
+        <v>714</v>
       </c>
       <c r="D28" t="n">
-        <v>169.2865607665154</v>
+        <v>185.5408029878618</v>
       </c>
       <c r="E28" t="n">
-        <v>20.45</v>
+        <v>20.44166666666667</v>
       </c>
       <c r="F28" t="n">
-        <v>2.821442679441923</v>
+        <v>3.092346716464363</v>
       </c>
       <c r="G28" t="n">
-        <v>0.3408333333333333</v>
+        <v>0.3406944444444444</v>
       </c>
       <c r="H28" t="n">
-        <v>881.4934753211629</v>
+        <v>875.1335518102371</v>
       </c>
       <c r="I28" t="n">
-        <v>882.05</v>
+        <v>886.2249999999999</v>
       </c>
       <c r="J28" t="n">
-        <v>14.69155792201938</v>
+        <v>14.58555919683729</v>
       </c>
       <c r="K28" t="n">
-        <v>14.70083333333333</v>
+        <v>14.77041666666667</v>
       </c>
       <c r="L28" t="n">
-        <v>672.5099729546992</v>
+        <v>647.0578027465668</v>
       </c>
       <c r="M28" t="n">
-        <v>754.9666666666667</v>
+        <v>725.4416666666666</v>
       </c>
       <c r="N28" t="n">
-        <v>11.20849954924499</v>
+        <v>10.78429671244278</v>
       </c>
       <c r="O28" t="n">
-        <v>12.58277777777778</v>
+        <v>12.09069444444444</v>
       </c>
     </row>
     <row r="29">
@@ -3704,43 +3704,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>603</v>
+        <v>632</v>
       </c>
       <c r="D29" t="n">
-        <v>712.1982310668877</v>
+        <v>708.7461497890295</v>
       </c>
       <c r="E29" t="n">
-        <v>223.3333333333333</v>
+        <v>224.3833333333333</v>
       </c>
       <c r="F29" t="n">
-        <v>11.86997051778146</v>
+        <v>11.81243582981716</v>
       </c>
       <c r="G29" t="n">
-        <v>3.722222222222222</v>
+        <v>3.739722222222222</v>
       </c>
       <c r="H29" t="n">
-        <v>1511.047916666667</v>
+        <v>1501.085416666667</v>
       </c>
       <c r="I29" t="n">
-        <v>1134.358333333333</v>
+        <v>1144.508333333333</v>
       </c>
       <c r="J29" t="n">
-        <v>25.18413194444444</v>
+        <v>25.01809027777778</v>
       </c>
       <c r="K29" t="n">
-        <v>18.90597222222222</v>
+        <v>19.07513888888889</v>
       </c>
       <c r="L29" t="n">
-        <v>795.2763513513514</v>
+        <v>793.7133387445887</v>
       </c>
       <c r="M29" t="n">
-        <v>825.475</v>
+        <v>831.5833333333334</v>
       </c>
       <c r="N29" t="n">
-        <v>13.25460585585586</v>
+        <v>13.22855564574315</v>
       </c>
       <c r="O29" t="n">
-        <v>13.75791666666667</v>
+        <v>13.85972222222222</v>
       </c>
     </row>
     <row r="30">
@@ -3755,43 +3755,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>9388</v>
+        <v>10005</v>
       </c>
       <c r="D30" t="n">
-        <v>15.85036216446528</v>
+        <v>14.9563901382642</v>
       </c>
       <c r="E30" t="n">
-        <v>20.25</v>
+        <v>20.1</v>
       </c>
       <c r="F30" t="n">
-        <v>0.2641727027410879</v>
+        <v>0.24927316897107</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3375</v>
+        <v>0.335</v>
       </c>
       <c r="H30" t="n">
-        <v>443.0361457129404</v>
+        <v>436.943277176093</v>
       </c>
       <c r="I30" t="n">
-        <v>379.5</v>
+        <v>371.525</v>
       </c>
       <c r="J30" t="n">
-        <v>7.38393576188234</v>
+        <v>7.282387952934885</v>
       </c>
       <c r="K30" t="n">
-        <v>6.325</v>
+        <v>6.192083333333334</v>
       </c>
       <c r="L30" t="n">
-        <v>424.3640404948418</v>
+        <v>419.3479823505816</v>
       </c>
       <c r="M30" t="n">
-        <v>366.5666666666667</v>
+        <v>360.9666666666667</v>
       </c>
       <c r="N30" t="n">
-        <v>7.072734008247363</v>
+        <v>6.989133039176362</v>
       </c>
       <c r="O30" t="n">
-        <v>6.109444444444445</v>
+        <v>6.016111111111111</v>
       </c>
     </row>
     <row r="31">
@@ -3806,40 +3806,40 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3017</v>
+        <v>3193</v>
       </c>
       <c r="D31" t="n">
-        <v>1912.681626339631</v>
+        <v>1886.441048126109</v>
       </c>
       <c r="E31" t="n">
-        <v>1480.5</v>
+        <v>1466.233333333333</v>
       </c>
       <c r="F31" t="n">
-        <v>31.87802710566051</v>
+        <v>31.44068413543515</v>
       </c>
       <c r="G31" t="n">
-        <v>24.675</v>
+        <v>24.43722222222222</v>
       </c>
       <c r="H31" t="n">
-        <v>2121.648593335639</v>
+        <v>2090.825733289717</v>
       </c>
       <c r="I31" t="n">
-        <v>1660.916666666667</v>
+        <v>1646.516666666667</v>
       </c>
       <c r="J31" t="n">
-        <v>35.36080988892732</v>
+        <v>34.84709555482862</v>
       </c>
       <c r="K31" t="n">
-        <v>27.68194444444445</v>
+        <v>27.44194444444445</v>
       </c>
       <c r="L31" t="n">
-        <v>207.3172258734002</v>
+        <v>201.4531894013739</v>
       </c>
       <c r="M31" t="n">
         <v>234.8166666666667</v>
       </c>
       <c r="N31" t="n">
-        <v>3.455287097890004</v>
+        <v>3.357553156689565</v>
       </c>
       <c r="O31" t="n">
         <v>3.913611111111111</v>
@@ -3857,43 +3857,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6230</v>
+        <v>6833</v>
       </c>
       <c r="D32" t="n">
-        <v>340.4267067950776</v>
+        <v>330.3981560076101</v>
       </c>
       <c r="E32" t="n">
-        <v>20.425</v>
+        <v>20.28333333333333</v>
       </c>
       <c r="F32" t="n">
-        <v>5.673778446584625</v>
+        <v>5.506635933460168</v>
       </c>
       <c r="G32" t="n">
-        <v>0.3404166666666667</v>
+        <v>0.3380555555555556</v>
       </c>
       <c r="H32" t="n">
-        <v>694.0605051985207</v>
+        <v>688.690564122089</v>
       </c>
       <c r="I32" t="n">
-        <v>435.2166666666666</v>
+        <v>435.7833333333334</v>
       </c>
       <c r="J32" t="n">
-        <v>11.56767508664201</v>
+        <v>11.47817606870148</v>
       </c>
       <c r="K32" t="n">
-        <v>7.253611111111111</v>
+        <v>7.263055555555556</v>
       </c>
       <c r="L32" t="n">
-        <v>253.6920696392436</v>
+        <v>262.4696332254585</v>
       </c>
       <c r="M32" t="n">
-        <v>70.81666666666666</v>
+        <v>71.06666666666666</v>
       </c>
       <c r="N32" t="n">
-        <v>4.228201160654059</v>
+        <v>4.374493887090975</v>
       </c>
       <c r="O32" t="n">
-        <v>1.180277777777778</v>
+        <v>1.184444444444444</v>
       </c>
     </row>
     <row r="33">
@@ -3908,43 +3908,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>9241</v>
+        <v>9778</v>
       </c>
       <c r="D33" t="n">
-        <v>401.3472585939472</v>
+        <v>402.4027186882117</v>
       </c>
       <c r="E33" t="n">
-        <v>62.76666666666667</v>
+        <v>65.92500000000001</v>
       </c>
       <c r="F33" t="n">
-        <v>6.689120976565787</v>
+        <v>6.706711978136861</v>
       </c>
       <c r="G33" t="n">
-        <v>1.046111111111111</v>
+        <v>1.09875</v>
       </c>
       <c r="H33" t="n">
-        <v>678.7645575771712</v>
+        <v>685.7487735918337</v>
       </c>
       <c r="I33" t="n">
-        <v>330.9</v>
+        <v>342.0833333333334</v>
       </c>
       <c r="J33" t="n">
-        <v>11.31274262628619</v>
+        <v>11.42914622653056</v>
       </c>
       <c r="K33" t="n">
-        <v>5.515000000000001</v>
+        <v>5.701388888888889</v>
       </c>
       <c r="L33" t="n">
-        <v>254.4889996889822</v>
+        <v>262.7073474333553</v>
       </c>
       <c r="M33" t="n">
-        <v>67.68333333333334</v>
+        <v>69.45833333333334</v>
       </c>
       <c r="N33" t="n">
-        <v>4.241483328149704</v>
+        <v>4.378455790555923</v>
       </c>
       <c r="O33" t="n">
-        <v>1.128055555555556</v>
+        <v>1.157638888888889</v>
       </c>
     </row>
     <row r="34">
@@ -3959,43 +3959,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1972</v>
+        <v>2129</v>
       </c>
       <c r="D34" t="n">
-        <v>1457.845884043272</v>
+        <v>1429.859769844998</v>
       </c>
       <c r="E34" t="n">
-        <v>1044.225</v>
+        <v>1036.633333333333</v>
       </c>
       <c r="F34" t="n">
-        <v>24.29743140072121</v>
+        <v>23.8309961640833</v>
       </c>
       <c r="G34" t="n">
-        <v>17.40375</v>
+        <v>17.27722222222222</v>
       </c>
       <c r="H34" t="n">
-        <v>2149.565047114252</v>
+        <v>2117.60903231663</v>
       </c>
       <c r="I34" t="n">
-        <v>1648.433333333333</v>
+        <v>1642.291666666667</v>
       </c>
       <c r="J34" t="n">
-        <v>35.82608411857087</v>
+        <v>35.29348387194383</v>
       </c>
       <c r="K34" t="n">
-        <v>27.47388888888889</v>
+        <v>27.37152777777778</v>
       </c>
       <c r="L34" t="n">
-        <v>539.3833333333333</v>
+        <v>543.6460330428467</v>
       </c>
       <c r="M34" t="n">
-        <v>442.525</v>
+        <v>444.6333333333333</v>
       </c>
       <c r="N34" t="n">
-        <v>8.989722222222223</v>
+        <v>9.06076721738078</v>
       </c>
       <c r="O34" t="n">
-        <v>7.375416666666666</v>
+        <v>7.410555555555556</v>
       </c>
     </row>
     <row r="35">
@@ -4010,43 +4010,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2307</v>
+        <v>2472</v>
       </c>
       <c r="D35" t="n">
-        <v>1909.514658286375</v>
+        <v>1861.983656957929</v>
       </c>
       <c r="E35" t="n">
-        <v>1900.133333333333</v>
+        <v>1824.408333333333</v>
       </c>
       <c r="F35" t="n">
-        <v>31.82524430477292</v>
+        <v>31.03306094929881</v>
       </c>
       <c r="G35" t="n">
-        <v>31.66888888888889</v>
+        <v>30.40680555555556</v>
       </c>
       <c r="H35" t="n">
-        <v>2459.743304254668</v>
+        <v>2434.428471328471</v>
       </c>
       <c r="I35" t="n">
-        <v>2366.15</v>
+        <v>2332.366666666667</v>
       </c>
       <c r="J35" t="n">
-        <v>40.9957217375778</v>
+        <v>40.57380785547452</v>
       </c>
       <c r="K35" t="n">
-        <v>39.43583333333333</v>
+        <v>38.87277777777778</v>
       </c>
       <c r="L35" t="n">
-        <v>536.72842822161</v>
+        <v>561.1538038038037</v>
       </c>
       <c r="M35" t="n">
-        <v>443.8916666666667</v>
+        <v>445.5333333333334</v>
       </c>
       <c r="N35" t="n">
-        <v>8.945473803693501</v>
+        <v>9.352563396730064</v>
       </c>
       <c r="O35" t="n">
-        <v>7.398194444444444</v>
+        <v>7.425555555555556</v>
       </c>
     </row>
     <row r="36">
@@ -4061,43 +4061,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1138</v>
+        <v>1265</v>
       </c>
       <c r="D36" t="n">
-        <v>17.06802870533099</v>
+        <v>15.49750988142292</v>
       </c>
       <c r="E36" t="n">
-        <v>20.35</v>
+        <v>20.18333333333333</v>
       </c>
       <c r="F36" t="n">
-        <v>0.2844671450888498</v>
+        <v>0.2582918313570488</v>
       </c>
       <c r="G36" t="n">
-        <v>0.3391666666666667</v>
+        <v>0.3363888888888889</v>
       </c>
       <c r="H36" t="n">
-        <v>2460.456875</v>
+        <v>2556.419755116959</v>
       </c>
       <c r="I36" t="n">
-        <v>1819.216666666667</v>
+        <v>2165.8</v>
       </c>
       <c r="J36" t="n">
-        <v>41.00761458333332</v>
+        <v>42.60699591861598</v>
       </c>
       <c r="K36" t="n">
-        <v>30.32027777777778</v>
+        <v>36.09666666666666</v>
       </c>
       <c r="L36" t="n">
-        <v>2437.4168125</v>
+        <v>2536.012097953216</v>
       </c>
       <c r="M36" t="n">
-        <v>1786.433333333333</v>
+        <v>2137.683333333333</v>
       </c>
       <c r="N36" t="n">
-        <v>40.62361354166666</v>
+        <v>42.26686829922027</v>
       </c>
       <c r="O36" t="n">
-        <v>29.77388888888889</v>
+        <v>35.62805555555556</v>
       </c>
     </row>
     <row r="37">
@@ -4112,43 +4112,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>489</v>
+        <v>547</v>
       </c>
       <c r="D37" t="n">
-        <v>2751.817246080436</v>
+        <v>2752.072699573431</v>
       </c>
       <c r="E37" t="n">
-        <v>2518.9</v>
+        <v>2551.266666666667</v>
       </c>
       <c r="F37" t="n">
-        <v>45.86362076800727</v>
+        <v>45.86787832622384</v>
       </c>
       <c r="G37" t="n">
-        <v>41.98166666666667</v>
+        <v>42.52111111111112</v>
       </c>
       <c r="H37" t="n">
-        <v>3183.666215199398</v>
+        <v>3175.70348759222</v>
       </c>
       <c r="I37" t="n">
-        <v>2858.5</v>
+        <v>2885.716666666667</v>
       </c>
       <c r="J37" t="n">
-        <v>53.06110358665664</v>
+        <v>52.92839145987033</v>
       </c>
       <c r="K37" t="n">
-        <v>47.64166666666667</v>
+        <v>48.09527777777778</v>
       </c>
       <c r="L37" t="n">
-        <v>286.4480060195636</v>
+        <v>273.2040576794098</v>
       </c>
       <c r="M37" t="n">
-        <v>289.4</v>
+        <v>230.2333333333333</v>
       </c>
       <c r="N37" t="n">
-        <v>4.774133433659394</v>
+        <v>4.553400961323497</v>
       </c>
       <c r="O37" t="n">
-        <v>4.823333333333333</v>
+        <v>3.837222222222222</v>
       </c>
     </row>
     <row r="38">
@@ -4163,43 +4163,43 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>302</v>
+        <v>337</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>0.06602373887240356</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>0.001100395647873393</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>380.6364583333333</v>
+        <v>288.5324324324324</v>
       </c>
       <c r="I38" t="n">
-        <v>130.7833333333333</v>
+        <v>79.36666666666666</v>
       </c>
       <c r="J38" t="n">
-        <v>6.343940972222223</v>
+        <v>4.808873873873874</v>
       </c>
       <c r="K38" t="n">
-        <v>2.179722222222222</v>
+        <v>1.322777777777778</v>
       </c>
       <c r="L38" t="n">
-        <v>380.6364583333333</v>
+        <v>287.9310810810811</v>
       </c>
       <c r="M38" t="n">
-        <v>130.7833333333333</v>
+        <v>78.06666666666666</v>
       </c>
       <c r="N38" t="n">
-        <v>6.343940972222223</v>
+        <v>4.798851351351352</v>
       </c>
       <c r="O38" t="n">
-        <v>2.179722222222222</v>
+        <v>1.301111111111111</v>
       </c>
     </row>
     <row r="39">
@@ -4214,43 +4214,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1111</v>
+        <v>1192</v>
       </c>
       <c r="D39" t="n">
-        <v>218.8424542454246</v>
+        <v>215.794966442953</v>
       </c>
       <c r="E39" t="n">
-        <v>89.98333333333333</v>
+        <v>90.38333333333333</v>
       </c>
       <c r="F39" t="n">
-        <v>3.647374237423743</v>
+        <v>3.596582774049217</v>
       </c>
       <c r="G39" t="n">
-        <v>1.499722222222222</v>
+        <v>1.506388888888889</v>
       </c>
       <c r="H39" t="n">
-        <v>544.346152676399</v>
+        <v>544.1107558965616</v>
       </c>
       <c r="I39" t="n">
-        <v>469.2416666666667</v>
+        <v>485.65</v>
       </c>
       <c r="J39" t="n">
-        <v>9.072435877939983</v>
+        <v>9.068512598276024</v>
       </c>
       <c r="K39" t="n">
-        <v>7.820694444444444</v>
+        <v>8.094166666666666</v>
       </c>
       <c r="L39" t="n">
-        <v>324.2905717761557</v>
+        <v>327.724978687127</v>
       </c>
       <c r="M39" t="n">
-        <v>205.95</v>
+        <v>225.1166666666667</v>
       </c>
       <c r="N39" t="n">
-        <v>5.404842862935928</v>
+        <v>5.462082978118783</v>
       </c>
       <c r="O39" t="n">
-        <v>3.4325</v>
+        <v>3.751944444444445</v>
       </c>
     </row>
     <row r="40">
@@ -4265,40 +4265,40 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>32716</v>
+        <v>34880</v>
       </c>
       <c r="D40" t="n">
-        <v>125.122158882504</v>
+        <v>118.6896081804281</v>
       </c>
       <c r="E40" t="n">
-        <v>2.016666666666667</v>
+        <v>1.933333333333333</v>
       </c>
       <c r="F40" t="n">
-        <v>2.0853693147084</v>
+        <v>1.978160136340469</v>
       </c>
       <c r="G40" t="n">
-        <v>0.03361111111111111</v>
+        <v>0.03222222222222222</v>
       </c>
       <c r="H40" t="n">
-        <v>196.1111803203785</v>
+        <v>190.2468324139147</v>
       </c>
       <c r="I40" t="n">
-        <v>20.81666666666667</v>
+        <v>20.76666666666667</v>
       </c>
       <c r="J40" t="n">
-        <v>3.268519672006307</v>
+        <v>3.170780540231912</v>
       </c>
       <c r="K40" t="n">
-        <v>0.3469444444444444</v>
+        <v>0.3461111111111111</v>
       </c>
       <c r="L40" t="n">
-        <v>32.9230863301618</v>
+        <v>35.56440149625935</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.5487181055026966</v>
+        <v>0.5927400249376558</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -4316,43 +4316,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>9261</v>
+        <v>9823</v>
       </c>
       <c r="D41" t="n">
-        <v>798.685127596012</v>
+        <v>779.5033730360718</v>
       </c>
       <c r="E41" t="n">
-        <v>664.8166666666667</v>
+        <v>647.65</v>
       </c>
       <c r="F41" t="n">
-        <v>13.31141879326687</v>
+        <v>12.99172288393453</v>
       </c>
       <c r="G41" t="n">
-        <v>11.08027777777778</v>
+        <v>10.79416666666667</v>
       </c>
       <c r="H41" t="n">
-        <v>895.375662270319</v>
+        <v>876.9706051512877</v>
       </c>
       <c r="I41" t="n">
-        <v>765.25</v>
+        <v>746.8666666666667</v>
       </c>
       <c r="J41" t="n">
-        <v>14.92292770450532</v>
+        <v>14.61617675252146</v>
       </c>
       <c r="K41" t="n">
-        <v>12.75416666666667</v>
+        <v>12.44777777777778</v>
       </c>
       <c r="L41" t="n">
-        <v>91.06264043888325</v>
+        <v>89.83725752866788</v>
       </c>
       <c r="M41" t="n">
-        <v>73.86666666666666</v>
+        <v>72.76666666666667</v>
       </c>
       <c r="N41" t="n">
-        <v>1.517710673981387</v>
+        <v>1.497287625477798</v>
       </c>
       <c r="O41" t="n">
-        <v>1.231111111111111</v>
+        <v>1.212777777777778</v>
       </c>
     </row>
     <row r="42">
@@ -4367,43 +4367,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>67663</v>
+        <v>72965</v>
       </c>
       <c r="D42" t="n">
-        <v>17.49177196793915</v>
+        <v>16.33591333744489</v>
       </c>
       <c r="E42" t="n">
-        <v>20.41666666666667</v>
+        <v>20.31666666666667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.2915295327989857</v>
+        <v>0.2722652222907482</v>
       </c>
       <c r="G42" t="n">
-        <v>0.3402777777777778</v>
+        <v>0.3386111111111111</v>
       </c>
       <c r="H42" t="n">
-        <v>496.4281213396886</v>
+        <v>487.7713662845229</v>
       </c>
       <c r="I42" t="n">
-        <v>184.7833333333333</v>
+        <v>185.2</v>
       </c>
       <c r="J42" t="n">
-        <v>8.273802022328141</v>
+        <v>8.129522771408716</v>
       </c>
       <c r="K42" t="n">
-        <v>3.079722222222222</v>
+        <v>3.086666666666666</v>
       </c>
       <c r="L42" t="n">
-        <v>477.3967122429809</v>
+        <v>470.05796579465</v>
       </c>
       <c r="M42" t="n">
-        <v>165.6833333333333</v>
+        <v>167.4666666666667</v>
       </c>
       <c r="N42" t="n">
-        <v>7.956611870716349</v>
+        <v>7.834299429910832</v>
       </c>
       <c r="O42" t="n">
-        <v>2.761388888888889</v>
+        <v>2.791111111111111</v>
       </c>
     </row>
     <row r="43">
@@ -4418,43 +4418,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>46450</v>
+        <v>49780</v>
       </c>
       <c r="D43" t="n">
-        <v>150.1527922497309</v>
+        <v>155.1284608946029</v>
       </c>
       <c r="E43" t="n">
-        <v>79.34999999999999</v>
+        <v>80.65000000000001</v>
       </c>
       <c r="F43" t="n">
-        <v>2.502546537495515</v>
+        <v>2.585474348243382</v>
       </c>
       <c r="G43" t="n">
-        <v>1.3225</v>
+        <v>1.344166666666667</v>
       </c>
       <c r="H43" t="n">
-        <v>546.2368451085314</v>
+        <v>542.2905018953537</v>
       </c>
       <c r="I43" t="n">
-        <v>232.4833333333333</v>
+        <v>234.6333333333333</v>
       </c>
       <c r="J43" t="n">
-        <v>9.103947418475522</v>
+        <v>9.03817503158923</v>
       </c>
       <c r="K43" t="n">
-        <v>3.874722222222222</v>
+        <v>3.910555555555555</v>
       </c>
       <c r="L43" t="n">
-        <v>394.9053736622528</v>
+        <v>389.7402636426352</v>
       </c>
       <c r="M43" t="n">
-        <v>114.5333333333333</v>
+        <v>114.4166666666667</v>
       </c>
       <c r="N43" t="n">
-        <v>6.581756227704214</v>
+        <v>6.495671060710585</v>
       </c>
       <c r="O43" t="n">
-        <v>1.908888888888889</v>
+        <v>1.906944444444445</v>
       </c>
     </row>
     <row r="44">
@@ -4469,43 +4469,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>7653</v>
+        <v>8409</v>
       </c>
       <c r="D44" t="n">
-        <v>13.17853565050743</v>
+        <v>12.10447139969081</v>
       </c>
       <c r="E44" t="n">
-        <v>1.95</v>
+        <v>1.866666666666667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.2196422608417904</v>
+        <v>0.2017411899948468</v>
       </c>
       <c r="G44" t="n">
-        <v>0.0325</v>
+        <v>0.03111111111111111</v>
       </c>
       <c r="H44" t="n">
-        <v>820.3296343402226</v>
+        <v>803.1863700359258</v>
       </c>
       <c r="I44" t="n">
-        <v>799.7583333333333</v>
+        <v>787.2916666666667</v>
       </c>
       <c r="J44" t="n">
-        <v>13.67216057233704</v>
+        <v>13.38643950059877</v>
       </c>
       <c r="K44" t="n">
-        <v>13.32930555555556</v>
+        <v>13.12152777777778</v>
       </c>
       <c r="L44" t="n">
-        <v>804.6955219925809</v>
+        <v>788.7304689775707</v>
       </c>
       <c r="M44" t="n">
-        <v>783.9333333333334</v>
+        <v>772.2333333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>13.41159203320968</v>
+        <v>13.14550781629285</v>
       </c>
       <c r="O44" t="n">
-        <v>13.06555555555556</v>
+        <v>12.87055555555556</v>
       </c>
     </row>
     <row r="45">
@@ -4520,43 +4520,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>13779</v>
+        <v>14118</v>
       </c>
       <c r="D45" t="n">
-        <v>221.0427534654184</v>
+        <v>223.9100651650375</v>
       </c>
       <c r="E45" t="n">
-        <v>27.71666666666667</v>
+        <v>29.25</v>
       </c>
       <c r="F45" t="n">
-        <v>3.684045891090307</v>
+        <v>3.731834419417292</v>
       </c>
       <c r="G45" t="n">
-        <v>0.4619444444444444</v>
+        <v>0.4875</v>
       </c>
       <c r="H45" t="n">
-        <v>822.5919505577328</v>
+        <v>829.3605793049321</v>
       </c>
       <c r="I45" t="n">
-        <v>856.5083333333333</v>
+        <v>862.5166666666667</v>
       </c>
       <c r="J45" t="n">
-        <v>13.70986584262888</v>
+        <v>13.82267632174887</v>
       </c>
       <c r="K45" t="n">
-        <v>14.27513888888889</v>
+        <v>14.37527777777778</v>
       </c>
       <c r="L45" t="n">
-        <v>601.0616759622148</v>
+        <v>604.9602862188212</v>
       </c>
       <c r="M45" t="n">
-        <v>437.0083333333333</v>
+        <v>441.95</v>
       </c>
       <c r="N45" t="n">
-        <v>10.01769459937025</v>
+        <v>10.08267143698035</v>
       </c>
       <c r="O45" t="n">
-        <v>7.283472222222223</v>
+        <v>7.365833333333333</v>
       </c>
     </row>
     <row r="46">
@@ -4571,43 +4571,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>981</v>
+        <v>1241</v>
       </c>
       <c r="D46" t="n">
-        <v>16.45504587155963</v>
+        <v>13.30096696212732</v>
       </c>
       <c r="E46" t="n">
-        <v>20.4</v>
+        <v>1.966666666666667</v>
       </c>
       <c r="F46" t="n">
-        <v>0.2742507645259939</v>
+        <v>0.221682782702122</v>
       </c>
       <c r="G46" t="n">
-        <v>0.34</v>
+        <v>0.03277777777777777</v>
       </c>
       <c r="H46" t="n">
-        <v>3269.677423822715</v>
+        <v>3337.216862117981</v>
       </c>
       <c r="I46" t="n">
-        <v>2943.358333333334</v>
+        <v>3245</v>
       </c>
       <c r="J46" t="n">
-        <v>54.49462373037858</v>
+        <v>55.62028103529969</v>
       </c>
       <c r="K46" t="n">
-        <v>49.05597222222222</v>
+        <v>54.08333333333333</v>
       </c>
       <c r="L46" t="n">
-        <v>3247.938481071099</v>
+        <v>3320.112117981521</v>
       </c>
       <c r="M46" t="n">
-        <v>2922.858333333333</v>
+        <v>3218.608333333334</v>
       </c>
       <c r="N46" t="n">
-        <v>54.13230801785164</v>
+        <v>55.33520196635868</v>
       </c>
       <c r="O46" t="n">
-        <v>48.71430555555555</v>
+        <v>53.64347222222223</v>
       </c>
     </row>
     <row r="47">
@@ -4622,43 +4622,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1297</v>
+        <v>1509</v>
       </c>
       <c r="D47" t="n">
-        <v>215.2599460292984</v>
+        <v>233.5916832339297</v>
       </c>
       <c r="E47" t="n">
-        <v>42.2</v>
+        <v>50.31666666666667</v>
       </c>
       <c r="F47" t="n">
-        <v>3.587665767154973</v>
+        <v>3.893194720565496</v>
       </c>
       <c r="G47" t="n">
-        <v>0.7033333333333334</v>
+        <v>0.8386111111111112</v>
       </c>
       <c r="H47" t="n">
-        <v>3262.960426796326</v>
+        <v>3298.929506685108</v>
       </c>
       <c r="I47" t="n">
-        <v>2963.741666666667</v>
+        <v>3011.716666666667</v>
       </c>
       <c r="J47" t="n">
-        <v>54.38267377993878</v>
+        <v>54.9821584447518</v>
       </c>
       <c r="K47" t="n">
-        <v>49.39569444444444</v>
+        <v>50.19527777777778</v>
       </c>
       <c r="L47" t="n">
-        <v>3048.287722852512</v>
+        <v>3064.575945136007</v>
       </c>
       <c r="M47" t="n">
-        <v>2876.583333333333</v>
+        <v>2885.058333333333</v>
       </c>
       <c r="N47" t="n">
-        <v>50.80479538087521</v>
+        <v>51.07626575226679</v>
       </c>
       <c r="O47" t="n">
-        <v>47.94305555555555</v>
+        <v>48.08430555555555</v>
       </c>
     </row>
     <row r="48">
@@ -4673,43 +4673,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>5390</v>
+        <v>5753</v>
       </c>
       <c r="D48" t="n">
-        <v>16.43401669758812</v>
+        <v>15.49175212932383</v>
       </c>
       <c r="E48" t="n">
-        <v>20.275</v>
+        <v>20.1</v>
       </c>
       <c r="F48" t="n">
-        <v>0.2739002782931355</v>
+        <v>0.2581958688220638</v>
       </c>
       <c r="G48" t="n">
-        <v>0.3379166666666667</v>
+        <v>0.335</v>
       </c>
       <c r="H48" t="n">
-        <v>418.4459716496709</v>
+        <v>411.585717653398</v>
       </c>
       <c r="I48" t="n">
-        <v>353.15</v>
+        <v>345.9333333333333</v>
       </c>
       <c r="J48" t="n">
-        <v>6.974099527494515</v>
+        <v>6.859761960889967</v>
       </c>
       <c r="K48" t="n">
-        <v>5.885833333333333</v>
+        <v>5.765555555555555</v>
       </c>
       <c r="L48" t="n">
-        <v>399.4396940768062</v>
+        <v>393.7757156327878</v>
       </c>
       <c r="M48" t="n">
-        <v>327.8666666666667</v>
+        <v>324.8166666666667</v>
       </c>
       <c r="N48" t="n">
-        <v>6.657328234613438</v>
+        <v>6.562928593879796</v>
       </c>
       <c r="O48" t="n">
-        <v>5.464444444444444</v>
+        <v>5.413611111111111</v>
       </c>
     </row>
     <row r="49">
@@ -4724,43 +4724,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2456</v>
+        <v>2569</v>
       </c>
       <c r="D49" t="n">
-        <v>295.0677049402823</v>
+        <v>290.0281951472687</v>
       </c>
       <c r="E49" t="n">
-        <v>112.0916666666667</v>
+        <v>109.7166666666667</v>
       </c>
       <c r="F49" t="n">
-        <v>4.917795082338039</v>
+        <v>4.833803252454478</v>
       </c>
       <c r="G49" t="n">
-        <v>1.868194444444444</v>
+        <v>1.828611111111111</v>
       </c>
       <c r="H49" t="n">
-        <v>663.9142130584193</v>
+        <v>658.5903297858363</v>
       </c>
       <c r="I49" t="n">
-        <v>558.9833333333333</v>
+        <v>554.9333333333333</v>
       </c>
       <c r="J49" t="n">
-        <v>11.06523688430699</v>
+        <v>10.9765054964306</v>
       </c>
       <c r="K49" t="n">
-        <v>9.316388888888889</v>
+        <v>9.248888888888889</v>
       </c>
       <c r="L49" t="n">
-        <v>368.1101580756014</v>
+        <v>367.8139534883721</v>
       </c>
       <c r="M49" t="n">
-        <v>194.1333333333333</v>
+        <v>196.5166666666667</v>
       </c>
       <c r="N49" t="n">
-        <v>6.135169301260023</v>
+        <v>6.130232558139536</v>
       </c>
       <c r="O49" t="n">
-        <v>3.235555555555556</v>
+        <v>3.275277777777778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard mié 02/09/2026 11:02:08,23
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -699,28 +699,28 @@
         <v>65.29306173417623</v>
       </c>
       <c r="W2" t="n">
-        <v>9832</v>
+        <v>9849</v>
       </c>
       <c r="X2" t="n">
-        <v>25.56956875508544</v>
+        <v>25.69804041019393</v>
       </c>
       <c r="Y2" t="n">
-        <v>71.60292921074044</v>
+        <v>71.65194435983349</v>
       </c>
       <c r="Z2" t="n">
-        <v>52</v>
+        <v>455</v>
       </c>
       <c r="AA2" t="n">
-        <v>40.38461538461539</v>
+        <v>34.72527472527472</v>
       </c>
       <c r="AB2" t="n">
-        <v>76.92307692307693</v>
+        <v>68.57142857142857</v>
       </c>
       <c r="AC2" t="n">
-        <v>14.81504662952995</v>
+        <v>9.027234315080793</v>
       </c>
       <c r="AD2" t="n">
-        <v>-99.47111472742066</v>
+        <v>-95.38024164889836</v>
       </c>
     </row>
     <row r="3">
@@ -802,19 +802,19 @@
         <v>79.51807228915662</v>
       </c>
       <c r="Z3" t="n">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="AA3" t="n">
-        <v>50</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="AB3" t="n">
-        <v>100</v>
+        <v>91.48936170212765</v>
       </c>
       <c r="AC3" t="n">
-        <v>24.18244406196213</v>
+        <v>31.62925257260044</v>
       </c>
       <c r="AD3" t="n">
-        <v>-98.96729776247849</v>
+        <v>-91.91049913941481</v>
       </c>
     </row>
     <row r="4">
@@ -887,28 +887,28 @@
         <v>34.85881207400195</v>
       </c>
       <c r="W4" t="n">
-        <v>373</v>
+        <v>457</v>
       </c>
       <c r="X4" t="n">
-        <v>23.32439678284182</v>
+        <v>19.47483588621444</v>
       </c>
       <c r="Y4" t="n">
-        <v>65.41554959785523</v>
+        <v>63.45733041575492</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AB4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="AC4" t="n">
-        <v>-23.32439678284182</v>
+        <v>80.52516411378556</v>
       </c>
       <c r="AD4" t="n">
-        <v>-100</v>
+        <v>-99.78118161925602</v>
       </c>
     </row>
     <row r="5">
@@ -981,28 +981,28 @@
         <v>52.69410267288927</v>
       </c>
       <c r="W5" t="n">
-        <v>1950</v>
+        <v>1988</v>
       </c>
       <c r="X5" t="n">
-        <v>55.43589743589744</v>
+        <v>55.73440643863179</v>
       </c>
       <c r="Y5" t="n">
-        <v>62.15384615384615</v>
+        <v>62.37424547283702</v>
       </c>
       <c r="Z5" t="n">
-        <v>6</v>
+        <v>94</v>
       </c>
       <c r="AA5" t="n">
-        <v>100</v>
+        <v>60.63829787234043</v>
       </c>
       <c r="AB5" t="n">
-        <v>100</v>
+        <v>64.8936170212766</v>
       </c>
       <c r="AC5" t="n">
-        <v>44.56410256410256</v>
+        <v>4.903891433708644</v>
       </c>
       <c r="AD5" t="n">
-        <v>-99.69230769230769</v>
+        <v>-95.27162977867204</v>
       </c>
     </row>
     <row r="6">
@@ -1075,28 +1075,28 @@
         <v>64.41954378433441</v>
       </c>
       <c r="W6" t="n">
-        <v>19755</v>
+        <v>19863</v>
       </c>
       <c r="X6" t="n">
-        <v>78.95216400911161</v>
+        <v>79.06660625283189</v>
       </c>
       <c r="Y6" t="n">
-        <v>82.45001265502404</v>
+        <v>82.54543623823189</v>
       </c>
       <c r="Z6" t="n">
-        <v>5</v>
+        <v>1383</v>
       </c>
       <c r="AA6" t="n">
-        <v>100</v>
+        <v>36.73174258857556</v>
       </c>
       <c r="AB6" t="n">
-        <v>100</v>
+        <v>45.98698481561822</v>
       </c>
       <c r="AC6" t="n">
-        <v>21.04783599088839</v>
+        <v>-42.33486366425632</v>
       </c>
       <c r="AD6" t="n">
-        <v>-99.97468995191092</v>
+        <v>-93.03730554296934</v>
       </c>
     </row>
     <row r="7">
@@ -1169,28 +1169,28 @@
         <v>61.85549639414975</v>
       </c>
       <c r="W7" t="n">
-        <v>24881</v>
+        <v>24906</v>
       </c>
       <c r="X7" t="n">
-        <v>44.49580000803826</v>
+        <v>44.49931743355015</v>
       </c>
       <c r="Y7" t="n">
-        <v>64.36236485671797</v>
+        <v>64.37806151128243</v>
       </c>
       <c r="Z7" t="n">
-        <v>129</v>
+        <v>1480</v>
       </c>
       <c r="AA7" t="n">
-        <v>72.86821705426357</v>
+        <v>58.51351351351352</v>
       </c>
       <c r="AB7" t="n">
-        <v>86.82170542635659</v>
+        <v>67.70270270270269</v>
       </c>
       <c r="AC7" t="n">
-        <v>28.37241704622531</v>
+        <v>14.01419607996336</v>
       </c>
       <c r="AD7" t="n">
-        <v>-99.48153209276155</v>
+        <v>-94.05765678952864</v>
       </c>
     </row>
     <row r="8">
@@ -1263,28 +1263,28 @@
         <v>53.9494851994852</v>
       </c>
       <c r="W8" t="n">
-        <v>7676</v>
+        <v>7735</v>
       </c>
       <c r="X8" t="n">
-        <v>49.36164669098489</v>
+        <v>49.41176470588236</v>
       </c>
       <c r="Y8" t="n">
-        <v>63.23606044815008</v>
+        <v>63.24499030381383</v>
       </c>
       <c r="Z8" t="n">
-        <v>359</v>
+        <v>474</v>
       </c>
       <c r="AA8" t="n">
-        <v>54.87465181058496</v>
+        <v>54.85232067510548</v>
       </c>
       <c r="AB8" t="n">
-        <v>65.18105849582173</v>
+        <v>64.55696202531645</v>
       </c>
       <c r="AC8" t="n">
-        <v>5.513005119600074</v>
+        <v>5.440555969223126</v>
       </c>
       <c r="AD8" t="n">
-        <v>-95.32308494007296</v>
+        <v>-93.87201034259857</v>
       </c>
     </row>
     <row r="9">
@@ -1357,28 +1357,28 @@
         <v>68.22074215033301</v>
       </c>
       <c r="W9" t="n">
-        <v>2559</v>
+        <v>2668</v>
       </c>
       <c r="X9" t="n">
-        <v>69.51934349355217</v>
+        <v>70.76461769115441</v>
       </c>
       <c r="Y9" t="n">
-        <v>75.69363032434545</v>
+        <v>76.68665667166417</v>
       </c>
       <c r="Z9" t="n">
-        <v>5</v>
+        <v>92</v>
       </c>
       <c r="AA9" t="n">
-        <v>100</v>
+        <v>41.30434782608695</v>
       </c>
       <c r="AB9" t="n">
-        <v>100</v>
+        <v>52.17391304347826</v>
       </c>
       <c r="AC9" t="n">
-        <v>30.48065650644783</v>
+        <v>-29.46026986506746</v>
       </c>
       <c r="AD9" t="n">
-        <v>-99.80461117624073</v>
+        <v>-96.55172413793103</v>
       </c>
     </row>
     <row r="10">
@@ -1451,28 +1451,28 @@
         <v>36.93293885601578</v>
       </c>
       <c r="W10" t="n">
-        <v>2705</v>
+        <v>2706</v>
       </c>
       <c r="X10" t="n">
-        <v>33.45656192236599</v>
+        <v>33.48115299334812</v>
       </c>
       <c r="Y10" t="n">
-        <v>54.63955637707948</v>
+        <v>54.65631929046562</v>
       </c>
       <c r="Z10" t="n">
-        <v>11</v>
+        <v>182</v>
       </c>
       <c r="AA10" t="n">
-        <v>100</v>
+        <v>56.04395604395604</v>
       </c>
       <c r="AB10" t="n">
-        <v>100</v>
+        <v>62.63736263736264</v>
       </c>
       <c r="AC10" t="n">
-        <v>66.54343807763401</v>
+        <v>22.56280305060793</v>
       </c>
       <c r="AD10" t="n">
-        <v>-99.59334565619223</v>
+        <v>-93.27420546932743</v>
       </c>
     </row>
     <row r="11">
@@ -1545,28 +1545,28 @@
         <v>73.6447415973979</v>
       </c>
       <c r="W11" t="n">
-        <v>71059</v>
+        <v>71097</v>
       </c>
       <c r="X11" t="n">
-        <v>78.40667614236058</v>
+        <v>78.41259124857589</v>
       </c>
       <c r="Y11" t="n">
-        <v>81.92065748181089</v>
+        <v>81.92610096065937</v>
       </c>
       <c r="Z11" t="n">
-        <v>426</v>
+        <v>3441</v>
       </c>
       <c r="AA11" t="n">
-        <v>100</v>
+        <v>77.44841615809358</v>
       </c>
       <c r="AB11" t="n">
-        <v>100</v>
+        <v>80.76140656785819</v>
       </c>
       <c r="AC11" t="n">
-        <v>21.59332385763942</v>
+        <v>-0.9641750904823141</v>
       </c>
       <c r="AD11" t="n">
-        <v>-99.40049817757075</v>
+        <v>-95.16013333895945</v>
       </c>
     </row>
     <row r="12">
@@ -1639,28 +1639,28 @@
         <v>74.93570456560008</v>
       </c>
       <c r="W12" t="n">
-        <v>198454</v>
+        <v>200009</v>
       </c>
       <c r="X12" t="n">
-        <v>62.25876021647334</v>
+        <v>62.27519761610728</v>
       </c>
       <c r="Y12" t="n">
-        <v>79.34836284479023</v>
+        <v>79.34442950067246</v>
       </c>
       <c r="Z12" t="n">
-        <v>1146</v>
+        <v>8108</v>
       </c>
       <c r="AA12" t="n">
-        <v>62.30366492146597</v>
+        <v>64.29452392698569</v>
       </c>
       <c r="AB12" t="n">
-        <v>78.53403141361257</v>
+        <v>79.18105574740997</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.04490470499263211</v>
+        <v>2.019326310878412</v>
       </c>
       <c r="AD12" t="n">
-        <v>-99.4225362048636</v>
+        <v>-95.94618242179102</v>
       </c>
     </row>
     <row r="13">
@@ -1733,28 +1733,28 @@
         <v>60.82532992468735</v>
       </c>
       <c r="W13" t="n">
-        <v>37012</v>
+        <v>38714</v>
       </c>
       <c r="X13" t="n">
-        <v>42.42678050362045</v>
+        <v>42.86304695975616</v>
       </c>
       <c r="Y13" t="n">
-        <v>66.87290608451313</v>
+        <v>67.14883504675311</v>
       </c>
       <c r="Z13" t="n">
-        <v>33</v>
+        <v>2024</v>
       </c>
       <c r="AA13" t="n">
-        <v>69.6969696969697</v>
+        <v>45.35573122529645</v>
       </c>
       <c r="AB13" t="n">
-        <v>78.78787878787878</v>
+        <v>65.26679841897233</v>
       </c>
       <c r="AC13" t="n">
-        <v>27.27018919334925</v>
+        <v>2.492684265540284</v>
       </c>
       <c r="AD13" t="n">
-        <v>-99.9108397276559</v>
+        <v>-94.77191713591982</v>
       </c>
     </row>
     <row r="14">
@@ -1827,28 +1827,28 @@
         <v>60.31513970110461</v>
       </c>
       <c r="W14" t="n">
-        <v>3573</v>
+        <v>4118</v>
       </c>
       <c r="X14" t="n">
-        <v>48.30674503218584</v>
+        <v>48.64011656143759</v>
       </c>
       <c r="Y14" t="n">
-        <v>71.70445004198153</v>
+        <v>71.97668771248179</v>
       </c>
       <c r="Z14" t="n">
-        <v>11</v>
+        <v>59</v>
       </c>
       <c r="AA14" t="n">
-        <v>81.81818181818183</v>
+        <v>71.1864406779661</v>
       </c>
       <c r="AB14" t="n">
-        <v>90.90909090909091</v>
+        <v>83.05084745762711</v>
       </c>
       <c r="AC14" t="n">
-        <v>33.51143678599599</v>
+        <v>22.54632411652851</v>
       </c>
       <c r="AD14" t="n">
-        <v>-99.69213546039742</v>
+        <v>-98.56726566294317</v>
       </c>
     </row>
     <row r="15">
@@ -1921,28 +1921,28 @@
         <v>74.15969011620642</v>
       </c>
       <c r="W15" t="n">
-        <v>13021</v>
+        <v>13328</v>
       </c>
       <c r="X15" t="n">
-        <v>70.06374318408724</v>
+        <v>69.77791116446579</v>
       </c>
       <c r="Y15" t="n">
-        <v>78.55003455955763</v>
+        <v>78.45138055222088</v>
       </c>
       <c r="Z15" t="n">
-        <v>11</v>
+        <v>423</v>
       </c>
       <c r="AA15" t="n">
-        <v>100</v>
+        <v>68.32151300236407</v>
       </c>
       <c r="AB15" t="n">
-        <v>100</v>
+        <v>74.70449172576832</v>
       </c>
       <c r="AC15" t="n">
-        <v>29.93625681591276</v>
+        <v>-1.456398162101721</v>
       </c>
       <c r="AD15" t="n">
-        <v>-99.91552108133016</v>
+        <v>-96.82623049219687</v>
       </c>
     </row>
   </sheetData>
@@ -3863,19 +3863,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22</v>
+        <v>297</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="D4" t="n">
-        <v>4.545454545454546</v>
+        <v>8.080808080808081</v>
       </c>
       <c r="E4" t="n">
-        <v>95</v>
+        <v>1041.718333333333</v>
       </c>
       <c r="F4" t="n">
-        <v>99.77809523809525</v>
+        <v>2839.077032967033</v>
       </c>
     </row>
     <row r="5">
@@ -3885,19 +3885,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1680</v>
+        <v>12598</v>
       </c>
       <c r="C5" t="n">
-        <v>1413</v>
+        <v>10334</v>
       </c>
       <c r="D5" t="n">
-        <v>84.10714285714286</v>
+        <v>82.02889347515479</v>
       </c>
       <c r="E5" t="n">
-        <v>954.2693276716207</v>
+        <v>3645.505887362105</v>
       </c>
       <c r="F5" t="n">
-        <v>934.7420973782771</v>
+        <v>20112.23494257951</v>
       </c>
     </row>
     <row r="6">
@@ -3907,19 +3907,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>422</v>
+        <v>4469</v>
       </c>
       <c r="C6" t="n">
-        <v>79</v>
+        <v>490</v>
       </c>
       <c r="D6" t="n">
-        <v>18.72037914691943</v>
+        <v>10.96442157082121</v>
       </c>
       <c r="E6" t="n">
-        <v>44938.69860759494</v>
+        <v>11002.56659183674</v>
       </c>
       <c r="F6" t="n">
-        <v>340.415860058309</v>
+        <v>10697.80345061573</v>
       </c>
     </row>
     <row r="7">
@@ -3929,19 +3929,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>76</v>
+        <v>899</v>
       </c>
       <c r="C7" t="n">
-        <v>32</v>
+        <v>296</v>
       </c>
       <c r="D7" t="n">
-        <v>42.10526315789473</v>
+        <v>32.92547274749722</v>
       </c>
       <c r="E7" t="n">
-        <v>161.0778125</v>
+        <v>2195.769020270271</v>
       </c>
       <c r="F7" t="n">
-        <v>65.49636363636364</v>
+        <v>7539.56167495854</v>
       </c>
     </row>
     <row r="8"/>
@@ -3999,19 +3999,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8077</v>
+        <v>8170</v>
       </c>
       <c r="C12" t="n">
-        <v>1182</v>
+        <v>1186</v>
       </c>
       <c r="D12" t="n">
-        <v>14.63414634146341</v>
+        <v>14.51652386780906</v>
       </c>
       <c r="E12" t="n">
-        <v>714.5970558375634</v>
+        <v>712.7015767284992</v>
       </c>
       <c r="F12" t="n">
-        <v>1211.36404350979</v>
+        <v>1297.363880297823</v>
       </c>
     </row>
     <row r="13">
@@ -4021,19 +4021,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>282365</v>
+        <v>285775</v>
       </c>
       <c r="C13" t="n">
-        <v>222408</v>
+        <v>225004</v>
       </c>
       <c r="D13" t="n">
-        <v>78.76613602960707</v>
+        <v>78.73466888286239</v>
       </c>
       <c r="E13" t="n">
-        <v>4126.47125965298</v>
+        <v>4125.764280132353</v>
       </c>
       <c r="F13" t="n">
-        <v>6215.480429474456</v>
+        <v>6151.237982261277</v>
       </c>
     </row>
     <row r="14">
@@ -4043,19 +4043,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>84020</v>
+        <v>84889</v>
       </c>
       <c r="C14" t="n">
-        <v>11210</v>
+        <v>11243</v>
       </c>
       <c r="D14" t="n">
-        <v>13.34206141394906</v>
+        <v>13.24435439220629</v>
       </c>
       <c r="E14" t="n">
-        <v>9712.2407279215</v>
+        <v>9704.806294583297</v>
       </c>
       <c r="F14" t="n">
-        <v>3767.443206549925</v>
+        <v>3741.013305527795</v>
       </c>
     </row>
     <row r="15">
@@ -4065,19 +4065,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18969</v>
+        <v>19185</v>
       </c>
       <c r="C15" t="n">
-        <v>7995</v>
+        <v>8051</v>
       </c>
       <c r="D15" t="n">
-        <v>42.14771469239285</v>
+        <v>41.96507688298149</v>
       </c>
       <c r="E15" t="n">
-        <v>887.474268292683</v>
+        <v>895.4252720158987</v>
       </c>
       <c r="F15" t="n">
-        <v>3334.587063058138</v>
+        <v>3312.71680977187</v>
       </c>
     </row>
     <row r="16"/>
@@ -5043,7 +5043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5119,19 +5119,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>52</v>
+        <v>455</v>
       </c>
       <c r="C4" t="n">
-        <v>21</v>
+        <v>158</v>
       </c>
       <c r="D4" t="n">
-        <v>40.38461538461539</v>
+        <v>34.72527472527472</v>
       </c>
       <c r="E4" t="n">
-        <v>40</v>
+        <v>312</v>
       </c>
       <c r="F4" t="n">
-        <v>76.92307692307693</v>
+        <v>68.57142857142857</v>
       </c>
     </row>
     <row r="5">
@@ -5141,38 +5141,38 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>47</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="D5" t="n">
-        <v>50</v>
+        <v>57.44680851063831</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="F5" t="n">
-        <v>100</v>
+        <v>91.48936170212765</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Doradobet Chile</t>
+          <t>Doradobet Bolivia</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>100</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>100</v>
@@ -5181,224 +5181,245 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Doradobet Costa Rica</t>
+          <t>Doradobet Chile</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>94</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>57</v>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>60.63829787234043</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>64.8936170212766</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Doradobet Ecuador</t>
+          <t>Doradobet Costa Rica</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>129</v>
+        <v>1383</v>
       </c>
       <c r="C8" t="n">
-        <v>94</v>
+        <v>508</v>
       </c>
       <c r="D8" t="n">
-        <v>72.86821705426357</v>
+        <v>36.73174258857556</v>
       </c>
       <c r="E8" t="n">
-        <v>112</v>
+        <v>636</v>
       </c>
       <c r="F8" t="n">
-        <v>86.82170542635659</v>
+        <v>45.98698481561822</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Doradobet El Salvador</t>
+          <t>Doradobet Ecuador</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>359</v>
+        <v>1480</v>
       </c>
       <c r="C9" t="n">
-        <v>197</v>
+        <v>866</v>
       </c>
       <c r="D9" t="n">
-        <v>54.87465181058496</v>
+        <v>58.51351351351352</v>
       </c>
       <c r="E9" t="n">
-        <v>234</v>
+        <v>1002</v>
       </c>
       <c r="F9" t="n">
-        <v>65.18105849582173</v>
+        <v>67.70270270270269</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Doradobet Guatemala</t>
+          <t>Doradobet El Salvador</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>474</v>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>260</v>
       </c>
       <c r="D10" t="n">
-        <v>100</v>
+        <v>54.85232067510548</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>306</v>
       </c>
       <c r="F10" t="n">
-        <v>100</v>
+        <v>64.55696202531645</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Doradobet Honduras</t>
+          <t>Doradobet Guatemala</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>11</v>
+        <v>92</v>
       </c>
       <c r="C11" t="n">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="D11" t="n">
-        <v>100</v>
+        <v>41.30434782608695</v>
       </c>
       <c r="E11" t="n">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="F11" t="n">
-        <v>100</v>
+        <v>52.17391304347826</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Doradobet Perú</t>
+          <t>Doradobet Honduras</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>426</v>
+        <v>182</v>
       </c>
       <c r="C12" t="n">
-        <v>426</v>
+        <v>102</v>
       </c>
       <c r="D12" t="n">
-        <v>100</v>
+        <v>56.04395604395604</v>
       </c>
       <c r="E12" t="n">
-        <v>426</v>
+        <v>114</v>
       </c>
       <c r="F12" t="n">
-        <v>100</v>
+        <v>62.63736263736264</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ecuabet Ecuador</t>
+          <t>Doradobet Perú</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1146</v>
+        <v>3441</v>
       </c>
       <c r="C13" t="n">
-        <v>714</v>
+        <v>2665</v>
       </c>
       <c r="D13" t="n">
-        <v>62.30366492146597</v>
+        <v>77.44841615809358</v>
       </c>
       <c r="E13" t="n">
-        <v>900</v>
+        <v>2779</v>
       </c>
       <c r="F13" t="n">
-        <v>78.53403141361257</v>
+        <v>80.76140656785819</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GanaPlay El Salvador</t>
+          <t>Ecuabet Ecuador</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>33</v>
+        <v>8108</v>
       </c>
       <c r="C14" t="n">
-        <v>23</v>
+        <v>5213</v>
       </c>
       <c r="D14" t="n">
-        <v>69.6969696969697</v>
+        <v>64.29452392698569</v>
       </c>
       <c r="E14" t="n">
-        <v>26</v>
+        <v>6420</v>
       </c>
       <c r="F14" t="n">
-        <v>78.78787878787878</v>
+        <v>79.18105574740997</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GanaPlay Guatemala</t>
+          <t>GanaPlay El Salvador</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11</v>
+        <v>2024</v>
       </c>
       <c r="C15" t="n">
-        <v>9</v>
+        <v>918</v>
       </c>
       <c r="D15" t="n">
-        <v>81.81818181818183</v>
+        <v>45.35573122529645</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>1321</v>
       </c>
       <c r="F15" t="n">
-        <v>90.90909090909091</v>
+        <v>65.26679841897233</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>GanaPlay Guatemala</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>59</v>
+      </c>
+      <c r="C16" t="n">
+        <v>42</v>
+      </c>
+      <c r="D16" t="n">
+        <v>71.1864406779661</v>
+      </c>
+      <c r="E16" t="n">
+        <v>49</v>
+      </c>
+      <c r="F16" t="n">
+        <v>83.05084745762711</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Paniplay Honduras</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>11</v>
-      </c>
-      <c r="C16" t="n">
-        <v>11</v>
-      </c>
-      <c r="D16" t="n">
-        <v>100</v>
-      </c>
-      <c r="E16" t="n">
-        <v>11</v>
-      </c>
-      <c r="F16" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="17"/>
+      <c r="B17" t="n">
+        <v>423</v>
+      </c>
+      <c r="C17" t="n">
+        <v>289</v>
+      </c>
+      <c r="D17" t="n">
+        <v>68.32151300236407</v>
+      </c>
+      <c r="E17" t="n">
+        <v>316</v>
+      </c>
+      <c r="F17" t="n">
+        <v>74.70449172576832</v>
+      </c>
+    </row>
     <row r="18"/>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5497,43 +5518,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>21</v>
+        <v>158</v>
       </c>
       <c r="D22" t="n">
-        <v>2.219047619047619</v>
+        <v>2.39831223628692</v>
       </c>
       <c r="E22" t="n">
         <v>2.533333333333333</v>
       </c>
       <c r="F22" t="n">
-        <v>0.03698412698412699</v>
+        <v>0.03997187060478201</v>
       </c>
       <c r="G22" t="n">
         <v>0.04222222222222222</v>
       </c>
       <c r="H22" t="n">
-        <v>233.5882352941176</v>
+        <v>239.4075342465754</v>
       </c>
       <c r="I22" t="n">
-        <v>197.1</v>
+        <v>108.7666666666667</v>
       </c>
       <c r="J22" t="n">
-        <v>3.89313725490196</v>
+        <v>3.990125570776256</v>
       </c>
       <c r="K22" t="n">
-        <v>3.285</v>
+        <v>1.812777777777778</v>
       </c>
       <c r="L22" t="n">
-        <v>230.9813725490196</v>
+        <v>236.8277397260274</v>
       </c>
       <c r="M22" t="n">
-        <v>194.2833333333333</v>
+        <v>105.9583333333333</v>
       </c>
       <c r="N22" t="n">
-        <v>3.849689542483659</v>
+        <v>3.947128995433789</v>
       </c>
       <c r="O22" t="n">
-        <v>3.238055555555555</v>
+        <v>1.765972222222222</v>
       </c>
     </row>
     <row r="23">
@@ -5548,43 +5569,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>31</v>
+        <v>297</v>
       </c>
       <c r="D23" t="n">
-        <v>523.8118279569892</v>
+        <v>258.8453423120091</v>
       </c>
       <c r="E23" t="n">
-        <v>569.1833333333333</v>
+        <v>75.13333333333334</v>
       </c>
       <c r="F23" t="n">
-        <v>8.730197132616485</v>
+        <v>4.314089038533483</v>
       </c>
       <c r="G23" t="n">
-        <v>9.486388888888888</v>
+        <v>1.252222222222222</v>
       </c>
       <c r="H23" t="n">
-        <v>541.3677419354838</v>
+        <v>286.4700458190149</v>
       </c>
       <c r="I23" t="n">
-        <v>587.9</v>
+        <v>109.8166666666667</v>
       </c>
       <c r="J23" t="n">
-        <v>9.022795698924732</v>
+        <v>4.774500763650248</v>
       </c>
       <c r="K23" t="n">
-        <v>9.798333333333334</v>
+        <v>1.830277777777778</v>
       </c>
       <c r="L23" t="n">
-        <v>17.55591397849462</v>
+        <v>23.07605956471936</v>
       </c>
       <c r="M23" t="n">
-        <v>17.91666666666667</v>
+        <v>7.516666666666667</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2925985663082437</v>
+        <v>0.3846009927453226</v>
       </c>
       <c r="O23" t="n">
-        <v>0.2986111111111111</v>
+        <v>0.1252777777777778</v>
       </c>
     </row>
     <row r="24">
@@ -5599,43 +5620,43 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="D24" t="n">
-        <v>2.75</v>
+        <v>2.34320987654321</v>
       </c>
       <c r="E24" t="n">
-        <v>2.666666666666667</v>
+        <v>2.633333333333333</v>
       </c>
       <c r="F24" t="n">
-        <v>0.04583333333333334</v>
+        <v>0.03905349794238683</v>
       </c>
       <c r="G24" t="n">
-        <v>0.04444444444444444</v>
+        <v>0.04388888888888889</v>
       </c>
       <c r="H24" t="n">
-        <v>12.16666666666667</v>
+        <v>41.13205128205129</v>
       </c>
       <c r="I24" t="n">
-        <v>12.16666666666667</v>
+        <v>11.1</v>
       </c>
       <c r="J24" t="n">
-        <v>0.2027777777777778</v>
+        <v>0.685534188034188</v>
       </c>
       <c r="K24" t="n">
-        <v>0.2027777777777778</v>
+        <v>0.185</v>
       </c>
       <c r="L24" t="n">
-        <v>9.5</v>
+        <v>38.42179487179487</v>
       </c>
       <c r="M24" t="n">
-        <v>9.5</v>
+        <v>8.566666666666666</v>
       </c>
       <c r="N24" t="n">
-        <v>0.1583333333333333</v>
+        <v>0.6403632478632478</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1583333333333333</v>
+        <v>0.1427777777777778</v>
       </c>
     </row>
     <row r="25">
@@ -5650,49 +5671,49 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="D25" t="n">
-        <v>104.3333333333333</v>
+        <v>300.6</v>
       </c>
       <c r="E25" t="n">
-        <v>18.98333333333333</v>
+        <v>38.91666666666667</v>
       </c>
       <c r="F25" t="n">
-        <v>1.738888888888889</v>
+        <v>5.01</v>
       </c>
       <c r="G25" t="n">
-        <v>0.3163888888888889</v>
+        <v>0.6486111111111111</v>
       </c>
       <c r="H25" t="n">
-        <v>106.6944444444444</v>
+        <v>302.5733333333333</v>
       </c>
       <c r="I25" t="n">
-        <v>22.51666666666667</v>
+        <v>44.65</v>
       </c>
       <c r="J25" t="n">
-        <v>1.778240740740741</v>
+        <v>5.042888888888888</v>
       </c>
       <c r="K25" t="n">
-        <v>0.3752777777777778</v>
+        <v>0.7441666666666666</v>
       </c>
       <c r="L25" t="n">
-        <v>2.361111111111111</v>
+        <v>1.973333333333333</v>
       </c>
       <c r="M25" t="n">
-        <v>1.916666666666667</v>
+        <v>1.541666666666667</v>
       </c>
       <c r="N25" t="n">
-        <v>0.03935185185185185</v>
+        <v>0.03288888888888889</v>
       </c>
       <c r="O25" t="n">
-        <v>0.03194444444444445</v>
+        <v>0.02569444444444444</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Doradobet Chile</t>
+          <t>Doradobet Bolivia</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5701,7 +5722,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -5719,7 +5740,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Doradobet Chile</t>
+          <t>Doradobet Bolivia</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5734,7 +5755,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Doradobet Costa Rica</t>
+          <t>Doradobet Chile</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5743,25 +5764,49 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>5</v>
+        <v>57</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>419.6833333333333</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>2.983333333333333</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>6.994722222222222</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>0.04972222222222222</v>
+      </c>
+      <c r="H28" t="n">
+        <v>708.9813492063493</v>
+      </c>
+      <c r="I28" t="n">
+        <v>830.6916666666666</v>
+      </c>
+      <c r="J28" t="n">
+        <v>11.81635582010582</v>
+      </c>
+      <c r="K28" t="n">
+        <v>13.84486111111111</v>
+      </c>
+      <c r="L28" t="n">
+        <v>139.4111111111111</v>
+      </c>
+      <c r="M28" t="n">
+        <v>6.208333333333334</v>
+      </c>
+      <c r="N28" t="n">
+        <v>2.323518518518518</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.1034722222222222</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Doradobet Costa Rica</t>
+          <t>Doradobet Chile</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5770,13 +5815,49 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>37</v>
+      </c>
+      <c r="D29" t="n">
+        <v>647.3923423423422</v>
+      </c>
+      <c r="E29" t="n">
+        <v>639.55</v>
+      </c>
+      <c r="F29" t="n">
+        <v>10.78987237237237</v>
+      </c>
+      <c r="G29" t="n">
+        <v>10.65916666666667</v>
+      </c>
+      <c r="H29" t="n">
+        <v>715.714864864865</v>
+      </c>
+      <c r="I29" t="n">
+        <v>859.2333333333333</v>
+      </c>
+      <c r="J29" t="n">
+        <v>11.92858108108108</v>
+      </c>
+      <c r="K29" t="n">
+        <v>14.32055555555556</v>
+      </c>
+      <c r="L29" t="n">
+        <v>68.32252252252252</v>
+      </c>
+      <c r="M29" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="N29" t="n">
+        <v>1.138708708708709</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.1033333333333333</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Doradobet Ecuador</t>
+          <t>Doradobet Costa Rica</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5785,49 +5866,49 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>94</v>
+        <v>508</v>
       </c>
       <c r="D30" t="n">
-        <v>2.312056737588652</v>
+        <v>2.259383202099737</v>
       </c>
       <c r="E30" t="n">
-        <v>2.566666666666667</v>
+        <v>2.575</v>
       </c>
       <c r="F30" t="n">
-        <v>0.03853427895981087</v>
+        <v>0.03765638670166229</v>
       </c>
       <c r="G30" t="n">
-        <v>0.04277777777777778</v>
+        <v>0.04291666666666667</v>
       </c>
       <c r="H30" t="n">
-        <v>191.0424242424242</v>
+        <v>196.9045232273839</v>
       </c>
       <c r="I30" t="n">
-        <v>94.90833333333333</v>
+        <v>88.36666666666666</v>
       </c>
       <c r="J30" t="n">
-        <v>3.184040404040404</v>
+        <v>3.281742053789731</v>
       </c>
       <c r="K30" t="n">
-        <v>1.581805555555555</v>
+        <v>1.472777777777778</v>
       </c>
       <c r="L30" t="n">
-        <v>188.4560606060606</v>
+        <v>194.2876935615322</v>
       </c>
       <c r="M30" t="n">
-        <v>92.58333333333334</v>
+        <v>85.38333333333334</v>
       </c>
       <c r="N30" t="n">
-        <v>3.140934343434343</v>
+        <v>3.238128226025536</v>
       </c>
       <c r="O30" t="n">
-        <v>1.543055555555556</v>
+        <v>1.423055555555556</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Doradobet Ecuador</t>
+          <t>Doradobet Costa Rica</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5836,49 +5917,49 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>35</v>
+        <v>875</v>
       </c>
       <c r="D31" t="n">
-        <v>440.2809523809523</v>
+        <v>3176.798457142856</v>
       </c>
       <c r="E31" t="n">
-        <v>590.3666666666667</v>
+        <v>2856.35</v>
       </c>
       <c r="F31" t="n">
-        <v>7.338015873015872</v>
+        <v>52.94664095238095</v>
       </c>
       <c r="G31" t="n">
-        <v>9.839444444444444</v>
+        <v>47.60583333333333</v>
       </c>
       <c r="H31" t="n">
-        <v>475.2119047619048</v>
+        <v>3535.979122182681</v>
       </c>
       <c r="I31" t="n">
-        <v>609.0333333333333</v>
+        <v>3212.583333333333</v>
       </c>
       <c r="J31" t="n">
-        <v>7.920198412698412</v>
+        <v>58.93298536971135</v>
       </c>
       <c r="K31" t="n">
-        <v>10.15055555555555</v>
+        <v>53.54305555555556</v>
       </c>
       <c r="L31" t="n">
-        <v>14.27380952380952</v>
+        <v>352.7267497034401</v>
       </c>
       <c r="M31" t="n">
-        <v>14.06666666666667</v>
+        <v>352.5833333333333</v>
       </c>
       <c r="N31" t="n">
-        <v>0.2378968253968254</v>
+        <v>5.878779161724001</v>
       </c>
       <c r="O31" t="n">
-        <v>0.2344444444444444</v>
+        <v>5.876388888888888</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Doradobet El Salvador</t>
+          <t>Doradobet Ecuador</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5887,25 +5968,49 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>197</v>
+        <v>866</v>
       </c>
       <c r="D32" t="n">
-        <v>831.5466159052452</v>
+        <v>258.2367975365666</v>
       </c>
       <c r="E32" t="n">
-        <v>901.7833333333333</v>
+        <v>2.741666666666667</v>
       </c>
       <c r="F32" t="n">
-        <v>13.85911026508743</v>
+        <v>4.303946625609443</v>
       </c>
       <c r="G32" t="n">
-        <v>15.02972222222222</v>
+        <v>0.04569444444444444</v>
+      </c>
+      <c r="H32" t="n">
+        <v>528.9238178633975</v>
+      </c>
+      <c r="I32" t="n">
+        <v>320.8166666666667</v>
+      </c>
+      <c r="J32" t="n">
+        <v>8.815396964389958</v>
+      </c>
+      <c r="K32" t="n">
+        <v>5.346944444444444</v>
+      </c>
+      <c r="L32" t="n">
+        <v>140.332545242265</v>
+      </c>
+      <c r="M32" t="n">
+        <v>36.43333333333333</v>
+      </c>
+      <c r="N32" t="n">
+        <v>2.338875754037751</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.6072222222222222</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Doradobet El Salvador</t>
+          <t>Doradobet Ecuador</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5914,25 +6019,49 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>162</v>
+        <v>614</v>
       </c>
       <c r="D33" t="n">
-        <v>1132.975205761317</v>
+        <v>425.0889522258415</v>
       </c>
       <c r="E33" t="n">
-        <v>1010.158333333333</v>
+        <v>147.925</v>
       </c>
       <c r="F33" t="n">
-        <v>18.88292009602195</v>
+        <v>7.084815870430692</v>
       </c>
       <c r="G33" t="n">
-        <v>16.83597222222222</v>
+        <v>2.465416666666667</v>
+      </c>
+      <c r="H33" t="n">
+        <v>601.8411388355726</v>
+      </c>
+      <c r="I33" t="n">
+        <v>485.8166666666667</v>
+      </c>
+      <c r="J33" t="n">
+        <v>10.03068564725954</v>
+      </c>
+      <c r="K33" t="n">
+        <v>8.096944444444444</v>
+      </c>
+      <c r="L33" t="n">
+        <v>130.2832373640435</v>
+      </c>
+      <c r="M33" t="n">
+        <v>36.46666666666667</v>
+      </c>
+      <c r="N33" t="n">
+        <v>2.171387289400725</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.6077777777777779</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Doradobet Guatemala</t>
+          <t>Doradobet El Salvador</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5941,25 +6070,49 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>5</v>
+        <v>260</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>792.2355128205128</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>834.2333333333333</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>13.20392521367521</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>13.90388888888889</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1402.207042253521</v>
+      </c>
+      <c r="I34" t="n">
+        <v>1463.283333333333</v>
+      </c>
+      <c r="J34" t="n">
+        <v>23.37011737089202</v>
+      </c>
+      <c r="K34" t="n">
+        <v>24.38805555555556</v>
+      </c>
+      <c r="L34" t="n">
+        <v>565.0092331768387</v>
+      </c>
+      <c r="M34" t="n">
+        <v>563.75</v>
+      </c>
+      <c r="N34" t="n">
+        <v>9.416820552947312</v>
+      </c>
+      <c r="O34" t="n">
+        <v>9.395833333333334</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Doradobet Guatemala</t>
+          <t>Doradobet El Salvador</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5968,13 +6121,49 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>214</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1115.859501557632</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1001.583333333333</v>
+      </c>
+      <c r="F35" t="n">
+        <v>18.59765835929387</v>
+      </c>
+      <c r="G35" t="n">
+        <v>16.69305555555556</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1683.434638554217</v>
+      </c>
+      <c r="I35" t="n">
+        <v>1569.491666666667</v>
+      </c>
+      <c r="J35" t="n">
+        <v>28.05724397590361</v>
+      </c>
+      <c r="K35" t="n">
+        <v>26.15819444444445</v>
+      </c>
+      <c r="L35" t="n">
+        <v>564.335642570281</v>
+      </c>
+      <c r="M35" t="n">
+        <v>563.75</v>
+      </c>
+      <c r="N35" t="n">
+        <v>9.405594042838018</v>
+      </c>
+      <c r="O35" t="n">
+        <v>9.395833333333334</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Doradobet Honduras</t>
+          <t>Doradobet Guatemala</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5983,49 +6172,49 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="D36" t="n">
-        <v>1.428787878787879</v>
+        <v>0.637719298245614</v>
       </c>
       <c r="E36" t="n">
-        <v>2.416666666666667</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0.02381313131313131</v>
+        <v>0.01062865497076023</v>
       </c>
       <c r="G36" t="n">
-        <v>0.04027777777777777</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>447.4133333333333</v>
+        <v>159.0738095238095</v>
       </c>
       <c r="I36" t="n">
-        <v>482.45</v>
+        <v>142.7</v>
       </c>
       <c r="J36" t="n">
-        <v>7.456888888888889</v>
+        <v>2.651230158730158</v>
       </c>
       <c r="K36" t="n">
-        <v>8.040833333333333</v>
+        <v>2.378333333333333</v>
       </c>
       <c r="L36" t="n">
-        <v>444.7566666666667</v>
+        <v>156.4452380952381</v>
       </c>
       <c r="M36" t="n">
-        <v>480.0166666666667</v>
+        <v>140.4</v>
       </c>
       <c r="N36" t="n">
-        <v>7.41261111111111</v>
+        <v>2.607420634920635</v>
       </c>
       <c r="O36" t="n">
-        <v>8.000277777777777</v>
+        <v>2.34</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Doradobet Honduras</t>
+          <t>Doradobet Guatemala</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6034,13 +6223,49 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>54</v>
+      </c>
+      <c r="D37" t="n">
+        <v>5610.661419753086</v>
+      </c>
+      <c r="E37" t="n">
+        <v>6823.466666666667</v>
+      </c>
+      <c r="F37" t="n">
+        <v>93.51102366255145</v>
+      </c>
+      <c r="G37" t="n">
+        <v>113.7244444444444</v>
+      </c>
+      <c r="H37" t="n">
+        <v>6468.867006802721</v>
+      </c>
+      <c r="I37" t="n">
+        <v>7226.016666666666</v>
+      </c>
+      <c r="J37" t="n">
+        <v>107.8144501133787</v>
+      </c>
+      <c r="K37" t="n">
+        <v>120.4336111111111</v>
+      </c>
+      <c r="L37" t="n">
+        <v>296.5472789115645</v>
+      </c>
+      <c r="M37" t="n">
+        <v>330.9</v>
+      </c>
+      <c r="N37" t="n">
+        <v>4.942454648526077</v>
+      </c>
+      <c r="O37" t="n">
+        <v>5.515</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Doradobet Perú</t>
+          <t>Doradobet Honduras</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6049,49 +6274,49 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>426</v>
+        <v>102</v>
       </c>
       <c r="D38" t="n">
-        <v>2.266079812206573</v>
+        <v>1.801797385620915</v>
       </c>
       <c r="E38" t="n">
-        <v>2.483333333333333</v>
+        <v>2.408333333333333</v>
       </c>
       <c r="F38" t="n">
-        <v>0.03776799687010955</v>
+        <v>0.03002995642701525</v>
       </c>
       <c r="G38" t="n">
-        <v>0.04138888888888889</v>
+        <v>0.04013888888888889</v>
       </c>
       <c r="H38" t="n">
-        <v>3.321235721703011</v>
+        <v>374.6587962962963</v>
       </c>
       <c r="I38" t="n">
-        <v>2.766666666666667</v>
+        <v>356.5916666666667</v>
       </c>
       <c r="J38" t="n">
-        <v>0.05535392869505019</v>
+        <v>6.244313271604939</v>
       </c>
       <c r="K38" t="n">
-        <v>0.04611111111111111</v>
+        <v>5.943194444444445</v>
       </c>
       <c r="L38" t="n">
-        <v>0.7954309449636552</v>
+        <v>372.2446759259259</v>
       </c>
       <c r="M38" t="n">
-        <v>0.2333333333333333</v>
+        <v>353.9666666666667</v>
       </c>
       <c r="N38" t="n">
-        <v>0.01325718241606092</v>
+        <v>6.204077932098766</v>
       </c>
       <c r="O38" t="n">
-        <v>0.003888888888888889</v>
+        <v>5.899444444444445</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Doradobet Perú</t>
+          <t>Doradobet Honduras</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6100,13 +6325,49 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>80</v>
+      </c>
+      <c r="D39" t="n">
+        <v>201.6135416666667</v>
+      </c>
+      <c r="E39" t="n">
+        <v>52.88333333333333</v>
+      </c>
+      <c r="F39" t="n">
+        <v>3.360225694444444</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.8813888888888889</v>
+      </c>
+      <c r="H39" t="n">
+        <v>600.9472222222222</v>
+      </c>
+      <c r="I39" t="n">
+        <v>531.85</v>
+      </c>
+      <c r="J39" t="n">
+        <v>10.01578703703704</v>
+      </c>
+      <c r="K39" t="n">
+        <v>8.864166666666668</v>
+      </c>
+      <c r="L39" t="n">
+        <v>396.2326923076923</v>
+      </c>
+      <c r="M39" t="n">
+        <v>469.525</v>
+      </c>
+      <c r="N39" t="n">
+        <v>6.603878205128205</v>
+      </c>
+      <c r="O39" t="n">
+        <v>7.825416666666667</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ecuabet Ecuador</t>
+          <t>Doradobet Perú</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6115,49 +6376,49 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>714</v>
+        <v>2665</v>
       </c>
       <c r="D40" t="n">
-        <v>2.457446311858077</v>
+        <v>25.32980612883052</v>
       </c>
       <c r="E40" t="n">
-        <v>2.566666666666667</v>
+        <v>2.55</v>
       </c>
       <c r="F40" t="n">
-        <v>0.04095743853096794</v>
+        <v>0.4221634354805087</v>
       </c>
       <c r="G40" t="n">
-        <v>0.04277777777777778</v>
+        <v>0.0425</v>
       </c>
       <c r="H40" t="n">
-        <v>199.8486625514403</v>
+        <v>40.81043697205978</v>
       </c>
       <c r="I40" t="n">
-        <v>131.8916666666667</v>
+        <v>2.866666666666667</v>
       </c>
       <c r="J40" t="n">
-        <v>3.330811042524005</v>
+        <v>0.6801739495343296</v>
       </c>
       <c r="K40" t="n">
-        <v>2.198194444444445</v>
+        <v>0.04777777777777778</v>
       </c>
       <c r="L40" t="n">
-        <v>197.2991769547325</v>
+        <v>8.767357050032489</v>
       </c>
       <c r="M40" t="n">
-        <v>129.275</v>
+        <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>3.288319615912209</v>
+        <v>0.1461226175005415</v>
       </c>
       <c r="O40" t="n">
-        <v>2.154583333333333</v>
+        <v>0.003888888888888889</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Ecuabet Ecuador</t>
+          <t>Doradobet Perú</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6166,49 +6427,49 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>432</v>
+        <v>776</v>
       </c>
       <c r="D41" t="n">
-        <v>428.4212191358025</v>
+        <v>593.5414518900344</v>
       </c>
       <c r="E41" t="n">
-        <v>504.85</v>
+        <v>667.2</v>
       </c>
       <c r="F41" t="n">
-        <v>7.140353652263375</v>
+        <v>9.892357531500574</v>
       </c>
       <c r="G41" t="n">
-        <v>8.414166666666667</v>
+        <v>11.12</v>
       </c>
       <c r="H41" t="n">
-        <v>460.1957471264367</v>
+        <v>664.4059082892416</v>
       </c>
       <c r="I41" t="n">
-        <v>523.5833333333334</v>
+        <v>712.5916666666667</v>
       </c>
       <c r="J41" t="n">
-        <v>7.669929118773946</v>
+        <v>11.07343180482069</v>
       </c>
       <c r="K41" t="n">
-        <v>8.72638888888889</v>
+        <v>11.87652777777778</v>
       </c>
       <c r="L41" t="n">
-        <v>39.33126436781609</v>
+        <v>69.37429453262786</v>
       </c>
       <c r="M41" t="n">
-        <v>40</v>
+        <v>54.60833333333333</v>
       </c>
       <c r="N41" t="n">
-        <v>0.6555210727969348</v>
+        <v>1.156238242210464</v>
       </c>
       <c r="O41" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.9101388888888888</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GanaPlay El Salvador</t>
+          <t>Ecuabet Ecuador</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6217,25 +6478,49 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>23</v>
+        <v>5213</v>
       </c>
       <c r="D42" t="n">
-        <v>0.108695652173913</v>
+        <v>2.504706183259799</v>
       </c>
       <c r="E42" t="n">
-        <v>0</v>
+        <v>2.616666666666667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.001811594202898551</v>
+        <v>0.04174510305432998</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>0.04361111111111111</v>
+      </c>
+      <c r="H42" t="n">
+        <v>202.9883456334564</v>
+      </c>
+      <c r="I42" t="n">
+        <v>127.1083333333333</v>
+      </c>
+      <c r="J42" t="n">
+        <v>3.383139093890939</v>
+      </c>
+      <c r="K42" t="n">
+        <v>2.118472222222223</v>
+      </c>
+      <c r="L42" t="n">
+        <v>200.3730671235284</v>
+      </c>
+      <c r="M42" t="n">
+        <v>124.425</v>
+      </c>
+      <c r="N42" t="n">
+        <v>3.339551118725473</v>
+      </c>
+      <c r="O42" t="n">
+        <v>2.07375</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>GanaPlay El Salvador</t>
+          <t>Ecuabet Ecuador</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -6244,49 +6529,49 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>10</v>
+        <v>2895</v>
       </c>
       <c r="D43" t="n">
-        <v>442.6216666666666</v>
+        <v>206.4872654001151</v>
       </c>
       <c r="E43" t="n">
-        <v>496.6833333333334</v>
+        <v>102.6</v>
       </c>
       <c r="F43" t="n">
-        <v>7.377027777777778</v>
+        <v>3.441454423335253</v>
       </c>
       <c r="G43" t="n">
-        <v>8.278055555555556</v>
+        <v>1.71</v>
       </c>
       <c r="H43" t="n">
-        <v>563.5722222222222</v>
+        <v>327.6762283640425</v>
       </c>
       <c r="I43" t="n">
-        <v>824.75</v>
+        <v>211.8583333333333</v>
       </c>
       <c r="J43" t="n">
-        <v>9.392870370370369</v>
+        <v>5.461270472734041</v>
       </c>
       <c r="K43" t="n">
-        <v>13.74583333333333</v>
+        <v>3.530972222222222</v>
       </c>
       <c r="L43" t="n">
-        <v>7.594444444444444</v>
+        <v>137.781365159129</v>
       </c>
       <c r="M43" t="n">
-        <v>9.583333333333334</v>
+        <v>86.02500000000001</v>
       </c>
       <c r="N43" t="n">
-        <v>0.1265740740740741</v>
+        <v>2.296356085985483</v>
       </c>
       <c r="O43" t="n">
-        <v>0.1597222222222222</v>
+        <v>1.43375</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GanaPlay Guatemala</t>
+          <t>GanaPlay El Salvador</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -6295,25 +6580,49 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>9</v>
+        <v>918</v>
       </c>
       <c r="D44" t="n">
-        <v>0.2518518518518518</v>
+        <v>2.180319535221496</v>
       </c>
       <c r="E44" t="n">
-        <v>0</v>
+        <v>2.516666666666667</v>
       </c>
       <c r="F44" t="n">
-        <v>0.004197530864197531</v>
+        <v>0.03633865892035826</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>0.04194444444444444</v>
+      </c>
+      <c r="H44" t="n">
+        <v>571.8012582781456</v>
+      </c>
+      <c r="I44" t="n">
+        <v>538.9</v>
+      </c>
+      <c r="J44" t="n">
+        <v>9.530020971302429</v>
+      </c>
+      <c r="K44" t="n">
+        <v>8.981666666666666</v>
+      </c>
+      <c r="L44" t="n">
+        <v>569.202825607064</v>
+      </c>
+      <c r="M44" t="n">
+        <v>535.9</v>
+      </c>
+      <c r="N44" t="n">
+        <v>9.486713760117734</v>
+      </c>
+      <c r="O44" t="n">
+        <v>8.931666666666667</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GanaPlay Guatemala</t>
+          <t>GanaPlay El Salvador</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -6322,25 +6631,49 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>1106</v>
       </c>
       <c r="D45" t="n">
-        <v>54.15833333333333</v>
+        <v>335.2304098854732</v>
       </c>
       <c r="E45" t="n">
-        <v>54.15833333333333</v>
+        <v>205.1333333333333</v>
       </c>
       <c r="F45" t="n">
-        <v>0.9026388888888889</v>
+        <v>5.58717349809122</v>
       </c>
       <c r="G45" t="n">
-        <v>0.9026388888888889</v>
+        <v>3.418888888888889</v>
+      </c>
+      <c r="H45" t="n">
+        <v>891.7515023474178</v>
+      </c>
+      <c r="I45" t="n">
+        <v>781.2166666666667</v>
+      </c>
+      <c r="J45" t="n">
+        <v>14.86252503912363</v>
+      </c>
+      <c r="K45" t="n">
+        <v>13.02027777777778</v>
+      </c>
+      <c r="L45" t="n">
+        <v>560.297323943662</v>
+      </c>
+      <c r="M45" t="n">
+        <v>607.5333333333333</v>
+      </c>
+      <c r="N45" t="n">
+        <v>9.338288732394366</v>
+      </c>
+      <c r="O45" t="n">
+        <v>10.12555555555556</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Paniplay Honduras</t>
+          <t>GanaPlay Guatemala</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -6349,58 +6682,196 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>11</v>
+        <v>42</v>
       </c>
       <c r="D46" t="n">
-        <v>0.9924242424242423</v>
+        <v>0.7186507936507938</v>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>0.01654040404040404</v>
+        <v>0.01197751322751323</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>258.0375</v>
+        <v>43.25</v>
       </c>
       <c r="I46" t="n">
-        <v>252.8166666666667</v>
+        <v>29.85833333333333</v>
       </c>
       <c r="J46" t="n">
-        <v>4.300625</v>
+        <v>0.7208333333333333</v>
       </c>
       <c r="K46" t="n">
-        <v>4.213611111111112</v>
+        <v>0.4976388888888889</v>
       </c>
       <c r="L46" t="n">
-        <v>255.3083333333333</v>
+        <v>40.6875</v>
       </c>
       <c r="M46" t="n">
-        <v>250.2166666666667</v>
+        <v>27.38333333333333</v>
       </c>
       <c r="N46" t="n">
-        <v>4.255138888888889</v>
+        <v>0.678125</v>
       </c>
       <c r="O46" t="n">
-        <v>4.170277777777778</v>
+        <v>0.4563888888888888</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>GanaPlay Guatemala</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>17</v>
+      </c>
+      <c r="D47" t="n">
+        <v>145.7098039215686</v>
+      </c>
+      <c r="E47" t="n">
+        <v>28.53333333333333</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2.428496732026144</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.4755555555555556</v>
+      </c>
+      <c r="H47" t="n">
+        <v>237.4409090909091</v>
+      </c>
+      <c r="I47" t="n">
+        <v>146.15</v>
+      </c>
+      <c r="J47" t="n">
+        <v>3.957348484848485</v>
+      </c>
+      <c r="K47" t="n">
+        <v>2.435833333333334</v>
+      </c>
+      <c r="L47" t="n">
+        <v>125.7</v>
+      </c>
+      <c r="M47" t="n">
+        <v>128.7833333333333</v>
+      </c>
+      <c r="N47" t="n">
+        <v>2.095</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.146388888888889</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>Paniplay Honduras</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Automatico</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>289</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2.315051903114187</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2.533333333333333</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.03858419838523645</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.04222222222222222</v>
+      </c>
+      <c r="H48" t="n">
+        <v>398.7149019607843</v>
+      </c>
+      <c r="I48" t="n">
+        <v>359.4333333333333</v>
+      </c>
+      <c r="J48" t="n">
+        <v>6.645248366013072</v>
+      </c>
+      <c r="K48" t="n">
+        <v>5.990555555555556</v>
+      </c>
+      <c r="L48" t="n">
+        <v>396.1299346405229</v>
+      </c>
+      <c r="M48" t="n">
+        <v>356.5</v>
+      </c>
+      <c r="N48" t="n">
+        <v>6.602165577342048</v>
+      </c>
+      <c r="O48" t="n">
+        <v>5.941666666666666</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Paniplay Honduras</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>Manual</t>
         </is>
       </c>
-      <c r="C47" t="n">
-        <v>0</v>
+      <c r="C49" t="n">
+        <v>134</v>
+      </c>
+      <c r="D49" t="n">
+        <v>177.9324626865672</v>
+      </c>
+      <c r="E49" t="n">
+        <v>70.04166666666667</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2.965541044776119</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.167361111111111</v>
+      </c>
+      <c r="H49" t="n">
+        <v>496.6455128205127</v>
+      </c>
+      <c r="I49" t="n">
+        <v>419.325</v>
+      </c>
+      <c r="J49" t="n">
+        <v>8.277425213675215</v>
+      </c>
+      <c r="K49" t="n">
+        <v>6.98875</v>
+      </c>
+      <c r="L49" t="n">
+        <v>320.381282051282</v>
+      </c>
+      <c r="M49" t="n">
+        <v>316.825</v>
+      </c>
+      <c r="N49" t="n">
+        <v>5.339688034188034</v>
+      </c>
+      <c r="O49" t="n">
+        <v>5.280416666666667</v>
       </c>
     </row>
   </sheetData>
@@ -6490,19 +6961,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9832</v>
+        <v>9849</v>
       </c>
       <c r="C4" t="n">
-        <v>2514</v>
+        <v>2531</v>
       </c>
       <c r="D4" t="n">
-        <v>25.56956875508544</v>
+        <v>25.69804041019393</v>
       </c>
       <c r="E4" t="n">
-        <v>7040</v>
+        <v>7057</v>
       </c>
       <c r="F4" t="n">
-        <v>71.60292921074044</v>
+        <v>71.65194435983349</v>
       </c>
     </row>
     <row r="5">
@@ -6534,19 +7005,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>373</v>
+        <v>457</v>
       </c>
       <c r="C6" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D6" t="n">
-        <v>23.32439678284182</v>
+        <v>19.47483588621444</v>
       </c>
       <c r="E6" t="n">
-        <v>244</v>
+        <v>290</v>
       </c>
       <c r="F6" t="n">
-        <v>65.41554959785523</v>
+        <v>63.45733041575492</v>
       </c>
     </row>
     <row r="7">
@@ -6556,19 +7027,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1950</v>
+        <v>1988</v>
       </c>
       <c r="C7" t="n">
-        <v>1081</v>
+        <v>1108</v>
       </c>
       <c r="D7" t="n">
-        <v>55.43589743589744</v>
+        <v>55.73440643863179</v>
       </c>
       <c r="E7" t="n">
-        <v>1212</v>
+        <v>1240</v>
       </c>
       <c r="F7" t="n">
-        <v>62.15384615384615</v>
+        <v>62.37424547283702</v>
       </c>
     </row>
     <row r="8">
@@ -6578,19 +7049,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19755</v>
+        <v>19863</v>
       </c>
       <c r="C8" t="n">
-        <v>15597</v>
+        <v>15705</v>
       </c>
       <c r="D8" t="n">
-        <v>78.95216400911161</v>
+        <v>79.06660625283189</v>
       </c>
       <c r="E8" t="n">
-        <v>16288</v>
+        <v>16396</v>
       </c>
       <c r="F8" t="n">
-        <v>82.45001265502404</v>
+        <v>82.54543623823189</v>
       </c>
     </row>
     <row r="9">
@@ -6600,19 +7071,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24881</v>
+        <v>24906</v>
       </c>
       <c r="C9" t="n">
-        <v>11071</v>
+        <v>11083</v>
       </c>
       <c r="D9" t="n">
-        <v>44.49580000803826</v>
+        <v>44.49931743355015</v>
       </c>
       <c r="E9" t="n">
-        <v>16014</v>
+        <v>16034</v>
       </c>
       <c r="F9" t="n">
-        <v>64.36236485671797</v>
+        <v>64.37806151128243</v>
       </c>
     </row>
     <row r="10">
@@ -6622,19 +7093,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7676</v>
+        <v>7735</v>
       </c>
       <c r="C10" t="n">
-        <v>3789</v>
+        <v>3822</v>
       </c>
       <c r="D10" t="n">
-        <v>49.36164669098489</v>
+        <v>49.41176470588236</v>
       </c>
       <c r="E10" t="n">
-        <v>4854</v>
+        <v>4892</v>
       </c>
       <c r="F10" t="n">
-        <v>63.23606044815008</v>
+        <v>63.24499030381383</v>
       </c>
     </row>
     <row r="11">
@@ -6644,19 +7115,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2559</v>
+        <v>2668</v>
       </c>
       <c r="C11" t="n">
-        <v>1779</v>
+        <v>1888</v>
       </c>
       <c r="D11" t="n">
-        <v>69.51934349355217</v>
+        <v>70.76461769115441</v>
       </c>
       <c r="E11" t="n">
-        <v>1937</v>
+        <v>2046</v>
       </c>
       <c r="F11" t="n">
-        <v>75.69363032434545</v>
+        <v>76.68665667166417</v>
       </c>
     </row>
     <row r="12">
@@ -6666,19 +7137,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2705</v>
+        <v>2706</v>
       </c>
       <c r="C12" t="n">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="D12" t="n">
-        <v>33.45656192236599</v>
+        <v>33.48115299334812</v>
       </c>
       <c r="E12" t="n">
-        <v>1478</v>
+        <v>1479</v>
       </c>
       <c r="F12" t="n">
-        <v>54.63955637707948</v>
+        <v>54.65631929046562</v>
       </c>
     </row>
     <row r="13">
@@ -6688,19 +7159,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>71059</v>
+        <v>71097</v>
       </c>
       <c r="C13" t="n">
-        <v>55715</v>
+        <v>55749</v>
       </c>
       <c r="D13" t="n">
-        <v>78.40667614236058</v>
+        <v>78.41259124857589</v>
       </c>
       <c r="E13" t="n">
-        <v>58212</v>
+        <v>58247</v>
       </c>
       <c r="F13" t="n">
-        <v>81.92065748181089</v>
+        <v>81.92610096065937</v>
       </c>
     </row>
     <row r="14">
@@ -6710,19 +7181,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>198454</v>
+        <v>200009</v>
       </c>
       <c r="C14" t="n">
-        <v>123555</v>
+        <v>124556</v>
       </c>
       <c r="D14" t="n">
-        <v>62.25876021647334</v>
+        <v>62.27519761610728</v>
       </c>
       <c r="E14" t="n">
-        <v>157470</v>
+        <v>158696</v>
       </c>
       <c r="F14" t="n">
-        <v>79.34836284479023</v>
+        <v>79.34442950067246</v>
       </c>
     </row>
     <row r="15">
@@ -6732,19 +7203,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>37012</v>
+        <v>38714</v>
       </c>
       <c r="C15" t="n">
-        <v>15703</v>
+        <v>16594</v>
       </c>
       <c r="D15" t="n">
-        <v>42.42678050362045</v>
+        <v>42.86304695975616</v>
       </c>
       <c r="E15" t="n">
-        <v>24751</v>
+        <v>25996</v>
       </c>
       <c r="F15" t="n">
-        <v>66.87290608451313</v>
+        <v>67.14883504675311</v>
       </c>
     </row>
     <row r="16">
@@ -6754,19 +7225,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3573</v>
+        <v>4118</v>
       </c>
       <c r="C16" t="n">
-        <v>1726</v>
+        <v>2003</v>
       </c>
       <c r="D16" t="n">
-        <v>48.30674503218584</v>
+        <v>48.64011656143759</v>
       </c>
       <c r="E16" t="n">
-        <v>2562</v>
+        <v>2964</v>
       </c>
       <c r="F16" t="n">
-        <v>71.70445004198153</v>
+        <v>71.97668771248179</v>
       </c>
     </row>
     <row r="17">
@@ -6776,19 +7247,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13021</v>
+        <v>13328</v>
       </c>
       <c r="C17" t="n">
-        <v>9123</v>
+        <v>9300</v>
       </c>
       <c r="D17" t="n">
-        <v>70.06374318408724</v>
+        <v>69.77791116446579</v>
       </c>
       <c r="E17" t="n">
-        <v>10228</v>
+        <v>10456</v>
       </c>
       <c r="F17" t="n">
-        <v>78.55003455955763</v>
+        <v>78.45138055222088</v>
       </c>
     </row>
     <row r="18"/>
@@ -6889,43 +7360,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2514</v>
+        <v>2531</v>
       </c>
       <c r="D22" t="n">
-        <v>4.821850967913019</v>
+        <v>4.805985776372975</v>
       </c>
       <c r="E22" t="n">
-        <v>1.816666666666667</v>
+        <v>1.833333333333333</v>
       </c>
       <c r="F22" t="n">
-        <v>0.08036418279855034</v>
+        <v>0.08009976293954958</v>
       </c>
       <c r="G22" t="n">
-        <v>0.03027777777777778</v>
+        <v>0.03055555555555555</v>
       </c>
       <c r="H22" t="n">
-        <v>221.1542890591741</v>
+        <v>225.8820780590717</v>
       </c>
       <c r="I22" t="n">
-        <v>88.56666666666666</v>
+        <v>89.46666666666667</v>
       </c>
       <c r="J22" t="n">
-        <v>3.685904817652902</v>
+        <v>3.764701300984528</v>
       </c>
       <c r="K22" t="n">
-        <v>1.476111111111111</v>
+        <v>1.491111111111111</v>
       </c>
       <c r="L22" t="n">
-        <v>213.8695934440187</v>
+        <v>218.6354641350211</v>
       </c>
       <c r="M22" t="n">
-        <v>79.45</v>
+        <v>80.34999999999999</v>
       </c>
       <c r="N22" t="n">
-        <v>3.564493224066979</v>
+        <v>3.643924402250352</v>
       </c>
       <c r="O22" t="n">
-        <v>1.324166666666667</v>
+        <v>1.339166666666667</v>
       </c>
     </row>
     <row r="23">
@@ -7006,28 +7477,28 @@
         <v>0.03791666666666667</v>
       </c>
       <c r="H24" t="n">
-        <v>119.5997916666667</v>
+        <v>170.3943775100401</v>
       </c>
       <c r="I24" t="n">
-        <v>17.86666666666667</v>
+        <v>20.31666666666667</v>
       </c>
       <c r="J24" t="n">
-        <v>1.993329861111111</v>
+        <v>2.839906291834003</v>
       </c>
       <c r="K24" t="n">
-        <v>0.2977777777777778</v>
+        <v>0.3386111111111111</v>
       </c>
       <c r="L24" t="n">
-        <v>116.8585416666667</v>
+        <v>167.6485943775101</v>
       </c>
       <c r="M24" t="n">
-        <v>11.8</v>
+        <v>17.4</v>
       </c>
       <c r="N24" t="n">
-        <v>1.947642361111112</v>
+        <v>2.794143239625167</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1966666666666667</v>
+        <v>0.29</v>
       </c>
     </row>
     <row r="25">
@@ -7063,7 +7534,7 @@
         <v>22.78333333333333</v>
       </c>
       <c r="J25" t="n">
-        <v>4.982369242779078</v>
+        <v>4.982369242779079</v>
       </c>
       <c r="K25" t="n">
         <v>0.3797222222222222</v>
@@ -7093,7 +7564,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
@@ -7120,43 +7591,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>286</v>
+        <v>368</v>
       </c>
       <c r="D27" t="n">
-        <v>792.8872377622378</v>
+        <v>680.657472826087</v>
       </c>
       <c r="E27" t="n">
-        <v>145.4083333333333</v>
+        <v>162.8</v>
       </c>
       <c r="F27" t="n">
-        <v>13.2147872960373</v>
+        <v>11.34429121376811</v>
       </c>
       <c r="G27" t="n">
-        <v>2.423472222222222</v>
+        <v>2.713333333333333</v>
       </c>
       <c r="H27" t="n">
-        <v>4366.379938271604</v>
+        <v>4311.782998084292</v>
       </c>
       <c r="I27" t="n">
-        <v>2911.158333333333</v>
+        <v>3150.391666666666</v>
       </c>
       <c r="J27" t="n">
-        <v>72.77299897119342</v>
+        <v>71.86304996807152</v>
       </c>
       <c r="K27" t="n">
-        <v>48.51930555555555</v>
+        <v>52.50652777777778</v>
       </c>
       <c r="L27" t="n">
-        <v>3534.369320987654</v>
+        <v>3599.365900383142</v>
       </c>
       <c r="M27" t="n">
-        <v>2640.058333333333</v>
+        <v>2760.925</v>
       </c>
       <c r="N27" t="n">
-        <v>58.90615534979424</v>
+        <v>59.98943167305237</v>
       </c>
       <c r="O27" t="n">
-        <v>44.00097222222222</v>
+        <v>46.01541666666667</v>
       </c>
     </row>
     <row r="28">
@@ -7171,43 +7642,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1081</v>
+        <v>1108</v>
       </c>
       <c r="D28" t="n">
-        <v>160.0812827628739</v>
+        <v>156.2555204572804</v>
       </c>
       <c r="E28" t="n">
-        <v>2.766666666666667</v>
+        <v>2.75</v>
       </c>
       <c r="F28" t="n">
-        <v>2.668021379381231</v>
+        <v>2.604258674288006</v>
       </c>
       <c r="G28" t="n">
-        <v>0.04611111111111111</v>
+        <v>0.04583333333333333</v>
       </c>
       <c r="H28" t="n">
-        <v>887.658655394525</v>
+        <v>894.4853239656518</v>
       </c>
       <c r="I28" t="n">
-        <v>918.6833333333334</v>
+        <v>934.6500000000001</v>
       </c>
       <c r="J28" t="n">
-        <v>14.79431092324208</v>
+        <v>14.90808873276086</v>
       </c>
       <c r="K28" t="n">
-        <v>15.31138888888889</v>
+        <v>15.5775</v>
       </c>
       <c r="L28" t="n">
-        <v>697.0822665056361</v>
+        <v>709.6165690866511</v>
       </c>
       <c r="M28" t="n">
-        <v>793.8666666666667</v>
+        <v>818.475</v>
       </c>
       <c r="N28" t="n">
-        <v>11.61803777509393</v>
+        <v>11.82694281811085</v>
       </c>
       <c r="O28" t="n">
-        <v>13.23111111111111</v>
+        <v>13.64125</v>
       </c>
     </row>
     <row r="29">
@@ -7222,43 +7693,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>869</v>
+        <v>880</v>
       </c>
       <c r="D29" t="n">
-        <v>630.9640583045646</v>
+        <v>624.1741856060607</v>
       </c>
       <c r="E29" t="n">
-        <v>236.6666666666667</v>
+        <v>232.2833333333333</v>
       </c>
       <c r="F29" t="n">
-        <v>10.51606763840941</v>
+        <v>10.40290309343434</v>
       </c>
       <c r="G29" t="n">
-        <v>3.944444444444444</v>
+        <v>3.871388888888889</v>
       </c>
       <c r="H29" t="n">
-        <v>1383.5427949327</v>
+        <v>1381.629953106682</v>
       </c>
       <c r="I29" t="n">
-        <v>1115.341666666667</v>
+        <v>1121.816666666667</v>
       </c>
       <c r="J29" t="n">
-        <v>23.05904658221166</v>
+        <v>23.02716588511137</v>
       </c>
       <c r="K29" t="n">
-        <v>18.58902777777778</v>
+        <v>18.69694444444444</v>
       </c>
       <c r="L29" t="n">
-        <v>752.3356294536817</v>
+        <v>757.430715123095</v>
       </c>
       <c r="M29" t="n">
-        <v>813.6833333333334</v>
+        <v>815.6166666666667</v>
       </c>
       <c r="N29" t="n">
-        <v>12.53892715756136</v>
+        <v>12.62384525205158</v>
       </c>
       <c r="O29" t="n">
-        <v>13.56138888888889</v>
+        <v>13.59361111111111</v>
       </c>
     </row>
     <row r="30">
@@ -7273,43 +7744,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>15597</v>
+        <v>15705</v>
       </c>
       <c r="D30" t="n">
-        <v>10.50590498172725</v>
+        <v>10.45028547171814</v>
       </c>
       <c r="E30" t="n">
         <v>2.55</v>
       </c>
       <c r="F30" t="n">
-        <v>0.1750984163621209</v>
+        <v>0.1741714245286356</v>
       </c>
       <c r="G30" t="n">
         <v>0.0425</v>
       </c>
       <c r="H30" t="n">
-        <v>422.629699872286</v>
+        <v>424.7645747755972</v>
       </c>
       <c r="I30" t="n">
-        <v>288.225</v>
+        <v>301.9416666666667</v>
       </c>
       <c r="J30" t="n">
-        <v>7.043828331204769</v>
+        <v>7.079409579593285</v>
       </c>
       <c r="K30" t="n">
-        <v>4.803750000000001</v>
+        <v>5.032361111111111</v>
       </c>
       <c r="L30" t="n">
-        <v>410.3589961685824</v>
+        <v>412.5641716111364</v>
       </c>
       <c r="M30" t="n">
-        <v>278.3333333333333</v>
+        <v>290.2166666666667</v>
       </c>
       <c r="N30" t="n">
-        <v>6.839316602809707</v>
+        <v>6.876069526852274</v>
       </c>
       <c r="O30" t="n">
-        <v>4.638888888888888</v>
+        <v>4.836944444444445</v>
       </c>
     </row>
     <row r="31">
@@ -7375,43 +7846,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>11071</v>
+        <v>11083</v>
       </c>
       <c r="D32" t="n">
-        <v>313.5846114473248</v>
+        <v>313.2478856506962</v>
       </c>
       <c r="E32" t="n">
         <v>2.816666666666667</v>
       </c>
       <c r="F32" t="n">
-        <v>5.226410190788748</v>
+        <v>5.220798094178272</v>
       </c>
       <c r="G32" t="n">
         <v>0.04694444444444445</v>
       </c>
       <c r="H32" t="n">
-        <v>643.6331005962685</v>
+        <v>647.007467644027</v>
       </c>
       <c r="I32" t="n">
-        <v>383.7833333333334</v>
+        <v>394.9166666666667</v>
       </c>
       <c r="J32" t="n">
-        <v>10.72721834327114</v>
+        <v>10.78345779406712</v>
       </c>
       <c r="K32" t="n">
-        <v>6.39638888888889</v>
+        <v>6.581944444444445</v>
       </c>
       <c r="L32" t="n">
-        <v>246.9747816887863</v>
+        <v>253.3266273431833</v>
       </c>
       <c r="M32" t="n">
-        <v>71.08333333333333</v>
+        <v>71.26666666666667</v>
       </c>
       <c r="N32" t="n">
-        <v>4.116246361479772</v>
+        <v>4.222110455719721</v>
       </c>
       <c r="O32" t="n">
-        <v>1.184722222222222</v>
+        <v>1.187777777777778</v>
       </c>
     </row>
     <row r="33">
@@ -7426,43 +7897,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>13810</v>
+        <v>13823</v>
       </c>
       <c r="D33" t="n">
-        <v>400.3451979242095</v>
+        <v>400.0687031276375</v>
       </c>
       <c r="E33" t="n">
-        <v>72.04166666666666</v>
+        <v>72.03333333333333</v>
       </c>
       <c r="F33" t="n">
-        <v>6.672419965403491</v>
+        <v>6.667811718793959</v>
       </c>
       <c r="G33" t="n">
-        <v>1.200694444444444</v>
+        <v>1.200555555555556</v>
       </c>
       <c r="H33" t="n">
-        <v>674.6612554790231</v>
+        <v>679.4091485015384</v>
       </c>
       <c r="I33" t="n">
-        <v>350.175</v>
+        <v>360.5833333333333</v>
       </c>
       <c r="J33" t="n">
-        <v>11.24435425798372</v>
+        <v>11.32348580835898</v>
       </c>
       <c r="K33" t="n">
-        <v>5.83625</v>
+        <v>6.009722222222222</v>
       </c>
       <c r="L33" t="n">
-        <v>253.6091356188687</v>
+        <v>260.4465027280015</v>
       </c>
       <c r="M33" t="n">
-        <v>68.25</v>
+        <v>69.5</v>
       </c>
       <c r="N33" t="n">
-        <v>4.226818926981145</v>
+        <v>4.340775045466692</v>
       </c>
       <c r="O33" t="n">
-        <v>1.1375</v>
+        <v>1.158333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -7477,43 +7948,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>3789</v>
+        <v>3822</v>
       </c>
       <c r="D34" t="n">
-        <v>1176.947211225477</v>
+        <v>1166.810430839002</v>
       </c>
       <c r="E34" t="n">
-        <v>911.9166666666666</v>
+        <v>904.525</v>
       </c>
       <c r="F34" t="n">
-        <v>19.61578685375795</v>
+        <v>19.44684051398337</v>
       </c>
       <c r="G34" t="n">
-        <v>15.19861111111111</v>
+        <v>15.07541666666667</v>
       </c>
       <c r="H34" t="n">
-        <v>1807.82438537185</v>
+        <v>1818.155462568472</v>
       </c>
       <c r="I34" t="n">
-        <v>1454.416666666667</v>
+        <v>1456.95</v>
       </c>
       <c r="J34" t="n">
-        <v>30.13040642286417</v>
+        <v>30.30259104280787</v>
       </c>
       <c r="K34" t="n">
-        <v>24.24027777777778</v>
+        <v>24.2825</v>
       </c>
       <c r="L34" t="n">
-        <v>511.1862784265519</v>
+        <v>534.1150233313045</v>
       </c>
       <c r="M34" t="n">
-        <v>477.8833333333333</v>
+        <v>478.0333333333334</v>
       </c>
       <c r="N34" t="n">
-        <v>8.519771307109199</v>
+        <v>8.901917055521741</v>
       </c>
       <c r="O34" t="n">
-        <v>7.964722222222222</v>
+        <v>7.967222222222222</v>
       </c>
     </row>
     <row r="35">
@@ -7528,43 +7999,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>3887</v>
+        <v>3913</v>
       </c>
       <c r="D35" t="n">
-        <v>1673.227510505103</v>
+        <v>1663.589300621859</v>
       </c>
       <c r="E35" t="n">
-        <v>1341.966666666667</v>
+        <v>1336.45</v>
       </c>
       <c r="F35" t="n">
-        <v>27.88712517508504</v>
+        <v>27.72648834369765</v>
       </c>
       <c r="G35" t="n">
-        <v>22.36611111111111</v>
+        <v>22.27416666666667</v>
       </c>
       <c r="H35" t="n">
-        <v>2227.539973237357</v>
+        <v>2236.593251786696</v>
       </c>
       <c r="I35" t="n">
-        <v>1934.133333333333</v>
+        <v>1948.075</v>
       </c>
       <c r="J35" t="n">
-        <v>37.12566622062262</v>
+        <v>37.27655419644493</v>
       </c>
       <c r="K35" t="n">
-        <v>32.23555555555556</v>
+        <v>32.46791666666667</v>
       </c>
       <c r="L35" t="n">
-        <v>534.2950489110373</v>
+        <v>553.8581592450064</v>
       </c>
       <c r="M35" t="n">
-        <v>478.1083333333333</v>
+        <v>478.2166666666666</v>
       </c>
       <c r="N35" t="n">
-        <v>8.904917481850621</v>
+        <v>9.230969320750106</v>
       </c>
       <c r="O35" t="n">
-        <v>7.968472222222223</v>
+        <v>7.970277777777778</v>
       </c>
     </row>
     <row r="36">
@@ -7579,43 +8050,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1779</v>
+        <v>1888</v>
       </c>
       <c r="D36" t="n">
-        <v>11.57439572793704</v>
+        <v>11.11486581920904</v>
       </c>
       <c r="E36" t="n">
-        <v>2.233333333333333</v>
+        <v>2.4</v>
       </c>
       <c r="F36" t="n">
-        <v>0.1929065954656174</v>
+        <v>0.185247763653484</v>
       </c>
       <c r="G36" t="n">
-        <v>0.03722222222222223</v>
+        <v>0.04</v>
       </c>
       <c r="H36" t="n">
-        <v>2699.619936457506</v>
+        <v>2929.286748027613</v>
       </c>
       <c r="I36" t="n">
-        <v>2504.483333333333</v>
+        <v>2632.05</v>
       </c>
       <c r="J36" t="n">
-        <v>44.9936656076251</v>
+        <v>48.82144580046022</v>
       </c>
       <c r="K36" t="n">
-        <v>41.74138888888888</v>
+        <v>43.8675</v>
       </c>
       <c r="L36" t="n">
-        <v>2684.089634630659</v>
+        <v>2914.533407297831</v>
       </c>
       <c r="M36" t="n">
-        <v>2500.283333333333</v>
+        <v>2620.45</v>
       </c>
       <c r="N36" t="n">
-        <v>44.73482724384433</v>
+        <v>48.57555678829718</v>
       </c>
       <c r="O36" t="n">
-        <v>41.67138888888889</v>
+        <v>43.67416666666666</v>
       </c>
     </row>
     <row r="37">
@@ -7645,28 +8116,28 @@
         <v>49.10194444444444</v>
       </c>
       <c r="H37" t="n">
-        <v>3514.511378659112</v>
+        <v>3511.772395096652</v>
       </c>
       <c r="I37" t="n">
-        <v>3664.833333333333</v>
+        <v>3650.95</v>
       </c>
       <c r="J37" t="n">
-        <v>58.57518964431854</v>
+        <v>58.52953991827754</v>
       </c>
       <c r="K37" t="n">
-        <v>61.08055555555555</v>
+        <v>60.84916666666666</v>
       </c>
       <c r="L37" t="n">
-        <v>293.6152030217186</v>
+        <v>295.4250353606789</v>
       </c>
       <c r="M37" t="n">
-        <v>244.7166666666667</v>
+        <v>245.05</v>
       </c>
       <c r="N37" t="n">
-        <v>4.893586717028644</v>
+        <v>4.92375058934465</v>
       </c>
       <c r="O37" t="n">
-        <v>4.078611111111111</v>
+        <v>4.084166666666667</v>
       </c>
     </row>
     <row r="38">
@@ -7681,16 +8152,16 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="D38" t="n">
-        <v>1.247569060773481</v>
+        <v>1.246192052980132</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0.02079281767955801</v>
+        <v>0.02076986754966888</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -7714,7 +8185,7 @@
         <v>397.9666666666666</v>
       </c>
       <c r="N38" t="n">
-        <v>7.590093205788571</v>
+        <v>7.590093205788569</v>
       </c>
       <c r="O38" t="n">
         <v>6.632777777777777</v>
@@ -7747,7 +8218,7 @@
         <v>1.83375</v>
       </c>
       <c r="H39" t="n">
-        <v>602.7895047833429</v>
+        <v>602.7895047833426</v>
       </c>
       <c r="I39" t="n">
         <v>595.3</v>
@@ -7783,40 +8254,40 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>55715</v>
+        <v>55749</v>
       </c>
       <c r="D40" t="n">
-        <v>88.41074516138683</v>
+        <v>88.35809252183897</v>
       </c>
       <c r="E40" t="n">
         <v>2.483333333333333</v>
       </c>
       <c r="F40" t="n">
-        <v>1.473512419356448</v>
+        <v>1.472634875363983</v>
       </c>
       <c r="G40" t="n">
         <v>0.04138888888888889</v>
       </c>
       <c r="H40" t="n">
-        <v>140.7716753082688</v>
+        <v>141.3187099098262</v>
       </c>
       <c r="I40" t="n">
         <v>3.183333333333333</v>
       </c>
       <c r="J40" t="n">
-        <v>2.346194588471147</v>
+        <v>2.355311831830436</v>
       </c>
       <c r="K40" t="n">
         <v>0.05305555555555555</v>
       </c>
       <c r="L40" t="n">
-        <v>27.91211451866663</v>
+        <v>28.50747187877661</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.4652019086444439</v>
+        <v>0.4751245313129435</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -7834,43 +8305,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>15344</v>
+        <v>15348</v>
       </c>
       <c r="D41" t="n">
-        <v>754.268514294404</v>
+        <v>754.0881960733212</v>
       </c>
       <c r="E41" t="n">
-        <v>631.9083333333333</v>
+        <v>631.3</v>
       </c>
       <c r="F41" t="n">
-        <v>12.57114190490673</v>
+        <v>12.56813660122202</v>
       </c>
       <c r="G41" t="n">
-        <v>10.53180555555556</v>
+        <v>10.52166666666667</v>
       </c>
       <c r="H41" t="n">
-        <v>833.2983020918228</v>
+        <v>833.3736499637877</v>
       </c>
       <c r="I41" t="n">
-        <v>714.0916666666667</v>
+        <v>714.8</v>
       </c>
       <c r="J41" t="n">
-        <v>13.88830503486371</v>
+        <v>13.8895608327298</v>
       </c>
       <c r="K41" t="n">
-        <v>11.90152777777778</v>
+        <v>11.91333333333333</v>
       </c>
       <c r="L41" t="n">
-        <v>76.06556189441277</v>
+        <v>76.32962384573601</v>
       </c>
       <c r="M41" t="n">
-        <v>61.31666666666667</v>
+        <v>61.325</v>
       </c>
       <c r="N41" t="n">
-        <v>1.267759364906879</v>
+        <v>1.272160397428933</v>
       </c>
       <c r="O41" t="n">
-        <v>1.021944444444445</v>
+        <v>1.022083333333333</v>
       </c>
     </row>
     <row r="42">
@@ -7885,43 +8356,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>123555</v>
+        <v>124556</v>
       </c>
       <c r="D42" t="n">
-        <v>10.90193017954218</v>
+        <v>10.84058923964589</v>
       </c>
       <c r="E42" t="n">
         <v>2.733333333333333</v>
       </c>
       <c r="F42" t="n">
-        <v>0.1816988363257029</v>
+        <v>0.1806764873274315</v>
       </c>
       <c r="G42" t="n">
         <v>0.04555555555555556</v>
       </c>
       <c r="H42" t="n">
-        <v>464.0093607476986</v>
+        <v>472.3386509467931</v>
       </c>
       <c r="I42" t="n">
-        <v>167.4166666666667</v>
+        <v>171.8166666666667</v>
       </c>
       <c r="J42" t="n">
-        <v>7.733489345794977</v>
+        <v>7.872310849113219</v>
       </c>
       <c r="K42" t="n">
-        <v>2.790277777777777</v>
+        <v>2.863611111111111</v>
       </c>
       <c r="L42" t="n">
-        <v>452.358217129764</v>
+        <v>460.8076949827506</v>
       </c>
       <c r="M42" t="n">
-        <v>156.55</v>
+        <v>160.85</v>
       </c>
       <c r="N42" t="n">
-        <v>7.5393036188294</v>
+        <v>7.680128249712509</v>
       </c>
       <c r="O42" t="n">
-        <v>2.609166666666667</v>
+        <v>2.680833333333333</v>
       </c>
     </row>
     <row r="43">
@@ -7936,43 +8407,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>74899</v>
+        <v>75453</v>
       </c>
       <c r="D43" t="n">
-        <v>159.0232161533087</v>
+        <v>158.4405384809087</v>
       </c>
       <c r="E43" t="n">
-        <v>85.8</v>
+        <v>85.73333333333333</v>
       </c>
       <c r="F43" t="n">
-        <v>2.650386935888478</v>
+        <v>2.640675641348477</v>
       </c>
       <c r="G43" t="n">
-        <v>1.43</v>
+        <v>1.428888888888889</v>
       </c>
       <c r="H43" t="n">
-        <v>537.9934669966996</v>
+        <v>546.1492319809115</v>
       </c>
       <c r="I43" t="n">
-        <v>231.375</v>
+        <v>235.9416666666667</v>
       </c>
       <c r="J43" t="n">
-        <v>8.966557783278327</v>
+        <v>9.102487199681857</v>
       </c>
       <c r="K43" t="n">
-        <v>3.85625</v>
+        <v>3.932361111111111</v>
       </c>
       <c r="L43" t="n">
-        <v>380.1026178689297</v>
+        <v>389.1404997250416</v>
       </c>
       <c r="M43" t="n">
-        <v>110.3916666666667</v>
+        <v>112.7333333333333</v>
       </c>
       <c r="N43" t="n">
-        <v>6.335043631148829</v>
+        <v>6.485674995417361</v>
       </c>
       <c r="O43" t="n">
-        <v>1.839861111111111</v>
+        <v>1.878888888888889</v>
       </c>
     </row>
     <row r="44">
@@ -7987,43 +8458,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>15703</v>
+        <v>16594</v>
       </c>
       <c r="D44" t="n">
-        <v>7.562211042475959</v>
+        <v>7.318905427664618</v>
       </c>
       <c r="E44" t="n">
-        <v>2.4</v>
+        <v>2.45</v>
       </c>
       <c r="F44" t="n">
-        <v>0.1260368507079327</v>
+        <v>0.1219817571277436</v>
       </c>
       <c r="G44" t="n">
-        <v>0.04</v>
+        <v>0.04083333333333334</v>
       </c>
       <c r="H44" t="n">
-        <v>804.9544844070111</v>
+        <v>837.6443158894031</v>
       </c>
       <c r="I44" t="n">
-        <v>828.1666666666666</v>
+        <v>853.4</v>
       </c>
       <c r="J44" t="n">
-        <v>13.41590807345019</v>
+        <v>13.96073859815672</v>
       </c>
       <c r="K44" t="n">
-        <v>13.80277777777778</v>
+        <v>14.22333333333333</v>
       </c>
       <c r="L44" t="n">
-        <v>796.1613640387485</v>
+        <v>829.2039527708556</v>
       </c>
       <c r="M44" t="n">
-        <v>819.7</v>
+        <v>844.2166666666667</v>
       </c>
       <c r="N44" t="n">
-        <v>13.26935606731248</v>
+        <v>13.82006587951426</v>
       </c>
       <c r="O44" t="n">
-        <v>13.66166666666667</v>
+        <v>14.07027777777778</v>
       </c>
     </row>
     <row r="45">
@@ -8038,43 +8509,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>21309</v>
+        <v>22120</v>
       </c>
       <c r="D45" t="n">
-        <v>238.909257434261</v>
+        <v>232.5550821277878</v>
       </c>
       <c r="E45" t="n">
-        <v>35.76666666666667</v>
+        <v>33.60833333333333</v>
       </c>
       <c r="F45" t="n">
-        <v>3.981820957237682</v>
+        <v>3.87591803546313</v>
       </c>
       <c r="G45" t="n">
-        <v>0.5961111111111111</v>
+        <v>0.560138888888889</v>
       </c>
       <c r="H45" t="n">
-        <v>844.3830725750287</v>
+        <v>862.0196887432717</v>
       </c>
       <c r="I45" t="n">
-        <v>898.5166666666667</v>
+        <v>919.7166666666667</v>
       </c>
       <c r="J45" t="n">
-        <v>14.07305120958381</v>
+        <v>14.36699481238786</v>
       </c>
       <c r="K45" t="n">
-        <v>14.97527777777778</v>
+        <v>15.32861111111111</v>
       </c>
       <c r="L45" t="n">
-        <v>604.782314594367</v>
+        <v>628.9955316327326</v>
       </c>
       <c r="M45" t="n">
-        <v>450.8166666666667</v>
+        <v>461.0833333333333</v>
       </c>
       <c r="N45" t="n">
-        <v>10.07970524323945</v>
+        <v>10.48325886054554</v>
       </c>
       <c r="O45" t="n">
-        <v>7.513611111111111</v>
+        <v>7.684722222222222</v>
       </c>
     </row>
     <row r="46">
@@ -8089,43 +8560,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1726</v>
+        <v>2003</v>
       </c>
       <c r="D46" t="n">
-        <v>10.11962147547316</v>
+        <v>9.174912631053418</v>
       </c>
       <c r="E46" t="n">
-        <v>1.95</v>
+        <v>2.433333333333333</v>
       </c>
       <c r="F46" t="n">
-        <v>0.1686603579245526</v>
+        <v>0.152915210517557</v>
       </c>
       <c r="G46" t="n">
-        <v>0.0325</v>
+        <v>0.04055555555555555</v>
       </c>
       <c r="H46" t="n">
-        <v>3060.106052141527</v>
+        <v>3320.401501305483</v>
       </c>
       <c r="I46" t="n">
-        <v>2711.566666666667</v>
+        <v>2954.375</v>
       </c>
       <c r="J46" t="n">
-        <v>51.00176753569211</v>
+        <v>55.34002502175805</v>
       </c>
       <c r="K46" t="n">
-        <v>45.19277777777778</v>
+        <v>49.23958333333333</v>
       </c>
       <c r="L46" t="n">
-        <v>3046.590117052408</v>
+        <v>3308.746910356832</v>
       </c>
       <c r="M46" t="n">
-        <v>2691.65</v>
+        <v>2950.708333333333</v>
       </c>
       <c r="N46" t="n">
-        <v>50.77650195087346</v>
+        <v>55.14578183928054</v>
       </c>
       <c r="O46" t="n">
-        <v>44.86083333333333</v>
+        <v>49.17847222222223</v>
       </c>
     </row>
     <row r="47">
@@ -8140,43 +8611,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1847</v>
+        <v>2115</v>
       </c>
       <c r="D47" t="n">
-        <v>243.872513986645</v>
+        <v>253.1741922773838</v>
       </c>
       <c r="E47" t="n">
-        <v>59.56666666666667</v>
+        <v>76.18333333333334</v>
       </c>
       <c r="F47" t="n">
-        <v>4.064541899777416</v>
+        <v>4.219569871289729</v>
       </c>
       <c r="G47" t="n">
-        <v>0.9927777777777779</v>
+        <v>1.269722222222222</v>
       </c>
       <c r="H47" t="n">
-        <v>3100.174174684022</v>
+        <v>3299.089833005894</v>
       </c>
       <c r="I47" t="n">
-        <v>2828.683333333333</v>
+        <v>2956.458333333333</v>
       </c>
       <c r="J47" t="n">
-        <v>51.66956957806703</v>
+        <v>54.98483055009823</v>
       </c>
       <c r="K47" t="n">
-        <v>47.14472222222222</v>
+        <v>49.27430555555556</v>
       </c>
       <c r="L47" t="n">
-        <v>2854.73588945482</v>
+        <v>3044.33881794368</v>
       </c>
       <c r="M47" t="n">
-        <v>2745.833333333333</v>
+        <v>2888.425</v>
       </c>
       <c r="N47" t="n">
-        <v>47.57893149091366</v>
+        <v>50.73898029906134</v>
       </c>
       <c r="O47" t="n">
-        <v>45.76388888888889</v>
+        <v>48.14041666666667</v>
       </c>
     </row>
     <row r="48">
@@ -8191,43 +8662,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9123</v>
+        <v>9300</v>
       </c>
       <c r="D48" t="n">
-        <v>10.75505864299025</v>
+        <v>10.60408422939068</v>
       </c>
       <c r="E48" t="n">
         <v>2.583333333333333</v>
       </c>
       <c r="F48" t="n">
-        <v>0.1792509773831708</v>
+        <v>0.1767347371565114</v>
       </c>
       <c r="G48" t="n">
         <v>0.04305555555555556</v>
       </c>
       <c r="H48" t="n">
-        <v>401.9185352891156</v>
+        <v>416.414008817902</v>
       </c>
       <c r="I48" t="n">
-        <v>307.1083333333333</v>
+        <v>317.1</v>
       </c>
       <c r="J48" t="n">
-        <v>6.698642254818594</v>
+        <v>6.940233480298367</v>
       </c>
       <c r="K48" t="n">
-        <v>5.118472222222222</v>
+        <v>5.285</v>
       </c>
       <c r="L48" t="n">
-        <v>389.5431802721089</v>
+        <v>404.2452707761417</v>
       </c>
       <c r="M48" t="n">
-        <v>291.3166666666667</v>
+        <v>303.05</v>
       </c>
       <c r="N48" t="n">
-        <v>6.492386337868481</v>
+        <v>6.737421179602363</v>
       </c>
       <c r="O48" t="n">
-        <v>4.855277777777777</v>
+        <v>5.050833333333333</v>
       </c>
     </row>
     <row r="49">
@@ -8242,43 +8713,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3898</v>
+        <v>4028</v>
       </c>
       <c r="D49" t="n">
-        <v>339.5726782965623</v>
+        <v>334.8714208871235</v>
       </c>
       <c r="E49" t="n">
-        <v>161.725</v>
+        <v>156.8833333333333</v>
       </c>
       <c r="F49" t="n">
-        <v>5.659544638276039</v>
+        <v>5.581190348118724</v>
       </c>
       <c r="G49" t="n">
-        <v>2.695416666666667</v>
+        <v>2.614722222222222</v>
       </c>
       <c r="H49" t="n">
-        <v>773.5009083007388</v>
+        <v>803.9068919146074</v>
       </c>
       <c r="I49" t="n">
-        <v>645.3666666666667</v>
+        <v>667.4083333333333</v>
       </c>
       <c r="J49" t="n">
-        <v>12.89168180501231</v>
+        <v>13.39844819857679</v>
       </c>
       <c r="K49" t="n">
-        <v>10.75611111111111</v>
+        <v>11.12347222222222</v>
       </c>
       <c r="L49" t="n">
-        <v>432.9362538026945</v>
+        <v>468.1192721465793</v>
       </c>
       <c r="M49" t="n">
-        <v>298.2333333333333</v>
+        <v>321.325</v>
       </c>
       <c r="N49" t="n">
-        <v>7.215604230044907</v>
+        <v>7.801987869109654</v>
       </c>
       <c r="O49" t="n">
-        <v>4.970555555555555</v>
+        <v>5.355416666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica dashboard vie 04/09/2026 11:24:12,90
</commit_message>
<xml_diff>
--- a/Reporte_Efectividad_Automatizacion.xlsx
+++ b/Reporte_Efectividad_Automatizacion.xlsx
@@ -708,19 +708,19 @@
         <v>71.65194435983349</v>
       </c>
       <c r="Z2" t="n">
-        <v>455</v>
+        <v>1280</v>
       </c>
       <c r="AA2" t="n">
-        <v>34.72527472527472</v>
+        <v>36.25</v>
       </c>
       <c r="AB2" t="n">
-        <v>68.57142857142857</v>
+        <v>69.765625</v>
       </c>
       <c r="AC2" t="n">
-        <v>9.027234315080793</v>
+        <v>10.55195958980607</v>
       </c>
       <c r="AD2" t="n">
-        <v>-95.38024164889836</v>
+        <v>-87.00375672657123</v>
       </c>
     </row>
     <row r="3">
@@ -802,19 +802,19 @@
         <v>79.51807228915662</v>
       </c>
       <c r="Z3" t="n">
-        <v>47</v>
+        <v>98</v>
       </c>
       <c r="AA3" t="n">
-        <v>57.44680851063831</v>
+        <v>50</v>
       </c>
       <c r="AB3" t="n">
-        <v>91.48936170212765</v>
+        <v>91.83673469387756</v>
       </c>
       <c r="AC3" t="n">
-        <v>31.62925257260044</v>
+        <v>24.18244406196213</v>
       </c>
       <c r="AD3" t="n">
-        <v>-91.91049913941481</v>
+        <v>-83.13253012048193</v>
       </c>
     </row>
     <row r="4">
@@ -887,28 +887,28 @@
         <v>34.85881207400195</v>
       </c>
       <c r="W4" t="n">
-        <v>457</v>
+        <v>479</v>
       </c>
       <c r="X4" t="n">
-        <v>19.47483588621444</v>
+        <v>18.580375782881</v>
       </c>
       <c r="Y4" t="n">
-        <v>63.45733041575492</v>
+        <v>62.42171189979123</v>
       </c>
       <c r="Z4" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="AA4" t="n">
-        <v>100</v>
+        <v>72.22222222222221</v>
       </c>
       <c r="AB4" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
       <c r="AC4" t="n">
-        <v>80.52516411378556</v>
+        <v>53.64184643934121</v>
       </c>
       <c r="AD4" t="n">
-        <v>-99.78118161925602</v>
+        <v>-96.24217118997912</v>
       </c>
     </row>
     <row r="5">
@@ -990,19 +990,19 @@
         <v>62.37424547283702</v>
       </c>
       <c r="Z5" t="n">
-        <v>94</v>
+        <v>286</v>
       </c>
       <c r="AA5" t="n">
-        <v>60.63829787234043</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="AB5" t="n">
-        <v>64.8936170212766</v>
+        <v>59.09090909090909</v>
       </c>
       <c r="AC5" t="n">
-        <v>4.903891433708644</v>
+        <v>-1.188951893177247</v>
       </c>
       <c r="AD5" t="n">
-        <v>-95.27162977867204</v>
+        <v>-85.61368209255534</v>
       </c>
     </row>
     <row r="6">
@@ -1084,19 +1084,19 @@
         <v>82.54543623823189</v>
       </c>
       <c r="Z6" t="n">
-        <v>1383</v>
+        <v>3125</v>
       </c>
       <c r="AA6" t="n">
-        <v>36.73174258857556</v>
+        <v>58.11199999999999</v>
       </c>
       <c r="AB6" t="n">
-        <v>45.98698481561822</v>
+        <v>64.096</v>
       </c>
       <c r="AC6" t="n">
-        <v>-42.33486366425632</v>
+        <v>-20.95460625283189</v>
       </c>
       <c r="AD6" t="n">
-        <v>-93.03730554296934</v>
+        <v>-84.2672305291245</v>
       </c>
     </row>
     <row r="7">
@@ -1169,28 +1169,28 @@
         <v>61.85549639414975</v>
       </c>
       <c r="W7" t="n">
-        <v>24906</v>
+        <v>24907</v>
       </c>
       <c r="X7" t="n">
-        <v>44.49931743355015</v>
+        <v>44.49753081463042</v>
       </c>
       <c r="Y7" t="n">
-        <v>64.37806151128243</v>
+        <v>64.37949170915806</v>
       </c>
       <c r="Z7" t="n">
-        <v>1480</v>
+        <v>3808</v>
       </c>
       <c r="AA7" t="n">
-        <v>58.51351351351352</v>
+        <v>54.51680672268907</v>
       </c>
       <c r="AB7" t="n">
-        <v>67.70270270270269</v>
+        <v>65.30987394957984</v>
       </c>
       <c r="AC7" t="n">
-        <v>14.01419607996336</v>
+        <v>10.01927590805865</v>
       </c>
       <c r="AD7" t="n">
-        <v>-94.05765678952864</v>
+        <v>-84.71112538643754</v>
       </c>
     </row>
     <row r="8">
@@ -1272,19 +1272,19 @@
         <v>63.24499030381383</v>
       </c>
       <c r="Z8" t="n">
-        <v>474</v>
+        <v>1660</v>
       </c>
       <c r="AA8" t="n">
-        <v>54.85232067510548</v>
+        <v>50.96385542168674</v>
       </c>
       <c r="AB8" t="n">
-        <v>64.55696202531645</v>
+        <v>60.12048192771084</v>
       </c>
       <c r="AC8" t="n">
-        <v>5.440555969223126</v>
+        <v>1.55209071580439</v>
       </c>
       <c r="AD8" t="n">
-        <v>-93.87201034259857</v>
+        <v>-78.53910795087266</v>
       </c>
     </row>
     <row r="9">
@@ -1357,28 +1357,28 @@
         <v>68.22074215033301</v>
       </c>
       <c r="W9" t="n">
-        <v>2668</v>
+        <v>2877</v>
       </c>
       <c r="X9" t="n">
-        <v>70.76461769115441</v>
+        <v>72.88842544316996</v>
       </c>
       <c r="Y9" t="n">
-        <v>76.68665667166417</v>
+        <v>78.380257212374</v>
       </c>
       <c r="Z9" t="n">
-        <v>92</v>
+        <v>309</v>
       </c>
       <c r="AA9" t="n">
-        <v>41.30434782608695</v>
+        <v>42.39482200647249</v>
       </c>
       <c r="AB9" t="n">
-        <v>52.17391304347826</v>
+        <v>57.28155339805825</v>
       </c>
       <c r="AC9" t="n">
-        <v>-29.46026986506746</v>
+        <v>-30.49360343669747</v>
       </c>
       <c r="AD9" t="n">
-        <v>-96.55172413793103</v>
+        <v>-89.25964546402503</v>
       </c>
     </row>
     <row r="10">
@@ -1460,19 +1460,19 @@
         <v>54.65631929046562</v>
       </c>
       <c r="Z10" t="n">
-        <v>182</v>
+        <v>433</v>
       </c>
       <c r="AA10" t="n">
-        <v>56.04395604395604</v>
+        <v>51.73210161662818</v>
       </c>
       <c r="AB10" t="n">
-        <v>62.63736263736264</v>
+        <v>57.27482678983834</v>
       </c>
       <c r="AC10" t="n">
-        <v>22.56280305060793</v>
+        <v>18.25094862328006</v>
       </c>
       <c r="AD10" t="n">
-        <v>-93.27420546932743</v>
+        <v>-83.99852180339985</v>
       </c>
     </row>
     <row r="11">
@@ -1545,28 +1545,28 @@
         <v>73.6447415973979</v>
       </c>
       <c r="W11" t="n">
-        <v>71097</v>
+        <v>71099</v>
       </c>
       <c r="X11" t="n">
-        <v>78.41259124857589</v>
+        <v>78.41038551878367</v>
       </c>
       <c r="Y11" t="n">
-        <v>81.92610096065937</v>
+        <v>81.92520288611654</v>
       </c>
       <c r="Z11" t="n">
-        <v>3441</v>
+        <v>9221</v>
       </c>
       <c r="AA11" t="n">
-        <v>77.44841615809358</v>
+        <v>76.90055308534866</v>
       </c>
       <c r="AB11" t="n">
-        <v>80.76140656785819</v>
+        <v>80.34920290640927</v>
       </c>
       <c r="AC11" t="n">
-        <v>-0.9641750904823141</v>
+        <v>-1.509832433435008</v>
       </c>
       <c r="AD11" t="n">
-        <v>-95.16013333895945</v>
+        <v>-87.03075992629995</v>
       </c>
     </row>
     <row r="12">
@@ -1639,28 +1639,28 @@
         <v>74.93570456560008</v>
       </c>
       <c r="W12" t="n">
-        <v>200009</v>
+        <v>200042</v>
       </c>
       <c r="X12" t="n">
-        <v>62.27519761610728</v>
+        <v>62.27442237130203</v>
       </c>
       <c r="Y12" t="n">
-        <v>79.34442950067246</v>
+        <v>79.3433378990412</v>
       </c>
       <c r="Z12" t="n">
-        <v>8108</v>
+        <v>24739</v>
       </c>
       <c r="AA12" t="n">
-        <v>64.29452392698569</v>
+        <v>65.6453373216379</v>
       </c>
       <c r="AB12" t="n">
-        <v>79.18105574740997</v>
+        <v>79.80920813290754</v>
       </c>
       <c r="AC12" t="n">
-        <v>2.019326310878412</v>
+        <v>3.370914950335866</v>
       </c>
       <c r="AD12" t="n">
-        <v>-95.94618242179102</v>
+        <v>-87.63309704961958</v>
       </c>
     </row>
     <row r="13">
@@ -1742,19 +1742,19 @@
         <v>67.14883504675311</v>
       </c>
       <c r="Z13" t="n">
-        <v>2024</v>
+        <v>5816</v>
       </c>
       <c r="AA13" t="n">
-        <v>45.35573122529645</v>
+        <v>46.56121045392022</v>
       </c>
       <c r="AB13" t="n">
-        <v>65.26679841897233</v>
+        <v>66.23108665749656</v>
       </c>
       <c r="AC13" t="n">
-        <v>2.492684265540284</v>
+        <v>3.698163494164056</v>
       </c>
       <c r="AD13" t="n">
-        <v>-94.77191713591982</v>
+        <v>-84.97701090044944</v>
       </c>
     </row>
     <row r="14">
@@ -1827,28 +1827,28 @@
         <v>60.31513970110461</v>
       </c>
       <c r="W14" t="n">
-        <v>4118</v>
+        <v>4414</v>
       </c>
       <c r="X14" t="n">
-        <v>48.64011656143759</v>
+        <v>48.7313094698686</v>
       </c>
       <c r="Y14" t="n">
-        <v>71.97668771248179</v>
+        <v>72.04349796103308</v>
       </c>
       <c r="Z14" t="n">
-        <v>59</v>
+        <v>432</v>
       </c>
       <c r="AA14" t="n">
-        <v>71.1864406779661</v>
+        <v>53.00925925925925</v>
       </c>
       <c r="AB14" t="n">
-        <v>83.05084745762711</v>
+        <v>73.14814814814815</v>
       </c>
       <c r="AC14" t="n">
-        <v>22.54632411652851</v>
+        <v>4.277949789390654</v>
       </c>
       <c r="AD14" t="n">
-        <v>-98.56726566294317</v>
+        <v>-90.21295876755777</v>
       </c>
     </row>
     <row r="15">
@@ -1921,28 +1921,28 @@
         <v>74.15969011620642</v>
       </c>
       <c r="W15" t="n">
-        <v>13328</v>
+        <v>13344</v>
       </c>
       <c r="X15" t="n">
-        <v>69.77791116446579</v>
+        <v>69.73171462829735</v>
       </c>
       <c r="Y15" t="n">
-        <v>78.45138055222088</v>
+        <v>78.43225419664267</v>
       </c>
       <c r="Z15" t="n">
-        <v>423</v>
+        <v>1522</v>
       </c>
       <c r="AA15" t="n">
-        <v>68.32151300236407</v>
+        <v>67.47700394218134</v>
       </c>
       <c r="AB15" t="n">
-        <v>74.70449172576832</v>
+        <v>73.25886990801577</v>
       </c>
       <c r="AC15" t="n">
-        <v>-1.456398162101721</v>
+        <v>-2.254710686116013</v>
       </c>
       <c r="AD15" t="n">
-        <v>-96.82623049219687</v>
+        <v>-88.5941247002398</v>
       </c>
     </row>
   </sheetData>
@@ -2497,7 +2497,7 @@
         <v>2.425833333333334</v>
       </c>
       <c r="H23" t="n">
-        <v>378.110467671061</v>
+        <v>378.1104676710609</v>
       </c>
       <c r="I23" t="n">
         <v>181.55</v>
@@ -2869,7 +2869,7 @@
         <v>32.50861111111111</v>
       </c>
       <c r="H31" t="n">
-        <v>2605.974803101902</v>
+        <v>2605.974803101903</v>
       </c>
       <c r="I31" t="n">
         <v>2260.533333333333</v>
@@ -2887,7 +2887,7 @@
         <v>333.5833333333333</v>
       </c>
       <c r="N31" t="n">
-        <v>5.414959004806335</v>
+        <v>5.414959004806334</v>
       </c>
       <c r="O31" t="n">
         <v>5.559722222222222</v>
@@ -3298,7 +3298,7 @@
         <v>419.8583333333333</v>
       </c>
       <c r="F40" t="n">
-        <v>11.1580480527115</v>
+        <v>11.15804805271149</v>
       </c>
       <c r="G40" t="n">
         <v>6.997638888888889</v>
@@ -3406,25 +3406,25 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>511.5223548146922</v>
+        <v>511.5223548146923</v>
       </c>
       <c r="I42" t="n">
         <v>178.9666666666667</v>
       </c>
       <c r="J42" t="n">
-        <v>8.52537258024487</v>
+        <v>8.525372580244872</v>
       </c>
       <c r="K42" t="n">
         <v>2.982777777777778</v>
       </c>
       <c r="L42" t="n">
-        <v>511.5223548146922</v>
+        <v>511.5223548146923</v>
       </c>
       <c r="M42" t="n">
         <v>178.9666666666667</v>
       </c>
       <c r="N42" t="n">
-        <v>8.52537258024487</v>
+        <v>8.525372580244872</v>
       </c>
       <c r="O42" t="n">
         <v>2.982777777777778</v>
@@ -3457,7 +3457,7 @@
         <v>1.447222222222222</v>
       </c>
       <c r="H43" t="n">
-        <v>630.0103297602134</v>
+        <v>630.0103297602135</v>
       </c>
       <c r="I43" t="n">
         <v>248.175</v>
@@ -3475,7 +3475,7 @@
         <v>124.8416666666667</v>
       </c>
       <c r="N43" t="n">
-        <v>8.105845548667613</v>
+        <v>8.105845548667615</v>
       </c>
       <c r="O43" t="n">
         <v>2.080694444444444</v>
@@ -3571,13 +3571,13 @@
         <v>52.98138888888889</v>
       </c>
       <c r="L45" t="n">
-        <v>4027.889167021226</v>
+        <v>4027.889167021227</v>
       </c>
       <c r="M45" t="n">
         <v>3093.05</v>
       </c>
       <c r="N45" t="n">
-        <v>67.13148611702043</v>
+        <v>67.13148611702044</v>
       </c>
       <c r="O45" t="n">
         <v>51.55083333333334</v>
@@ -3863,19 +3863,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>297</v>
+        <v>890</v>
       </c>
       <c r="C4" t="n">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="D4" t="n">
-        <v>8.080808080808081</v>
+        <v>9.438202247191011</v>
       </c>
       <c r="E4" t="n">
-        <v>1041.718333333333</v>
+        <v>882.4149999999998</v>
       </c>
       <c r="F4" t="n">
-        <v>2839.077032967033</v>
+        <v>3131.372717121588</v>
       </c>
     </row>
     <row r="5">
@@ -3885,19 +3885,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12598</v>
+        <v>37249</v>
       </c>
       <c r="C5" t="n">
-        <v>10334</v>
+        <v>30802</v>
       </c>
       <c r="D5" t="n">
-        <v>82.02889347515479</v>
+        <v>82.69215280947139</v>
       </c>
       <c r="E5" t="n">
-        <v>3645.505887362105</v>
+        <v>3707.349971722616</v>
       </c>
       <c r="F5" t="n">
-        <v>20112.23494257951</v>
+        <v>11534.20088242593</v>
       </c>
     </row>
     <row r="6">
@@ -3907,19 +3907,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4469</v>
+        <v>12226</v>
       </c>
       <c r="C6" t="n">
-        <v>490</v>
+        <v>1349</v>
       </c>
       <c r="D6" t="n">
-        <v>10.96442157082121</v>
+        <v>11.03386226075577</v>
       </c>
       <c r="E6" t="n">
-        <v>11002.56659183674</v>
+        <v>10517.2290437361</v>
       </c>
       <c r="F6" t="n">
-        <v>10697.80345061573</v>
+        <v>6244.661888388342</v>
       </c>
     </row>
     <row r="7">
@@ -3929,19 +3929,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>899</v>
+        <v>2382</v>
       </c>
       <c r="C7" t="n">
-        <v>296</v>
+        <v>835</v>
       </c>
       <c r="D7" t="n">
-        <v>32.92547274749722</v>
+        <v>35.05457598656591</v>
       </c>
       <c r="E7" t="n">
-        <v>2195.769020270271</v>
+        <v>1869.074892215569</v>
       </c>
       <c r="F7" t="n">
-        <v>7539.56167495854</v>
+        <v>4984.897601809954</v>
       </c>
     </row>
     <row r="8"/>
@@ -3999,19 +3999,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8170</v>
+        <v>8175</v>
       </c>
       <c r="C12" t="n">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="D12" t="n">
-        <v>14.51652386780906</v>
+        <v>14.51987767584098</v>
       </c>
       <c r="E12" t="n">
-        <v>712.7015767284992</v>
+        <v>712.2696461668071</v>
       </c>
       <c r="F12" t="n">
-        <v>1297.363880297823</v>
+        <v>1298.332793360046</v>
       </c>
     </row>
     <row r="13">
@@ -4021,19 +4021,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>285775</v>
+        <v>286217</v>
       </c>
       <c r="C13" t="n">
-        <v>225004</v>
+        <v>225357</v>
       </c>
       <c r="D13" t="n">
-        <v>78.73466888286239</v>
+        <v>78.73641328083238</v>
       </c>
       <c r="E13" t="n">
-        <v>4125.764280132353</v>
+        <v>4120.778946812835</v>
       </c>
       <c r="F13" t="n">
-        <v>6151.237982261277</v>
+        <v>6146.60409217877</v>
       </c>
     </row>
     <row r="14">
@@ -4043,19 +4043,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>84889</v>
+        <v>84990</v>
       </c>
       <c r="C14" t="n">
-        <v>11243</v>
+        <v>11253</v>
       </c>
       <c r="D14" t="n">
-        <v>13.24435439220629</v>
+        <v>13.24038122132015</v>
       </c>
       <c r="E14" t="n">
-        <v>9704.806294583297</v>
+        <v>9697.071729316625</v>
       </c>
       <c r="F14" t="n">
-        <v>3741.013305527795</v>
+        <v>3738.809382655926</v>
       </c>
     </row>
     <row r="15">
@@ -4065,19 +4065,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>19185</v>
+        <v>19216</v>
       </c>
       <c r="C15" t="n">
-        <v>8051</v>
+        <v>8068</v>
       </c>
       <c r="D15" t="n">
-        <v>41.96507688298149</v>
+        <v>41.98584512905911</v>
       </c>
       <c r="E15" t="n">
-        <v>895.4252720158987</v>
+        <v>894.3062946207237</v>
       </c>
       <c r="F15" t="n">
-        <v>3312.71680977187</v>
+        <v>3309.067976318622</v>
       </c>
     </row>
     <row r="16"/>
@@ -4166,7 +4166,7 @@
         <v>72.71500426235504</v>
       </c>
       <c r="E21" t="n">
-        <v>2922.888139929873</v>
+        <v>2922.888139929872</v>
       </c>
       <c r="F21" t="n">
         <v>4919.188137725003</v>
@@ -4210,10 +4210,10 @@
         <v>29.51209150840977</v>
       </c>
       <c r="E23" t="n">
-        <v>537.9021183558139</v>
+        <v>537.902118355814</v>
       </c>
       <c r="F23" t="n">
-        <v>4341.150800669642</v>
+        <v>4341.150800669643</v>
       </c>
     </row>
     <row r="24"/>
@@ -4349,7 +4349,7 @@
         <v>1497.978539343367</v>
       </c>
       <c r="F31" t="n">
-        <v>5790.459127365586</v>
+        <v>5790.459127365587</v>
       </c>
     </row>
     <row r="32"/>
@@ -4438,7 +4438,7 @@
         <v>73.8886025622147</v>
       </c>
       <c r="E37" t="n">
-        <v>3245.465664772564</v>
+        <v>3245.465664772563</v>
       </c>
       <c r="F37" t="n">
         <v>5332.958196689648</v>
@@ -4463,7 +4463,7 @@
         <v>3021.038748</v>
       </c>
       <c r="F38" t="n">
-        <v>4188.860212739793</v>
+        <v>4188.860212739794</v>
       </c>
     </row>
     <row r="39">
@@ -4574,7 +4574,7 @@
         <v>64.44184402779122</v>
       </c>
       <c r="E45" t="n">
-        <v>2849.819069938493</v>
+        <v>2849.819069938494</v>
       </c>
       <c r="F45" t="n">
         <v>4340.007072489959</v>
@@ -4599,7 +4599,7 @@
         <v>1229.104427761094</v>
       </c>
       <c r="F46" t="n">
-        <v>4169.080603087387</v>
+        <v>4169.080603087389</v>
       </c>
     </row>
     <row r="47">
@@ -4618,10 +4618,10 @@
         <v>29.73658732013488</v>
       </c>
       <c r="E47" t="n">
-        <v>2038.200483889076</v>
+        <v>2038.200483889077</v>
       </c>
       <c r="F47" t="n">
-        <v>3167.130335930819</v>
+        <v>3167.130335930818</v>
       </c>
     </row>
     <row r="48"/>
@@ -4757,7 +4757,7 @@
         <v>725.1393298267328</v>
       </c>
       <c r="F55" t="n">
-        <v>2737.009878135031</v>
+        <v>2737.00987813503</v>
       </c>
     </row>
     <row r="56"/>
@@ -4827,7 +4827,7 @@
         <v>730.4016084977238</v>
       </c>
       <c r="F60" t="n">
-        <v>1487.580224330735</v>
+        <v>1487.580224330736</v>
       </c>
     </row>
     <row r="61">
@@ -4849,7 +4849,7 @@
         <v>2376.702662645152</v>
       </c>
       <c r="F61" t="n">
-        <v>4345.258339661355</v>
+        <v>4345.258339661354</v>
       </c>
     </row>
     <row r="62">
@@ -4893,7 +4893,7 @@
         <v>1281.145036051026</v>
       </c>
       <c r="F63" t="n">
-        <v>2680.31142581012</v>
+        <v>2680.311425810119</v>
       </c>
     </row>
     <row r="64"/>
@@ -4985,7 +4985,7 @@
         <v>1684.996463385178</v>
       </c>
       <c r="F69" t="n">
-        <v>4723.494139916261</v>
+        <v>4723.49413991626</v>
       </c>
     </row>
     <row r="70">
@@ -5119,19 +5119,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>455</v>
+        <v>1280</v>
       </c>
       <c r="C4" t="n">
-        <v>158</v>
+        <v>464</v>
       </c>
       <c r="D4" t="n">
-        <v>34.72527472527472</v>
+        <v>36.25</v>
       </c>
       <c r="E4" t="n">
-        <v>312</v>
+        <v>893</v>
       </c>
       <c r="F4" t="n">
-        <v>68.57142857142857</v>
+        <v>69.765625</v>
       </c>
     </row>
     <row r="5">
@@ -5141,19 +5141,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>47</v>
+        <v>98</v>
       </c>
       <c r="C5" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="D5" t="n">
-        <v>57.44680851063831</v>
+        <v>50</v>
       </c>
       <c r="E5" t="n">
-        <v>43</v>
+        <v>90</v>
       </c>
       <c r="F5" t="n">
-        <v>91.48936170212765</v>
+        <v>91.83673469387756</v>
       </c>
     </row>
     <row r="6">
@@ -5163,19 +5163,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D6" t="n">
-        <v>100</v>
+        <v>72.22222222222221</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>100</v>
+        <v>88.88888888888889</v>
       </c>
     </row>
     <row r="7">
@@ -5185,19 +5185,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>94</v>
+        <v>286</v>
       </c>
       <c r="C7" t="n">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="D7" t="n">
-        <v>60.63829787234043</v>
+        <v>54.54545454545454</v>
       </c>
       <c r="E7" t="n">
-        <v>61</v>
+        <v>169</v>
       </c>
       <c r="F7" t="n">
-        <v>64.8936170212766</v>
+        <v>59.09090909090909</v>
       </c>
     </row>
     <row r="8">
@@ -5207,19 +5207,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1383</v>
+        <v>3125</v>
       </c>
       <c r="C8" t="n">
-        <v>508</v>
+        <v>1816</v>
       </c>
       <c r="D8" t="n">
-        <v>36.73174258857556</v>
+        <v>58.11199999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>636</v>
+        <v>2003</v>
       </c>
       <c r="F8" t="n">
-        <v>45.98698481561822</v>
+        <v>64.096</v>
       </c>
     </row>
     <row r="9">
@@ -5229,19 +5229,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1480</v>
+        <v>3808</v>
       </c>
       <c r="C9" t="n">
-        <v>866</v>
+        <v>2076</v>
       </c>
       <c r="D9" t="n">
-        <v>58.51351351351352</v>
+        <v>54.51680672268907</v>
       </c>
       <c r="E9" t="n">
-        <v>1002</v>
+        <v>2487</v>
       </c>
       <c r="F9" t="n">
-        <v>67.70270270270269</v>
+        <v>65.30987394957984</v>
       </c>
     </row>
     <row r="10">
@@ -5251,19 +5251,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>474</v>
+        <v>1660</v>
       </c>
       <c r="C10" t="n">
-        <v>260</v>
+        <v>846</v>
       </c>
       <c r="D10" t="n">
-        <v>54.85232067510548</v>
+        <v>50.96385542168674</v>
       </c>
       <c r="E10" t="n">
-        <v>306</v>
+        <v>998</v>
       </c>
       <c r="F10" t="n">
-        <v>64.55696202531645</v>
+        <v>60.12048192771084</v>
       </c>
     </row>
     <row r="11">
@@ -5273,19 +5273,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>92</v>
+        <v>309</v>
       </c>
       <c r="C11" t="n">
-        <v>38</v>
+        <v>131</v>
       </c>
       <c r="D11" t="n">
-        <v>41.30434782608695</v>
+        <v>42.39482200647249</v>
       </c>
       <c r="E11" t="n">
-        <v>48</v>
+        <v>177</v>
       </c>
       <c r="F11" t="n">
-        <v>52.17391304347826</v>
+        <v>57.28155339805825</v>
       </c>
     </row>
     <row r="12">
@@ -5295,19 +5295,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>182</v>
+        <v>433</v>
       </c>
       <c r="C12" t="n">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="D12" t="n">
-        <v>56.04395604395604</v>
+        <v>51.73210161662818</v>
       </c>
       <c r="E12" t="n">
-        <v>114</v>
+        <v>248</v>
       </c>
       <c r="F12" t="n">
-        <v>62.63736263736264</v>
+        <v>57.27482678983834</v>
       </c>
     </row>
     <row r="13">
@@ -5317,19 +5317,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3441</v>
+        <v>9221</v>
       </c>
       <c r="C13" t="n">
-        <v>2665</v>
+        <v>7091</v>
       </c>
       <c r="D13" t="n">
-        <v>77.44841615809358</v>
+        <v>76.90055308534866</v>
       </c>
       <c r="E13" t="n">
-        <v>2779</v>
+        <v>7409</v>
       </c>
       <c r="F13" t="n">
-        <v>80.76140656785819</v>
+        <v>80.34920290640927</v>
       </c>
     </row>
     <row r="14">
@@ -5339,19 +5339,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>8108</v>
+        <v>24739</v>
       </c>
       <c r="C14" t="n">
-        <v>5213</v>
+        <v>16240</v>
       </c>
       <c r="D14" t="n">
-        <v>64.29452392698569</v>
+        <v>65.6453373216379</v>
       </c>
       <c r="E14" t="n">
-        <v>6420</v>
+        <v>19744</v>
       </c>
       <c r="F14" t="n">
-        <v>79.18105574740997</v>
+        <v>79.80920813290754</v>
       </c>
     </row>
     <row r="15">
@@ -5361,19 +5361,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2024</v>
+        <v>5816</v>
       </c>
       <c r="C15" t="n">
-        <v>918</v>
+        <v>2708</v>
       </c>
       <c r="D15" t="n">
-        <v>45.35573122529645</v>
+        <v>46.56121045392022</v>
       </c>
       <c r="E15" t="n">
-        <v>1321</v>
+        <v>3852</v>
       </c>
       <c r="F15" t="n">
-        <v>65.26679841897233</v>
+        <v>66.23108665749656</v>
       </c>
     </row>
     <row r="16">
@@ -5383,19 +5383,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>59</v>
+        <v>432</v>
       </c>
       <c r="C16" t="n">
-        <v>42</v>
+        <v>229</v>
       </c>
       <c r="D16" t="n">
-        <v>71.1864406779661</v>
+        <v>53.00925925925925</v>
       </c>
       <c r="E16" t="n">
-        <v>49</v>
+        <v>316</v>
       </c>
       <c r="F16" t="n">
-        <v>83.05084745762711</v>
+        <v>73.14814814814815</v>
       </c>
     </row>
     <row r="17">
@@ -5405,19 +5405,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>423</v>
+        <v>1522</v>
       </c>
       <c r="C17" t="n">
-        <v>289</v>
+        <v>1027</v>
       </c>
       <c r="D17" t="n">
-        <v>68.32151300236407</v>
+        <v>67.47700394218134</v>
       </c>
       <c r="E17" t="n">
-        <v>316</v>
+        <v>1115</v>
       </c>
       <c r="F17" t="n">
-        <v>74.70449172576832</v>
+        <v>73.25886990801577</v>
       </c>
     </row>
     <row r="18"/>
@@ -5518,43 +5518,43 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>158</v>
+        <v>464</v>
       </c>
       <c r="D22" t="n">
-        <v>2.39831223628692</v>
+        <v>2.283081896551724</v>
       </c>
       <c r="E22" t="n">
-        <v>2.533333333333333</v>
+        <v>2.566666666666667</v>
       </c>
       <c r="F22" t="n">
-        <v>0.03997187060478201</v>
+        <v>0.03805136494252874</v>
       </c>
       <c r="G22" t="n">
-        <v>0.04222222222222222</v>
+        <v>0.04277777777777778</v>
       </c>
       <c r="H22" t="n">
-        <v>239.4075342465754</v>
+        <v>213.1201265822785</v>
       </c>
       <c r="I22" t="n">
-        <v>108.7666666666667</v>
+        <v>87.28333333333333</v>
       </c>
       <c r="J22" t="n">
-        <v>3.990125570776256</v>
+        <v>3.552002109704642</v>
       </c>
       <c r="K22" t="n">
-        <v>1.812777777777778</v>
+        <v>1.454722222222222</v>
       </c>
       <c r="L22" t="n">
-        <v>236.8277397260274</v>
+        <v>210.5104219409283</v>
       </c>
       <c r="M22" t="n">
-        <v>105.9583333333333</v>
+        <v>85.13333333333334</v>
       </c>
       <c r="N22" t="n">
-        <v>3.947128995433789</v>
+        <v>3.508507032348805</v>
       </c>
       <c r="O22" t="n">
-        <v>1.765972222222222</v>
+        <v>1.418888888888889</v>
       </c>
     </row>
     <row r="23">
@@ -5569,43 +5569,43 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>297</v>
+        <v>816</v>
       </c>
       <c r="D23" t="n">
-        <v>258.8453423120091</v>
+        <v>238.7686887254902</v>
       </c>
       <c r="E23" t="n">
-        <v>75.13333333333334</v>
+        <v>70.19999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>4.314089038533483</v>
+        <v>3.979478145424837</v>
       </c>
       <c r="G23" t="n">
-        <v>1.252222222222222</v>
+        <v>1.17</v>
       </c>
       <c r="H23" t="n">
-        <v>286.4700458190149</v>
+        <v>275.6725563909774</v>
       </c>
       <c r="I23" t="n">
-        <v>109.8166666666667</v>
+        <v>106.0166666666667</v>
       </c>
       <c r="J23" t="n">
-        <v>4.774500763650248</v>
+        <v>4.59454260651629</v>
       </c>
       <c r="K23" t="n">
-        <v>1.830277777777778</v>
+        <v>1.766944444444444</v>
       </c>
       <c r="L23" t="n">
-        <v>23.07605956471936</v>
+        <v>32.26791979949875</v>
       </c>
       <c r="M23" t="n">
-        <v>7.516666666666667</v>
+        <v>7.441666666666666</v>
       </c>
       <c r="N23" t="n">
-        <v>0.3846009927453226</v>
+        <v>0.5377986633249792</v>
       </c>
       <c r="O23" t="n">
-        <v>0.1252777777777778</v>
+        <v>0.1240277777777778</v>
       </c>
     </row>
     <row r="24">
@@ -5620,43 +5620,43 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>27</v>
+        <v>49</v>
       </c>
       <c r="D24" t="n">
-        <v>2.34320987654321</v>
+        <v>2.169047619047619</v>
       </c>
       <c r="E24" t="n">
-        <v>2.633333333333333</v>
+        <v>2.533333333333333</v>
       </c>
       <c r="F24" t="n">
-        <v>0.03905349794238683</v>
+        <v>0.03615079365079365</v>
       </c>
       <c r="G24" t="n">
-        <v>0.04388888888888889</v>
+        <v>0.04222222222222222</v>
       </c>
       <c r="H24" t="n">
-        <v>41.13205128205129</v>
+        <v>267.8308823529412</v>
       </c>
       <c r="I24" t="n">
-        <v>11.1</v>
+        <v>16.55</v>
       </c>
       <c r="J24" t="n">
-        <v>0.685534188034188</v>
+        <v>4.463848039215685</v>
       </c>
       <c r="K24" t="n">
-        <v>0.185</v>
+        <v>0.2758333333333334</v>
       </c>
       <c r="L24" t="n">
-        <v>38.42179487179487</v>
+        <v>265.1759803921569</v>
       </c>
       <c r="M24" t="n">
-        <v>8.566666666666666</v>
+        <v>14.025</v>
       </c>
       <c r="N24" t="n">
-        <v>0.6403632478632478</v>
+        <v>4.419599673202614</v>
       </c>
       <c r="O24" t="n">
-        <v>0.1427777777777778</v>
+        <v>0.23375</v>
       </c>
     </row>
     <row r="25">
@@ -5671,43 +5671,43 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="D25" t="n">
-        <v>300.6</v>
+        <v>396.5632653061224</v>
       </c>
       <c r="E25" t="n">
-        <v>38.91666666666667</v>
+        <v>58.2</v>
       </c>
       <c r="F25" t="n">
-        <v>5.01</v>
+        <v>6.609387755102041</v>
       </c>
       <c r="G25" t="n">
-        <v>0.6486111111111111</v>
+        <v>0.9700000000000001</v>
       </c>
       <c r="H25" t="n">
-        <v>302.5733333333333</v>
+        <v>389.8354166666667</v>
       </c>
       <c r="I25" t="n">
-        <v>44.65</v>
+        <v>56.73333333333333</v>
       </c>
       <c r="J25" t="n">
-        <v>5.042888888888888</v>
+        <v>6.497256944444444</v>
       </c>
       <c r="K25" t="n">
-        <v>0.7441666666666666</v>
+        <v>0.9455555555555555</v>
       </c>
       <c r="L25" t="n">
-        <v>1.973333333333333</v>
+        <v>10.92847222222222</v>
       </c>
       <c r="M25" t="n">
-        <v>1.541666666666667</v>
+        <v>1.691666666666667</v>
       </c>
       <c r="N25" t="n">
-        <v>0.03288888888888889</v>
+        <v>0.1821412037037037</v>
       </c>
       <c r="O25" t="n">
-        <v>0.02569444444444444</v>
+        <v>0.02819444444444445</v>
       </c>
     </row>
     <row r="26">
@@ -5722,19 +5722,43 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>0.776923076923077</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>0.01294871794871795</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>1514.916666666667</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1539.35</v>
+      </c>
+      <c r="J26" t="n">
+        <v>25.24861111111111</v>
+      </c>
+      <c r="K26" t="n">
+        <v>25.65583333333333</v>
+      </c>
+      <c r="L26" t="n">
+        <v>1512.391666666667</v>
+      </c>
+      <c r="M26" t="n">
+        <v>1536.9</v>
+      </c>
+      <c r="N26" t="n">
+        <v>25.20652777777778</v>
+      </c>
+      <c r="O26" t="n">
+        <v>25.615</v>
       </c>
     </row>
     <row r="27">
@@ -5749,7 +5773,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="D27" t="n">
+        <v>531.3566666666667</v>
+      </c>
+      <c r="E27" t="n">
+        <v>294.6</v>
+      </c>
+      <c r="F27" t="n">
+        <v>8.855944444444443</v>
+      </c>
+      <c r="G27" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2136.71</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1899.9</v>
+      </c>
+      <c r="J27" t="n">
+        <v>35.61183333333334</v>
+      </c>
+      <c r="K27" t="n">
+        <v>31.665</v>
+      </c>
+      <c r="L27" t="n">
+        <v>1605.353333333333</v>
+      </c>
+      <c r="M27" t="n">
+        <v>1605.3</v>
+      </c>
+      <c r="N27" t="n">
+        <v>26.75588888888889</v>
+      </c>
+      <c r="O27" t="n">
+        <v>26.755</v>
       </c>
     </row>
     <row r="28">
@@ -5764,43 +5824,43 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>57</v>
+        <v>156</v>
       </c>
       <c r="D28" t="n">
-        <v>419.6833333333333</v>
+        <v>261.8352564102564</v>
       </c>
       <c r="E28" t="n">
-        <v>2.983333333333333</v>
+        <v>2.766666666666667</v>
       </c>
       <c r="F28" t="n">
-        <v>6.994722222222222</v>
+        <v>4.36392094017094</v>
       </c>
       <c r="G28" t="n">
-        <v>0.04972222222222222</v>
+        <v>0.04611111111111111</v>
       </c>
       <c r="H28" t="n">
-        <v>708.9813492063493</v>
+        <v>770.6377777777778</v>
       </c>
       <c r="I28" t="n">
-        <v>830.6916666666666</v>
+        <v>826.7416666666667</v>
       </c>
       <c r="J28" t="n">
-        <v>11.81635582010582</v>
+        <v>12.84396296296296</v>
       </c>
       <c r="K28" t="n">
-        <v>13.84486111111111</v>
+        <v>13.77902777777778</v>
       </c>
       <c r="L28" t="n">
-        <v>139.4111111111111</v>
+        <v>440.3436111111112</v>
       </c>
       <c r="M28" t="n">
-        <v>6.208333333333334</v>
+        <v>198.9666666666667</v>
       </c>
       <c r="N28" t="n">
-        <v>2.323518518518518</v>
+        <v>7.339060185185185</v>
       </c>
       <c r="O28" t="n">
-        <v>0.1034722222222222</v>
+        <v>3.316111111111111</v>
       </c>
     </row>
     <row r="29">
@@ -5815,43 +5875,43 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>37</v>
+        <v>130</v>
       </c>
       <c r="D29" t="n">
-        <v>647.3923423423422</v>
+        <v>411.6869230769231</v>
       </c>
       <c r="E29" t="n">
-        <v>639.55</v>
+        <v>159.025</v>
       </c>
       <c r="F29" t="n">
-        <v>10.78987237237237</v>
+        <v>6.861448717948718</v>
       </c>
       <c r="G29" t="n">
-        <v>10.65916666666667</v>
+        <v>2.650416666666667</v>
       </c>
       <c r="H29" t="n">
-        <v>715.714864864865</v>
+        <v>825.6088461538461</v>
       </c>
       <c r="I29" t="n">
-        <v>859.2333333333333</v>
+        <v>919.1083333333333</v>
       </c>
       <c r="J29" t="n">
-        <v>11.92858108108108</v>
+        <v>13.76014743589744</v>
       </c>
       <c r="K29" t="n">
-        <v>14.32055555555556</v>
+        <v>15.31847222222222</v>
       </c>
       <c r="L29" t="n">
-        <v>68.32252252252252</v>
+        <v>413.9219230769231</v>
       </c>
       <c r="M29" t="n">
-        <v>6.2</v>
+        <v>163.7416666666667</v>
       </c>
       <c r="N29" t="n">
-        <v>1.138708708708709</v>
+        <v>6.898698717948718</v>
       </c>
       <c r="O29" t="n">
-        <v>0.1033333333333333</v>
+        <v>2.729027777777778</v>
       </c>
     </row>
     <row r="30">
@@ -5866,43 +5926,43 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>508</v>
+        <v>1816</v>
       </c>
       <c r="D30" t="n">
-        <v>2.259383202099737</v>
+        <v>2.299045521292217</v>
       </c>
       <c r="E30" t="n">
-        <v>2.575</v>
+        <v>2.583333333333333</v>
       </c>
       <c r="F30" t="n">
-        <v>0.03765638670166229</v>
+        <v>0.03831742535487029</v>
       </c>
       <c r="G30" t="n">
-        <v>0.04291666666666667</v>
+        <v>0.04305555555555556</v>
       </c>
       <c r="H30" t="n">
-        <v>196.9045232273839</v>
+        <v>242.1395969498911</v>
       </c>
       <c r="I30" t="n">
-        <v>88.36666666666666</v>
+        <v>90.84166666666667</v>
       </c>
       <c r="J30" t="n">
-        <v>3.281742053789731</v>
+        <v>4.035659949164851</v>
       </c>
       <c r="K30" t="n">
-        <v>1.472777777777778</v>
+        <v>1.514027777777778</v>
       </c>
       <c r="L30" t="n">
-        <v>194.2876935615322</v>
+        <v>239.5165468409586</v>
       </c>
       <c r="M30" t="n">
-        <v>85.38333333333334</v>
+        <v>88.15833333333333</v>
       </c>
       <c r="N30" t="n">
-        <v>3.238128226025536</v>
+        <v>3.99194244734931</v>
       </c>
       <c r="O30" t="n">
-        <v>1.423055555555556</v>
+        <v>1.469305555555556</v>
       </c>
     </row>
     <row r="31">
@@ -5917,40 +5977,40 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>875</v>
+        <v>1309</v>
       </c>
       <c r="D31" t="n">
-        <v>3176.798457142856</v>
+        <v>2556.705449452509</v>
       </c>
       <c r="E31" t="n">
-        <v>2856.35</v>
+        <v>2044.233333333333</v>
       </c>
       <c r="F31" t="n">
-        <v>52.94664095238095</v>
+        <v>42.61175749087514</v>
       </c>
       <c r="G31" t="n">
-        <v>47.60583333333333</v>
+        <v>34.07055555555556</v>
       </c>
       <c r="H31" t="n">
-        <v>3535.979122182681</v>
+        <v>2894.496544876887</v>
       </c>
       <c r="I31" t="n">
-        <v>3212.583333333333</v>
+        <v>2372.7</v>
       </c>
       <c r="J31" t="n">
-        <v>58.93298536971135</v>
+        <v>48.24160908128145</v>
       </c>
       <c r="K31" t="n">
-        <v>53.54305555555556</v>
+        <v>39.54499999999999</v>
       </c>
       <c r="L31" t="n">
-        <v>352.7267497034401</v>
+        <v>331.1936060365369</v>
       </c>
       <c r="M31" t="n">
         <v>352.5833333333333</v>
       </c>
       <c r="N31" t="n">
-        <v>5.878779161724001</v>
+        <v>5.519893433942283</v>
       </c>
       <c r="O31" t="n">
         <v>5.876388888888888</v>
@@ -5968,43 +6028,43 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>866</v>
+        <v>2076</v>
       </c>
       <c r="D32" t="n">
-        <v>258.2367975365666</v>
+        <v>293.0092565831728</v>
       </c>
       <c r="E32" t="n">
-        <v>2.741666666666667</v>
+        <v>2.733333333333333</v>
       </c>
       <c r="F32" t="n">
-        <v>4.303946625609443</v>
+        <v>4.883487609719546</v>
       </c>
       <c r="G32" t="n">
-        <v>0.04569444444444444</v>
+        <v>0.04555555555555556</v>
       </c>
       <c r="H32" t="n">
-        <v>528.9238178633975</v>
+        <v>603.0128722970215</v>
       </c>
       <c r="I32" t="n">
-        <v>320.8166666666667</v>
+        <v>430.2416666666667</v>
       </c>
       <c r="J32" t="n">
-        <v>8.815396964389958</v>
+        <v>10.0502145382837</v>
       </c>
       <c r="K32" t="n">
-        <v>5.346944444444444</v>
+        <v>7.170694444444445</v>
       </c>
       <c r="L32" t="n">
-        <v>140.332545242265</v>
+        <v>232.5903814769482</v>
       </c>
       <c r="M32" t="n">
-        <v>36.43333333333333</v>
+        <v>58.64166666666667</v>
       </c>
       <c r="N32" t="n">
-        <v>2.338875754037751</v>
+        <v>3.876506357949137</v>
       </c>
       <c r="O32" t="n">
-        <v>0.6072222222222222</v>
+        <v>0.9773611111111111</v>
       </c>
     </row>
     <row r="33">
@@ -6019,43 +6079,43 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>614</v>
+        <v>1732</v>
       </c>
       <c r="D33" t="n">
-        <v>425.0889522258415</v>
+        <v>450.8132217090069</v>
       </c>
       <c r="E33" t="n">
-        <v>147.925</v>
+        <v>153.0583333333333</v>
       </c>
       <c r="F33" t="n">
-        <v>7.084815870430692</v>
+        <v>7.513553695150116</v>
       </c>
       <c r="G33" t="n">
-        <v>2.465416666666667</v>
+        <v>2.550972222222222</v>
       </c>
       <c r="H33" t="n">
-        <v>601.8411388355726</v>
+        <v>665.5287597857437</v>
       </c>
       <c r="I33" t="n">
-        <v>485.8166666666667</v>
+        <v>545.275</v>
       </c>
       <c r="J33" t="n">
-        <v>10.03068564725954</v>
+        <v>11.09214599642906</v>
       </c>
       <c r="K33" t="n">
-        <v>8.096944444444444</v>
+        <v>9.087916666666665</v>
       </c>
       <c r="L33" t="n">
-        <v>130.2832373640435</v>
+        <v>200.658941079522</v>
       </c>
       <c r="M33" t="n">
-        <v>36.46666666666667</v>
+        <v>44.8</v>
       </c>
       <c r="N33" t="n">
-        <v>2.171387289400725</v>
+        <v>3.344315684658701</v>
       </c>
       <c r="O33" t="n">
-        <v>0.6077777777777779</v>
+        <v>0.7466666666666666</v>
       </c>
     </row>
     <row r="34">
@@ -6070,43 +6130,43 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>260</v>
+        <v>846</v>
       </c>
       <c r="D34" t="n">
-        <v>792.2355128205128</v>
+        <v>1385.587765957447</v>
       </c>
       <c r="E34" t="n">
-        <v>834.2333333333333</v>
+        <v>1148.316666666667</v>
       </c>
       <c r="F34" t="n">
-        <v>13.20392521367521</v>
+        <v>23.09312943262411</v>
       </c>
       <c r="G34" t="n">
-        <v>13.90388888888889</v>
+        <v>19.13861111111111</v>
       </c>
       <c r="H34" t="n">
-        <v>1402.207042253521</v>
+        <v>1603.701923076923</v>
       </c>
       <c r="I34" t="n">
-        <v>1463.283333333333</v>
+        <v>1530.525</v>
       </c>
       <c r="J34" t="n">
-        <v>23.37011737089202</v>
+        <v>26.72836538461538</v>
       </c>
       <c r="K34" t="n">
-        <v>24.38805555555556</v>
+        <v>25.50875</v>
       </c>
       <c r="L34" t="n">
-        <v>565.0092331768387</v>
+        <v>452.9673076923077</v>
       </c>
       <c r="M34" t="n">
-        <v>563.75</v>
+        <v>562.1</v>
       </c>
       <c r="N34" t="n">
-        <v>9.416820552947312</v>
+        <v>7.549455128205129</v>
       </c>
       <c r="O34" t="n">
-        <v>9.395833333333334</v>
+        <v>9.368333333333334</v>
       </c>
     </row>
     <row r="35">
@@ -6121,43 +6181,43 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>214</v>
+        <v>814</v>
       </c>
       <c r="D35" t="n">
-        <v>1115.859501557632</v>
+        <v>1728.951842751843</v>
       </c>
       <c r="E35" t="n">
-        <v>1001.583333333333</v>
+        <v>1830.591666666667</v>
       </c>
       <c r="F35" t="n">
-        <v>18.59765835929387</v>
+        <v>28.81586404586405</v>
       </c>
       <c r="G35" t="n">
-        <v>16.69305555555556</v>
+        <v>30.50986111111111</v>
       </c>
       <c r="H35" t="n">
-        <v>1683.434638554217</v>
+        <v>1939.052753623188</v>
       </c>
       <c r="I35" t="n">
-        <v>1569.491666666667</v>
+        <v>1737</v>
       </c>
       <c r="J35" t="n">
-        <v>28.05724397590361</v>
+        <v>32.31754589371981</v>
       </c>
       <c r="K35" t="n">
-        <v>26.15819444444445</v>
+        <v>28.95</v>
       </c>
       <c r="L35" t="n">
-        <v>564.335642570281</v>
+        <v>474.3645893719806</v>
       </c>
       <c r="M35" t="n">
-        <v>563.75</v>
+        <v>562</v>
       </c>
       <c r="N35" t="n">
-        <v>9.405594042838018</v>
+        <v>7.906076489533012</v>
       </c>
       <c r="O35" t="n">
-        <v>9.395833333333334</v>
+        <v>9.366666666666667</v>
       </c>
     </row>
     <row r="36">
@@ -6172,43 +6232,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>38</v>
+        <v>131</v>
       </c>
       <c r="D36" t="n">
-        <v>0.637719298245614</v>
+        <v>1.233206106870229</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0.01062865497076023</v>
+        <v>0.02055343511450381</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>159.0738095238095</v>
+        <v>690.9660256410257</v>
       </c>
       <c r="I36" t="n">
-        <v>142.7</v>
+        <v>396.15</v>
       </c>
       <c r="J36" t="n">
-        <v>2.651230158730158</v>
+        <v>11.51610042735043</v>
       </c>
       <c r="K36" t="n">
-        <v>2.378333333333333</v>
+        <v>6.6025</v>
       </c>
       <c r="L36" t="n">
-        <v>156.4452380952381</v>
+        <v>688.3766025641027</v>
       </c>
       <c r="M36" t="n">
-        <v>140.4</v>
+        <v>393.4833333333333</v>
       </c>
       <c r="N36" t="n">
-        <v>2.607420634920635</v>
+        <v>11.47294337606838</v>
       </c>
       <c r="O36" t="n">
-        <v>2.34</v>
+        <v>6.558055555555556</v>
       </c>
     </row>
     <row r="37">
@@ -6223,43 +6283,43 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>54</v>
+        <v>178</v>
       </c>
       <c r="D37" t="n">
-        <v>5610.661419753086</v>
+        <v>5612.686235955057</v>
       </c>
       <c r="E37" t="n">
-        <v>6823.466666666667</v>
+        <v>6836.775</v>
       </c>
       <c r="F37" t="n">
-        <v>93.51102366255145</v>
+        <v>93.54477059925094</v>
       </c>
       <c r="G37" t="n">
-        <v>113.7244444444444</v>
+        <v>113.94625</v>
       </c>
       <c r="H37" t="n">
-        <v>6468.867006802721</v>
+        <v>6325.357723577235</v>
       </c>
       <c r="I37" t="n">
-        <v>7226.016666666666</v>
+        <v>7186.825000000001</v>
       </c>
       <c r="J37" t="n">
-        <v>107.8144501133787</v>
+        <v>105.4226287262873</v>
       </c>
       <c r="K37" t="n">
-        <v>120.4336111111111</v>
+        <v>119.7804166666667</v>
       </c>
       <c r="L37" t="n">
-        <v>296.5472789115645</v>
+        <v>293.5424796747968</v>
       </c>
       <c r="M37" t="n">
-        <v>330.9</v>
+        <v>303.6083333333333</v>
       </c>
       <c r="N37" t="n">
-        <v>4.942454648526077</v>
+        <v>4.892374661246611</v>
       </c>
       <c r="O37" t="n">
-        <v>5.515</v>
+        <v>5.06013888888889</v>
       </c>
     </row>
     <row r="38">
@@ -6274,43 +6334,43 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>102</v>
+        <v>224</v>
       </c>
       <c r="D38" t="n">
-        <v>1.801797385620915</v>
+        <v>1.953050595238095</v>
       </c>
       <c r="E38" t="n">
-        <v>2.408333333333333</v>
+        <v>2.433333333333333</v>
       </c>
       <c r="F38" t="n">
-        <v>0.03002995642701525</v>
+        <v>0.03255084325396825</v>
       </c>
       <c r="G38" t="n">
-        <v>0.04013888888888889</v>
+        <v>0.04055555555555555</v>
       </c>
       <c r="H38" t="n">
-        <v>374.6587962962963</v>
+        <v>388.2659763313609</v>
       </c>
       <c r="I38" t="n">
-        <v>356.5916666666667</v>
+        <v>411.2833333333334</v>
       </c>
       <c r="J38" t="n">
-        <v>6.244313271604939</v>
+        <v>6.471099605522682</v>
       </c>
       <c r="K38" t="n">
-        <v>5.943194444444445</v>
+        <v>6.854722222222223</v>
       </c>
       <c r="L38" t="n">
-        <v>372.2446759259259</v>
+        <v>385.8447731755424</v>
       </c>
       <c r="M38" t="n">
-        <v>353.9666666666667</v>
+        <v>409.05</v>
       </c>
       <c r="N38" t="n">
-        <v>6.204077932098766</v>
+        <v>6.430746219592375</v>
       </c>
       <c r="O38" t="n">
-        <v>5.899444444444445</v>
+        <v>6.8175</v>
       </c>
     </row>
     <row r="39">
@@ -6325,43 +6385,43 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>80</v>
+        <v>209</v>
       </c>
       <c r="D39" t="n">
-        <v>201.6135416666667</v>
+        <v>241.2178628389155</v>
       </c>
       <c r="E39" t="n">
-        <v>52.88333333333333</v>
+        <v>68.34999999999999</v>
       </c>
       <c r="F39" t="n">
-        <v>3.360225694444444</v>
+        <v>4.020297713981924</v>
       </c>
       <c r="G39" t="n">
-        <v>0.8813888888888889</v>
+        <v>1.139166666666667</v>
       </c>
       <c r="H39" t="n">
-        <v>600.9472222222222</v>
+        <v>626.7366834170854</v>
       </c>
       <c r="I39" t="n">
-        <v>531.85</v>
+        <v>535.4833333333333</v>
       </c>
       <c r="J39" t="n">
-        <v>10.01578703703704</v>
+        <v>10.44561139028476</v>
       </c>
       <c r="K39" t="n">
-        <v>8.864166666666668</v>
+        <v>8.924722222222222</v>
       </c>
       <c r="L39" t="n">
-        <v>396.2326923076923</v>
+        <v>379.7951423785595</v>
       </c>
       <c r="M39" t="n">
-        <v>469.525</v>
+        <v>297.2166666666666</v>
       </c>
       <c r="N39" t="n">
-        <v>6.603878205128205</v>
+        <v>6.329919039642657</v>
       </c>
       <c r="O39" t="n">
-        <v>7.825416666666667</v>
+        <v>4.953611111111111</v>
       </c>
     </row>
     <row r="40">
@@ -6376,40 +6436,40 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2665</v>
+        <v>7091</v>
       </c>
       <c r="D40" t="n">
-        <v>25.32980612883052</v>
+        <v>25.77965026089409</v>
       </c>
       <c r="E40" t="n">
-        <v>2.55</v>
+        <v>2.566666666666667</v>
       </c>
       <c r="F40" t="n">
-        <v>0.4221634354805087</v>
+        <v>0.4296608376815682</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0425</v>
+        <v>0.04277777777777778</v>
       </c>
       <c r="H40" t="n">
-        <v>40.81043697205978</v>
+        <v>40.47532175032175</v>
       </c>
       <c r="I40" t="n">
-        <v>2.866666666666667</v>
+        <v>2.9</v>
       </c>
       <c r="J40" t="n">
-        <v>0.6801739495343296</v>
+        <v>0.6745886958386959</v>
       </c>
       <c r="K40" t="n">
-        <v>0.04777777777777778</v>
+        <v>0.04833333333333333</v>
       </c>
       <c r="L40" t="n">
-        <v>8.767357050032489</v>
+        <v>8.916959166959169</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.1461226175005415</v>
+        <v>0.1486159861159861</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -6427,43 +6487,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>776</v>
+        <v>2130</v>
       </c>
       <c r="D41" t="n">
-        <v>593.5414518900344</v>
+        <v>541.180297339593</v>
       </c>
       <c r="E41" t="n">
-        <v>667.2</v>
+        <v>355.0583333333333</v>
       </c>
       <c r="F41" t="n">
-        <v>9.892357531500574</v>
+        <v>9.019671622326552</v>
       </c>
       <c r="G41" t="n">
-        <v>11.12</v>
+        <v>5.917638888888889</v>
       </c>
       <c r="H41" t="n">
-        <v>664.4059082892416</v>
+        <v>599.6213436194149</v>
       </c>
       <c r="I41" t="n">
-        <v>712.5916666666667</v>
+        <v>441.55</v>
       </c>
       <c r="J41" t="n">
-        <v>11.07343180482069</v>
+        <v>9.993689060323584</v>
       </c>
       <c r="K41" t="n">
-        <v>11.87652777777778</v>
+        <v>7.359166666666667</v>
       </c>
       <c r="L41" t="n">
-        <v>69.37429453262786</v>
+        <v>56.12655094824815</v>
       </c>
       <c r="M41" t="n">
-        <v>54.60833333333333</v>
+        <v>49.58333333333334</v>
       </c>
       <c r="N41" t="n">
-        <v>1.156238242210464</v>
+        <v>0.9354425158041357</v>
       </c>
       <c r="O41" t="n">
-        <v>0.9101388888888888</v>
+        <v>0.826388888888889</v>
       </c>
     </row>
     <row r="42">
@@ -6478,43 +6538,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>5213</v>
+        <v>16240</v>
       </c>
       <c r="D42" t="n">
-        <v>2.504706183259799</v>
+        <v>2.520657840722496</v>
       </c>
       <c r="E42" t="n">
         <v>2.616666666666667</v>
       </c>
       <c r="F42" t="n">
-        <v>0.04174510305432998</v>
+        <v>0.04201096401204159</v>
       </c>
       <c r="G42" t="n">
         <v>0.04361111111111111</v>
       </c>
       <c r="H42" t="n">
-        <v>202.9883456334564</v>
+        <v>304.2713635570186</v>
       </c>
       <c r="I42" t="n">
-        <v>127.1083333333333</v>
+        <v>155.4666666666667</v>
       </c>
       <c r="J42" t="n">
-        <v>3.383139093890939</v>
+        <v>5.071189392616975</v>
       </c>
       <c r="K42" t="n">
-        <v>2.118472222222223</v>
+        <v>2.591111111111111</v>
       </c>
       <c r="L42" t="n">
-        <v>200.3730671235284</v>
+        <v>301.6504039799506</v>
       </c>
       <c r="M42" t="n">
-        <v>124.425</v>
+        <v>152.7833333333333</v>
       </c>
       <c r="N42" t="n">
-        <v>3.339551118725473</v>
+        <v>5.027506732999177</v>
       </c>
       <c r="O42" t="n">
-        <v>2.07375</v>
+        <v>2.546388888888889</v>
       </c>
     </row>
     <row r="43">
@@ -6529,43 +6589,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2895</v>
+        <v>8499</v>
       </c>
       <c r="D43" t="n">
-        <v>206.4872654001151</v>
+        <v>183.9063615327293</v>
       </c>
       <c r="E43" t="n">
-        <v>102.6</v>
+        <v>94.81666666666666</v>
       </c>
       <c r="F43" t="n">
-        <v>3.441454423335253</v>
+        <v>3.065106025545489</v>
       </c>
       <c r="G43" t="n">
-        <v>1.71</v>
+        <v>1.580277777777778</v>
       </c>
       <c r="H43" t="n">
-        <v>327.6762283640425</v>
+        <v>401.2816377599448</v>
       </c>
       <c r="I43" t="n">
-        <v>211.8583333333333</v>
+        <v>234.75</v>
       </c>
       <c r="J43" t="n">
-        <v>5.461270472734041</v>
+        <v>6.688027295999079</v>
       </c>
       <c r="K43" t="n">
-        <v>3.530972222222222</v>
+        <v>3.9125</v>
       </c>
       <c r="L43" t="n">
-        <v>137.781365159129</v>
+        <v>224.0738998187937</v>
       </c>
       <c r="M43" t="n">
-        <v>86.02500000000001</v>
+        <v>106.8833333333333</v>
       </c>
       <c r="N43" t="n">
-        <v>2.296356085985483</v>
+        <v>3.734564996979895</v>
       </c>
       <c r="O43" t="n">
-        <v>1.43375</v>
+        <v>1.781388888888889</v>
       </c>
     </row>
     <row r="44">
@@ -6580,43 +6640,43 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>918</v>
+        <v>2708</v>
       </c>
       <c r="D44" t="n">
-        <v>2.180319535221496</v>
+        <v>2.301550960118169</v>
       </c>
       <c r="E44" t="n">
-        <v>2.516666666666667</v>
+        <v>2.55</v>
       </c>
       <c r="F44" t="n">
-        <v>0.03633865892035826</v>
+        <v>0.03835918266863614</v>
       </c>
       <c r="G44" t="n">
-        <v>0.04194444444444444</v>
+        <v>0.0425</v>
       </c>
       <c r="H44" t="n">
-        <v>571.8012582781456</v>
+        <v>623.2935766111823</v>
       </c>
       <c r="I44" t="n">
-        <v>538.9</v>
+        <v>638.5166666666667</v>
       </c>
       <c r="J44" t="n">
-        <v>9.530020971302429</v>
+        <v>10.38822627685304</v>
       </c>
       <c r="K44" t="n">
-        <v>8.981666666666666</v>
+        <v>10.64194444444444</v>
       </c>
       <c r="L44" t="n">
-        <v>569.202825607064</v>
+        <v>620.6899061032865</v>
       </c>
       <c r="M44" t="n">
-        <v>535.9</v>
+        <v>636.1333333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>9.486713760117734</v>
+        <v>10.34483176838811</v>
       </c>
       <c r="O44" t="n">
-        <v>8.931666666666667</v>
+        <v>10.60222222222222</v>
       </c>
     </row>
     <row r="45">
@@ -6631,43 +6691,43 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1106</v>
+        <v>3108</v>
       </c>
       <c r="D45" t="n">
-        <v>335.2304098854732</v>
+        <v>266.4696374946375</v>
       </c>
       <c r="E45" t="n">
-        <v>205.1333333333333</v>
+        <v>62.18333333333334</v>
       </c>
       <c r="F45" t="n">
-        <v>5.58717349809122</v>
+        <v>4.441160624910625</v>
       </c>
       <c r="G45" t="n">
-        <v>3.418888888888889</v>
+        <v>1.036388888888889</v>
       </c>
       <c r="H45" t="n">
-        <v>891.7515023474178</v>
+        <v>768.6591913806509</v>
       </c>
       <c r="I45" t="n">
-        <v>781.2166666666667</v>
+        <v>756.6166666666667</v>
       </c>
       <c r="J45" t="n">
-        <v>14.86252503912363</v>
+        <v>12.81098652301085</v>
       </c>
       <c r="K45" t="n">
-        <v>13.02027777777778</v>
+        <v>12.61027777777778</v>
       </c>
       <c r="L45" t="n">
-        <v>560.297323943662</v>
+        <v>503.5153004554038</v>
       </c>
       <c r="M45" t="n">
-        <v>607.5333333333333</v>
+        <v>459.1333333333333</v>
       </c>
       <c r="N45" t="n">
-        <v>9.338288732394366</v>
+        <v>8.391921674256729</v>
       </c>
       <c r="O45" t="n">
-        <v>10.12555555555556</v>
+        <v>7.652222222222222</v>
       </c>
     </row>
     <row r="46">
@@ -6682,43 +6742,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>42</v>
+        <v>229</v>
       </c>
       <c r="D46" t="n">
-        <v>0.7186507936507938</v>
+        <v>1.828311499272198</v>
       </c>
       <c r="E46" t="n">
-        <v>0</v>
+        <v>2.433333333333333</v>
       </c>
       <c r="F46" t="n">
-        <v>0.01197751322751323</v>
+        <v>0.0304718583212033</v>
       </c>
       <c r="G46" t="n">
-        <v>0</v>
+        <v>0.04055555555555555</v>
       </c>
       <c r="H46" t="n">
-        <v>43.25</v>
+        <v>2286.81326754386</v>
       </c>
       <c r="I46" t="n">
-        <v>29.85833333333333</v>
+        <v>2410.116666666667</v>
       </c>
       <c r="J46" t="n">
-        <v>0.7208333333333333</v>
+        <v>38.11355445906432</v>
       </c>
       <c r="K46" t="n">
-        <v>0.4976388888888889</v>
+        <v>40.16861111111111</v>
       </c>
       <c r="L46" t="n">
-        <v>40.6875</v>
+        <v>2284.205372807017</v>
       </c>
       <c r="M46" t="n">
-        <v>27.38333333333333</v>
+        <v>2407.791666666667</v>
       </c>
       <c r="N46" t="n">
-        <v>0.678125</v>
+        <v>38.07008954678363</v>
       </c>
       <c r="O46" t="n">
-        <v>0.4563888888888888</v>
+        <v>40.12986111111111</v>
       </c>
     </row>
     <row r="47">
@@ -6733,43 +6793,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>17</v>
+        <v>203</v>
       </c>
       <c r="D47" t="n">
-        <v>145.7098039215686</v>
+        <v>378.3878489326765</v>
       </c>
       <c r="E47" t="n">
-        <v>28.53333333333333</v>
+        <v>327.9333333333333</v>
       </c>
       <c r="F47" t="n">
-        <v>2.428496732026144</v>
+        <v>6.306464148877943</v>
       </c>
       <c r="G47" t="n">
-        <v>0.4755555555555556</v>
+        <v>5.465555555555556</v>
       </c>
       <c r="H47" t="n">
-        <v>237.4409090909091</v>
+        <v>2301.548395721925</v>
       </c>
       <c r="I47" t="n">
-        <v>146.15</v>
+        <v>2545.85</v>
       </c>
       <c r="J47" t="n">
-        <v>3.957348484848485</v>
+        <v>38.35913992869875</v>
       </c>
       <c r="K47" t="n">
-        <v>2.435833333333334</v>
+        <v>42.43083333333333</v>
       </c>
       <c r="L47" t="n">
-        <v>125.7</v>
+        <v>1911.210071301248</v>
       </c>
       <c r="M47" t="n">
-        <v>128.7833333333333</v>
+        <v>1856.466666666667</v>
       </c>
       <c r="N47" t="n">
-        <v>2.095</v>
+        <v>31.85350118835413</v>
       </c>
       <c r="O47" t="n">
-        <v>2.146388888888889</v>
+        <v>30.94111111111111</v>
       </c>
     </row>
     <row r="48">
@@ -6784,43 +6844,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>289</v>
+        <v>1027</v>
       </c>
       <c r="D48" t="n">
-        <v>2.315051903114187</v>
+        <v>2.400227198961376</v>
       </c>
       <c r="E48" t="n">
-        <v>2.533333333333333</v>
+        <v>2.6</v>
       </c>
       <c r="F48" t="n">
-        <v>0.03858419838523645</v>
+        <v>0.04000378664935628</v>
       </c>
       <c r="G48" t="n">
-        <v>0.04222222222222222</v>
+        <v>0.04333333333333333</v>
       </c>
       <c r="H48" t="n">
-        <v>398.7149019607843</v>
+        <v>387.2921736036997</v>
       </c>
       <c r="I48" t="n">
-        <v>359.4333333333333</v>
+        <v>302.75</v>
       </c>
       <c r="J48" t="n">
-        <v>6.645248366013072</v>
+        <v>6.454869560061662</v>
       </c>
       <c r="K48" t="n">
-        <v>5.990555555555556</v>
+        <v>5.045833333333333</v>
       </c>
       <c r="L48" t="n">
-        <v>396.1299346405229</v>
+        <v>384.6745464247599</v>
       </c>
       <c r="M48" t="n">
-        <v>356.5</v>
+        <v>299.9333333333333</v>
       </c>
       <c r="N48" t="n">
-        <v>6.602165577342048</v>
+        <v>6.411242440412664</v>
       </c>
       <c r="O48" t="n">
-        <v>5.941666666666666</v>
+        <v>4.998888888888889</v>
       </c>
     </row>
     <row r="49">
@@ -6835,43 +6895,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>134</v>
+        <v>495</v>
       </c>
       <c r="D49" t="n">
-        <v>177.9324626865672</v>
+        <v>230.5010101010101</v>
       </c>
       <c r="E49" t="n">
-        <v>70.04166666666667</v>
+        <v>71.36666666666666</v>
       </c>
       <c r="F49" t="n">
-        <v>2.965541044776119</v>
+        <v>3.841683501683502</v>
       </c>
       <c r="G49" t="n">
-        <v>1.167361111111111</v>
+        <v>1.189444444444444</v>
       </c>
       <c r="H49" t="n">
-        <v>496.6455128205127</v>
+        <v>621.4152173913044</v>
       </c>
       <c r="I49" t="n">
-        <v>419.325</v>
+        <v>529.5833333333334</v>
       </c>
       <c r="J49" t="n">
-        <v>8.277425213675215</v>
+        <v>10.35692028985507</v>
       </c>
       <c r="K49" t="n">
-        <v>6.98875</v>
+        <v>8.826388888888889</v>
       </c>
       <c r="L49" t="n">
-        <v>320.381282051282</v>
+        <v>391.1469289164942</v>
       </c>
       <c r="M49" t="n">
-        <v>316.825</v>
+        <v>253.0166666666667</v>
       </c>
       <c r="N49" t="n">
-        <v>5.339688034188034</v>
+        <v>6.519115481941569</v>
       </c>
       <c r="O49" t="n">
-        <v>5.280416666666667</v>
+        <v>4.216944444444445</v>
       </c>
     </row>
   </sheetData>
@@ -7005,19 +7065,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>457</v>
+        <v>479</v>
       </c>
       <c r="C6" t="n">
         <v>89</v>
       </c>
       <c r="D6" t="n">
-        <v>19.47483588621444</v>
+        <v>18.580375782881</v>
       </c>
       <c r="E6" t="n">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="F6" t="n">
-        <v>63.45733041575492</v>
+        <v>62.42171189979123</v>
       </c>
     </row>
     <row r="7">
@@ -7071,19 +7131,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24906</v>
+        <v>24907</v>
       </c>
       <c r="C9" t="n">
         <v>11083</v>
       </c>
       <c r="D9" t="n">
-        <v>44.49931743355015</v>
+        <v>44.49753081463042</v>
       </c>
       <c r="E9" t="n">
-        <v>16034</v>
+        <v>16035</v>
       </c>
       <c r="F9" t="n">
-        <v>64.37806151128243</v>
+        <v>64.37949170915806</v>
       </c>
     </row>
     <row r="10">
@@ -7115,19 +7175,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2668</v>
+        <v>2877</v>
       </c>
       <c r="C11" t="n">
-        <v>1888</v>
+        <v>2097</v>
       </c>
       <c r="D11" t="n">
-        <v>70.76461769115441</v>
+        <v>72.88842544316996</v>
       </c>
       <c r="E11" t="n">
-        <v>2046</v>
+        <v>2255</v>
       </c>
       <c r="F11" t="n">
-        <v>76.68665667166417</v>
+        <v>78.380257212374</v>
       </c>
     </row>
     <row r="12">
@@ -7159,19 +7219,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>71097</v>
+        <v>71099</v>
       </c>
       <c r="C13" t="n">
         <v>55749</v>
       </c>
       <c r="D13" t="n">
-        <v>78.41259124857589</v>
+        <v>78.41038551878367</v>
       </c>
       <c r="E13" t="n">
-        <v>58247</v>
+        <v>58248</v>
       </c>
       <c r="F13" t="n">
-        <v>81.92610096065937</v>
+        <v>81.92520288611654</v>
       </c>
     </row>
     <row r="14">
@@ -7181,19 +7241,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>200009</v>
+        <v>200042</v>
       </c>
       <c r="C14" t="n">
-        <v>124556</v>
+        <v>124575</v>
       </c>
       <c r="D14" t="n">
-        <v>62.27519761610728</v>
+        <v>62.27442237130203</v>
       </c>
       <c r="E14" t="n">
-        <v>158696</v>
+        <v>158720</v>
       </c>
       <c r="F14" t="n">
-        <v>79.34442950067246</v>
+        <v>79.3433378990412</v>
       </c>
     </row>
     <row r="15">
@@ -7225,19 +7285,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4118</v>
+        <v>4414</v>
       </c>
       <c r="C16" t="n">
-        <v>2003</v>
+        <v>2151</v>
       </c>
       <c r="D16" t="n">
-        <v>48.64011656143759</v>
+        <v>48.7313094698686</v>
       </c>
       <c r="E16" t="n">
-        <v>2964</v>
+        <v>3180</v>
       </c>
       <c r="F16" t="n">
-        <v>71.97668771248179</v>
+        <v>72.04349796103308</v>
       </c>
     </row>
     <row r="17">
@@ -7247,19 +7307,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13328</v>
+        <v>13344</v>
       </c>
       <c r="C17" t="n">
-        <v>9300</v>
+        <v>9305</v>
       </c>
       <c r="D17" t="n">
-        <v>69.77791116446579</v>
+        <v>69.73171462829735</v>
       </c>
       <c r="E17" t="n">
-        <v>10456</v>
+        <v>10466</v>
       </c>
       <c r="F17" t="n">
-        <v>78.45138055222088</v>
+        <v>78.43225419664267</v>
       </c>
     </row>
     <row r="18"/>
@@ -7477,19 +7537,19 @@
         <v>0.03791666666666667</v>
       </c>
       <c r="H24" t="n">
-        <v>170.3943775100401</v>
+        <v>170.3943775100402</v>
       </c>
       <c r="I24" t="n">
         <v>20.31666666666667</v>
       </c>
       <c r="J24" t="n">
-        <v>2.839906291834003</v>
+        <v>2.839906291834002</v>
       </c>
       <c r="K24" t="n">
         <v>0.3386111111111111</v>
       </c>
       <c r="L24" t="n">
-        <v>167.6485943775101</v>
+        <v>167.64859437751</v>
       </c>
       <c r="M24" t="n">
         <v>17.4</v>
@@ -7516,7 +7576,7 @@
         <v>431</v>
       </c>
       <c r="D25" t="n">
-        <v>291.1989945862335</v>
+        <v>291.1989945862336</v>
       </c>
       <c r="E25" t="n">
         <v>16.76666666666667</v>
@@ -7534,7 +7594,7 @@
         <v>22.78333333333333</v>
       </c>
       <c r="J25" t="n">
-        <v>4.982369242779079</v>
+        <v>4.982369242779078</v>
       </c>
       <c r="K25" t="n">
         <v>0.3797222222222222</v>
@@ -7591,43 +7651,43 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>368</v>
+        <v>390</v>
       </c>
       <c r="D27" t="n">
-        <v>680.657472826087</v>
+        <v>649.0805982905982</v>
       </c>
       <c r="E27" t="n">
-        <v>162.8</v>
+        <v>152.0916666666667</v>
       </c>
       <c r="F27" t="n">
-        <v>11.34429121376811</v>
+        <v>10.81800997150997</v>
       </c>
       <c r="G27" t="n">
-        <v>2.713333333333333</v>
+        <v>2.534861111111111</v>
       </c>
       <c r="H27" t="n">
-        <v>4311.782998084292</v>
+        <v>4228.452747747748</v>
       </c>
       <c r="I27" t="n">
-        <v>3150.391666666666</v>
+        <v>2994.808333333333</v>
       </c>
       <c r="J27" t="n">
-        <v>71.86304996807152</v>
+        <v>70.47421246246246</v>
       </c>
       <c r="K27" t="n">
-        <v>52.50652777777778</v>
+        <v>49.91347222222222</v>
       </c>
       <c r="L27" t="n">
-        <v>3599.365900383142</v>
+        <v>3551.207792792793</v>
       </c>
       <c r="M27" t="n">
-        <v>2760.925</v>
+        <v>2759.225</v>
       </c>
       <c r="N27" t="n">
-        <v>59.98943167305237</v>
+        <v>59.18679654654655</v>
       </c>
       <c r="O27" t="n">
-        <v>46.01541666666667</v>
+        <v>45.98708333333334</v>
       </c>
     </row>
     <row r="28">
@@ -7696,7 +7756,7 @@
         <v>880</v>
       </c>
       <c r="D29" t="n">
-        <v>624.1741856060607</v>
+        <v>624.1741856060606</v>
       </c>
       <c r="E29" t="n">
         <v>232.2833333333333</v>
@@ -7759,7 +7819,7 @@
         <v>0.0425</v>
       </c>
       <c r="H30" t="n">
-        <v>424.7645747755972</v>
+        <v>424.7645747755971</v>
       </c>
       <c r="I30" t="n">
         <v>301.9416666666667</v>
@@ -7810,7 +7870,7 @@
         <v>23.05652777777778</v>
       </c>
       <c r="H31" t="n">
-        <v>1959.900728277248</v>
+        <v>1959.900728277247</v>
       </c>
       <c r="I31" t="n">
         <v>1544.433333333333</v>
@@ -7861,28 +7921,28 @@
         <v>0.04694444444444445</v>
       </c>
       <c r="H32" t="n">
-        <v>647.007467644027</v>
+        <v>649.6601713021251</v>
       </c>
       <c r="I32" t="n">
-        <v>394.9166666666667</v>
+        <v>396.35</v>
       </c>
       <c r="J32" t="n">
-        <v>10.78345779406712</v>
+        <v>10.82766952170208</v>
       </c>
       <c r="K32" t="n">
-        <v>6.581944444444445</v>
+        <v>6.605833333333334</v>
       </c>
       <c r="L32" t="n">
-        <v>253.3266273431833</v>
+        <v>256.2472625996718</v>
       </c>
       <c r="M32" t="n">
-        <v>71.26666666666667</v>
+        <v>71.61666666666666</v>
       </c>
       <c r="N32" t="n">
-        <v>4.222110455719721</v>
+        <v>4.270787709994532</v>
       </c>
       <c r="O32" t="n">
-        <v>1.187777777777778</v>
+        <v>1.193611111111111</v>
       </c>
     </row>
     <row r="33">
@@ -7897,40 +7957,40 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>13823</v>
+        <v>13824</v>
       </c>
       <c r="D33" t="n">
-        <v>400.0687031276375</v>
+        <v>400.0459768036265</v>
       </c>
       <c r="E33" t="n">
-        <v>72.03333333333333</v>
+        <v>72.04166666666666</v>
       </c>
       <c r="F33" t="n">
-        <v>6.667811718793959</v>
+        <v>6.667432946727109</v>
       </c>
       <c r="G33" t="n">
-        <v>1.200555555555556</v>
+        <v>1.200694444444444</v>
       </c>
       <c r="H33" t="n">
-        <v>679.4091485015384</v>
+        <v>681.4709586563308</v>
       </c>
       <c r="I33" t="n">
-        <v>360.5833333333333</v>
+        <v>361.4583333333334</v>
       </c>
       <c r="J33" t="n">
-        <v>11.32348580835898</v>
+        <v>11.35784931093885</v>
       </c>
       <c r="K33" t="n">
-        <v>6.009722222222222</v>
+        <v>6.024305555555555</v>
       </c>
       <c r="L33" t="n">
-        <v>260.4465027280015</v>
+        <v>262.6570322997416</v>
       </c>
       <c r="M33" t="n">
         <v>69.5</v>
       </c>
       <c r="N33" t="n">
-        <v>4.340775045466692</v>
+        <v>4.377617204995694</v>
       </c>
       <c r="O33" t="n">
         <v>1.158333333333333</v>
@@ -8014,28 +8074,28 @@
         <v>22.27416666666667</v>
       </c>
       <c r="H35" t="n">
-        <v>2236.593251786696</v>
+        <v>2241.141305540318</v>
       </c>
       <c r="I35" t="n">
-        <v>1948.075</v>
+        <v>1954.65</v>
       </c>
       <c r="J35" t="n">
-        <v>37.27655419644493</v>
+        <v>37.35235509233863</v>
       </c>
       <c r="K35" t="n">
-        <v>32.46791666666667</v>
+        <v>32.5775</v>
       </c>
       <c r="L35" t="n">
-        <v>553.8581592450064</v>
+        <v>561.6724766867801</v>
       </c>
       <c r="M35" t="n">
-        <v>478.2166666666666</v>
+        <v>478.25</v>
       </c>
       <c r="N35" t="n">
-        <v>9.230969320750106</v>
+        <v>9.361207944779666</v>
       </c>
       <c r="O35" t="n">
-        <v>7.970277777777778</v>
+        <v>7.970833333333333</v>
       </c>
     </row>
     <row r="36">
@@ -8050,43 +8110,43 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1888</v>
+        <v>2097</v>
       </c>
       <c r="D36" t="n">
-        <v>11.11486581920904</v>
+        <v>10.27350182800827</v>
       </c>
       <c r="E36" t="n">
-        <v>2.4</v>
+        <v>2.516666666666667</v>
       </c>
       <c r="F36" t="n">
-        <v>0.185247763653484</v>
+        <v>0.1712250304668044</v>
       </c>
       <c r="G36" t="n">
-        <v>0.04</v>
+        <v>0.04194444444444444</v>
       </c>
       <c r="H36" t="n">
-        <v>2929.286748027613</v>
+        <v>3204.765762857758</v>
       </c>
       <c r="I36" t="n">
-        <v>2632.05</v>
+        <v>2857</v>
       </c>
       <c r="J36" t="n">
-        <v>48.82144580046022</v>
+        <v>53.41276271429596</v>
       </c>
       <c r="K36" t="n">
-        <v>43.8675</v>
+        <v>47.61666666666667</v>
       </c>
       <c r="L36" t="n">
-        <v>2914.533407297831</v>
+        <v>3191.5261889391</v>
       </c>
       <c r="M36" t="n">
-        <v>2620.45</v>
+        <v>2848.65</v>
       </c>
       <c r="N36" t="n">
-        <v>48.57555678829718</v>
+        <v>53.19210314898501</v>
       </c>
       <c r="O36" t="n">
-        <v>43.67416666666666</v>
+        <v>47.4775</v>
       </c>
     </row>
     <row r="37">
@@ -8155,7 +8215,7 @@
         <v>906</v>
       </c>
       <c r="D38" t="n">
-        <v>1.246192052980132</v>
+        <v>1.246192052980133</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
@@ -8167,7 +8227,7 @@
         <v>0</v>
       </c>
       <c r="H38" t="n">
-        <v>457.8752023546726</v>
+        <v>457.8752023546725</v>
       </c>
       <c r="I38" t="n">
         <v>400.1833333333333</v>
@@ -8185,7 +8245,7 @@
         <v>397.9666666666666</v>
       </c>
       <c r="N38" t="n">
-        <v>7.590093205788569</v>
+        <v>7.590093205788571</v>
       </c>
       <c r="O38" t="n">
         <v>6.632777777777777</v>
@@ -8218,7 +8278,7 @@
         <v>1.83375</v>
       </c>
       <c r="H39" t="n">
-        <v>602.7895047833426</v>
+        <v>602.7895047833429</v>
       </c>
       <c r="I39" t="n">
         <v>595.3</v>
@@ -8257,37 +8317,37 @@
         <v>55749</v>
       </c>
       <c r="D40" t="n">
-        <v>88.35809252183897</v>
+        <v>88.35809252183896</v>
       </c>
       <c r="E40" t="n">
         <v>2.483333333333333</v>
       </c>
       <c r="F40" t="n">
-        <v>1.472634875363983</v>
+        <v>1.472634875363982</v>
       </c>
       <c r="G40" t="n">
         <v>0.04138888888888889</v>
       </c>
       <c r="H40" t="n">
-        <v>141.3187099098262</v>
+        <v>141.4860005267765</v>
       </c>
       <c r="I40" t="n">
         <v>3.183333333333333</v>
       </c>
       <c r="J40" t="n">
-        <v>2.355311831830436</v>
+        <v>2.358100008779609</v>
       </c>
       <c r="K40" t="n">
         <v>0.05305555555555555</v>
       </c>
       <c r="L40" t="n">
-        <v>28.50747187877661</v>
+        <v>28.67731491164873</v>
       </c>
       <c r="M40" t="n">
         <v>0.2333333333333333</v>
       </c>
       <c r="N40" t="n">
-        <v>0.4751245313129435</v>
+        <v>0.4779552485274789</v>
       </c>
       <c r="O40" t="n">
         <v>0.003888888888888889</v>
@@ -8305,43 +8365,43 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>15348</v>
+        <v>15350</v>
       </c>
       <c r="D41" t="n">
-        <v>754.0881960733212</v>
+        <v>754.0832160694897</v>
       </c>
       <c r="E41" t="n">
         <v>631.3</v>
       </c>
       <c r="F41" t="n">
-        <v>12.56813660122202</v>
+        <v>12.56805360115816</v>
       </c>
       <c r="G41" t="n">
         <v>10.52166666666667</v>
       </c>
       <c r="H41" t="n">
-        <v>833.3736499637877</v>
+        <v>833.5321112544412</v>
       </c>
       <c r="I41" t="n">
-        <v>714.8</v>
+        <v>714.9166666666666</v>
       </c>
       <c r="J41" t="n">
-        <v>13.8895608327298</v>
+        <v>13.89220185424069</v>
       </c>
       <c r="K41" t="n">
-        <v>11.91333333333333</v>
+        <v>11.91527777777778</v>
       </c>
       <c r="L41" t="n">
-        <v>76.32962384573601</v>
+        <v>76.53031434584832</v>
       </c>
       <c r="M41" t="n">
-        <v>61.325</v>
+        <v>61.33333333333334</v>
       </c>
       <c r="N41" t="n">
-        <v>1.272160397428933</v>
+        <v>1.275505239097472</v>
       </c>
       <c r="O41" t="n">
-        <v>1.022083333333333</v>
+        <v>1.022222222222222</v>
       </c>
     </row>
     <row r="42">
@@ -8356,43 +8416,43 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>124556</v>
+        <v>124575</v>
       </c>
       <c r="D42" t="n">
-        <v>10.84058923964589</v>
+        <v>10.83935152853034</v>
       </c>
       <c r="E42" t="n">
         <v>2.733333333333333</v>
       </c>
       <c r="F42" t="n">
-        <v>0.1806764873274315</v>
+        <v>0.1806558588088389</v>
       </c>
       <c r="G42" t="n">
         <v>0.04555555555555556</v>
       </c>
       <c r="H42" t="n">
-        <v>472.3386509467931</v>
+        <v>473.7804100609663</v>
       </c>
       <c r="I42" t="n">
-        <v>171.8166666666667</v>
+        <v>171.975</v>
       </c>
       <c r="J42" t="n">
-        <v>7.872310849113219</v>
+        <v>7.89634016768277</v>
       </c>
       <c r="K42" t="n">
-        <v>2.863611111111111</v>
+        <v>2.86625</v>
       </c>
       <c r="L42" t="n">
-        <v>460.8076949827506</v>
+        <v>462.2537391801857</v>
       </c>
       <c r="M42" t="n">
-        <v>160.85</v>
+        <v>161.0333333333333</v>
       </c>
       <c r="N42" t="n">
-        <v>7.680128249712509</v>
+        <v>7.704228986336428</v>
       </c>
       <c r="O42" t="n">
-        <v>2.680833333333333</v>
+        <v>2.683888888888889</v>
       </c>
     </row>
     <row r="43">
@@ -8407,43 +8467,43 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>75453</v>
+        <v>75467</v>
       </c>
       <c r="D43" t="n">
-        <v>158.4405384809087</v>
+        <v>158.428003630726</v>
       </c>
       <c r="E43" t="n">
         <v>85.73333333333333</v>
       </c>
       <c r="F43" t="n">
-        <v>2.640675641348477</v>
+        <v>2.640466727178767</v>
       </c>
       <c r="G43" t="n">
         <v>1.428888888888889</v>
       </c>
       <c r="H43" t="n">
-        <v>546.1492319809115</v>
+        <v>547.4915743186276</v>
       </c>
       <c r="I43" t="n">
-        <v>235.9416666666667</v>
+        <v>236.3166666666667</v>
       </c>
       <c r="J43" t="n">
-        <v>9.102487199681857</v>
+        <v>9.124859571977124</v>
       </c>
       <c r="K43" t="n">
-        <v>3.932361111111111</v>
+        <v>3.938611111111111</v>
       </c>
       <c r="L43" t="n">
-        <v>389.1404997250416</v>
+        <v>390.5085330519804</v>
       </c>
       <c r="M43" t="n">
-        <v>112.7333333333333</v>
+        <v>112.8666666666667</v>
       </c>
       <c r="N43" t="n">
-        <v>6.485674995417361</v>
+        <v>6.50847555086634</v>
       </c>
       <c r="O43" t="n">
-        <v>1.878888888888889</v>
+        <v>1.881111111111111</v>
       </c>
     </row>
     <row r="44">
@@ -8461,7 +8521,7 @@
         <v>16594</v>
       </c>
       <c r="D44" t="n">
-        <v>7.318905427664618</v>
+        <v>7.318905427664617</v>
       </c>
       <c r="E44" t="n">
         <v>2.45</v>
@@ -8485,7 +8545,7 @@
         <v>14.22333333333333</v>
       </c>
       <c r="L44" t="n">
-        <v>829.2039527708556</v>
+        <v>829.2039527708555</v>
       </c>
       <c r="M44" t="n">
         <v>844.2166666666667</v>
@@ -8560,43 +8620,43 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2003</v>
+        <v>2151</v>
       </c>
       <c r="D46" t="n">
-        <v>9.174912631053418</v>
+        <v>8.765798853246551</v>
       </c>
       <c r="E46" t="n">
-        <v>2.433333333333333</v>
+        <v>2.483333333333333</v>
       </c>
       <c r="F46" t="n">
-        <v>0.152915210517557</v>
+        <v>0.1460966475541092</v>
       </c>
       <c r="G46" t="n">
-        <v>0.04055555555555555</v>
+        <v>0.04138888888888889</v>
       </c>
       <c r="H46" t="n">
-        <v>3320.401501305483</v>
+        <v>3297.18157842554</v>
       </c>
       <c r="I46" t="n">
-        <v>2954.375</v>
+        <v>2941.383333333333</v>
       </c>
       <c r="J46" t="n">
-        <v>55.34002502175805</v>
+        <v>54.95302630709234</v>
       </c>
       <c r="K46" t="n">
-        <v>49.23958333333333</v>
+        <v>49.02305555555555</v>
       </c>
       <c r="L46" t="n">
-        <v>3308.746910356832</v>
+        <v>3286.274043228237</v>
       </c>
       <c r="M46" t="n">
-        <v>2950.708333333333</v>
+        <v>2929.416666666667</v>
       </c>
       <c r="N46" t="n">
-        <v>55.14578183928054</v>
+        <v>54.77123405380395</v>
       </c>
       <c r="O46" t="n">
-        <v>49.17847222222223</v>
+        <v>48.82361111111111</v>
       </c>
     </row>
     <row r="47">
@@ -8611,43 +8671,43 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2115</v>
+        <v>2263</v>
       </c>
       <c r="D47" t="n">
-        <v>253.1741922773838</v>
+        <v>251.5135955221682</v>
       </c>
       <c r="E47" t="n">
-        <v>76.18333333333334</v>
+        <v>77.01666666666667</v>
       </c>
       <c r="F47" t="n">
-        <v>4.219569871289729</v>
+        <v>4.191893258702803</v>
       </c>
       <c r="G47" t="n">
-        <v>1.269722222222222</v>
+        <v>1.283611111111111</v>
       </c>
       <c r="H47" t="n">
-        <v>3299.089833005894</v>
+        <v>3293.311111111111</v>
       </c>
       <c r="I47" t="n">
-        <v>2956.458333333333</v>
+        <v>2972.85</v>
       </c>
       <c r="J47" t="n">
-        <v>54.98483055009823</v>
+        <v>54.88851851851852</v>
       </c>
       <c r="K47" t="n">
-        <v>49.27430555555556</v>
+        <v>49.5475</v>
       </c>
       <c r="L47" t="n">
-        <v>3044.33881794368</v>
+        <v>3040.387614468864</v>
       </c>
       <c r="M47" t="n">
-        <v>2888.425</v>
+        <v>2878.908333333333</v>
       </c>
       <c r="N47" t="n">
-        <v>50.73898029906134</v>
+        <v>50.67312690781441</v>
       </c>
       <c r="O47" t="n">
-        <v>48.14041666666667</v>
+        <v>47.98180555555555</v>
       </c>
     </row>
     <row r="48">
@@ -8662,43 +8722,43 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>9300</v>
+        <v>9305</v>
       </c>
       <c r="D48" t="n">
-        <v>10.60408422939068</v>
+        <v>10.59985312555973</v>
       </c>
       <c r="E48" t="n">
         <v>2.583333333333333</v>
       </c>
       <c r="F48" t="n">
-        <v>0.1767347371565114</v>
+        <v>0.1766642187593289</v>
       </c>
       <c r="G48" t="n">
         <v>0.04305555555555556</v>
       </c>
       <c r="H48" t="n">
-        <v>416.414008817902</v>
+        <v>418.1481793241052</v>
       </c>
       <c r="I48" t="n">
-        <v>317.1</v>
+        <v>317.4333333333333</v>
       </c>
       <c r="J48" t="n">
-        <v>6.940233480298367</v>
+        <v>6.969136322068421</v>
       </c>
       <c r="K48" t="n">
-        <v>5.285</v>
+        <v>5.290555555555556</v>
       </c>
       <c r="L48" t="n">
-        <v>404.2452707761417</v>
+        <v>405.9853265161908</v>
       </c>
       <c r="M48" t="n">
-        <v>303.05</v>
+        <v>303.2666666666667</v>
       </c>
       <c r="N48" t="n">
-        <v>6.737421179602363</v>
+        <v>6.766422108603179</v>
       </c>
       <c r="O48" t="n">
-        <v>5.050833333333333</v>
+        <v>5.054444444444444</v>
       </c>
     </row>
     <row r="49">
@@ -8713,43 +8773,43 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>4028</v>
+        <v>4039</v>
       </c>
       <c r="D49" t="n">
-        <v>334.8714208871235</v>
+        <v>335.4764380622266</v>
       </c>
       <c r="E49" t="n">
-        <v>156.8833333333333</v>
+        <v>157.0666666666667</v>
       </c>
       <c r="F49" t="n">
-        <v>5.581190348118724</v>
+        <v>5.591273967703777</v>
       </c>
       <c r="G49" t="n">
-        <v>2.614722222222222</v>
+        <v>2.617777777777778</v>
       </c>
       <c r="H49" t="n">
-        <v>803.9068919146074</v>
+        <v>812.6870505406085</v>
       </c>
       <c r="I49" t="n">
-        <v>667.4083333333333</v>
+        <v>668.7</v>
       </c>
       <c r="J49" t="n">
-        <v>13.39844819857679</v>
+        <v>13.54478417567681</v>
       </c>
       <c r="K49" t="n">
-        <v>11.12347222222222</v>
+        <v>11.145</v>
       </c>
       <c r="L49" t="n">
-        <v>468.1192721465793</v>
+        <v>476.2875157153634</v>
       </c>
       <c r="M49" t="n">
-        <v>321.325</v>
+        <v>326.4</v>
       </c>
       <c r="N49" t="n">
-        <v>7.801987869109654</v>
+        <v>7.938125261922722</v>
       </c>
       <c r="O49" t="n">
-        <v>5.355416666666667</v>
+        <v>5.44</v>
       </c>
     </row>
   </sheetData>
@@ -9310,13 +9370,13 @@
         <v>85.81666666666666</v>
       </c>
       <c r="J23" t="n">
-        <v>4.180780165727814</v>
+        <v>4.180780165727815</v>
       </c>
       <c r="K23" t="n">
         <v>1.430277777777778</v>
       </c>
       <c r="L23" t="n">
-        <v>13.79189780798433</v>
+        <v>13.79189780798432</v>
       </c>
       <c r="M23" t="n">
         <v>6.066666666666666</v>
@@ -9649,7 +9709,7 @@
         <v>3.915416666666666</v>
       </c>
       <c r="L30" t="n">
-        <v>378.6940673253775</v>
+        <v>378.6940673253774</v>
       </c>
       <c r="M30" t="n">
         <v>206.7</v>
@@ -9688,7 +9748,7 @@
         <v>21.33138888888889</v>
       </c>
       <c r="H31" t="n">
-        <v>1957.352044979763</v>
+        <v>1957.352044979762</v>
       </c>
       <c r="I31" t="n">
         <v>1507.958333333333</v>
@@ -9733,13 +9793,13 @@
         <v>35.31666666666667</v>
       </c>
       <c r="F32" t="n">
-        <v>5.370218737264492</v>
+        <v>5.370218737264491</v>
       </c>
       <c r="G32" t="n">
         <v>0.5886111111111112</v>
       </c>
       <c r="H32" t="n">
-        <v>656.6801168186909</v>
+        <v>656.680116818691</v>
       </c>
       <c r="I32" t="n">
         <v>408.3583333333333</v>
@@ -9808,7 +9868,7 @@
         <v>62.79166666666666</v>
       </c>
       <c r="N33" t="n">
-        <v>4.5091769412465</v>
+        <v>4.509176941246501</v>
       </c>
       <c r="O33" t="n">
         <v>1.046527777777778</v>
@@ -10135,7 +10195,7 @@
         <v>59921</v>
       </c>
       <c r="D40" t="n">
-        <v>490.567163153708</v>
+        <v>490.5671631537079</v>
       </c>
       <c r="E40" t="n">
         <v>45</v>
@@ -10147,7 +10207,7 @@
         <v>0.75</v>
       </c>
       <c r="H40" t="n">
-        <v>611.0832309299897</v>
+        <v>611.0832309299894</v>
       </c>
       <c r="I40" t="n">
         <v>200.3333333333333</v>
@@ -10159,7 +10219,7 @@
         <v>3.338888888888889</v>
       </c>
       <c r="L40" t="n">
-        <v>90.37999164054335</v>
+        <v>90.37999164054337</v>
       </c>
       <c r="M40" t="n">
         <v>48.58333333333334</v>
@@ -10186,7 +10246,7 @@
         <v>28623</v>
       </c>
       <c r="D41" t="n">
-        <v>830.8317151707832</v>
+        <v>830.8317151707834</v>
       </c>
       <c r="E41" t="n">
         <v>725.4666666666667</v>
@@ -10198,19 +10258,19 @@
         <v>12.09111111111111</v>
       </c>
       <c r="H41" t="n">
-        <v>946.3680715032921</v>
+        <v>946.3680715032922</v>
       </c>
       <c r="I41" t="n">
         <v>848.5166666666667</v>
       </c>
       <c r="J41" t="n">
-        <v>15.77280119172153</v>
+        <v>15.77280119172154</v>
       </c>
       <c r="K41" t="n">
         <v>14.14194444444444</v>
       </c>
       <c r="L41" t="n">
-        <v>108.6917365085226</v>
+        <v>108.6917365085225</v>
       </c>
       <c r="M41" t="n">
         <v>86.96666666666667</v>
@@ -10267,7 +10327,7 @@
         <v>172.8833333333333</v>
       </c>
       <c r="N42" t="n">
-        <v>7.362103963711153</v>
+        <v>7.362103963711149</v>
       </c>
       <c r="O42" t="n">
         <v>2.881388888888889</v>
@@ -10288,25 +10348,25 @@
         <v>137804</v>
       </c>
       <c r="D43" t="n">
-        <v>156.9309387487542</v>
+        <v>156.9309387487543</v>
       </c>
       <c r="E43" t="n">
         <v>88.96666666666667</v>
       </c>
       <c r="F43" t="n">
-        <v>2.615515645812572</v>
+        <v>2.615515645812571</v>
       </c>
       <c r="G43" t="n">
         <v>1.482777777777778</v>
       </c>
       <c r="H43" t="n">
-        <v>556.2643231660055</v>
+        <v>556.2643231660056</v>
       </c>
       <c r="I43" t="n">
         <v>263.475</v>
       </c>
       <c r="J43" t="n">
-        <v>9.271072052766758</v>
+        <v>9.27107205276676</v>
       </c>
       <c r="K43" t="n">
         <v>4.391249999999999</v>
@@ -10402,7 +10462,7 @@
         <v>0.4711111111111111</v>
       </c>
       <c r="H45" t="n">
-        <v>1102.18878353756</v>
+        <v>1102.188783537559</v>
       </c>
       <c r="I45" t="n">
         <v>937.7666666666667</v>
@@ -10414,7 +10474,7 @@
         <v>15.62944444444444</v>
       </c>
       <c r="L45" t="n">
-        <v>833.926264000069</v>
+        <v>833.9262640000692</v>
       </c>
       <c r="M45" t="n">
         <v>562.0333333333333</v>
@@ -10549,7 +10609,7 @@
         <v>35.15</v>
       </c>
       <c r="F48" t="n">
-        <v>0.4245496921723835</v>
+        <v>0.4245496921723834</v>
       </c>
       <c r="G48" t="n">
         <v>0.5858333333333333</v>
@@ -10561,7 +10621,7 @@
         <v>340.05</v>
       </c>
       <c r="J48" t="n">
-        <v>6.611753065674087</v>
+        <v>6.611753065674088</v>
       </c>
       <c r="K48" t="n">
         <v>5.6675</v>
@@ -11176,7 +11236,7 @@
         <v>116.6333333333333</v>
       </c>
       <c r="F23" t="n">
-        <v>5.534719646761214</v>
+        <v>5.534719646761215</v>
       </c>
       <c r="G23" t="n">
         <v>1.943888888888889</v>
@@ -11200,7 +11260,7 @@
         <v>6.316666666666666</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2447684015348261</v>
+        <v>0.244768401534826</v>
       </c>
       <c r="O23" t="n">
         <v>0.1052777777777778</v>
@@ -11509,7 +11569,7 @@
         <v>14.4</v>
       </c>
       <c r="F30" t="n">
-        <v>0.1870989473684211</v>
+        <v>0.187098947368421</v>
       </c>
       <c r="G30" t="n">
         <v>0.24</v>
@@ -11554,7 +11614,7 @@
         <v>12127</v>
       </c>
       <c r="D31" t="n">
-        <v>1803.942101646464</v>
+        <v>1803.942101646463</v>
       </c>
       <c r="E31" t="n">
         <v>1345.6</v>
@@ -11605,13 +11665,13 @@
         <v>13128</v>
       </c>
       <c r="D32" t="n">
-        <v>299.5310430631728</v>
+        <v>299.5310430631729</v>
       </c>
       <c r="E32" t="n">
         <v>14.45</v>
       </c>
       <c r="F32" t="n">
-        <v>4.992184051052881</v>
+        <v>4.992184051052882</v>
       </c>
       <c r="G32" t="n">
         <v>0.2408333333333333</v>
@@ -11629,7 +11689,7 @@
         <v>5.139861111111111</v>
       </c>
       <c r="L32" t="n">
-        <v>252.900874159462</v>
+        <v>252.9008741594621</v>
       </c>
       <c r="M32" t="n">
         <v>73.27500000000001</v>
@@ -11662,7 +11722,7 @@
         <v>137.3583333333333</v>
       </c>
       <c r="F33" t="n">
-        <v>7.00585628066947</v>
+        <v>7.005856280669471</v>
       </c>
       <c r="G33" t="n">
         <v>2.289305555555555</v>
@@ -12019,7 +12079,7 @@
         <v>68.75</v>
       </c>
       <c r="F40" t="n">
-        <v>8.080344958994358</v>
+        <v>8.080344958994356</v>
       </c>
       <c r="G40" t="n">
         <v>1.145833333333333</v>
@@ -12064,7 +12124,7 @@
         <v>25046</v>
       </c>
       <c r="D41" t="n">
-        <v>874.0449313263595</v>
+        <v>874.0449313263596</v>
       </c>
       <c r="E41" t="n">
         <v>769.3833333333333</v>
@@ -12127,25 +12187,25 @@
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>473.0165184347057</v>
+        <v>473.0165184347056</v>
       </c>
       <c r="I42" t="n">
         <v>172.05</v>
       </c>
       <c r="J42" t="n">
-        <v>7.883608640578425</v>
+        <v>7.883608640578426</v>
       </c>
       <c r="K42" t="n">
         <v>2.8675</v>
       </c>
       <c r="L42" t="n">
-        <v>473.0165184347057</v>
+        <v>473.0165184347056</v>
       </c>
       <c r="M42" t="n">
         <v>172.05</v>
       </c>
       <c r="N42" t="n">
-        <v>7.883608640578425</v>
+        <v>7.883608640578426</v>
       </c>
       <c r="O42" t="n">
         <v>2.8675</v>
@@ -12190,7 +12250,7 @@
         <v>4.594722222222222</v>
       </c>
       <c r="L43" t="n">
-        <v>470.612362582121</v>
+        <v>470.6123625821211</v>
       </c>
       <c r="M43" t="n">
         <v>123.7666666666667</v>
@@ -12235,13 +12295,13 @@
         <v>3118.85</v>
       </c>
       <c r="J44" t="n">
-        <v>53.04485702683022</v>
+        <v>53.04485702683023</v>
       </c>
       <c r="K44" t="n">
         <v>51.98083333333334</v>
       </c>
       <c r="L44" t="n">
-        <v>3171.043867977371</v>
+        <v>3171.04386797737</v>
       </c>
       <c r="M44" t="n">
         <v>3104.783333333333</v>
@@ -12274,13 +12334,13 @@
         <v>151.4583333333333</v>
       </c>
       <c r="F45" t="n">
-        <v>6.228881899070625</v>
+        <v>6.228881899070624</v>
       </c>
       <c r="G45" t="n">
         <v>2.524305555555555</v>
       </c>
       <c r="H45" t="n">
-        <v>3263.452867733505</v>
+        <v>3263.452867733504</v>
       </c>
       <c r="I45" t="n">
         <v>2515.583333333333</v>
@@ -13048,13 +13108,13 @@
         <v>9120</v>
       </c>
       <c r="D23" t="n">
-        <v>242.2425109649123</v>
+        <v>242.2425109649122</v>
       </c>
       <c r="E23" t="n">
         <v>71.48333333333333</v>
       </c>
       <c r="F23" t="n">
-        <v>4.037375182748539</v>
+        <v>4.037375182748538</v>
       </c>
       <c r="G23" t="n">
         <v>1.191388888888889</v>
@@ -13072,13 +13132,13 @@
         <v>1.475555555555556</v>
       </c>
       <c r="L23" t="n">
-        <v>16.65544133617945</v>
+        <v>16.65544133617946</v>
       </c>
       <c r="M23" t="n">
         <v>7.116666666666666</v>
       </c>
       <c r="N23" t="n">
-        <v>0.2775906889363243</v>
+        <v>0.2775906889363242</v>
       </c>
       <c r="O23" t="n">
         <v>0.1186111111111111</v>
@@ -13387,7 +13447,7 @@
         <v>2.183333333333333</v>
       </c>
       <c r="F30" t="n">
-        <v>0.6050886833757764</v>
+        <v>0.6050886833757763</v>
       </c>
       <c r="G30" t="n">
         <v>0.03638888888888889</v>
@@ -13411,7 +13471,7 @@
         <v>245.0833333333333</v>
       </c>
       <c r="N30" t="n">
-        <v>6.494622005589888</v>
+        <v>6.494622005589886</v>
       </c>
       <c r="O30" t="n">
         <v>4.084722222222222</v>
@@ -13495,7 +13555,7 @@
         <v>0.03861111111111112</v>
       </c>
       <c r="H32" t="n">
-        <v>702.4301408339267</v>
+        <v>702.4301408339268</v>
       </c>
       <c r="I32" t="n">
         <v>321.7</v>
@@ -13534,7 +13594,7 @@
         <v>15278</v>
       </c>
       <c r="D33" t="n">
-        <v>455.5605456647903</v>
+        <v>455.5605456647904</v>
       </c>
       <c r="E33" t="n">
         <v>111.9583333333333</v>
@@ -13879,7 +13939,7 @@
         <v>0.8127777777777778</v>
       </c>
       <c r="H40" t="n">
-        <v>693.4443901040598</v>
+        <v>693.4443901040597</v>
       </c>
       <c r="I40" t="n">
         <v>233.0166666666667</v>
@@ -13930,7 +13990,7 @@
         <v>10.39527777777778</v>
       </c>
       <c r="H41" t="n">
-        <v>891.433795162278</v>
+        <v>891.4337951622779</v>
       </c>
       <c r="I41" t="n">
         <v>752.8416666666667</v>
@@ -13948,7 +14008,7 @@
         <v>86.74166666666667</v>
       </c>
       <c r="N41" t="n">
-        <v>2.355245288154046</v>
+        <v>2.355245288154045</v>
       </c>
       <c r="O41" t="n">
         <v>1.445694444444444</v>
@@ -14020,7 +14080,7 @@
         <v>92767</v>
       </c>
       <c r="D43" t="n">
-        <v>162.3702329492169</v>
+        <v>162.3702329492168</v>
       </c>
       <c r="E43" t="n">
         <v>92.01666666666667</v>
@@ -14032,7 +14092,7 @@
         <v>1.533611111111111</v>
       </c>
       <c r="H43" t="n">
-        <v>622.608807824149</v>
+        <v>622.6088078241489</v>
       </c>
       <c r="I43" t="n">
         <v>255.1166666666667</v>
@@ -14050,7 +14110,7 @@
         <v>115.9</v>
       </c>
       <c r="N43" t="n">
-        <v>7.663797610921932</v>
+        <v>7.663797610921931</v>
       </c>
       <c r="O43" t="n">
         <v>1.931666666666667</v>
@@ -14122,7 +14182,7 @@
         <v>44395</v>
       </c>
       <c r="D45" t="n">
-        <v>258.6143529676765</v>
+        <v>258.6143529676766</v>
       </c>
       <c r="E45" t="n">
         <v>51.98333333333333</v>
@@ -14146,7 +14206,7 @@
         <v>17.42361111111111</v>
       </c>
       <c r="L45" t="n">
-        <v>929.04475961316</v>
+        <v>929.0447596131598</v>
       </c>
       <c r="M45" t="n">
         <v>545.4333333333334</v>
@@ -15265,7 +15325,7 @@
         <v>333.6166666666667</v>
       </c>
       <c r="N30" t="n">
-        <v>6.648160798856225</v>
+        <v>6.648160798856223</v>
       </c>
       <c r="O30" t="n">
         <v>5.560277777777778</v>
@@ -15388,7 +15448,7 @@
         <v>18478</v>
       </c>
       <c r="D33" t="n">
-        <v>340.8348802179168</v>
+        <v>340.8348802179167</v>
       </c>
       <c r="E33" t="n">
         <v>128.475</v>
@@ -15412,7 +15472,7 @@
         <v>5.245138888888889</v>
       </c>
       <c r="L33" t="n">
-        <v>293.6192615402325</v>
+        <v>293.6192615402326</v>
       </c>
       <c r="M33" t="n">
         <v>65.18333333333334</v>
@@ -15739,7 +15799,7 @@
         <v>99.67500000000001</v>
       </c>
       <c r="N40" t="n">
-        <v>2.767195660374124</v>
+        <v>2.767195660374123</v>
       </c>
       <c r="O40" t="n">
         <v>1.66125</v>
@@ -15760,7 +15820,7 @@
         <v>33976</v>
       </c>
       <c r="D41" t="n">
-        <v>645.5681392747821</v>
+        <v>645.5681392747822</v>
       </c>
       <c r="E41" t="n">
         <v>272.0583333333333</v>
@@ -15811,7 +15871,7 @@
         <v>151206</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1708009823243345</v>
+        <v>0.1708009823243346</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
@@ -15886,7 +15946,7 @@
         <v>4.155277777777778</v>
       </c>
       <c r="L43" t="n">
-        <v>462.1773911064036</v>
+        <v>462.1773911064035</v>
       </c>
       <c r="M43" t="n">
         <v>119.8916666666667</v>
@@ -15976,7 +16036,7 @@
         <v>0.5241666666666667</v>
       </c>
       <c r="H45" t="n">
-        <v>858.6822808104105</v>
+        <v>858.6822808104108</v>
       </c>
       <c r="I45" t="n">
         <v>770.175</v>
@@ -15994,7 +16054,7 @@
         <v>395.1333333333333</v>
       </c>
       <c r="N45" t="n">
-        <v>10.65539464567078</v>
+        <v>10.65539464567079</v>
       </c>
       <c r="O45" t="n">
         <v>6.585555555555556</v>
@@ -16129,25 +16189,25 @@
         <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>375.5856337635437</v>
+        <v>375.5856337635436</v>
       </c>
       <c r="I48" t="n">
         <v>278.3416666666667</v>
       </c>
       <c r="J48" t="n">
-        <v>6.259760562725728</v>
+        <v>6.259760562725727</v>
       </c>
       <c r="K48" t="n">
         <v>4.639027777777779</v>
       </c>
       <c r="L48" t="n">
-        <v>375.5856337635437</v>
+        <v>375.5856337635436</v>
       </c>
       <c r="M48" t="n">
         <v>278.3416666666667</v>
       </c>
       <c r="N48" t="n">
-        <v>6.259760562725728</v>
+        <v>6.259760562725727</v>
       </c>
       <c r="O48" t="n">
         <v>4.639027777777779</v>
@@ -16744,13 +16804,13 @@
         <v>10097</v>
       </c>
       <c r="D23" t="n">
-        <v>244.2034102538708</v>
+        <v>244.2034102538707</v>
       </c>
       <c r="E23" t="n">
         <v>68.55</v>
       </c>
       <c r="F23" t="n">
-        <v>4.070056837564514</v>
+        <v>4.070056837564513</v>
       </c>
       <c r="G23" t="n">
         <v>1.1425</v>
@@ -17077,25 +17137,25 @@
         <v>0.07305555555555557</v>
       </c>
       <c r="H30" t="n">
-        <v>333.3020398542416</v>
+        <v>333.3020398542415</v>
       </c>
       <c r="I30" t="n">
         <v>126.2</v>
       </c>
       <c r="J30" t="n">
-        <v>5.555033997570693</v>
+        <v>5.555033997570691</v>
       </c>
       <c r="K30" t="n">
         <v>2.103333333333333</v>
       </c>
       <c r="L30" t="n">
-        <v>328.4209120097851</v>
+        <v>328.4209120097852</v>
       </c>
       <c r="M30" t="n">
         <v>118.2666666666667</v>
       </c>
       <c r="N30" t="n">
-        <v>5.473681866829753</v>
+        <v>5.473681866829754</v>
       </c>
       <c r="O30" t="n">
         <v>1.971111111111111</v>
@@ -17197,7 +17257,7 @@
         <v>88.06666666666666</v>
       </c>
       <c r="N32" t="n">
-        <v>4.306319206076786</v>
+        <v>4.306319206076785</v>
       </c>
       <c r="O32" t="n">
         <v>1.467777777777778</v>
@@ -17539,7 +17599,7 @@
         <v>62166</v>
       </c>
       <c r="D40" t="n">
-        <v>517.3971066713852</v>
+        <v>517.3971066713851</v>
       </c>
       <c r="E40" t="n">
         <v>66.15000000000001</v>
@@ -17590,7 +17650,7 @@
         <v>25056</v>
       </c>
       <c r="D41" t="n">
-        <v>849.7250093124735</v>
+        <v>849.7250093124734</v>
       </c>
       <c r="E41" t="n">
         <v>759.0416666666667</v>
@@ -17614,7 +17674,7 @@
         <v>15.26166666666667</v>
       </c>
       <c r="L41" t="n">
-        <v>178.3548424435548</v>
+        <v>178.3548424435547</v>
       </c>
       <c r="M41" t="n">
         <v>77.95</v>
@@ -17716,7 +17776,7 @@
         <v>4.4375</v>
       </c>
       <c r="L43" t="n">
-        <v>453.3391468153862</v>
+        <v>453.3391468153861</v>
       </c>
       <c r="M43" t="n">
         <v>128.2583333333333</v>
@@ -17755,7 +17815,7 @@
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>873.4327828001856</v>
+        <v>873.4327828001855</v>
       </c>
       <c r="I44" t="n">
         <v>711.9833333333333</v>
@@ -17767,7 +17827,7 @@
         <v>11.86638888888889</v>
       </c>
       <c r="L44" t="n">
-        <v>873.4327828001856</v>
+        <v>873.4327828001855</v>
       </c>
       <c r="M44" t="n">
         <v>711.9833333333333</v>
@@ -17800,13 +17860,13 @@
         <v>28.96666666666667</v>
       </c>
       <c r="F45" t="n">
-        <v>3.527821013618819</v>
+        <v>3.52782101361882</v>
       </c>
       <c r="G45" t="n">
         <v>0.4827777777777778</v>
       </c>
       <c r="H45" t="n">
-        <v>867.5344391512265</v>
+        <v>867.5344391512264</v>
       </c>
       <c r="I45" t="n">
         <v>690.5333333333333</v>
@@ -18580,7 +18640,7 @@
         <v>74.71666666666667</v>
       </c>
       <c r="F23" t="n">
-        <v>4.290628479236812</v>
+        <v>4.290628479236813</v>
       </c>
       <c r="G23" t="n">
         <v>1.245277777777778</v>
@@ -18919,7 +18979,7 @@
         <v>7.781944444444445</v>
       </c>
       <c r="L30" t="n">
-        <v>647.5108654876741</v>
+        <v>647.5108654876742</v>
       </c>
       <c r="M30" t="n">
         <v>465.075</v>
@@ -19003,13 +19063,13 @@
         <v>1.733333333333333</v>
       </c>
       <c r="F32" t="n">
-        <v>5.236490125300804</v>
+        <v>5.236490125300805</v>
       </c>
       <c r="G32" t="n">
         <v>0.02888888888888889</v>
       </c>
       <c r="H32" t="n">
-        <v>711.8602964237904</v>
+        <v>711.8602964237903</v>
       </c>
       <c r="I32" t="n">
         <v>253.9333333333333</v>
@@ -19027,7 +19087,7 @@
         <v>112.5833333333333</v>
       </c>
       <c r="N32" t="n">
-        <v>5.475285586791611</v>
+        <v>5.475285586791612</v>
       </c>
       <c r="O32" t="n">
         <v>1.876388888888889</v>
@@ -19420,7 +19480,7 @@
         <v>21879</v>
       </c>
       <c r="D41" t="n">
-        <v>832.7047122811828</v>
+        <v>832.704712281183</v>
       </c>
       <c r="E41" t="n">
         <v>745.4166666666666</v>
@@ -19528,13 +19588,13 @@
         <v>92.43333333333334</v>
       </c>
       <c r="F43" t="n">
-        <v>2.573943913160413</v>
+        <v>2.573943913160412</v>
       </c>
       <c r="G43" t="n">
         <v>1.540555555555556</v>
       </c>
       <c r="H43" t="n">
-        <v>645.8540349690377</v>
+        <v>645.8540349690379</v>
       </c>
       <c r="I43" t="n">
         <v>268.6166666666667</v>
@@ -19795,7 +19855,7 @@
         <v>325.7333333333333</v>
       </c>
       <c r="J48" t="n">
-        <v>7.002995345788266</v>
+        <v>7.002995345788265</v>
       </c>
       <c r="K48" t="n">
         <v>5.428888888888889</v>
@@ -19807,7 +19867,7 @@
         <v>325.7333333333333</v>
       </c>
       <c r="N48" t="n">
-        <v>7.002995345788266</v>
+        <v>7.002995345788265</v>
       </c>
       <c r="O48" t="n">
         <v>5.428888888888889</v>

</xml_diff>